<commit_message>
UPDATE: New WS and RS May 2026
</commit_message>
<xml_diff>
--- a/gp-app-1.0/Pricelist Car.xlsx
+++ b/gp-app-1.0/Pricelist Car.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\Work\gp-app\gp-app-1.0\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{3EFE44EB-1462-4830-B9BF-68AC98C79D4F}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{5EDCD83A-DF63-4AEE-A38D-D2CB8BC50D2F}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-110" yWindow="-110" windowWidth="19420" windowHeight="11020" tabRatio="861" xr2:uid="{C4C7316A-D95F-426A-ADF9-AD32FA680374}"/>
   </bookViews>
@@ -2462,7 +2462,7 @@
     <t>520S P2D (4X2) A/T</t>
   </si>
   <si>
-    <t>520S P3D (4X2) A/T</t>
+    <t>520S P2C (4X2) A/T</t>
   </si>
 </sst>
 </file>
@@ -7567,15 +7567,15 @@
       </c>
       <c r="D58" s="9">
         <f t="shared" ref="D58:D65" si="13">I58/1.12</f>
-        <v>20089285.714285716</v>
+        <v>22321428.571428571</v>
       </c>
       <c r="E58" s="9">
         <f t="shared" ref="E58:E65" si="14">D58*90%</f>
-        <v>18080357.142857146</v>
+        <v>20089285.714285713</v>
       </c>
       <c r="F58" s="9">
         <f t="shared" ref="F58:F65" si="15">D58*70%</f>
-        <v>14062500</v>
+        <v>15624999.999999998</v>
       </c>
       <c r="G58" s="21">
         <v>262</v>
@@ -7584,8 +7584,7 @@
         <v>623</v>
       </c>
       <c r="I58" s="19">
-        <f>15625000/7*9*1.12</f>
-        <v>22500000.000000004</v>
+        <v>25000000</v>
       </c>
     </row>
     <row r="59" spans="1:9" x14ac:dyDescent="0.35">
@@ -7600,15 +7599,15 @@
       </c>
       <c r="D59" s="9">
         <f t="shared" si="13"/>
-        <v>28125000</v>
+        <v>31249999.999999996</v>
       </c>
       <c r="E59" s="9">
         <f t="shared" si="14"/>
-        <v>25312500</v>
+        <v>28124999.999999996</v>
       </c>
       <c r="F59" s="9">
         <f t="shared" si="15"/>
-        <v>19687500</v>
+        <v>21874999.999999996</v>
       </c>
       <c r="G59" s="21">
         <v>263</v>
@@ -7617,8 +7616,7 @@
         <v>625</v>
       </c>
       <c r="I59" s="19">
-        <f>21875000/7*9*1.12</f>
-        <v>31500000.000000004</v>
+        <v>35000000</v>
       </c>
     </row>
     <row r="60" spans="1:9" x14ac:dyDescent="0.35">
@@ -7633,15 +7631,15 @@
       </c>
       <c r="D60" s="9">
         <f t="shared" si="13"/>
-        <v>28125000</v>
+        <v>22321428.571428571</v>
       </c>
       <c r="E60" s="9">
         <f t="shared" si="14"/>
-        <v>25312500</v>
+        <v>20089285.714285713</v>
       </c>
       <c r="F60" s="9">
         <f t="shared" si="15"/>
-        <v>19687500</v>
+        <v>15624999.999999998</v>
       </c>
       <c r="G60" s="21">
         <v>264</v>
@@ -7650,8 +7648,7 @@
         <v>624</v>
       </c>
       <c r="I60" s="19">
-        <f>21875000/7*9*1.12</f>
-        <v>31500000.000000004</v>
+        <v>25000000</v>
       </c>
     </row>
     <row r="61" spans="1:9" x14ac:dyDescent="0.35">
@@ -7666,15 +7663,15 @@
       </c>
       <c r="D61" s="9">
         <f t="shared" si="13"/>
-        <v>0</v>
+        <v>31249999.999999996</v>
       </c>
       <c r="E61" s="9">
         <f t="shared" si="14"/>
-        <v>0</v>
+        <v>28124999.999999996</v>
       </c>
       <c r="F61" s="9">
         <f t="shared" si="15"/>
-        <v>0</v>
+        <v>21874999.999999996</v>
       </c>
       <c r="G61" s="21">
         <v>265</v>
@@ -7682,7 +7679,9 @@
       <c r="H61" s="17" t="s">
         <v>626</v>
       </c>
-      <c r="I61" s="19"/>
+      <c r="I61" s="19">
+        <v>35000000</v>
+      </c>
     </row>
     <row r="62" spans="1:9" x14ac:dyDescent="0.35">
       <c r="A62" s="16" t="s">
@@ -7696,15 +7695,15 @@
       </c>
       <c r="D62" s="9">
         <f t="shared" si="13"/>
-        <v>20089285.714285716</v>
+        <v>22321428.571428571</v>
       </c>
       <c r="E62" s="9">
         <f t="shared" si="14"/>
-        <v>18080357.142857146</v>
+        <v>20089285.714285713</v>
       </c>
       <c r="F62" s="9">
         <f t="shared" si="15"/>
-        <v>14062500</v>
+        <v>15624999.999999998</v>
       </c>
       <c r="G62" s="21">
         <v>262</v>
@@ -7713,8 +7712,7 @@
         <v>623</v>
       </c>
       <c r="I62" s="19">
-        <f>15625000/7*9*1.12</f>
-        <v>22500000.000000004</v>
+        <v>25000000</v>
       </c>
     </row>
     <row r="63" spans="1:9" x14ac:dyDescent="0.35">
@@ -7729,15 +7727,15 @@
       </c>
       <c r="D63" s="9">
         <f t="shared" si="13"/>
-        <v>28125000</v>
+        <v>31249999.999999996</v>
       </c>
       <c r="E63" s="9">
         <f t="shared" si="14"/>
-        <v>25312500</v>
+        <v>28124999.999999996</v>
       </c>
       <c r="F63" s="9">
         <f t="shared" si="15"/>
-        <v>19687500</v>
+        <v>21874999.999999996</v>
       </c>
       <c r="G63" s="21">
         <v>263</v>
@@ -7746,13 +7744,12 @@
         <v>625</v>
       </c>
       <c r="I63" s="19">
-        <f>21875000/7*9*1.12</f>
-        <v>31500000.000000004</v>
+        <v>35000000</v>
       </c>
     </row>
     <row r="64" spans="1:9" x14ac:dyDescent="0.35">
       <c r="A64" s="16" t="s">
-        <v>629</v>
+        <v>630</v>
       </c>
       <c r="B64" s="17" t="s">
         <v>624</v>
@@ -7762,15 +7759,15 @@
       </c>
       <c r="D64" s="9">
         <f t="shared" si="13"/>
-        <v>0</v>
+        <v>22321428.571428571</v>
       </c>
       <c r="E64" s="9">
         <f t="shared" si="14"/>
-        <v>0</v>
+        <v>20089285.714285713</v>
       </c>
       <c r="F64" s="9">
         <f t="shared" si="15"/>
-        <v>0</v>
+        <v>15624999.999999998</v>
       </c>
       <c r="G64" s="21">
         <v>264</v>
@@ -7778,11 +7775,13 @@
       <c r="H64" s="17" t="s">
         <v>624</v>
       </c>
-      <c r="I64" s="19"/>
+      <c r="I64" s="19">
+        <v>25000000</v>
+      </c>
     </row>
     <row r="65" spans="1:9" x14ac:dyDescent="0.35">
       <c r="A65" s="16" t="s">
-        <v>630</v>
+        <v>629</v>
       </c>
       <c r="B65" s="17" t="s">
         <v>626</v>
@@ -7792,15 +7791,15 @@
       </c>
       <c r="D65" s="9">
         <f t="shared" si="13"/>
-        <v>28125000</v>
+        <v>31249999.999999996</v>
       </c>
       <c r="E65" s="9">
         <f t="shared" si="14"/>
-        <v>25312500</v>
+        <v>28124999.999999996</v>
       </c>
       <c r="F65" s="9">
         <f t="shared" si="15"/>
-        <v>19687500</v>
+        <v>21874999.999999996</v>
       </c>
       <c r="G65" s="21">
         <v>265</v>
@@ -7809,8 +7808,7 @@
         <v>626</v>
       </c>
       <c r="I65" s="19">
-        <f>21875000/7*9*1.12</f>
-        <v>31500000.000000004</v>
+        <v>35000000</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
UPDATE: New WS and RS June 2026
</commit_message>
<xml_diff>
--- a/gp-app-1.0/Pricelist Car.xlsx
+++ b/gp-app-1.0/Pricelist Car.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\Work\gp-app\gp-app-1.0\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{5EDCD83A-DF63-4AEE-A38D-D2CB8BC50D2F}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{19E6A4A0-AAB1-4428-A3CE-4DB953D4763F}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-110" yWindow="-110" windowWidth="19420" windowHeight="11020" tabRatio="861" xr2:uid="{C4C7316A-D95F-426A-ADF9-AD32FA680374}"/>
   </bookViews>
@@ -490,7 +490,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1408" uniqueCount="631">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1417" uniqueCount="634">
   <si>
     <t>Column1</t>
   </si>
@@ -2463,6 +2463,15 @@
   </si>
   <si>
     <t>520S P2C (4X2) A/T</t>
+  </si>
+  <si>
+    <t>310S I2D1 (4X2) A/T</t>
+  </si>
+  <si>
+    <t>310S I1F1 (4X2) M/T</t>
+  </si>
+  <si>
+    <t>310S I2F1 (4X2) A/T</t>
   </si>
 </sst>
 </file>
@@ -2654,7 +2663,7 @@
     <xf numFmtId="43" fontId="2" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="25">
+  <cellXfs count="28">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="2" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
     <xf numFmtId="3" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
@@ -2696,6 +2705,9 @@
     <xf numFmtId="0" fontId="2" fillId="2" borderId="9" xfId="3" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="9" xfId="0" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="43" fontId="0" fillId="0" borderId="10" xfId="0" applyNumberFormat="1" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="8" xfId="0" applyFill="1" applyBorder="1"/>
   </cellXfs>
   <cellStyles count="4">
     <cellStyle name="Comma" xfId="2" builtinId="3"/>
@@ -2703,7 +2715,17 @@
     <cellStyle name="Normal 2" xfId="1" xr:uid="{DA2601EE-1999-4BF8-AF5E-538A4398209C}"/>
     <cellStyle name="Normal 2 2" xfId="3" xr:uid="{8C240942-BC33-4996-847D-14CFBB46F4A3}"/>
   </cellStyles>
-  <dxfs count="154">
+  <dxfs count="155">
+    <dxf>
+      <font>
+        <color rgb="FF9C0006"/>
+      </font>
+      <fill>
+        <patternFill>
+          <bgColor rgb="FFFFC7CE"/>
+        </patternFill>
+      </fill>
+    </dxf>
     <dxf>
       <font>
         <color rgb="FF9C0006"/>
@@ -5070,21 +5092,21 @@
 </file>
 
 <file path=xl/tables/table1.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="20" xr:uid="{DF067A72-54A6-48F4-972D-2DE4603D61A4}" name="Table20" displayName="Table20" ref="A1:I65" totalsRowShown="0" headerRowDxfId="153" headerRowBorderDxfId="152" tableBorderDxfId="151" totalsRowBorderDxfId="150">
-  <autoFilter ref="A1:I65" xr:uid="{DF067A72-54A6-48F4-972D-2DE4603D61A4}"/>
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="20" xr:uid="{DF067A72-54A6-48F4-972D-2DE4603D61A4}" name="Table20" displayName="Table20" ref="A1:I69" totalsRowShown="0" headerRowDxfId="154" headerRowBorderDxfId="153" tableBorderDxfId="152" totalsRowBorderDxfId="151">
+  <autoFilter ref="A1:I69" xr:uid="{DF067A72-54A6-48F4-972D-2DE4603D61A4}"/>
   <sortState xmlns:xlrd2="http://schemas.microsoft.com/office/spreadsheetml/2017/richdata2" ref="A2:I57">
     <sortCondition ref="H1:H57"/>
   </sortState>
   <tableColumns count="9">
-    <tableColumn id="1" xr3:uid="{0E6335F2-6B6A-436C-92FA-B48E61551308}" name="Merek/Type" dataDxfId="149"/>
-    <tableColumn id="2" xr3:uid="{5A4965DA-398A-4134-90BD-9CE4D8355880}" name="Tipe" dataDxfId="148"/>
-    <tableColumn id="3" xr3:uid="{010303D1-E0A2-4DE6-8E87-64ACC3102E09}" name="Harga OTR Awal" dataDxfId="147" dataCellStyle="Comma"/>
-    <tableColumn id="4" xr3:uid="{91C798B0-7964-436A-84A5-7687993F376F}" name="Dealer Margin" dataDxfId="146" dataCellStyle="Comma"/>
-    <tableColumn id="5" xr3:uid="{CD936623-36F3-4BAA-A615-AF79A61C51E8}" name="Dealer Margin 9 %" dataDxfId="145" dataCellStyle="Comma"/>
-    <tableColumn id="6" xr3:uid="{A36173E8-D9B2-4F38-A572-F5D32CDADEB8}" name="Dealer Margin 7 %" dataDxfId="144" dataCellStyle="Comma"/>
-    <tableColumn id="7" xr3:uid="{7A11B7F5-7683-492A-A8B5-D96984323DDD}" name="Code Unit" dataDxfId="143"/>
-    <tableColumn id="8" xr3:uid="{AF243BB3-2044-4D1E-9F0D-A1EC0D2C15CF}" name="Merk/Type" dataDxfId="142"/>
-    <tableColumn id="9" xr3:uid="{9E0E2E6A-108F-4ACE-959D-9EB0F753BD73}" name="Full Margin" dataDxfId="141"/>
+    <tableColumn id="1" xr3:uid="{0E6335F2-6B6A-436C-92FA-B48E61551308}" name="Merek/Type" dataDxfId="150"/>
+    <tableColumn id="2" xr3:uid="{5A4965DA-398A-4134-90BD-9CE4D8355880}" name="Tipe" dataDxfId="149"/>
+    <tableColumn id="3" xr3:uid="{010303D1-E0A2-4DE6-8E87-64ACC3102E09}" name="Harga OTR Awal" dataDxfId="148" dataCellStyle="Comma"/>
+    <tableColumn id="4" xr3:uid="{91C798B0-7964-436A-84A5-7687993F376F}" name="Dealer Margin" dataDxfId="147" dataCellStyle="Comma"/>
+    <tableColumn id="5" xr3:uid="{CD936623-36F3-4BAA-A615-AF79A61C51E8}" name="Dealer Margin 9 %" dataDxfId="146" dataCellStyle="Comma"/>
+    <tableColumn id="6" xr3:uid="{A36173E8-D9B2-4F38-A572-F5D32CDADEB8}" name="Dealer Margin 7 %" dataDxfId="145" dataCellStyle="Comma"/>
+    <tableColumn id="7" xr3:uid="{7A11B7F5-7683-492A-A8B5-D96984323DDD}" name="Code Unit" dataDxfId="144"/>
+    <tableColumn id="8" xr3:uid="{AF243BB3-2044-4D1E-9F0D-A1EC0D2C15CF}" name="Merk/Type" dataDxfId="143"/>
+    <tableColumn id="9" xr3:uid="{9E0E2E6A-108F-4ACE-959D-9EB0F753BD73}" name="Full Margin" dataDxfId="142"/>
   </tableColumns>
   <tableStyleInfo name="TableStyleMedium2" showFirstColumn="0" showLastColumn="0" showRowStripes="1" showColumnStripes="0"/>
 </table>
@@ -5094,15 +5116,15 @@
 <table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="9" xr:uid="{630D8221-A5B4-4162-BEFC-7BB63825B861}" name="Table009__Page_6" displayName="Table009__Page_6" ref="A1:I16" tableType="queryTable" totalsRowShown="0">
   <autoFilter ref="A1:I16" xr:uid="{630D8221-A5B4-4162-BEFC-7BB63825B861}"/>
   <tableColumns count="9">
-    <tableColumn id="1" xr3:uid="{5980B244-73E4-43AF-B863-305E8B039C33}" uniqueName="1" name="Column1" queryTableFieldId="1" dataDxfId="74"/>
-    <tableColumn id="2" xr3:uid="{549208EE-7E07-4F0F-ACFD-9606CC8F6B50}" uniqueName="2" name="Column2" queryTableFieldId="2" dataDxfId="73"/>
-    <tableColumn id="3" xr3:uid="{086F7B88-A201-47FD-B9A0-0C976108E144}" uniqueName="3" name="Column3" queryTableFieldId="3" dataDxfId="72"/>
-    <tableColumn id="4" xr3:uid="{CC912184-CE02-4DC9-8815-71C4295C86DF}" uniqueName="4" name="Column4" queryTableFieldId="4" dataDxfId="71"/>
-    <tableColumn id="5" xr3:uid="{8F3F2202-7C07-4D43-B483-871C9E242208}" uniqueName="5" name="Column5" queryTableFieldId="5" dataDxfId="70"/>
-    <tableColumn id="6" xr3:uid="{6D2190D6-B434-4BB9-95B1-A29148C453AF}" uniqueName="6" name="Column6" queryTableFieldId="6" dataDxfId="69"/>
-    <tableColumn id="7" xr3:uid="{A33DE0AF-7DA7-4623-87E7-DBA2BF4E404A}" uniqueName="7" name="Column7" queryTableFieldId="7" dataDxfId="68"/>
-    <tableColumn id="8" xr3:uid="{CD689B59-BA44-4F67-9FF9-E08337BE66FD}" uniqueName="8" name="Column8" queryTableFieldId="8" dataDxfId="67"/>
-    <tableColumn id="9" xr3:uid="{744F224A-BA1E-4758-B291-8D5C8D341610}" uniqueName="9" name="Column9" queryTableFieldId="9" dataDxfId="66"/>
+    <tableColumn id="1" xr3:uid="{5980B244-73E4-43AF-B863-305E8B039C33}" uniqueName="1" name="Column1" queryTableFieldId="1" dataDxfId="75"/>
+    <tableColumn id="2" xr3:uid="{549208EE-7E07-4F0F-ACFD-9606CC8F6B50}" uniqueName="2" name="Column2" queryTableFieldId="2" dataDxfId="74"/>
+    <tableColumn id="3" xr3:uid="{086F7B88-A201-47FD-B9A0-0C976108E144}" uniqueName="3" name="Column3" queryTableFieldId="3" dataDxfId="73"/>
+    <tableColumn id="4" xr3:uid="{CC912184-CE02-4DC9-8815-71C4295C86DF}" uniqueName="4" name="Column4" queryTableFieldId="4" dataDxfId="72"/>
+    <tableColumn id="5" xr3:uid="{8F3F2202-7C07-4D43-B483-871C9E242208}" uniqueName="5" name="Column5" queryTableFieldId="5" dataDxfId="71"/>
+    <tableColumn id="6" xr3:uid="{6D2190D6-B434-4BB9-95B1-A29148C453AF}" uniqueName="6" name="Column6" queryTableFieldId="6" dataDxfId="70"/>
+    <tableColumn id="7" xr3:uid="{A33DE0AF-7DA7-4623-87E7-DBA2BF4E404A}" uniqueName="7" name="Column7" queryTableFieldId="7" dataDxfId="69"/>
+    <tableColumn id="8" xr3:uid="{CD689B59-BA44-4F67-9FF9-E08337BE66FD}" uniqueName="8" name="Column8" queryTableFieldId="8" dataDxfId="68"/>
+    <tableColumn id="9" xr3:uid="{744F224A-BA1E-4758-B291-8D5C8D341610}" uniqueName="9" name="Column9" queryTableFieldId="9" dataDxfId="67"/>
   </tableColumns>
   <tableStyleInfo name="TableStyleMedium7" showFirstColumn="0" showLastColumn="0" showRowStripes="1" showColumnStripes="0"/>
 </table>
@@ -5112,15 +5134,15 @@
 <table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="10" xr:uid="{116BBD7B-F856-4C44-8F1F-EA66756E3A0B}" name="Table010__Page_6" displayName="Table010__Page_6" ref="A18:I20" tableType="queryTable" totalsRowShown="0">
   <autoFilter ref="A18:I20" xr:uid="{116BBD7B-F856-4C44-8F1F-EA66756E3A0B}"/>
   <tableColumns count="9">
-    <tableColumn id="1" xr3:uid="{D02866AC-7C8C-4041-B0D6-297717EA2BCA}" uniqueName="1" name="Column1" queryTableFieldId="1" dataDxfId="65"/>
-    <tableColumn id="2" xr3:uid="{F9BA0334-AC0F-4599-91DD-1D3B53530BA2}" uniqueName="2" name="Column2" queryTableFieldId="2" dataDxfId="64"/>
-    <tableColumn id="3" xr3:uid="{2E40CB08-FF90-4211-A5F6-3255AA5CEAED}" uniqueName="3" name="Column3" queryTableFieldId="3" dataDxfId="63"/>
-    <tableColumn id="4" xr3:uid="{951E49DE-3DB8-41C0-8F36-6E5A1649659D}" uniqueName="4" name="Column4" queryTableFieldId="4" dataDxfId="62"/>
-    <tableColumn id="5" xr3:uid="{D7FC7D23-AA29-4FAE-8DF4-B23A11020D8C}" uniqueName="5" name="Column5" queryTableFieldId="5" dataDxfId="61"/>
-    <tableColumn id="6" xr3:uid="{85DA6C7C-BC56-4316-BB56-3D2CA86DF4B0}" uniqueName="6" name="Column6" queryTableFieldId="6" dataDxfId="60"/>
-    <tableColumn id="7" xr3:uid="{47F39228-8CCC-4319-9964-568280350AF4}" uniqueName="7" name="Column7" queryTableFieldId="7" dataDxfId="59"/>
-    <tableColumn id="8" xr3:uid="{781188CD-5AC0-41B9-8575-2EACD4BA90A4}" uniqueName="8" name="Column8" queryTableFieldId="8" dataDxfId="58"/>
-    <tableColumn id="9" xr3:uid="{A2DFBEC8-960F-4613-A8B8-821CF42818AC}" uniqueName="9" name="Column9" queryTableFieldId="9" dataDxfId="57"/>
+    <tableColumn id="1" xr3:uid="{D02866AC-7C8C-4041-B0D6-297717EA2BCA}" uniqueName="1" name="Column1" queryTableFieldId="1" dataDxfId="66"/>
+    <tableColumn id="2" xr3:uid="{F9BA0334-AC0F-4599-91DD-1D3B53530BA2}" uniqueName="2" name="Column2" queryTableFieldId="2" dataDxfId="65"/>
+    <tableColumn id="3" xr3:uid="{2E40CB08-FF90-4211-A5F6-3255AA5CEAED}" uniqueName="3" name="Column3" queryTableFieldId="3" dataDxfId="64"/>
+    <tableColumn id="4" xr3:uid="{951E49DE-3DB8-41C0-8F36-6E5A1649659D}" uniqueName="4" name="Column4" queryTableFieldId="4" dataDxfId="63"/>
+    <tableColumn id="5" xr3:uid="{D7FC7D23-AA29-4FAE-8DF4-B23A11020D8C}" uniqueName="5" name="Column5" queryTableFieldId="5" dataDxfId="62"/>
+    <tableColumn id="6" xr3:uid="{85DA6C7C-BC56-4316-BB56-3D2CA86DF4B0}" uniqueName="6" name="Column6" queryTableFieldId="6" dataDxfId="61"/>
+    <tableColumn id="7" xr3:uid="{47F39228-8CCC-4319-9964-568280350AF4}" uniqueName="7" name="Column7" queryTableFieldId="7" dataDxfId="60"/>
+    <tableColumn id="8" xr3:uid="{781188CD-5AC0-41B9-8575-2EACD4BA90A4}" uniqueName="8" name="Column8" queryTableFieldId="8" dataDxfId="59"/>
+    <tableColumn id="9" xr3:uid="{A2DFBEC8-960F-4613-A8B8-821CF42818AC}" uniqueName="9" name="Column9" queryTableFieldId="9" dataDxfId="58"/>
   </tableColumns>
   <tableStyleInfo name="TableStyleMedium7" showFirstColumn="0" showLastColumn="0" showRowStripes="1" showColumnStripes="0"/>
 </table>
@@ -5130,9 +5152,9 @@
 <table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="11" xr:uid="{D5A80464-2F5E-4F81-BC09-642A89962C82}" name="Table011__Page_7" displayName="Table011__Page_7" ref="A1:C15" tableType="queryTable" totalsRowShown="0">
   <autoFilter ref="A1:C15" xr:uid="{D5A80464-2F5E-4F81-BC09-642A89962C82}"/>
   <tableColumns count="3">
-    <tableColumn id="1" xr3:uid="{384F6B08-E7B1-4ECD-BC7E-1F8C8FC9CD11}" uniqueName="1" name="Column1" queryTableFieldId="1" dataDxfId="56"/>
-    <tableColumn id="2" xr3:uid="{BD116665-54B3-487B-82AD-7E260403FB1A}" uniqueName="2" name="Column2" queryTableFieldId="2" dataDxfId="55"/>
-    <tableColumn id="3" xr3:uid="{A0C72322-3C63-446F-A7B0-E45538411191}" uniqueName="3" name="Column3" queryTableFieldId="3" dataDxfId="54"/>
+    <tableColumn id="1" xr3:uid="{384F6B08-E7B1-4ECD-BC7E-1F8C8FC9CD11}" uniqueName="1" name="Column1" queryTableFieldId="1" dataDxfId="57"/>
+    <tableColumn id="2" xr3:uid="{BD116665-54B3-487B-82AD-7E260403FB1A}" uniqueName="2" name="Column2" queryTableFieldId="2" dataDxfId="56"/>
+    <tableColumn id="3" xr3:uid="{A0C72322-3C63-446F-A7B0-E45538411191}" uniqueName="3" name="Column3" queryTableFieldId="3" dataDxfId="55"/>
   </tableColumns>
   <tableStyleInfo name="TableStyleMedium7" showFirstColumn="0" showLastColumn="0" showRowStripes="1" showColumnStripes="0"/>
 </table>
@@ -5142,9 +5164,9 @@
 <table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="12" xr:uid="{BF5A7D5F-42BD-4927-9517-2459449E72C6}" name="Table012__Page_7" displayName="Table012__Page_7" ref="A17:C19" tableType="queryTable" totalsRowShown="0">
   <autoFilter ref="A17:C19" xr:uid="{BF5A7D5F-42BD-4927-9517-2459449E72C6}"/>
   <tableColumns count="3">
-    <tableColumn id="1" xr3:uid="{92B56AD9-FE6F-4702-B777-811CB1B6E64F}" uniqueName="1" name="Column1" queryTableFieldId="1" dataDxfId="53"/>
-    <tableColumn id="2" xr3:uid="{C37743D7-7886-43A1-BB26-C0F3914426C9}" uniqueName="2" name="Column2" queryTableFieldId="2" dataDxfId="52"/>
-    <tableColumn id="3" xr3:uid="{DFF6BFBF-623A-4318-86AF-C5448FC821A5}" uniqueName="3" name="Column3" queryTableFieldId="3" dataDxfId="51"/>
+    <tableColumn id="1" xr3:uid="{92B56AD9-FE6F-4702-B777-811CB1B6E64F}" uniqueName="1" name="Column1" queryTableFieldId="1" dataDxfId="54"/>
+    <tableColumn id="2" xr3:uid="{C37743D7-7886-43A1-BB26-C0F3914426C9}" uniqueName="2" name="Column2" queryTableFieldId="2" dataDxfId="53"/>
+    <tableColumn id="3" xr3:uid="{DFF6BFBF-623A-4318-86AF-C5448FC821A5}" uniqueName="3" name="Column3" queryTableFieldId="3" dataDxfId="52"/>
   </tableColumns>
   <tableStyleInfo name="TableStyleMedium7" showFirstColumn="0" showLastColumn="0" showRowStripes="1" showColumnStripes="0"/>
 </table>
@@ -5154,11 +5176,11 @@
 <table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="13" xr:uid="{4DAA9679-BE71-4F3A-B608-132984AF6DF1}" name="Table013__Page_8" displayName="Table013__Page_8" ref="A1:E16" tableType="queryTable" totalsRowShown="0">
   <autoFilter ref="A1:E16" xr:uid="{4DAA9679-BE71-4F3A-B608-132984AF6DF1}"/>
   <tableColumns count="5">
-    <tableColumn id="1" xr3:uid="{811DEB23-A3B8-4E1E-AF98-CBD4FE9515C8}" uniqueName="1" name="Column1" queryTableFieldId="1" dataDxfId="50"/>
-    <tableColumn id="2" xr3:uid="{D1233A63-9D37-45F3-9DC7-52977AC06ADC}" uniqueName="2" name="Column2" queryTableFieldId="2" dataDxfId="49"/>
-    <tableColumn id="3" xr3:uid="{400191B1-4CF8-4D78-82E7-FED7CD6730E6}" uniqueName="3" name="Column3" queryTableFieldId="3" dataDxfId="48"/>
-    <tableColumn id="4" xr3:uid="{3D829CC4-4292-4CD0-80B8-3490D4014AC9}" uniqueName="4" name="Column4" queryTableFieldId="4" dataDxfId="47"/>
-    <tableColumn id="5" xr3:uid="{9BC50CF1-EF44-42B4-9129-E887F74428C9}" uniqueName="5" name="Column5" queryTableFieldId="5" dataDxfId="46"/>
+    <tableColumn id="1" xr3:uid="{811DEB23-A3B8-4E1E-AF98-CBD4FE9515C8}" uniqueName="1" name="Column1" queryTableFieldId="1" dataDxfId="51"/>
+    <tableColumn id="2" xr3:uid="{D1233A63-9D37-45F3-9DC7-52977AC06ADC}" uniqueName="2" name="Column2" queryTableFieldId="2" dataDxfId="50"/>
+    <tableColumn id="3" xr3:uid="{400191B1-4CF8-4D78-82E7-FED7CD6730E6}" uniqueName="3" name="Column3" queryTableFieldId="3" dataDxfId="49"/>
+    <tableColumn id="4" xr3:uid="{3D829CC4-4292-4CD0-80B8-3490D4014AC9}" uniqueName="4" name="Column4" queryTableFieldId="4" dataDxfId="48"/>
+    <tableColumn id="5" xr3:uid="{9BC50CF1-EF44-42B4-9129-E887F74428C9}" uniqueName="5" name="Column5" queryTableFieldId="5" dataDxfId="47"/>
   </tableColumns>
   <tableStyleInfo name="TableStyleMedium7" showFirstColumn="0" showLastColumn="0" showRowStripes="1" showColumnStripes="0"/>
 </table>
@@ -5168,11 +5190,11 @@
 <table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="14" xr:uid="{9D3195A8-F1BD-4429-B95A-60FCF241B775}" name="Table014__Page_8" displayName="Table014__Page_8" ref="A18:E21" tableType="queryTable" totalsRowShown="0">
   <autoFilter ref="A18:E21" xr:uid="{9D3195A8-F1BD-4429-B95A-60FCF241B775}"/>
   <tableColumns count="5">
-    <tableColumn id="1" xr3:uid="{98A6121C-2EC1-48CA-8A40-28DAFD66423E}" uniqueName="1" name="Column1" queryTableFieldId="1" dataDxfId="45"/>
-    <tableColumn id="2" xr3:uid="{6B521FB3-E639-4556-B8C5-473A63201BC1}" uniqueName="2" name="Column2" queryTableFieldId="2" dataDxfId="44"/>
-    <tableColumn id="3" xr3:uid="{3D07F9E9-4DA3-41C6-98A7-BC28F0C8BFB5}" uniqueName="3" name="Column3" queryTableFieldId="3" dataDxfId="43"/>
-    <tableColumn id="4" xr3:uid="{89F1E0D5-9B1D-4170-BB1D-3FBA7855FC27}" uniqueName="4" name="Column4" queryTableFieldId="4" dataDxfId="42"/>
-    <tableColumn id="5" xr3:uid="{68E29A0D-4E20-4E2A-A030-157EF3C69E97}" uniqueName="5" name="Column5" queryTableFieldId="5" dataDxfId="41"/>
+    <tableColumn id="1" xr3:uid="{98A6121C-2EC1-48CA-8A40-28DAFD66423E}" uniqueName="1" name="Column1" queryTableFieldId="1" dataDxfId="46"/>
+    <tableColumn id="2" xr3:uid="{6B521FB3-E639-4556-B8C5-473A63201BC1}" uniqueName="2" name="Column2" queryTableFieldId="2" dataDxfId="45"/>
+    <tableColumn id="3" xr3:uid="{3D07F9E9-4DA3-41C6-98A7-BC28F0C8BFB5}" uniqueName="3" name="Column3" queryTableFieldId="3" dataDxfId="44"/>
+    <tableColumn id="4" xr3:uid="{89F1E0D5-9B1D-4170-BB1D-3FBA7855FC27}" uniqueName="4" name="Column4" queryTableFieldId="4" dataDxfId="43"/>
+    <tableColumn id="5" xr3:uid="{68E29A0D-4E20-4E2A-A030-157EF3C69E97}" uniqueName="5" name="Column5" queryTableFieldId="5" dataDxfId="42"/>
   </tableColumns>
   <tableStyleInfo name="TableStyleMedium7" showFirstColumn="0" showLastColumn="0" showRowStripes="1" showColumnStripes="0"/>
 </table>
@@ -5182,12 +5204,12 @@
 <table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="15" xr:uid="{F2B12C92-B774-477F-98C9-509526BBDEE5}" name="Table015__Page_9" displayName="Table015__Page_9" ref="A1:F16" tableType="queryTable" totalsRowShown="0">
   <autoFilter ref="A1:F16" xr:uid="{F2B12C92-B774-477F-98C9-509526BBDEE5}"/>
   <tableColumns count="6">
-    <tableColumn id="1" xr3:uid="{B9D47F1B-922B-4B02-855C-93AF62167342}" uniqueName="1" name="Column1" queryTableFieldId="1" dataDxfId="40"/>
-    <tableColumn id="2" xr3:uid="{9915D8BD-1C99-4D36-BE7E-9EBEAD6D7B12}" uniqueName="2" name="Column2" queryTableFieldId="2" dataDxfId="39"/>
-    <tableColumn id="3" xr3:uid="{D353D58B-6A1D-4079-A9EC-77376B67A375}" uniqueName="3" name="Column3" queryTableFieldId="3" dataDxfId="38"/>
-    <tableColumn id="4" xr3:uid="{ACF53426-7425-4D38-9673-B3197A3F9292}" uniqueName="4" name="Column4" queryTableFieldId="4" dataDxfId="37"/>
-    <tableColumn id="5" xr3:uid="{673A9374-D6DA-46D7-AAD2-6F2220F4ED8C}" uniqueName="5" name="Column5" queryTableFieldId="5" dataDxfId="36"/>
-    <tableColumn id="6" xr3:uid="{37C428F9-0692-44D1-B8CF-2CBC7901020B}" uniqueName="6" name="Column6" queryTableFieldId="6" dataDxfId="35"/>
+    <tableColumn id="1" xr3:uid="{B9D47F1B-922B-4B02-855C-93AF62167342}" uniqueName="1" name="Column1" queryTableFieldId="1" dataDxfId="41"/>
+    <tableColumn id="2" xr3:uid="{9915D8BD-1C99-4D36-BE7E-9EBEAD6D7B12}" uniqueName="2" name="Column2" queryTableFieldId="2" dataDxfId="40"/>
+    <tableColumn id="3" xr3:uid="{D353D58B-6A1D-4079-A9EC-77376B67A375}" uniqueName="3" name="Column3" queryTableFieldId="3" dataDxfId="39"/>
+    <tableColumn id="4" xr3:uid="{ACF53426-7425-4D38-9673-B3197A3F9292}" uniqueName="4" name="Column4" queryTableFieldId="4" dataDxfId="38"/>
+    <tableColumn id="5" xr3:uid="{673A9374-D6DA-46D7-AAD2-6F2220F4ED8C}" uniqueName="5" name="Column5" queryTableFieldId="5" dataDxfId="37"/>
+    <tableColumn id="6" xr3:uid="{37C428F9-0692-44D1-B8CF-2CBC7901020B}" uniqueName="6" name="Column6" queryTableFieldId="6" dataDxfId="36"/>
   </tableColumns>
   <tableStyleInfo name="TableStyleMedium7" showFirstColumn="0" showLastColumn="0" showRowStripes="1" showColumnStripes="0"/>
 </table>
@@ -5197,12 +5219,12 @@
 <table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="16" xr:uid="{3C596C1A-3A31-47DF-B534-2A3593167FFF}" name="Table016__Page_9" displayName="Table016__Page_9" ref="A18:F20" tableType="queryTable" totalsRowShown="0">
   <autoFilter ref="A18:F20" xr:uid="{3C596C1A-3A31-47DF-B534-2A3593167FFF}"/>
   <tableColumns count="6">
-    <tableColumn id="1" xr3:uid="{48EBD4D1-26EB-449F-8D09-DF1A8D9D96A3}" uniqueName="1" name="Column1" queryTableFieldId="1" dataDxfId="34"/>
-    <tableColumn id="2" xr3:uid="{671AE648-452F-44F1-9A65-8468F7B19950}" uniqueName="2" name="Column2" queryTableFieldId="2" dataDxfId="33"/>
-    <tableColumn id="3" xr3:uid="{C3287937-E8A8-4D80-A27C-D2A5C0E44D68}" uniqueName="3" name="Column3" queryTableFieldId="3" dataDxfId="32"/>
-    <tableColumn id="4" xr3:uid="{49CAB777-0355-40CC-9F2D-C41408ED9E98}" uniqueName="4" name="Column4" queryTableFieldId="4" dataDxfId="31"/>
-    <tableColumn id="5" xr3:uid="{A19C49CB-F2CF-4D60-B082-761FE4F0ABC5}" uniqueName="5" name="Column5" queryTableFieldId="5" dataDxfId="30"/>
-    <tableColumn id="6" xr3:uid="{801427E9-2562-451E-AE45-ACF6DAAAFFFB}" uniqueName="6" name="Column6" queryTableFieldId="6" dataDxfId="29"/>
+    <tableColumn id="1" xr3:uid="{48EBD4D1-26EB-449F-8D09-DF1A8D9D96A3}" uniqueName="1" name="Column1" queryTableFieldId="1" dataDxfId="35"/>
+    <tableColumn id="2" xr3:uid="{671AE648-452F-44F1-9A65-8468F7B19950}" uniqueName="2" name="Column2" queryTableFieldId="2" dataDxfId="34"/>
+    <tableColumn id="3" xr3:uid="{C3287937-E8A8-4D80-A27C-D2A5C0E44D68}" uniqueName="3" name="Column3" queryTableFieldId="3" dataDxfId="33"/>
+    <tableColumn id="4" xr3:uid="{49CAB777-0355-40CC-9F2D-C41408ED9E98}" uniqueName="4" name="Column4" queryTableFieldId="4" dataDxfId="32"/>
+    <tableColumn id="5" xr3:uid="{A19C49CB-F2CF-4D60-B082-761FE4F0ABC5}" uniqueName="5" name="Column5" queryTableFieldId="5" dataDxfId="31"/>
+    <tableColumn id="6" xr3:uid="{801427E9-2562-451E-AE45-ACF6DAAAFFFB}" uniqueName="6" name="Column6" queryTableFieldId="6" dataDxfId="30"/>
   </tableColumns>
   <tableStyleInfo name="TableStyleMedium7" showFirstColumn="0" showLastColumn="0" showRowStripes="1" showColumnStripes="0"/>
 </table>
@@ -5212,11 +5234,11 @@
 <table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="17" xr:uid="{510F87AB-8378-4FE2-9EBF-7361BA7DB6B8}" name="Table017__Page_10" displayName="Table017__Page_10" ref="A1:E15" tableType="queryTable" totalsRowShown="0">
   <autoFilter ref="A1:E15" xr:uid="{510F87AB-8378-4FE2-9EBF-7361BA7DB6B8}"/>
   <tableColumns count="5">
-    <tableColumn id="1" xr3:uid="{626476ED-551C-48ED-A0F5-9CB680097EF0}" uniqueName="1" name="Column1" queryTableFieldId="1" dataDxfId="28"/>
-    <tableColumn id="2" xr3:uid="{9215A7DD-9718-48E5-BA20-B6B9989DD0D2}" uniqueName="2" name="Column2" queryTableFieldId="2" dataDxfId="27"/>
-    <tableColumn id="3" xr3:uid="{AE2AC56F-3587-4342-A60B-0B4A30905DD3}" uniqueName="3" name="Column3" queryTableFieldId="3" dataDxfId="26"/>
-    <tableColumn id="4" xr3:uid="{F7BE237D-2C3F-4C27-92EF-2601ABCBA887}" uniqueName="4" name="Column4" queryTableFieldId="4" dataDxfId="25"/>
-    <tableColumn id="5" xr3:uid="{7950C4F9-8FA4-4C6E-B03A-A0235ECC51FF}" uniqueName="5" name="Column5" queryTableFieldId="5" dataDxfId="24"/>
+    <tableColumn id="1" xr3:uid="{626476ED-551C-48ED-A0F5-9CB680097EF0}" uniqueName="1" name="Column1" queryTableFieldId="1" dataDxfId="29"/>
+    <tableColumn id="2" xr3:uid="{9215A7DD-9718-48E5-BA20-B6B9989DD0D2}" uniqueName="2" name="Column2" queryTableFieldId="2" dataDxfId="28"/>
+    <tableColumn id="3" xr3:uid="{AE2AC56F-3587-4342-A60B-0B4A30905DD3}" uniqueName="3" name="Column3" queryTableFieldId="3" dataDxfId="27"/>
+    <tableColumn id="4" xr3:uid="{F7BE237D-2C3F-4C27-92EF-2601ABCBA887}" uniqueName="4" name="Column4" queryTableFieldId="4" dataDxfId="26"/>
+    <tableColumn id="5" xr3:uid="{7950C4F9-8FA4-4C6E-B03A-A0235ECC51FF}" uniqueName="5" name="Column5" queryTableFieldId="5" dataDxfId="25"/>
   </tableColumns>
   <tableStyleInfo name="TableStyleMedium7" showFirstColumn="0" showLastColumn="0" showRowStripes="1" showColumnStripes="0"/>
 </table>
@@ -5226,11 +5248,11 @@
 <table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="18" xr:uid="{14CF879A-74C7-4F0C-8E76-F1430C9579CD}" name="Table018__Page_10" displayName="Table018__Page_10" ref="A17:E19" tableType="queryTable" totalsRowShown="0">
   <autoFilter ref="A17:E19" xr:uid="{14CF879A-74C7-4F0C-8E76-F1430C9579CD}"/>
   <tableColumns count="5">
-    <tableColumn id="1" xr3:uid="{210B1486-2DC9-4D94-98AC-6BEB874B7545}" uniqueName="1" name="Column1" queryTableFieldId="1" dataDxfId="23"/>
-    <tableColumn id="2" xr3:uid="{BB67F395-3AAE-4514-BCCE-DE32693EB37D}" uniqueName="2" name="Column2" queryTableFieldId="2" dataDxfId="22"/>
-    <tableColumn id="3" xr3:uid="{230B22CA-5CA3-4E2D-92CC-C75BC5831FF2}" uniqueName="3" name="Column3" queryTableFieldId="3" dataDxfId="21"/>
-    <tableColumn id="4" xr3:uid="{42788CA6-A70D-442A-9072-79E0D19F0B28}" uniqueName="4" name="Column4" queryTableFieldId="4" dataDxfId="20"/>
-    <tableColumn id="5" xr3:uid="{E37C1038-7442-4E7D-BB43-162AD6FA4195}" uniqueName="5" name="Column5" queryTableFieldId="5" dataDxfId="19"/>
+    <tableColumn id="1" xr3:uid="{210B1486-2DC9-4D94-98AC-6BEB874B7545}" uniqueName="1" name="Column1" queryTableFieldId="1" dataDxfId="24"/>
+    <tableColumn id="2" xr3:uid="{BB67F395-3AAE-4514-BCCE-DE32693EB37D}" uniqueName="2" name="Column2" queryTableFieldId="2" dataDxfId="23"/>
+    <tableColumn id="3" xr3:uid="{230B22CA-5CA3-4E2D-92CC-C75BC5831FF2}" uniqueName="3" name="Column3" queryTableFieldId="3" dataDxfId="22"/>
+    <tableColumn id="4" xr3:uid="{42788CA6-A70D-442A-9072-79E0D19F0B28}" uniqueName="4" name="Column4" queryTableFieldId="4" dataDxfId="21"/>
+    <tableColumn id="5" xr3:uid="{E37C1038-7442-4E7D-BB43-162AD6FA4195}" uniqueName="5" name="Column5" queryTableFieldId="5" dataDxfId="20"/>
   </tableColumns>
   <tableStyleInfo name="TableStyleMedium7" showFirstColumn="0" showLastColumn="0" showRowStripes="1" showColumnStripes="0"/>
 </table>
@@ -5240,13 +5262,13 @@
 <table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="1" xr:uid="{8D8C9D73-217D-4974-B35A-0740746DA27F}" name="Table001__Page_2" displayName="Table001__Page_2" ref="A1:G16" tableType="queryTable" totalsRowShown="0">
   <autoFilter ref="A1:G16" xr:uid="{8D8C9D73-217D-4974-B35A-0740746DA27F}"/>
   <tableColumns count="7">
-    <tableColumn id="1" xr3:uid="{A26CE965-72B2-472B-B9FF-D68F7847F3C5}" uniqueName="1" name="Column1" queryTableFieldId="1" dataDxfId="140"/>
-    <tableColumn id="2" xr3:uid="{375BF78E-5806-424A-B7BD-C63C40843BE9}" uniqueName="2" name="Column2" queryTableFieldId="2" dataDxfId="139"/>
-    <tableColumn id="3" xr3:uid="{CD1FFC74-B097-42B5-B1FA-08D3BD4531B9}" uniqueName="3" name="Column3" queryTableFieldId="3" dataDxfId="138"/>
-    <tableColumn id="4" xr3:uid="{EA6F5C08-47B3-4BE3-8F9B-3167F2B34338}" uniqueName="4" name="Column4" queryTableFieldId="4" dataDxfId="137"/>
-    <tableColumn id="5" xr3:uid="{67D1B145-6151-4A54-9C79-A6B0381CDA09}" uniqueName="5" name="Column5" queryTableFieldId="5" dataDxfId="136"/>
-    <tableColumn id="6" xr3:uid="{E8D8899E-ED32-4A2F-B13D-18F4C289A59B}" uniqueName="6" name="Column6" queryTableFieldId="6" dataDxfId="135"/>
-    <tableColumn id="7" xr3:uid="{CD1BCBB0-10DE-4DDA-903D-C14D16829749}" uniqueName="7" name="Column7" queryTableFieldId="7" dataDxfId="134"/>
+    <tableColumn id="1" xr3:uid="{A26CE965-72B2-472B-B9FF-D68F7847F3C5}" uniqueName="1" name="Column1" queryTableFieldId="1" dataDxfId="141"/>
+    <tableColumn id="2" xr3:uid="{375BF78E-5806-424A-B7BD-C63C40843BE9}" uniqueName="2" name="Column2" queryTableFieldId="2" dataDxfId="140"/>
+    <tableColumn id="3" xr3:uid="{CD1FFC74-B097-42B5-B1FA-08D3BD4531B9}" uniqueName="3" name="Column3" queryTableFieldId="3" dataDxfId="139"/>
+    <tableColumn id="4" xr3:uid="{EA6F5C08-47B3-4BE3-8F9B-3167F2B34338}" uniqueName="4" name="Column4" queryTableFieldId="4" dataDxfId="138"/>
+    <tableColumn id="5" xr3:uid="{67D1B145-6151-4A54-9C79-A6B0381CDA09}" uniqueName="5" name="Column5" queryTableFieldId="5" dataDxfId="137"/>
+    <tableColumn id="6" xr3:uid="{E8D8899E-ED32-4A2F-B13D-18F4C289A59B}" uniqueName="6" name="Column6" queryTableFieldId="6" dataDxfId="136"/>
+    <tableColumn id="7" xr3:uid="{CD1BCBB0-10DE-4DDA-903D-C14D16829749}" uniqueName="7" name="Column7" queryTableFieldId="7" dataDxfId="135"/>
   </tableColumns>
   <tableStyleInfo name="TableStyleMedium7" showFirstColumn="0" showLastColumn="0" showRowStripes="1" showColumnStripes="0"/>
 </table>
@@ -5256,11 +5278,11 @@
 <table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="19" xr:uid="{A8D65B7F-C1B3-4E37-BFF7-03252131F371}" name="Table019__Page_11" displayName="Table019__Page_11" ref="A1:E16" tableType="queryTable" totalsRowShown="0">
   <autoFilter ref="A1:E16" xr:uid="{A8D65B7F-C1B3-4E37-BFF7-03252131F371}"/>
   <tableColumns count="5">
-    <tableColumn id="1" xr3:uid="{60EAA1C9-E43C-458C-A33C-365CF023541D}" uniqueName="1" name="Column1" queryTableFieldId="1" dataDxfId="18"/>
-    <tableColumn id="2" xr3:uid="{BF4ECEAF-8998-4833-A444-7DD2840947AB}" uniqueName="2" name="Column2" queryTableFieldId="2" dataDxfId="17"/>
-    <tableColumn id="3" xr3:uid="{A77E13C5-CB25-43C0-9678-51A378FA64FC}" uniqueName="3" name="Column3" queryTableFieldId="3" dataDxfId="16"/>
-    <tableColumn id="4" xr3:uid="{46713ABC-AA6E-45DD-9BBE-03C863D6B1D1}" uniqueName="4" name="Column4" queryTableFieldId="4" dataDxfId="15"/>
-    <tableColumn id="5" xr3:uid="{85365AB6-280F-40C4-AB42-3455547D61F1}" uniqueName="5" name="Column5" queryTableFieldId="5" dataDxfId="14"/>
+    <tableColumn id="1" xr3:uid="{60EAA1C9-E43C-458C-A33C-365CF023541D}" uniqueName="1" name="Column1" queryTableFieldId="1" dataDxfId="19"/>
+    <tableColumn id="2" xr3:uid="{BF4ECEAF-8998-4833-A444-7DD2840947AB}" uniqueName="2" name="Column2" queryTableFieldId="2" dataDxfId="18"/>
+    <tableColumn id="3" xr3:uid="{A77E13C5-CB25-43C0-9678-51A378FA64FC}" uniqueName="3" name="Column3" queryTableFieldId="3" dataDxfId="17"/>
+    <tableColumn id="4" xr3:uid="{46713ABC-AA6E-45DD-9BBE-03C863D6B1D1}" uniqueName="4" name="Column4" queryTableFieldId="4" dataDxfId="16"/>
+    <tableColumn id="5" xr3:uid="{85365AB6-280F-40C4-AB42-3455547D61F1}" uniqueName="5" name="Column5" queryTableFieldId="5" dataDxfId="15"/>
   </tableColumns>
   <tableStyleInfo name="TableStyleMedium7" showFirstColumn="0" showLastColumn="0" showRowStripes="1" showColumnStripes="0"/>
 </table>
@@ -5270,11 +5292,11 @@
 <table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="21" xr:uid="{0B4290D5-7CEE-4DDC-B997-690EEF6D9589}" name="Table020__Page_11" displayName="Table020__Page_11" ref="A18:E20" tableType="queryTable" totalsRowShown="0">
   <autoFilter ref="A18:E20" xr:uid="{0B4290D5-7CEE-4DDC-B997-690EEF6D9589}"/>
   <tableColumns count="5">
-    <tableColumn id="1" xr3:uid="{344C3D84-8C5A-4C60-ADD3-4EE73F83858B}" uniqueName="1" name="Column1" queryTableFieldId="1" dataDxfId="13"/>
-    <tableColumn id="2" xr3:uid="{3470DF86-5A38-429A-95CF-F5FF5E59449C}" uniqueName="2" name="Column2" queryTableFieldId="2" dataDxfId="12"/>
-    <tableColumn id="3" xr3:uid="{BC1BD851-46F6-4634-95EE-ED117E75EBB6}" uniqueName="3" name="Column3" queryTableFieldId="3" dataDxfId="11"/>
-    <tableColumn id="4" xr3:uid="{FF5D3D34-BBDB-4113-8340-C737255ED1BD}" uniqueName="4" name="Column4" queryTableFieldId="4" dataDxfId="10"/>
-    <tableColumn id="5" xr3:uid="{F05FA152-C9D6-4773-B0A5-5B18B60C7102}" uniqueName="5" name="Column5" queryTableFieldId="5" dataDxfId="9"/>
+    <tableColumn id="1" xr3:uid="{344C3D84-8C5A-4C60-ADD3-4EE73F83858B}" uniqueName="1" name="Column1" queryTableFieldId="1" dataDxfId="14"/>
+    <tableColumn id="2" xr3:uid="{3470DF86-5A38-429A-95CF-F5FF5E59449C}" uniqueName="2" name="Column2" queryTableFieldId="2" dataDxfId="13"/>
+    <tableColumn id="3" xr3:uid="{BC1BD851-46F6-4634-95EE-ED117E75EBB6}" uniqueName="3" name="Column3" queryTableFieldId="3" dataDxfId="12"/>
+    <tableColumn id="4" xr3:uid="{FF5D3D34-BBDB-4113-8340-C737255ED1BD}" uniqueName="4" name="Column4" queryTableFieldId="4" dataDxfId="11"/>
+    <tableColumn id="5" xr3:uid="{F05FA152-C9D6-4773-B0A5-5B18B60C7102}" uniqueName="5" name="Column5" queryTableFieldId="5" dataDxfId="10"/>
   </tableColumns>
   <tableStyleInfo name="TableStyleMedium7" showFirstColumn="0" showLastColumn="0" showRowStripes="1" showColumnStripes="0"/>
 </table>
@@ -5284,13 +5306,13 @@
 <table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="2" xr:uid="{D4474760-F3B7-4070-AE77-2962D090A5AB}" name="Table002__Page_2" displayName="Table002__Page_2" ref="A19:G21" tableType="queryTable" totalsRowShown="0">
   <autoFilter ref="A19:G21" xr:uid="{D4474760-F3B7-4070-AE77-2962D090A5AB}"/>
   <tableColumns count="7">
-    <tableColumn id="1" xr3:uid="{8A3681DA-5FE9-4564-BCAB-75CCDF2C3A51}" uniqueName="1" name="Column1" queryTableFieldId="1" dataDxfId="133"/>
-    <tableColumn id="2" xr3:uid="{44D6563C-A88C-4FEE-9427-B5252DF8FA5D}" uniqueName="2" name="Column6" queryTableFieldId="2" dataDxfId="132"/>
-    <tableColumn id="3" xr3:uid="{2514D758-49E4-4E3E-A628-2B2D894F398E}" uniqueName="3" name="Column2" queryTableFieldId="3" dataDxfId="131"/>
-    <tableColumn id="4" xr3:uid="{062470EA-CB73-435C-8DF3-28DE262C8D69}" uniqueName="4" name="Column3" queryTableFieldId="4" dataDxfId="130"/>
-    <tableColumn id="5" xr3:uid="{CDE500EE-B268-43D9-A30D-9E6CC1608CD0}" uniqueName="5" name="Column4" queryTableFieldId="5" dataDxfId="129"/>
-    <tableColumn id="6" xr3:uid="{699F51E2-9A1B-4953-91BE-8D6434D76B20}" uniqueName="6" name="Column5" queryTableFieldId="6" dataDxfId="128"/>
-    <tableColumn id="7" xr3:uid="{C62D0670-E212-49FF-BA61-22C41F21B60E}" uniqueName="7" name="Column62" queryTableFieldId="7" dataDxfId="127"/>
+    <tableColumn id="1" xr3:uid="{8A3681DA-5FE9-4564-BCAB-75CCDF2C3A51}" uniqueName="1" name="Column1" queryTableFieldId="1" dataDxfId="134"/>
+    <tableColumn id="2" xr3:uid="{44D6563C-A88C-4FEE-9427-B5252DF8FA5D}" uniqueName="2" name="Column6" queryTableFieldId="2" dataDxfId="133"/>
+    <tableColumn id="3" xr3:uid="{2514D758-49E4-4E3E-A628-2B2D894F398E}" uniqueName="3" name="Column2" queryTableFieldId="3" dataDxfId="132"/>
+    <tableColumn id="4" xr3:uid="{062470EA-CB73-435C-8DF3-28DE262C8D69}" uniqueName="4" name="Column3" queryTableFieldId="4" dataDxfId="131"/>
+    <tableColumn id="5" xr3:uid="{CDE500EE-B268-43D9-A30D-9E6CC1608CD0}" uniqueName="5" name="Column4" queryTableFieldId="5" dataDxfId="130"/>
+    <tableColumn id="6" xr3:uid="{699F51E2-9A1B-4953-91BE-8D6434D76B20}" uniqueName="6" name="Column5" queryTableFieldId="6" dataDxfId="129"/>
+    <tableColumn id="7" xr3:uid="{C62D0670-E212-49FF-BA61-22C41F21B60E}" uniqueName="7" name="Column62" queryTableFieldId="7" dataDxfId="128"/>
   </tableColumns>
   <tableStyleInfo name="TableStyleMedium7" showFirstColumn="0" showLastColumn="0" showRowStripes="1" showColumnStripes="0"/>
 </table>
@@ -5300,14 +5322,14 @@
 <table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="3" xr:uid="{EE92A61D-8549-4453-B707-7BA76D39611E}" name="Table003__Page_3" displayName="Table003__Page_3" ref="A1:H16" tableType="queryTable" totalsRowShown="0">
   <autoFilter ref="A1:H16" xr:uid="{EE92A61D-8549-4453-B707-7BA76D39611E}"/>
   <tableColumns count="8">
-    <tableColumn id="1" xr3:uid="{5E78ED26-3040-4033-A95F-3AC09118D17C}" uniqueName="1" name="Column1" queryTableFieldId="1" dataDxfId="126"/>
-    <tableColumn id="2" xr3:uid="{52F60F93-88D4-4F60-A15A-4B2113E53BE2}" uniqueName="2" name="Column2" queryTableFieldId="2" dataDxfId="125"/>
-    <tableColumn id="3" xr3:uid="{2A66B2A9-165C-4995-937F-8E0D8B01B3D8}" uniqueName="3" name="Column3" queryTableFieldId="3" dataDxfId="124"/>
-    <tableColumn id="4" xr3:uid="{937ED0C3-8277-4EC6-BFD2-C6699696538D}" uniqueName="4" name="Column4" queryTableFieldId="4" dataDxfId="123"/>
-    <tableColumn id="5" xr3:uid="{37EAAABA-4FEF-4D28-B237-360AD0A7194A}" uniqueName="5" name="Column5" queryTableFieldId="5" dataDxfId="122"/>
-    <tableColumn id="6" xr3:uid="{6E7D50A0-6329-4797-9F9A-628D251C7CA5}" uniqueName="6" name="Column6" queryTableFieldId="6" dataDxfId="121"/>
-    <tableColumn id="7" xr3:uid="{F8F31C01-9522-488B-915F-110987168D09}" uniqueName="7" name="Column7" queryTableFieldId="7" dataDxfId="120"/>
-    <tableColumn id="8" xr3:uid="{FFD35FDD-AAE7-4F54-8AF3-197380BC0AEB}" uniqueName="8" name="Column8" queryTableFieldId="8" dataDxfId="119"/>
+    <tableColumn id="1" xr3:uid="{5E78ED26-3040-4033-A95F-3AC09118D17C}" uniqueName="1" name="Column1" queryTableFieldId="1" dataDxfId="127"/>
+    <tableColumn id="2" xr3:uid="{52F60F93-88D4-4F60-A15A-4B2113E53BE2}" uniqueName="2" name="Column2" queryTableFieldId="2" dataDxfId="126"/>
+    <tableColumn id="3" xr3:uid="{2A66B2A9-165C-4995-937F-8E0D8B01B3D8}" uniqueName="3" name="Column3" queryTableFieldId="3" dataDxfId="125"/>
+    <tableColumn id="4" xr3:uid="{937ED0C3-8277-4EC6-BFD2-C6699696538D}" uniqueName="4" name="Column4" queryTableFieldId="4" dataDxfId="124"/>
+    <tableColumn id="5" xr3:uid="{37EAAABA-4FEF-4D28-B237-360AD0A7194A}" uniqueName="5" name="Column5" queryTableFieldId="5" dataDxfId="123"/>
+    <tableColumn id="6" xr3:uid="{6E7D50A0-6329-4797-9F9A-628D251C7CA5}" uniqueName="6" name="Column6" queryTableFieldId="6" dataDxfId="122"/>
+    <tableColumn id="7" xr3:uid="{F8F31C01-9522-488B-915F-110987168D09}" uniqueName="7" name="Column7" queryTableFieldId="7" dataDxfId="121"/>
+    <tableColumn id="8" xr3:uid="{FFD35FDD-AAE7-4F54-8AF3-197380BC0AEB}" uniqueName="8" name="Column8" queryTableFieldId="8" dataDxfId="120"/>
   </tableColumns>
   <tableStyleInfo name="TableStyleMedium7" showFirstColumn="0" showLastColumn="0" showRowStripes="1" showColumnStripes="0"/>
 </table>
@@ -5317,14 +5339,14 @@
 <table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="4" xr:uid="{1C7E55B7-7D73-418F-9229-407F52A253A6}" name="Table004__Page_3" displayName="Table004__Page_3" ref="A18:H20" tableType="queryTable" totalsRowShown="0">
   <autoFilter ref="A18:H20" xr:uid="{1C7E55B7-7D73-418F-9229-407F52A253A6}"/>
   <tableColumns count="8">
-    <tableColumn id="1" xr3:uid="{A8A6FCCE-AE43-4EDA-82DC-831809E03401}" uniqueName="1" name="Column1" queryTableFieldId="1" dataDxfId="118"/>
-    <tableColumn id="2" xr3:uid="{0231594E-DA9E-47DE-A01C-22488210A4CF}" uniqueName="2" name="Column2" queryTableFieldId="2" dataDxfId="117"/>
-    <tableColumn id="3" xr3:uid="{7A06306A-69AF-482D-910F-86D0EF88F740}" uniqueName="3" name="Column3" queryTableFieldId="3" dataDxfId="116"/>
-    <tableColumn id="4" xr3:uid="{E96F3603-E9D2-4710-BDE5-6FE3E6A378D8}" uniqueName="4" name="Column4" queryTableFieldId="4" dataDxfId="115"/>
-    <tableColumn id="5" xr3:uid="{37151140-CC9F-4EBB-B58D-F87E1081314A}" uniqueName="5" name="Column5" queryTableFieldId="5" dataDxfId="114"/>
-    <tableColumn id="6" xr3:uid="{F0AAEEC2-014D-412A-B58D-24C71FEC9A66}" uniqueName="6" name="Column6" queryTableFieldId="6" dataDxfId="113"/>
-    <tableColumn id="7" xr3:uid="{A4B4F3F0-B14D-498F-B185-AA3E2BAE729A}" uniqueName="7" name="Column7" queryTableFieldId="7" dataDxfId="112"/>
-    <tableColumn id="8" xr3:uid="{0C517BB9-44A4-4BBA-AA88-B86BB679F208}" uniqueName="8" name="Column8" queryTableFieldId="8" dataDxfId="111"/>
+    <tableColumn id="1" xr3:uid="{A8A6FCCE-AE43-4EDA-82DC-831809E03401}" uniqueName="1" name="Column1" queryTableFieldId="1" dataDxfId="119"/>
+    <tableColumn id="2" xr3:uid="{0231594E-DA9E-47DE-A01C-22488210A4CF}" uniqueName="2" name="Column2" queryTableFieldId="2" dataDxfId="118"/>
+    <tableColumn id="3" xr3:uid="{7A06306A-69AF-482D-910F-86D0EF88F740}" uniqueName="3" name="Column3" queryTableFieldId="3" dataDxfId="117"/>
+    <tableColumn id="4" xr3:uid="{E96F3603-E9D2-4710-BDE5-6FE3E6A378D8}" uniqueName="4" name="Column4" queryTableFieldId="4" dataDxfId="116"/>
+    <tableColumn id="5" xr3:uid="{37151140-CC9F-4EBB-B58D-F87E1081314A}" uniqueName="5" name="Column5" queryTableFieldId="5" dataDxfId="115"/>
+    <tableColumn id="6" xr3:uid="{F0AAEEC2-014D-412A-B58D-24C71FEC9A66}" uniqueName="6" name="Column6" queryTableFieldId="6" dataDxfId="114"/>
+    <tableColumn id="7" xr3:uid="{A4B4F3F0-B14D-498F-B185-AA3E2BAE729A}" uniqueName="7" name="Column7" queryTableFieldId="7" dataDxfId="113"/>
+    <tableColumn id="8" xr3:uid="{0C517BB9-44A4-4BBA-AA88-B86BB679F208}" uniqueName="8" name="Column8" queryTableFieldId="8" dataDxfId="112"/>
   </tableColumns>
   <tableStyleInfo name="TableStyleMedium7" showFirstColumn="0" showLastColumn="0" showRowStripes="1" showColumnStripes="0"/>
 </table>
@@ -5334,12 +5356,12 @@
 <table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="5" xr:uid="{2EB30D60-3074-4922-8217-6B97953C0F87}" name="Table005__Page_4" displayName="Table005__Page_4" ref="A1:F16" tableType="queryTable" totalsRowShown="0">
   <autoFilter ref="A1:F16" xr:uid="{2EB30D60-3074-4922-8217-6B97953C0F87}"/>
   <tableColumns count="6">
-    <tableColumn id="1" xr3:uid="{AB42FEA9-5A85-4A69-B46D-444C53C4B4EF}" uniqueName="1" name="Column1" queryTableFieldId="1" dataDxfId="110"/>
-    <tableColumn id="2" xr3:uid="{0D7919B1-FB5E-4192-8675-3D57B39D9AB0}" uniqueName="2" name="Column2" queryTableFieldId="2" dataDxfId="109"/>
-    <tableColumn id="3" xr3:uid="{94F12F3D-88BF-4BEB-85E7-FF6313F6B88E}" uniqueName="3" name="Column3" queryTableFieldId="3" dataDxfId="108"/>
-    <tableColumn id="4" xr3:uid="{2B04EEA3-DC55-4C69-860F-9571D35E352D}" uniqueName="4" name="Column4" queryTableFieldId="4" dataDxfId="107"/>
-    <tableColumn id="5" xr3:uid="{461C5084-182B-40CC-B479-24798E48D0F4}" uniqueName="5" name="Column5" queryTableFieldId="5" dataDxfId="106"/>
-    <tableColumn id="6" xr3:uid="{258F7EB6-7345-43CA-BF8A-5E088D06FF8F}" uniqueName="6" name="Column6" queryTableFieldId="6" dataDxfId="105"/>
+    <tableColumn id="1" xr3:uid="{AB42FEA9-5A85-4A69-B46D-444C53C4B4EF}" uniqueName="1" name="Column1" queryTableFieldId="1" dataDxfId="111"/>
+    <tableColumn id="2" xr3:uid="{0D7919B1-FB5E-4192-8675-3D57B39D9AB0}" uniqueName="2" name="Column2" queryTableFieldId="2" dataDxfId="110"/>
+    <tableColumn id="3" xr3:uid="{94F12F3D-88BF-4BEB-85E7-FF6313F6B88E}" uniqueName="3" name="Column3" queryTableFieldId="3" dataDxfId="109"/>
+    <tableColumn id="4" xr3:uid="{2B04EEA3-DC55-4C69-860F-9571D35E352D}" uniqueName="4" name="Column4" queryTableFieldId="4" dataDxfId="108"/>
+    <tableColumn id="5" xr3:uid="{461C5084-182B-40CC-B479-24798E48D0F4}" uniqueName="5" name="Column5" queryTableFieldId="5" dataDxfId="107"/>
+    <tableColumn id="6" xr3:uid="{258F7EB6-7345-43CA-BF8A-5E088D06FF8F}" uniqueName="6" name="Column6" queryTableFieldId="6" dataDxfId="106"/>
   </tableColumns>
   <tableStyleInfo name="TableStyleMedium7" showFirstColumn="0" showLastColumn="0" showRowStripes="1" showColumnStripes="0"/>
 </table>
@@ -5349,12 +5371,12 @@
 <table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="6" xr:uid="{BA3E356C-A98F-4646-B7E8-7B0C3904E2A4}" name="Table006__Page_4" displayName="Table006__Page_4" ref="A18:F20" tableType="queryTable" totalsRowShown="0">
   <autoFilter ref="A18:F20" xr:uid="{BA3E356C-A98F-4646-B7E8-7B0C3904E2A4}"/>
   <tableColumns count="6">
-    <tableColumn id="1" xr3:uid="{55987721-40E8-4E11-9B6F-67EE503D78F4}" uniqueName="1" name="Column1" queryTableFieldId="1" dataDxfId="104"/>
-    <tableColumn id="2" xr3:uid="{15260D47-39CC-4501-9656-F8DBE6AD3AB1}" uniqueName="2" name="Column2" queryTableFieldId="2" dataDxfId="103"/>
-    <tableColumn id="3" xr3:uid="{06C8B30C-3DD3-49E6-8BE6-C8A9D39F2FC4}" uniqueName="3" name="Column3" queryTableFieldId="3" dataDxfId="102"/>
-    <tableColumn id="4" xr3:uid="{40A070F6-4BDB-49A7-9394-4D63F3A9E318}" uniqueName="4" name="Column4" queryTableFieldId="4" dataDxfId="101"/>
-    <tableColumn id="5" xr3:uid="{C5E0BAEF-796C-4C71-ACA7-889E63543C2D}" uniqueName="5" name="Column5" queryTableFieldId="5" dataDxfId="100"/>
-    <tableColumn id="6" xr3:uid="{1BA75280-A961-41F1-B113-5935891BA00A}" uniqueName="6" name="Column6" queryTableFieldId="6" dataDxfId="99"/>
+    <tableColumn id="1" xr3:uid="{55987721-40E8-4E11-9B6F-67EE503D78F4}" uniqueName="1" name="Column1" queryTableFieldId="1" dataDxfId="105"/>
+    <tableColumn id="2" xr3:uid="{15260D47-39CC-4501-9656-F8DBE6AD3AB1}" uniqueName="2" name="Column2" queryTableFieldId="2" dataDxfId="104"/>
+    <tableColumn id="3" xr3:uid="{06C8B30C-3DD3-49E6-8BE6-C8A9D39F2FC4}" uniqueName="3" name="Column3" queryTableFieldId="3" dataDxfId="103"/>
+    <tableColumn id="4" xr3:uid="{40A070F6-4BDB-49A7-9394-4D63F3A9E318}" uniqueName="4" name="Column4" queryTableFieldId="4" dataDxfId="102"/>
+    <tableColumn id="5" xr3:uid="{C5E0BAEF-796C-4C71-ACA7-889E63543C2D}" uniqueName="5" name="Column5" queryTableFieldId="5" dataDxfId="101"/>
+    <tableColumn id="6" xr3:uid="{1BA75280-A961-41F1-B113-5935891BA00A}" uniqueName="6" name="Column6" queryTableFieldId="6" dataDxfId="100"/>
   </tableColumns>
   <tableStyleInfo name="TableStyleMedium7" showFirstColumn="0" showLastColumn="0" showRowStripes="1" showColumnStripes="0"/>
 </table>
@@ -5364,18 +5386,18 @@
 <table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="7" xr:uid="{6040FF08-DFFC-4D6C-87C0-7C33D5281777}" name="Table007__Page_5" displayName="Table007__Page_5" ref="A1:L16" tableType="queryTable" totalsRowShown="0">
   <autoFilter ref="A1:L16" xr:uid="{6040FF08-DFFC-4D6C-87C0-7C33D5281777}"/>
   <tableColumns count="12">
-    <tableColumn id="1" xr3:uid="{9561388E-64AE-4A76-863E-A0B2091E2F9F}" uniqueName="1" name="Column1" queryTableFieldId="1" dataDxfId="98"/>
-    <tableColumn id="2" xr3:uid="{151810A9-7DD3-4FD0-91D6-6608DF85A8CF}" uniqueName="2" name="Column2" queryTableFieldId="2" dataDxfId="97"/>
-    <tableColumn id="3" xr3:uid="{94D629BF-F745-493D-8F74-FA7EEFDEAA84}" uniqueName="3" name="Column3" queryTableFieldId="3" dataDxfId="96"/>
-    <tableColumn id="4" xr3:uid="{AE87299A-170F-4661-BD08-B108394E2F7C}" uniqueName="4" name="Column4" queryTableFieldId="4" dataDxfId="95"/>
-    <tableColumn id="5" xr3:uid="{708CB468-5E3F-4D0C-B6BD-C2C44C7191EC}" uniqueName="5" name="Column5" queryTableFieldId="5" dataDxfId="94"/>
-    <tableColumn id="6" xr3:uid="{5D4BD3CB-C344-4155-B3C1-ECC49F86CED1}" uniqueName="6" name="Column6" queryTableFieldId="6" dataDxfId="93"/>
-    <tableColumn id="7" xr3:uid="{61DF1122-5C54-47A3-98F9-27CA1B50CA9D}" uniqueName="7" name="Column7" queryTableFieldId="7" dataDxfId="92"/>
-    <tableColumn id="8" xr3:uid="{130590EE-DDCB-43DB-A020-385B521DA018}" uniqueName="8" name="Column8" queryTableFieldId="8" dataDxfId="91"/>
-    <tableColumn id="9" xr3:uid="{06B903F7-5E22-476D-A116-655599D2C518}" uniqueName="9" name="Column9" queryTableFieldId="9" dataDxfId="90"/>
-    <tableColumn id="10" xr3:uid="{CED96D55-8B0D-492D-B0EC-F3E56EFB2649}" uniqueName="10" name="Column10" queryTableFieldId="10" dataDxfId="89"/>
-    <tableColumn id="11" xr3:uid="{346823E9-F305-4F11-941F-1C42A8AB0C99}" uniqueName="11" name="Column11" queryTableFieldId="11" dataDxfId="88"/>
-    <tableColumn id="12" xr3:uid="{7B421AA8-C9DB-4E35-A456-DF0F56050B79}" uniqueName="12" name="Column12" queryTableFieldId="12" dataDxfId="87"/>
+    <tableColumn id="1" xr3:uid="{9561388E-64AE-4A76-863E-A0B2091E2F9F}" uniqueName="1" name="Column1" queryTableFieldId="1" dataDxfId="99"/>
+    <tableColumn id="2" xr3:uid="{151810A9-7DD3-4FD0-91D6-6608DF85A8CF}" uniqueName="2" name="Column2" queryTableFieldId="2" dataDxfId="98"/>
+    <tableColumn id="3" xr3:uid="{94D629BF-F745-493D-8F74-FA7EEFDEAA84}" uniqueName="3" name="Column3" queryTableFieldId="3" dataDxfId="97"/>
+    <tableColumn id="4" xr3:uid="{AE87299A-170F-4661-BD08-B108394E2F7C}" uniqueName="4" name="Column4" queryTableFieldId="4" dataDxfId="96"/>
+    <tableColumn id="5" xr3:uid="{708CB468-5E3F-4D0C-B6BD-C2C44C7191EC}" uniqueName="5" name="Column5" queryTableFieldId="5" dataDxfId="95"/>
+    <tableColumn id="6" xr3:uid="{5D4BD3CB-C344-4155-B3C1-ECC49F86CED1}" uniqueName="6" name="Column6" queryTableFieldId="6" dataDxfId="94"/>
+    <tableColumn id="7" xr3:uid="{61DF1122-5C54-47A3-98F9-27CA1B50CA9D}" uniqueName="7" name="Column7" queryTableFieldId="7" dataDxfId="93"/>
+    <tableColumn id="8" xr3:uid="{130590EE-DDCB-43DB-A020-385B521DA018}" uniqueName="8" name="Column8" queryTableFieldId="8" dataDxfId="92"/>
+    <tableColumn id="9" xr3:uid="{06B903F7-5E22-476D-A116-655599D2C518}" uniqueName="9" name="Column9" queryTableFieldId="9" dataDxfId="91"/>
+    <tableColumn id="10" xr3:uid="{CED96D55-8B0D-492D-B0EC-F3E56EFB2649}" uniqueName="10" name="Column10" queryTableFieldId="10" dataDxfId="90"/>
+    <tableColumn id="11" xr3:uid="{346823E9-F305-4F11-941F-1C42A8AB0C99}" uniqueName="11" name="Column11" queryTableFieldId="11" dataDxfId="89"/>
+    <tableColumn id="12" xr3:uid="{7B421AA8-C9DB-4E35-A456-DF0F56050B79}" uniqueName="12" name="Column12" queryTableFieldId="12" dataDxfId="88"/>
   </tableColumns>
   <tableStyleInfo name="TableStyleMedium7" showFirstColumn="0" showLastColumn="0" showRowStripes="1" showColumnStripes="0"/>
 </table>
@@ -5385,18 +5407,18 @@
 <table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="8" xr:uid="{DBF54861-4823-4965-9BF8-BF4D83A85FD1}" name="Table008__Page_5" displayName="Table008__Page_5" ref="A18:L20" tableType="queryTable" totalsRowShown="0">
   <autoFilter ref="A18:L20" xr:uid="{DBF54861-4823-4965-9BF8-BF4D83A85FD1}"/>
   <tableColumns count="12">
-    <tableColumn id="1" xr3:uid="{01D3C90B-BA67-46B4-BD1D-5C53486CAE57}" uniqueName="1" name="Column1" queryTableFieldId="1" dataDxfId="86"/>
-    <tableColumn id="2" xr3:uid="{166854EB-0B50-4420-BB3F-7A5A2C9FB7F7}" uniqueName="2" name="Column2" queryTableFieldId="2" dataDxfId="85"/>
-    <tableColumn id="3" xr3:uid="{638857E5-1EB4-4FBE-9FFE-2951F2F4ABD0}" uniqueName="3" name="Column3" queryTableFieldId="3" dataDxfId="84"/>
-    <tableColumn id="4" xr3:uid="{F4EFE2EF-AC84-40F8-BE68-0B6B520F8EA8}" uniqueName="4" name="Column4" queryTableFieldId="4" dataDxfId="83"/>
-    <tableColumn id="5" xr3:uid="{38D026D2-A47E-46EA-BA10-AF890A55BF2B}" uniqueName="5" name="Column5" queryTableFieldId="5" dataDxfId="82"/>
-    <tableColumn id="6" xr3:uid="{025C6DA2-37A6-491F-904E-DDE12948D35B}" uniqueName="6" name="Column6" queryTableFieldId="6" dataDxfId="81"/>
-    <tableColumn id="7" xr3:uid="{AC28B573-67B7-4468-A6A2-F648D17079B6}" uniqueName="7" name="Column7" queryTableFieldId="7" dataDxfId="80"/>
-    <tableColumn id="8" xr3:uid="{F6F06554-210B-472F-95F2-8E89D931E4C1}" uniqueName="8" name="Column8" queryTableFieldId="8" dataDxfId="79"/>
-    <tableColumn id="9" xr3:uid="{F0A8F323-36C1-4290-980B-8F6F5DC6A41E}" uniqueName="9" name="Column9" queryTableFieldId="9" dataDxfId="78"/>
-    <tableColumn id="10" xr3:uid="{25D60007-5007-4174-85F5-572E3C29FE33}" uniqueName="10" name="Column10" queryTableFieldId="10" dataDxfId="77"/>
-    <tableColumn id="11" xr3:uid="{2071EB9B-B14E-4EF0-9B86-0D5FDA96828D}" uniqueName="11" name="Column11" queryTableFieldId="11" dataDxfId="76"/>
-    <tableColumn id="12" xr3:uid="{1660C180-EE6B-48E8-9880-55F02CC623C4}" uniqueName="12" name="Column12" queryTableFieldId="12" dataDxfId="75"/>
+    <tableColumn id="1" xr3:uid="{01D3C90B-BA67-46B4-BD1D-5C53486CAE57}" uniqueName="1" name="Column1" queryTableFieldId="1" dataDxfId="87"/>
+    <tableColumn id="2" xr3:uid="{166854EB-0B50-4420-BB3F-7A5A2C9FB7F7}" uniqueName="2" name="Column2" queryTableFieldId="2" dataDxfId="86"/>
+    <tableColumn id="3" xr3:uid="{638857E5-1EB4-4FBE-9FFE-2951F2F4ABD0}" uniqueName="3" name="Column3" queryTableFieldId="3" dataDxfId="85"/>
+    <tableColumn id="4" xr3:uid="{F4EFE2EF-AC84-40F8-BE68-0B6B520F8EA8}" uniqueName="4" name="Column4" queryTableFieldId="4" dataDxfId="84"/>
+    <tableColumn id="5" xr3:uid="{38D026D2-A47E-46EA-BA10-AF890A55BF2B}" uniqueName="5" name="Column5" queryTableFieldId="5" dataDxfId="83"/>
+    <tableColumn id="6" xr3:uid="{025C6DA2-37A6-491F-904E-DDE12948D35B}" uniqueName="6" name="Column6" queryTableFieldId="6" dataDxfId="82"/>
+    <tableColumn id="7" xr3:uid="{AC28B573-67B7-4468-A6A2-F648D17079B6}" uniqueName="7" name="Column7" queryTableFieldId="7" dataDxfId="81"/>
+    <tableColumn id="8" xr3:uid="{F6F06554-210B-472F-95F2-8E89D931E4C1}" uniqueName="8" name="Column8" queryTableFieldId="8" dataDxfId="80"/>
+    <tableColumn id="9" xr3:uid="{F0A8F323-36C1-4290-980B-8F6F5DC6A41E}" uniqueName="9" name="Column9" queryTableFieldId="9" dataDxfId="79"/>
+    <tableColumn id="10" xr3:uid="{25D60007-5007-4174-85F5-572E3C29FE33}" uniqueName="10" name="Column10" queryTableFieldId="10" dataDxfId="78"/>
+    <tableColumn id="11" xr3:uid="{2071EB9B-B14E-4EF0-9B86-0D5FDA96828D}" uniqueName="11" name="Column11" queryTableFieldId="11" dataDxfId="77"/>
+    <tableColumn id="12" xr3:uid="{1660C180-EE6B-48E8-9880-55F02CC623C4}" uniqueName="12" name="Column12" queryTableFieldId="12" dataDxfId="76"/>
   </tableColumns>
   <tableStyleInfo name="TableStyleMedium7" showFirstColumn="0" showLastColumn="0" showRowStripes="1" showColumnStripes="0"/>
 </table>
@@ -5699,7 +5721,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{3B05C9E0-A64E-40AC-B9F4-C919ED5906CC}">
-  <dimension ref="A1:I65"/>
+  <dimension ref="A1:I69"/>
   <sheetFormatPr defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
   <cols>
     <col min="1" max="1" width="51.453125" bestFit="1" customWidth="1"/>
@@ -7578,7 +7600,7 @@
         <v>15624999.999999998</v>
       </c>
       <c r="G58" s="21">
-        <v>262</v>
+        <v>265</v>
       </c>
       <c r="H58" s="17" t="s">
         <v>623</v>
@@ -7610,7 +7632,7 @@
         <v>21874999.999999996</v>
       </c>
       <c r="G59" s="21">
-        <v>263</v>
+        <v>266</v>
       </c>
       <c r="H59" s="17" t="s">
         <v>625</v>
@@ -7642,7 +7664,7 @@
         <v>15624999.999999998</v>
       </c>
       <c r="G60" s="21">
-        <v>264</v>
+        <v>267</v>
       </c>
       <c r="H60" s="17" t="s">
         <v>624</v>
@@ -7674,7 +7696,7 @@
         <v>21874999.999999996</v>
       </c>
       <c r="G61" s="21">
-        <v>265</v>
+        <v>268</v>
       </c>
       <c r="H61" s="17" t="s">
         <v>626</v>
@@ -7706,7 +7728,7 @@
         <v>15624999.999999998</v>
       </c>
       <c r="G62" s="21">
-        <v>262</v>
+        <v>265</v>
       </c>
       <c r="H62" s="17" t="s">
         <v>623</v>
@@ -7738,7 +7760,7 @@
         <v>21874999.999999996</v>
       </c>
       <c r="G63" s="21">
-        <v>263</v>
+        <v>266</v>
       </c>
       <c r="H63" s="17" t="s">
         <v>625</v>
@@ -7770,7 +7792,7 @@
         <v>15624999.999999998</v>
       </c>
       <c r="G64" s="21">
-        <v>264</v>
+        <v>267</v>
       </c>
       <c r="H64" s="17" t="s">
         <v>624</v>
@@ -7802,7 +7824,7 @@
         <v>21874999.999999996</v>
       </c>
       <c r="G65" s="21">
-        <v>265</v>
+        <v>268</v>
       </c>
       <c r="H65" s="17" t="s">
         <v>626</v>
@@ -7811,23 +7833,130 @@
         <v>35000000</v>
       </c>
     </row>
+    <row r="66" spans="1:9" x14ac:dyDescent="0.35">
+      <c r="A66" s="16" t="s">
+        <v>631</v>
+      </c>
+      <c r="B66" s="25" t="s">
+        <v>615</v>
+      </c>
+      <c r="C66" s="18">
+        <v>303000000</v>
+      </c>
+      <c r="D66" s="9">
+        <f t="shared" ref="D66:D68" si="16">I66/1.12</f>
+        <v>20535714.285714284</v>
+      </c>
+      <c r="E66" s="9">
+        <f t="shared" ref="E66:E68" si="17">D66*90%</f>
+        <v>18482142.857142854</v>
+      </c>
+      <c r="F66" s="9">
+        <f t="shared" ref="F66:F68" si="18">D66*70%</f>
+        <v>14374999.999999998</v>
+      </c>
+      <c r="G66" s="3">
+        <v>264</v>
+      </c>
+      <c r="H66" s="17" t="s">
+        <v>566</v>
+      </c>
+      <c r="I66" s="26">
+        <v>23000000</v>
+      </c>
+    </row>
+    <row r="67" spans="1:9" x14ac:dyDescent="0.35">
+      <c r="A67" s="27" t="s">
+        <v>632</v>
+      </c>
+      <c r="B67" s="4" t="s">
+        <v>613</v>
+      </c>
+      <c r="C67" s="5">
+        <v>217000000</v>
+      </c>
+      <c r="D67" s="5">
+        <f t="shared" si="16"/>
+        <v>11607142.857142856</v>
+      </c>
+      <c r="E67" s="5">
+        <f t="shared" si="17"/>
+        <v>10446428.571428571</v>
+      </c>
+      <c r="F67" s="5">
+        <f t="shared" si="18"/>
+        <v>8124999.9999999991</v>
+      </c>
+      <c r="G67" s="3">
+        <v>262</v>
+      </c>
+      <c r="H67" s="4" t="s">
+        <v>566</v>
+      </c>
+      <c r="I67" s="12">
+        <v>13000000</v>
+      </c>
+    </row>
+    <row r="68" spans="1:9" x14ac:dyDescent="0.35">
+      <c r="A68" s="27" t="s">
+        <v>633</v>
+      </c>
+      <c r="B68" s="4" t="s">
+        <v>614</v>
+      </c>
+      <c r="C68" s="5">
+        <v>263000000</v>
+      </c>
+      <c r="D68" s="5">
+        <f t="shared" si="16"/>
+        <v>17857142.857142854</v>
+      </c>
+      <c r="E68" s="5">
+        <f t="shared" si="17"/>
+        <v>16071428.571428569</v>
+      </c>
+      <c r="F68" s="5">
+        <f t="shared" si="18"/>
+        <v>12499999.999999998</v>
+      </c>
+      <c r="G68" s="3">
+        <v>263</v>
+      </c>
+      <c r="H68" s="4" t="s">
+        <v>566</v>
+      </c>
+      <c r="I68" s="12">
+        <v>20000000</v>
+      </c>
+    </row>
+    <row r="69" spans="1:9" x14ac:dyDescent="0.35">
+      <c r="A69" s="27"/>
+      <c r="B69" s="25"/>
+      <c r="C69" s="18"/>
+      <c r="D69" s="18"/>
+      <c r="E69" s="18"/>
+      <c r="F69" s="18"/>
+      <c r="G69" s="17"/>
+      <c r="H69" s="17"/>
+      <c r="I69" s="26"/>
+    </row>
   </sheetData>
   <conditionalFormatting sqref="A1:A1048576">
-    <cfRule type="duplicateValues" dxfId="8" priority="1"/>
+    <cfRule type="duplicateValues" dxfId="9" priority="2"/>
   </conditionalFormatting>
   <conditionalFormatting sqref="A33:A41 A43:A46 A2:A31">
-    <cfRule type="duplicateValues" dxfId="7" priority="13"/>
+    <cfRule type="duplicateValues" dxfId="8" priority="14"/>
   </conditionalFormatting>
   <conditionalFormatting sqref="A33:A46 A2:A31">
-    <cfRule type="duplicateValues" dxfId="6" priority="17"/>
+    <cfRule type="duplicateValues" dxfId="7" priority="18"/>
   </conditionalFormatting>
   <conditionalFormatting sqref="H43:H46">
-    <cfRule type="duplicateValues" dxfId="5" priority="6"/>
-    <cfRule type="duplicateValues" dxfId="4" priority="7"/>
+    <cfRule type="duplicateValues" dxfId="6" priority="7"/>
+    <cfRule type="duplicateValues" dxfId="5" priority="8"/>
   </conditionalFormatting>
   <conditionalFormatting sqref="H51:H54">
-    <cfRule type="duplicateValues" dxfId="3" priority="2"/>
-    <cfRule type="duplicateValues" dxfId="2" priority="3"/>
+    <cfRule type="duplicateValues" dxfId="4" priority="3"/>
+    <cfRule type="duplicateValues" dxfId="3" priority="4"/>
   </conditionalFormatting>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <pageSetup paperSize="9" orientation="portrait" horizontalDpi="0" verticalDpi="0" r:id="rId1"/>
@@ -9825,10 +9954,10 @@
     </row>
   </sheetData>
   <conditionalFormatting sqref="A2:A33">
-    <cfRule type="duplicateValues" dxfId="1" priority="1"/>
+    <cfRule type="duplicateValues" dxfId="2" priority="1"/>
   </conditionalFormatting>
   <conditionalFormatting sqref="A2:A34">
-    <cfRule type="duplicateValues" dxfId="0" priority="2"/>
+    <cfRule type="duplicateValues" dxfId="1" priority="2"/>
   </conditionalFormatting>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>

</xml_diff>

<commit_message>
Update: New Pricelist for Aira EV
</commit_message>
<xml_diff>
--- a/gp-app-1.0/Pricelist Car.xlsx
+++ b/gp-app-1.0/Pricelist Car.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="27029"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="30228"/>
   <workbookPr hidePivotFieldList="1" defaultThemeVersion="166925"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\Work\gp-app\gp-app-1.0\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="G:\Other computers\My Laptop\Work\gp-app\gp-app-1.0\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{19E6A4A0-AAB1-4428-A3CE-4DB953D4763F}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{29A2033F-A2F0-4A1F-A376-25BE6D563462}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-110" yWindow="-110" windowWidth="19420" windowHeight="11020" tabRatio="861" xr2:uid="{C4C7316A-D95F-426A-ADF9-AD32FA680374}"/>
+    <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="16440" tabRatio="861" xr2:uid="{C4C7316A-D95F-426A-ADF9-AD32FA680374}"/>
   </bookViews>
   <sheets>
     <sheet name="Pricelist" sheetId="11" r:id="rId1"/>
@@ -490,7 +490,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1417" uniqueCount="634">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1423" uniqueCount="640">
   <si>
     <t>Column1</t>
   </si>
@@ -2472,6 +2472,24 @@
   </si>
   <si>
     <t>310S I2F1 (4X2) A/T</t>
+  </si>
+  <si>
+    <t>112C E1C (4x2) A/T</t>
+  </si>
+  <si>
+    <t>112C E2D (4x2) A/T</t>
+  </si>
+  <si>
+    <t>Aira EV LV 1</t>
+  </si>
+  <si>
+    <t>Aira EV LV 2</t>
+  </si>
+  <si>
+    <t>AIRA EV LV1</t>
+  </si>
+  <si>
+    <t>AIRA EV LV2</t>
   </si>
 </sst>
 </file>
@@ -2479,9 +2497,9 @@
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
   <numFmts count="1">
-    <numFmt numFmtId="43" formatCode="_-* #,##0.00_-;\-* #,##0.00_-;_-* &quot;-&quot;??_-;_-@_-"/>
+    <numFmt numFmtId="164" formatCode="_-* #,##0.00_-;\-* #,##0.00_-;_-* &quot;-&quot;??_-;_-@_-"/>
   </numFmts>
-  <fonts count="4" x14ac:knownFonts="1">
+  <fonts count="5" x14ac:knownFonts="1">
     <font>
       <sz val="11"/>
       <color theme="1"/>
@@ -2507,6 +2525,12 @@
       <b/>
       <sz val="11"/>
       <color theme="1"/>
+      <name val="Calibri"/>
+      <family val="2"/>
+      <scheme val="minor"/>
+    </font>
+    <font>
+      <sz val="8"/>
       <name val="Calibri"/>
       <family val="2"/>
       <scheme val="minor"/>
@@ -2660,10 +2684,10 @@
   <cellStyleXfs count="4">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0"/>
-    <xf numFmtId="43" fontId="2" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
+    <xf numFmtId="164" fontId="2" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="28">
+  <cellXfs count="25">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="2" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
     <xf numFmtId="3" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
@@ -2671,7 +2695,7 @@
       <alignment horizontal="center" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyBorder="1"/>
-    <xf numFmtId="43" fontId="0" fillId="0" borderId="1" xfId="2" applyFont="1" applyBorder="1"/>
+    <xf numFmtId="164" fontId="0" fillId="0" borderId="1" xfId="2" applyFont="1" applyBorder="1"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left"/>
     </xf>
@@ -2679,19 +2703,19 @@
       <alignment horizontal="center"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="2" xfId="0" applyBorder="1"/>
-    <xf numFmtId="43" fontId="0" fillId="0" borderId="1" xfId="2" applyFont="1" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="164" fontId="0" fillId="0" borderId="1" xfId="2" applyFont="1" applyFill="1" applyBorder="1"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="3" xfId="0" applyBorder="1"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="3" xfId="0" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left"/>
     </xf>
-    <xf numFmtId="43" fontId="0" fillId="0" borderId="4" xfId="0" applyNumberFormat="1" applyBorder="1"/>
+    <xf numFmtId="164" fontId="0" fillId="0" borderId="4" xfId="0" applyNumberFormat="1" applyBorder="1"/>
     <xf numFmtId="0" fontId="3" fillId="0" borderId="5" xfId="0" applyFont="1" applyBorder="1"/>
     <xf numFmtId="0" fontId="3" fillId="0" borderId="6" xfId="0" applyFont="1" applyBorder="1"/>
     <xf numFmtId="0" fontId="3" fillId="0" borderId="7" xfId="0" applyFont="1" applyBorder="1"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="8" xfId="0" applyBorder="1"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="9" xfId="0" applyBorder="1"/>
-    <xf numFmtId="43" fontId="0" fillId="0" borderId="9" xfId="2" applyFont="1" applyFill="1" applyBorder="1"/>
-    <xf numFmtId="43" fontId="0" fillId="0" borderId="10" xfId="0" applyNumberFormat="1" applyBorder="1"/>
+    <xf numFmtId="164" fontId="0" fillId="0" borderId="9" xfId="2" applyFont="1" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="164" fontId="0" fillId="0" borderId="10" xfId="0" applyNumberFormat="1" applyBorder="1"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
@@ -2701,13 +2725,10 @@
     <xf numFmtId="0" fontId="0" fillId="0" borderId="3" xfId="0" applyBorder="1" applyAlignment="1">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="43" fontId="0" fillId="0" borderId="9" xfId="2" applyFont="1" applyBorder="1"/>
+    <xf numFmtId="164" fontId="0" fillId="0" borderId="9" xfId="2" applyFont="1" applyBorder="1"/>
     <xf numFmtId="0" fontId="2" fillId="2" borderId="9" xfId="3" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="9" xfId="0" applyFill="1" applyBorder="1"/>
-    <xf numFmtId="43" fontId="0" fillId="0" borderId="10" xfId="0" applyNumberFormat="1" applyFill="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="8" xfId="0" applyFill="1" applyBorder="1"/>
   </cellXfs>
   <cellStyles count="4">
     <cellStyle name="Comma" xfId="2" builtinId="3"/>
@@ -2715,7 +2736,7 @@
     <cellStyle name="Normal 2" xfId="1" xr:uid="{DA2601EE-1999-4BF8-AF5E-538A4398209C}"/>
     <cellStyle name="Normal 2 2" xfId="3" xr:uid="{8C240942-BC33-4996-847D-14CFBB46F4A3}"/>
   </cellStyles>
-  <dxfs count="155">
+  <dxfs count="154">
     <dxf>
       <font>
         <color rgb="FF9C0006"/>
@@ -2807,413 +2828,403 @@
       </fill>
     </dxf>
     <dxf>
-      <font>
-        <color rgb="FF9C0006"/>
-      </font>
-      <fill>
-        <patternFill>
-          <bgColor rgb="FFFFC7CE"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <numFmt numFmtId="0" formatCode="General"/>
-    </dxf>
-    <dxf>
-      <numFmt numFmtId="0" formatCode="General"/>
-    </dxf>
-    <dxf>
-      <numFmt numFmtId="0" formatCode="General"/>
-    </dxf>
-    <dxf>
-      <numFmt numFmtId="0" formatCode="General"/>
-    </dxf>
-    <dxf>
-      <numFmt numFmtId="0" formatCode="General"/>
-    </dxf>
-    <dxf>
-      <numFmt numFmtId="0" formatCode="General"/>
-    </dxf>
-    <dxf>
-      <numFmt numFmtId="0" formatCode="General"/>
-    </dxf>
-    <dxf>
-      <numFmt numFmtId="0" formatCode="General"/>
-    </dxf>
-    <dxf>
-      <numFmt numFmtId="0" formatCode="General"/>
-    </dxf>
-    <dxf>
-      <numFmt numFmtId="0" formatCode="General"/>
-    </dxf>
-    <dxf>
-      <numFmt numFmtId="0" formatCode="General"/>
-    </dxf>
-    <dxf>
-      <numFmt numFmtId="0" formatCode="General"/>
-    </dxf>
-    <dxf>
-      <numFmt numFmtId="0" formatCode="General"/>
-    </dxf>
-    <dxf>
-      <numFmt numFmtId="0" formatCode="General"/>
-    </dxf>
-    <dxf>
-      <numFmt numFmtId="0" formatCode="General"/>
-    </dxf>
-    <dxf>
-      <numFmt numFmtId="0" formatCode="General"/>
-    </dxf>
-    <dxf>
-      <numFmt numFmtId="0" formatCode="General"/>
-    </dxf>
-    <dxf>
-      <numFmt numFmtId="0" formatCode="General"/>
-    </dxf>
-    <dxf>
-      <numFmt numFmtId="0" formatCode="General"/>
-    </dxf>
-    <dxf>
-      <numFmt numFmtId="0" formatCode="General"/>
-    </dxf>
-    <dxf>
-      <numFmt numFmtId="0" formatCode="General"/>
-    </dxf>
-    <dxf>
-      <numFmt numFmtId="0" formatCode="General"/>
-    </dxf>
-    <dxf>
-      <numFmt numFmtId="0" formatCode="General"/>
-    </dxf>
-    <dxf>
-      <numFmt numFmtId="0" formatCode="General"/>
-    </dxf>
-    <dxf>
-      <numFmt numFmtId="0" formatCode="General"/>
-    </dxf>
-    <dxf>
-      <numFmt numFmtId="0" formatCode="General"/>
-    </dxf>
-    <dxf>
-      <numFmt numFmtId="0" formatCode="General"/>
-    </dxf>
-    <dxf>
-      <numFmt numFmtId="0" formatCode="General"/>
-    </dxf>
-    <dxf>
-      <numFmt numFmtId="0" formatCode="General"/>
-    </dxf>
-    <dxf>
-      <numFmt numFmtId="0" formatCode="General"/>
-    </dxf>
-    <dxf>
-      <numFmt numFmtId="0" formatCode="General"/>
-    </dxf>
-    <dxf>
-      <numFmt numFmtId="0" formatCode="General"/>
-    </dxf>
-    <dxf>
-      <numFmt numFmtId="0" formatCode="General"/>
-    </dxf>
-    <dxf>
-      <numFmt numFmtId="0" formatCode="General"/>
-    </dxf>
-    <dxf>
-      <numFmt numFmtId="0" formatCode="General"/>
-    </dxf>
-    <dxf>
-      <numFmt numFmtId="0" formatCode="General"/>
-    </dxf>
-    <dxf>
-      <numFmt numFmtId="0" formatCode="General"/>
-    </dxf>
-    <dxf>
-      <numFmt numFmtId="0" formatCode="General"/>
-    </dxf>
-    <dxf>
-      <numFmt numFmtId="0" formatCode="General"/>
-    </dxf>
-    <dxf>
-      <numFmt numFmtId="0" formatCode="General"/>
-    </dxf>
-    <dxf>
-      <numFmt numFmtId="0" formatCode="General"/>
-    </dxf>
-    <dxf>
-      <numFmt numFmtId="0" formatCode="General"/>
-    </dxf>
-    <dxf>
-      <numFmt numFmtId="0" formatCode="General"/>
-    </dxf>
-    <dxf>
-      <numFmt numFmtId="0" formatCode="General"/>
-    </dxf>
-    <dxf>
-      <numFmt numFmtId="0" formatCode="General"/>
-    </dxf>
-    <dxf>
-      <numFmt numFmtId="0" formatCode="General"/>
-    </dxf>
-    <dxf>
-      <numFmt numFmtId="0" formatCode="General"/>
-    </dxf>
-    <dxf>
-      <numFmt numFmtId="0" formatCode="General"/>
-    </dxf>
-    <dxf>
-      <numFmt numFmtId="0" formatCode="General"/>
-    </dxf>
-    <dxf>
-      <numFmt numFmtId="0" formatCode="General"/>
-    </dxf>
-    <dxf>
-      <numFmt numFmtId="0" formatCode="General"/>
-    </dxf>
-    <dxf>
-      <numFmt numFmtId="0" formatCode="General"/>
-    </dxf>
-    <dxf>
-      <numFmt numFmtId="0" formatCode="General"/>
-    </dxf>
-    <dxf>
-      <numFmt numFmtId="0" formatCode="General"/>
-    </dxf>
-    <dxf>
-      <numFmt numFmtId="0" formatCode="General"/>
-    </dxf>
-    <dxf>
-      <numFmt numFmtId="0" formatCode="General"/>
-    </dxf>
-    <dxf>
-      <numFmt numFmtId="0" formatCode="General"/>
-    </dxf>
-    <dxf>
-      <numFmt numFmtId="0" formatCode="General"/>
-    </dxf>
-    <dxf>
-      <numFmt numFmtId="0" formatCode="General"/>
-    </dxf>
-    <dxf>
-      <numFmt numFmtId="0" formatCode="General"/>
-    </dxf>
-    <dxf>
-      <numFmt numFmtId="0" formatCode="General"/>
-    </dxf>
-    <dxf>
-      <numFmt numFmtId="0" formatCode="General"/>
-    </dxf>
-    <dxf>
-      <numFmt numFmtId="0" formatCode="General"/>
-    </dxf>
-    <dxf>
-      <numFmt numFmtId="0" formatCode="General"/>
-    </dxf>
-    <dxf>
-      <numFmt numFmtId="0" formatCode="General"/>
-    </dxf>
-    <dxf>
-      <numFmt numFmtId="0" formatCode="General"/>
-    </dxf>
-    <dxf>
-      <numFmt numFmtId="0" formatCode="General"/>
-    </dxf>
-    <dxf>
-      <numFmt numFmtId="0" formatCode="General"/>
-    </dxf>
-    <dxf>
-      <numFmt numFmtId="0" formatCode="General"/>
-    </dxf>
-    <dxf>
-      <numFmt numFmtId="0" formatCode="General"/>
-    </dxf>
-    <dxf>
-      <numFmt numFmtId="0" formatCode="General"/>
-    </dxf>
-    <dxf>
-      <numFmt numFmtId="0" formatCode="General"/>
-    </dxf>
-    <dxf>
-      <numFmt numFmtId="0" formatCode="General"/>
-    </dxf>
-    <dxf>
-      <numFmt numFmtId="0" formatCode="General"/>
-    </dxf>
-    <dxf>
-      <numFmt numFmtId="0" formatCode="General"/>
-    </dxf>
-    <dxf>
-      <numFmt numFmtId="0" formatCode="General"/>
-    </dxf>
-    <dxf>
-      <numFmt numFmtId="0" formatCode="General"/>
-    </dxf>
-    <dxf>
-      <numFmt numFmtId="0" formatCode="General"/>
-    </dxf>
-    <dxf>
-      <numFmt numFmtId="0" formatCode="General"/>
-    </dxf>
-    <dxf>
-      <numFmt numFmtId="0" formatCode="General"/>
-    </dxf>
-    <dxf>
-      <numFmt numFmtId="0" formatCode="General"/>
-    </dxf>
-    <dxf>
-      <numFmt numFmtId="0" formatCode="General"/>
-    </dxf>
-    <dxf>
-      <numFmt numFmtId="0" formatCode="General"/>
-    </dxf>
-    <dxf>
-      <numFmt numFmtId="0" formatCode="General"/>
-    </dxf>
-    <dxf>
-      <numFmt numFmtId="0" formatCode="General"/>
-    </dxf>
-    <dxf>
-      <numFmt numFmtId="0" formatCode="General"/>
-    </dxf>
-    <dxf>
-      <numFmt numFmtId="0" formatCode="General"/>
-    </dxf>
-    <dxf>
-      <numFmt numFmtId="0" formatCode="General"/>
-    </dxf>
-    <dxf>
-      <numFmt numFmtId="0" formatCode="General"/>
-    </dxf>
-    <dxf>
-      <numFmt numFmtId="0" formatCode="General"/>
-    </dxf>
-    <dxf>
-      <numFmt numFmtId="0" formatCode="General"/>
-    </dxf>
-    <dxf>
-      <numFmt numFmtId="0" formatCode="General"/>
-    </dxf>
-    <dxf>
-      <numFmt numFmtId="0" formatCode="General"/>
-    </dxf>
-    <dxf>
-      <numFmt numFmtId="0" formatCode="General"/>
-    </dxf>
-    <dxf>
-      <numFmt numFmtId="0" formatCode="General"/>
-    </dxf>
-    <dxf>
-      <numFmt numFmtId="0" formatCode="General"/>
-    </dxf>
-    <dxf>
-      <numFmt numFmtId="0" formatCode="General"/>
-    </dxf>
-    <dxf>
-      <numFmt numFmtId="0" formatCode="General"/>
-    </dxf>
-    <dxf>
-      <numFmt numFmtId="0" formatCode="General"/>
-    </dxf>
-    <dxf>
-      <numFmt numFmtId="0" formatCode="General"/>
-    </dxf>
-    <dxf>
-      <numFmt numFmtId="0" formatCode="General"/>
-    </dxf>
-    <dxf>
-      <numFmt numFmtId="0" formatCode="General"/>
-    </dxf>
-    <dxf>
-      <numFmt numFmtId="0" formatCode="General"/>
-    </dxf>
-    <dxf>
-      <numFmt numFmtId="0" formatCode="General"/>
-    </dxf>
-    <dxf>
-      <numFmt numFmtId="0" formatCode="General"/>
-    </dxf>
-    <dxf>
-      <numFmt numFmtId="0" formatCode="General"/>
-    </dxf>
-    <dxf>
-      <numFmt numFmtId="0" formatCode="General"/>
-    </dxf>
-    <dxf>
-      <numFmt numFmtId="0" formatCode="General"/>
-    </dxf>
-    <dxf>
-      <numFmt numFmtId="0" formatCode="General"/>
-    </dxf>
-    <dxf>
-      <numFmt numFmtId="0" formatCode="General"/>
-    </dxf>
-    <dxf>
-      <numFmt numFmtId="0" formatCode="General"/>
-    </dxf>
-    <dxf>
-      <numFmt numFmtId="0" formatCode="General"/>
-    </dxf>
-    <dxf>
-      <numFmt numFmtId="0" formatCode="General"/>
-    </dxf>
-    <dxf>
-      <numFmt numFmtId="0" formatCode="General"/>
-    </dxf>
-    <dxf>
-      <numFmt numFmtId="0" formatCode="General"/>
-    </dxf>
-    <dxf>
-      <numFmt numFmtId="0" formatCode="General"/>
-    </dxf>
-    <dxf>
-      <numFmt numFmtId="0" formatCode="General"/>
-    </dxf>
-    <dxf>
-      <numFmt numFmtId="0" formatCode="General"/>
-    </dxf>
-    <dxf>
-      <numFmt numFmtId="0" formatCode="General"/>
-    </dxf>
-    <dxf>
-      <numFmt numFmtId="0" formatCode="General"/>
-    </dxf>
-    <dxf>
-      <numFmt numFmtId="0" formatCode="General"/>
-    </dxf>
-    <dxf>
-      <numFmt numFmtId="0" formatCode="General"/>
-    </dxf>
-    <dxf>
-      <numFmt numFmtId="0" formatCode="General"/>
-    </dxf>
-    <dxf>
-      <numFmt numFmtId="0" formatCode="General"/>
-    </dxf>
-    <dxf>
-      <numFmt numFmtId="0" formatCode="General"/>
-    </dxf>
-    <dxf>
-      <numFmt numFmtId="0" formatCode="General"/>
-    </dxf>
-    <dxf>
-      <numFmt numFmtId="0" formatCode="General"/>
-    </dxf>
-    <dxf>
-      <numFmt numFmtId="0" formatCode="General"/>
-    </dxf>
-    <dxf>
-      <numFmt numFmtId="0" formatCode="General"/>
-    </dxf>
-    <dxf>
-      <numFmt numFmtId="0" formatCode="General"/>
-    </dxf>
-    <dxf>
-      <numFmt numFmtId="0" formatCode="General"/>
-    </dxf>
-    <dxf>
-      <numFmt numFmtId="0" formatCode="General"/>
-    </dxf>
-    <dxf>
-      <numFmt numFmtId="35" formatCode="_-* #,##0.00_-;\-* #,##0.00_-;_-* &quot;-&quot;??_-;_-@_-"/>
+      <numFmt numFmtId="0" formatCode="General"/>
+    </dxf>
+    <dxf>
+      <numFmt numFmtId="0" formatCode="General"/>
+    </dxf>
+    <dxf>
+      <numFmt numFmtId="0" formatCode="General"/>
+    </dxf>
+    <dxf>
+      <numFmt numFmtId="0" formatCode="General"/>
+    </dxf>
+    <dxf>
+      <numFmt numFmtId="0" formatCode="General"/>
+    </dxf>
+    <dxf>
+      <numFmt numFmtId="0" formatCode="General"/>
+    </dxf>
+    <dxf>
+      <numFmt numFmtId="0" formatCode="General"/>
+    </dxf>
+    <dxf>
+      <numFmt numFmtId="0" formatCode="General"/>
+    </dxf>
+    <dxf>
+      <numFmt numFmtId="0" formatCode="General"/>
+    </dxf>
+    <dxf>
+      <numFmt numFmtId="0" formatCode="General"/>
+    </dxf>
+    <dxf>
+      <numFmt numFmtId="0" formatCode="General"/>
+    </dxf>
+    <dxf>
+      <numFmt numFmtId="0" formatCode="General"/>
+    </dxf>
+    <dxf>
+      <numFmt numFmtId="0" formatCode="General"/>
+    </dxf>
+    <dxf>
+      <numFmt numFmtId="0" formatCode="General"/>
+    </dxf>
+    <dxf>
+      <numFmt numFmtId="0" formatCode="General"/>
+    </dxf>
+    <dxf>
+      <numFmt numFmtId="0" formatCode="General"/>
+    </dxf>
+    <dxf>
+      <numFmt numFmtId="0" formatCode="General"/>
+    </dxf>
+    <dxf>
+      <numFmt numFmtId="0" formatCode="General"/>
+    </dxf>
+    <dxf>
+      <numFmt numFmtId="0" formatCode="General"/>
+    </dxf>
+    <dxf>
+      <numFmt numFmtId="0" formatCode="General"/>
+    </dxf>
+    <dxf>
+      <numFmt numFmtId="0" formatCode="General"/>
+    </dxf>
+    <dxf>
+      <numFmt numFmtId="0" formatCode="General"/>
+    </dxf>
+    <dxf>
+      <numFmt numFmtId="0" formatCode="General"/>
+    </dxf>
+    <dxf>
+      <numFmt numFmtId="0" formatCode="General"/>
+    </dxf>
+    <dxf>
+      <numFmt numFmtId="0" formatCode="General"/>
+    </dxf>
+    <dxf>
+      <numFmt numFmtId="0" formatCode="General"/>
+    </dxf>
+    <dxf>
+      <numFmt numFmtId="0" formatCode="General"/>
+    </dxf>
+    <dxf>
+      <numFmt numFmtId="0" formatCode="General"/>
+    </dxf>
+    <dxf>
+      <numFmt numFmtId="0" formatCode="General"/>
+    </dxf>
+    <dxf>
+      <numFmt numFmtId="0" formatCode="General"/>
+    </dxf>
+    <dxf>
+      <numFmt numFmtId="0" formatCode="General"/>
+    </dxf>
+    <dxf>
+      <numFmt numFmtId="0" formatCode="General"/>
+    </dxf>
+    <dxf>
+      <numFmt numFmtId="0" formatCode="General"/>
+    </dxf>
+    <dxf>
+      <numFmt numFmtId="0" formatCode="General"/>
+    </dxf>
+    <dxf>
+      <numFmt numFmtId="0" formatCode="General"/>
+    </dxf>
+    <dxf>
+      <numFmt numFmtId="0" formatCode="General"/>
+    </dxf>
+    <dxf>
+      <numFmt numFmtId="0" formatCode="General"/>
+    </dxf>
+    <dxf>
+      <numFmt numFmtId="0" formatCode="General"/>
+    </dxf>
+    <dxf>
+      <numFmt numFmtId="0" formatCode="General"/>
+    </dxf>
+    <dxf>
+      <numFmt numFmtId="0" formatCode="General"/>
+    </dxf>
+    <dxf>
+      <numFmt numFmtId="0" formatCode="General"/>
+    </dxf>
+    <dxf>
+      <numFmt numFmtId="0" formatCode="General"/>
+    </dxf>
+    <dxf>
+      <numFmt numFmtId="0" formatCode="General"/>
+    </dxf>
+    <dxf>
+      <numFmt numFmtId="0" formatCode="General"/>
+    </dxf>
+    <dxf>
+      <numFmt numFmtId="0" formatCode="General"/>
+    </dxf>
+    <dxf>
+      <numFmt numFmtId="0" formatCode="General"/>
+    </dxf>
+    <dxf>
+      <numFmt numFmtId="0" formatCode="General"/>
+    </dxf>
+    <dxf>
+      <numFmt numFmtId="0" formatCode="General"/>
+    </dxf>
+    <dxf>
+      <numFmt numFmtId="0" formatCode="General"/>
+    </dxf>
+    <dxf>
+      <numFmt numFmtId="0" formatCode="General"/>
+    </dxf>
+    <dxf>
+      <numFmt numFmtId="0" formatCode="General"/>
+    </dxf>
+    <dxf>
+      <numFmt numFmtId="0" formatCode="General"/>
+    </dxf>
+    <dxf>
+      <numFmt numFmtId="0" formatCode="General"/>
+    </dxf>
+    <dxf>
+      <numFmt numFmtId="0" formatCode="General"/>
+    </dxf>
+    <dxf>
+      <numFmt numFmtId="0" formatCode="General"/>
+    </dxf>
+    <dxf>
+      <numFmt numFmtId="0" formatCode="General"/>
+    </dxf>
+    <dxf>
+      <numFmt numFmtId="0" formatCode="General"/>
+    </dxf>
+    <dxf>
+      <numFmt numFmtId="0" formatCode="General"/>
+    </dxf>
+    <dxf>
+      <numFmt numFmtId="0" formatCode="General"/>
+    </dxf>
+    <dxf>
+      <numFmt numFmtId="0" formatCode="General"/>
+    </dxf>
+    <dxf>
+      <numFmt numFmtId="0" formatCode="General"/>
+    </dxf>
+    <dxf>
+      <numFmt numFmtId="0" formatCode="General"/>
+    </dxf>
+    <dxf>
+      <numFmt numFmtId="0" formatCode="General"/>
+    </dxf>
+    <dxf>
+      <numFmt numFmtId="0" formatCode="General"/>
+    </dxf>
+    <dxf>
+      <numFmt numFmtId="0" formatCode="General"/>
+    </dxf>
+    <dxf>
+      <numFmt numFmtId="0" formatCode="General"/>
+    </dxf>
+    <dxf>
+      <numFmt numFmtId="0" formatCode="General"/>
+    </dxf>
+    <dxf>
+      <numFmt numFmtId="0" formatCode="General"/>
+    </dxf>
+    <dxf>
+      <numFmt numFmtId="0" formatCode="General"/>
+    </dxf>
+    <dxf>
+      <numFmt numFmtId="0" formatCode="General"/>
+    </dxf>
+    <dxf>
+      <numFmt numFmtId="0" formatCode="General"/>
+    </dxf>
+    <dxf>
+      <numFmt numFmtId="0" formatCode="General"/>
+    </dxf>
+    <dxf>
+      <numFmt numFmtId="0" formatCode="General"/>
+    </dxf>
+    <dxf>
+      <numFmt numFmtId="0" formatCode="General"/>
+    </dxf>
+    <dxf>
+      <numFmt numFmtId="0" formatCode="General"/>
+    </dxf>
+    <dxf>
+      <numFmt numFmtId="0" formatCode="General"/>
+    </dxf>
+    <dxf>
+      <numFmt numFmtId="0" formatCode="General"/>
+    </dxf>
+    <dxf>
+      <numFmt numFmtId="0" formatCode="General"/>
+    </dxf>
+    <dxf>
+      <numFmt numFmtId="0" formatCode="General"/>
+    </dxf>
+    <dxf>
+      <numFmt numFmtId="0" formatCode="General"/>
+    </dxf>
+    <dxf>
+      <numFmt numFmtId="0" formatCode="General"/>
+    </dxf>
+    <dxf>
+      <numFmt numFmtId="0" formatCode="General"/>
+    </dxf>
+    <dxf>
+      <numFmt numFmtId="0" formatCode="General"/>
+    </dxf>
+    <dxf>
+      <numFmt numFmtId="0" formatCode="General"/>
+    </dxf>
+    <dxf>
+      <numFmt numFmtId="0" formatCode="General"/>
+    </dxf>
+    <dxf>
+      <numFmt numFmtId="0" formatCode="General"/>
+    </dxf>
+    <dxf>
+      <numFmt numFmtId="0" formatCode="General"/>
+    </dxf>
+    <dxf>
+      <numFmt numFmtId="0" formatCode="General"/>
+    </dxf>
+    <dxf>
+      <numFmt numFmtId="0" formatCode="General"/>
+    </dxf>
+    <dxf>
+      <numFmt numFmtId="0" formatCode="General"/>
+    </dxf>
+    <dxf>
+      <numFmt numFmtId="0" formatCode="General"/>
+    </dxf>
+    <dxf>
+      <numFmt numFmtId="0" formatCode="General"/>
+    </dxf>
+    <dxf>
+      <numFmt numFmtId="0" formatCode="General"/>
+    </dxf>
+    <dxf>
+      <numFmt numFmtId="0" formatCode="General"/>
+    </dxf>
+    <dxf>
+      <numFmt numFmtId="0" formatCode="General"/>
+    </dxf>
+    <dxf>
+      <numFmt numFmtId="0" formatCode="General"/>
+    </dxf>
+    <dxf>
+      <numFmt numFmtId="0" formatCode="General"/>
+    </dxf>
+    <dxf>
+      <numFmt numFmtId="0" formatCode="General"/>
+    </dxf>
+    <dxf>
+      <numFmt numFmtId="0" formatCode="General"/>
+    </dxf>
+    <dxf>
+      <numFmt numFmtId="0" formatCode="General"/>
+    </dxf>
+    <dxf>
+      <numFmt numFmtId="0" formatCode="General"/>
+    </dxf>
+    <dxf>
+      <numFmt numFmtId="0" formatCode="General"/>
+    </dxf>
+    <dxf>
+      <numFmt numFmtId="0" formatCode="General"/>
+    </dxf>
+    <dxf>
+      <numFmt numFmtId="0" formatCode="General"/>
+    </dxf>
+    <dxf>
+      <numFmt numFmtId="0" formatCode="General"/>
+    </dxf>
+    <dxf>
+      <numFmt numFmtId="0" formatCode="General"/>
+    </dxf>
+    <dxf>
+      <numFmt numFmtId="0" formatCode="General"/>
+    </dxf>
+    <dxf>
+      <numFmt numFmtId="0" formatCode="General"/>
+    </dxf>
+    <dxf>
+      <numFmt numFmtId="0" formatCode="General"/>
+    </dxf>
+    <dxf>
+      <numFmt numFmtId="0" formatCode="General"/>
+    </dxf>
+    <dxf>
+      <numFmt numFmtId="0" formatCode="General"/>
+    </dxf>
+    <dxf>
+      <numFmt numFmtId="0" formatCode="General"/>
+    </dxf>
+    <dxf>
+      <numFmt numFmtId="0" formatCode="General"/>
+    </dxf>
+    <dxf>
+      <numFmt numFmtId="0" formatCode="General"/>
+    </dxf>
+    <dxf>
+      <numFmt numFmtId="0" formatCode="General"/>
+    </dxf>
+    <dxf>
+      <numFmt numFmtId="0" formatCode="General"/>
+    </dxf>
+    <dxf>
+      <numFmt numFmtId="0" formatCode="General"/>
+    </dxf>
+    <dxf>
+      <numFmt numFmtId="0" formatCode="General"/>
+    </dxf>
+    <dxf>
+      <numFmt numFmtId="0" formatCode="General"/>
+    </dxf>
+    <dxf>
+      <numFmt numFmtId="0" formatCode="General"/>
+    </dxf>
+    <dxf>
+      <numFmt numFmtId="0" formatCode="General"/>
+    </dxf>
+    <dxf>
+      <numFmt numFmtId="0" formatCode="General"/>
+    </dxf>
+    <dxf>
+      <numFmt numFmtId="0" formatCode="General"/>
+    </dxf>
+    <dxf>
+      <numFmt numFmtId="0" formatCode="General"/>
+    </dxf>
+    <dxf>
+      <numFmt numFmtId="0" formatCode="General"/>
+    </dxf>
+    <dxf>
+      <numFmt numFmtId="0" formatCode="General"/>
+    </dxf>
+    <dxf>
+      <numFmt numFmtId="0" formatCode="General"/>
+    </dxf>
+    <dxf>
+      <numFmt numFmtId="0" formatCode="General"/>
+    </dxf>
+    <dxf>
+      <numFmt numFmtId="0" formatCode="General"/>
+    </dxf>
+    <dxf>
+      <numFmt numFmtId="0" formatCode="General"/>
+    </dxf>
+    <dxf>
+      <numFmt numFmtId="0" formatCode="General"/>
+    </dxf>
+    <dxf>
+      <numFmt numFmtId="0" formatCode="General"/>
+    </dxf>
+    <dxf>
+      <numFmt numFmtId="164" formatCode="_-* #,##0.00_-;\-* #,##0.00_-;_-* &quot;-&quot;??_-;_-@_-"/>
       <fill>
         <patternFill patternType="none">
           <fgColor indexed="64"/>
@@ -5092,21 +5103,21 @@
 </file>
 
 <file path=xl/tables/table1.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="20" xr:uid="{DF067A72-54A6-48F4-972D-2DE4603D61A4}" name="Table20" displayName="Table20" ref="A1:I69" totalsRowShown="0" headerRowDxfId="154" headerRowBorderDxfId="153" tableBorderDxfId="152" totalsRowBorderDxfId="151">
-  <autoFilter ref="A1:I69" xr:uid="{DF067A72-54A6-48F4-972D-2DE4603D61A4}"/>
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="20" xr:uid="{DF067A72-54A6-48F4-972D-2DE4603D61A4}" name="Table20" displayName="Table20" ref="A1:I70" totalsRowShown="0" headerRowDxfId="153" headerRowBorderDxfId="152" tableBorderDxfId="151" totalsRowBorderDxfId="150">
+  <autoFilter ref="A1:I70" xr:uid="{DF067A72-54A6-48F4-972D-2DE4603D61A4}"/>
   <sortState xmlns:xlrd2="http://schemas.microsoft.com/office/spreadsheetml/2017/richdata2" ref="A2:I57">
     <sortCondition ref="H1:H57"/>
   </sortState>
   <tableColumns count="9">
-    <tableColumn id="1" xr3:uid="{0E6335F2-6B6A-436C-92FA-B48E61551308}" name="Merek/Type" dataDxfId="150"/>
-    <tableColumn id="2" xr3:uid="{5A4965DA-398A-4134-90BD-9CE4D8355880}" name="Tipe" dataDxfId="149"/>
-    <tableColumn id="3" xr3:uid="{010303D1-E0A2-4DE6-8E87-64ACC3102E09}" name="Harga OTR Awal" dataDxfId="148" dataCellStyle="Comma"/>
-    <tableColumn id="4" xr3:uid="{91C798B0-7964-436A-84A5-7687993F376F}" name="Dealer Margin" dataDxfId="147" dataCellStyle="Comma"/>
-    <tableColumn id="5" xr3:uid="{CD936623-36F3-4BAA-A615-AF79A61C51E8}" name="Dealer Margin 9 %" dataDxfId="146" dataCellStyle="Comma"/>
-    <tableColumn id="6" xr3:uid="{A36173E8-D9B2-4F38-A572-F5D32CDADEB8}" name="Dealer Margin 7 %" dataDxfId="145" dataCellStyle="Comma"/>
-    <tableColumn id="7" xr3:uid="{7A11B7F5-7683-492A-A8B5-D96984323DDD}" name="Code Unit" dataDxfId="144"/>
-    <tableColumn id="8" xr3:uid="{AF243BB3-2044-4D1E-9F0D-A1EC0D2C15CF}" name="Merk/Type" dataDxfId="143"/>
-    <tableColumn id="9" xr3:uid="{9E0E2E6A-108F-4ACE-959D-9EB0F753BD73}" name="Full Margin" dataDxfId="142"/>
+    <tableColumn id="1" xr3:uid="{0E6335F2-6B6A-436C-92FA-B48E61551308}" name="Merek/Type" dataDxfId="149"/>
+    <tableColumn id="2" xr3:uid="{5A4965DA-398A-4134-90BD-9CE4D8355880}" name="Tipe" dataDxfId="148"/>
+    <tableColumn id="3" xr3:uid="{010303D1-E0A2-4DE6-8E87-64ACC3102E09}" name="Harga OTR Awal" dataDxfId="147" dataCellStyle="Comma"/>
+    <tableColumn id="4" xr3:uid="{91C798B0-7964-436A-84A5-7687993F376F}" name="Dealer Margin" dataDxfId="146" dataCellStyle="Comma"/>
+    <tableColumn id="5" xr3:uid="{CD936623-36F3-4BAA-A615-AF79A61C51E8}" name="Dealer Margin 9 %" dataDxfId="145" dataCellStyle="Comma"/>
+    <tableColumn id="6" xr3:uid="{A36173E8-D9B2-4F38-A572-F5D32CDADEB8}" name="Dealer Margin 7 %" dataDxfId="144" dataCellStyle="Comma"/>
+    <tableColumn id="7" xr3:uid="{7A11B7F5-7683-492A-A8B5-D96984323DDD}" name="Code Unit" dataDxfId="143"/>
+    <tableColumn id="8" xr3:uid="{AF243BB3-2044-4D1E-9F0D-A1EC0D2C15CF}" name="Merk/Type" dataDxfId="142"/>
+    <tableColumn id="9" xr3:uid="{9E0E2E6A-108F-4ACE-959D-9EB0F753BD73}" name="Full Margin" dataDxfId="141"/>
   </tableColumns>
   <tableStyleInfo name="TableStyleMedium2" showFirstColumn="0" showLastColumn="0" showRowStripes="1" showColumnStripes="0"/>
 </table>
@@ -5116,15 +5127,15 @@
 <table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="9" xr:uid="{630D8221-A5B4-4162-BEFC-7BB63825B861}" name="Table009__Page_6" displayName="Table009__Page_6" ref="A1:I16" tableType="queryTable" totalsRowShown="0">
   <autoFilter ref="A1:I16" xr:uid="{630D8221-A5B4-4162-BEFC-7BB63825B861}"/>
   <tableColumns count="9">
-    <tableColumn id="1" xr3:uid="{5980B244-73E4-43AF-B863-305E8B039C33}" uniqueName="1" name="Column1" queryTableFieldId="1" dataDxfId="75"/>
-    <tableColumn id="2" xr3:uid="{549208EE-7E07-4F0F-ACFD-9606CC8F6B50}" uniqueName="2" name="Column2" queryTableFieldId="2" dataDxfId="74"/>
-    <tableColumn id="3" xr3:uid="{086F7B88-A201-47FD-B9A0-0C976108E144}" uniqueName="3" name="Column3" queryTableFieldId="3" dataDxfId="73"/>
-    <tableColumn id="4" xr3:uid="{CC912184-CE02-4DC9-8815-71C4295C86DF}" uniqueName="4" name="Column4" queryTableFieldId="4" dataDxfId="72"/>
-    <tableColumn id="5" xr3:uid="{8F3F2202-7C07-4D43-B483-871C9E242208}" uniqueName="5" name="Column5" queryTableFieldId="5" dataDxfId="71"/>
-    <tableColumn id="6" xr3:uid="{6D2190D6-B434-4BB9-95B1-A29148C453AF}" uniqueName="6" name="Column6" queryTableFieldId="6" dataDxfId="70"/>
-    <tableColumn id="7" xr3:uid="{A33DE0AF-7DA7-4623-87E7-DBA2BF4E404A}" uniqueName="7" name="Column7" queryTableFieldId="7" dataDxfId="69"/>
-    <tableColumn id="8" xr3:uid="{CD689B59-BA44-4F67-9FF9-E08337BE66FD}" uniqueName="8" name="Column8" queryTableFieldId="8" dataDxfId="68"/>
-    <tableColumn id="9" xr3:uid="{744F224A-BA1E-4758-B291-8D5C8D341610}" uniqueName="9" name="Column9" queryTableFieldId="9" dataDxfId="67"/>
+    <tableColumn id="1" xr3:uid="{5980B244-73E4-43AF-B863-305E8B039C33}" uniqueName="1" name="Column1" queryTableFieldId="1" dataDxfId="74"/>
+    <tableColumn id="2" xr3:uid="{549208EE-7E07-4F0F-ACFD-9606CC8F6B50}" uniqueName="2" name="Column2" queryTableFieldId="2" dataDxfId="73"/>
+    <tableColumn id="3" xr3:uid="{086F7B88-A201-47FD-B9A0-0C976108E144}" uniqueName="3" name="Column3" queryTableFieldId="3" dataDxfId="72"/>
+    <tableColumn id="4" xr3:uid="{CC912184-CE02-4DC9-8815-71C4295C86DF}" uniqueName="4" name="Column4" queryTableFieldId="4" dataDxfId="71"/>
+    <tableColumn id="5" xr3:uid="{8F3F2202-7C07-4D43-B483-871C9E242208}" uniqueName="5" name="Column5" queryTableFieldId="5" dataDxfId="70"/>
+    <tableColumn id="6" xr3:uid="{6D2190D6-B434-4BB9-95B1-A29148C453AF}" uniqueName="6" name="Column6" queryTableFieldId="6" dataDxfId="69"/>
+    <tableColumn id="7" xr3:uid="{A33DE0AF-7DA7-4623-87E7-DBA2BF4E404A}" uniqueName="7" name="Column7" queryTableFieldId="7" dataDxfId="68"/>
+    <tableColumn id="8" xr3:uid="{CD689B59-BA44-4F67-9FF9-E08337BE66FD}" uniqueName="8" name="Column8" queryTableFieldId="8" dataDxfId="67"/>
+    <tableColumn id="9" xr3:uid="{744F224A-BA1E-4758-B291-8D5C8D341610}" uniqueName="9" name="Column9" queryTableFieldId="9" dataDxfId="66"/>
   </tableColumns>
   <tableStyleInfo name="TableStyleMedium7" showFirstColumn="0" showLastColumn="0" showRowStripes="1" showColumnStripes="0"/>
 </table>
@@ -5134,15 +5145,15 @@
 <table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="10" xr:uid="{116BBD7B-F856-4C44-8F1F-EA66756E3A0B}" name="Table010__Page_6" displayName="Table010__Page_6" ref="A18:I20" tableType="queryTable" totalsRowShown="0">
   <autoFilter ref="A18:I20" xr:uid="{116BBD7B-F856-4C44-8F1F-EA66756E3A0B}"/>
   <tableColumns count="9">
-    <tableColumn id="1" xr3:uid="{D02866AC-7C8C-4041-B0D6-297717EA2BCA}" uniqueName="1" name="Column1" queryTableFieldId="1" dataDxfId="66"/>
-    <tableColumn id="2" xr3:uid="{F9BA0334-AC0F-4599-91DD-1D3B53530BA2}" uniqueName="2" name="Column2" queryTableFieldId="2" dataDxfId="65"/>
-    <tableColumn id="3" xr3:uid="{2E40CB08-FF90-4211-A5F6-3255AA5CEAED}" uniqueName="3" name="Column3" queryTableFieldId="3" dataDxfId="64"/>
-    <tableColumn id="4" xr3:uid="{951E49DE-3DB8-41C0-8F36-6E5A1649659D}" uniqueName="4" name="Column4" queryTableFieldId="4" dataDxfId="63"/>
-    <tableColumn id="5" xr3:uid="{D7FC7D23-AA29-4FAE-8DF4-B23A11020D8C}" uniqueName="5" name="Column5" queryTableFieldId="5" dataDxfId="62"/>
-    <tableColumn id="6" xr3:uid="{85DA6C7C-BC56-4316-BB56-3D2CA86DF4B0}" uniqueName="6" name="Column6" queryTableFieldId="6" dataDxfId="61"/>
-    <tableColumn id="7" xr3:uid="{47F39228-8CCC-4319-9964-568280350AF4}" uniqueName="7" name="Column7" queryTableFieldId="7" dataDxfId="60"/>
-    <tableColumn id="8" xr3:uid="{781188CD-5AC0-41B9-8575-2EACD4BA90A4}" uniqueName="8" name="Column8" queryTableFieldId="8" dataDxfId="59"/>
-    <tableColumn id="9" xr3:uid="{A2DFBEC8-960F-4613-A8B8-821CF42818AC}" uniqueName="9" name="Column9" queryTableFieldId="9" dataDxfId="58"/>
+    <tableColumn id="1" xr3:uid="{D02866AC-7C8C-4041-B0D6-297717EA2BCA}" uniqueName="1" name="Column1" queryTableFieldId="1" dataDxfId="65"/>
+    <tableColumn id="2" xr3:uid="{F9BA0334-AC0F-4599-91DD-1D3B53530BA2}" uniqueName="2" name="Column2" queryTableFieldId="2" dataDxfId="64"/>
+    <tableColumn id="3" xr3:uid="{2E40CB08-FF90-4211-A5F6-3255AA5CEAED}" uniqueName="3" name="Column3" queryTableFieldId="3" dataDxfId="63"/>
+    <tableColumn id="4" xr3:uid="{951E49DE-3DB8-41C0-8F36-6E5A1649659D}" uniqueName="4" name="Column4" queryTableFieldId="4" dataDxfId="62"/>
+    <tableColumn id="5" xr3:uid="{D7FC7D23-AA29-4FAE-8DF4-B23A11020D8C}" uniqueName="5" name="Column5" queryTableFieldId="5" dataDxfId="61"/>
+    <tableColumn id="6" xr3:uid="{85DA6C7C-BC56-4316-BB56-3D2CA86DF4B0}" uniqueName="6" name="Column6" queryTableFieldId="6" dataDxfId="60"/>
+    <tableColumn id="7" xr3:uid="{47F39228-8CCC-4319-9964-568280350AF4}" uniqueName="7" name="Column7" queryTableFieldId="7" dataDxfId="59"/>
+    <tableColumn id="8" xr3:uid="{781188CD-5AC0-41B9-8575-2EACD4BA90A4}" uniqueName="8" name="Column8" queryTableFieldId="8" dataDxfId="58"/>
+    <tableColumn id="9" xr3:uid="{A2DFBEC8-960F-4613-A8B8-821CF42818AC}" uniqueName="9" name="Column9" queryTableFieldId="9" dataDxfId="57"/>
   </tableColumns>
   <tableStyleInfo name="TableStyleMedium7" showFirstColumn="0" showLastColumn="0" showRowStripes="1" showColumnStripes="0"/>
 </table>
@@ -5152,9 +5163,9 @@
 <table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="11" xr:uid="{D5A80464-2F5E-4F81-BC09-642A89962C82}" name="Table011__Page_7" displayName="Table011__Page_7" ref="A1:C15" tableType="queryTable" totalsRowShown="0">
   <autoFilter ref="A1:C15" xr:uid="{D5A80464-2F5E-4F81-BC09-642A89962C82}"/>
   <tableColumns count="3">
-    <tableColumn id="1" xr3:uid="{384F6B08-E7B1-4ECD-BC7E-1F8C8FC9CD11}" uniqueName="1" name="Column1" queryTableFieldId="1" dataDxfId="57"/>
-    <tableColumn id="2" xr3:uid="{BD116665-54B3-487B-82AD-7E260403FB1A}" uniqueName="2" name="Column2" queryTableFieldId="2" dataDxfId="56"/>
-    <tableColumn id="3" xr3:uid="{A0C72322-3C63-446F-A7B0-E45538411191}" uniqueName="3" name="Column3" queryTableFieldId="3" dataDxfId="55"/>
+    <tableColumn id="1" xr3:uid="{384F6B08-E7B1-4ECD-BC7E-1F8C8FC9CD11}" uniqueName="1" name="Column1" queryTableFieldId="1" dataDxfId="56"/>
+    <tableColumn id="2" xr3:uid="{BD116665-54B3-487B-82AD-7E260403FB1A}" uniqueName="2" name="Column2" queryTableFieldId="2" dataDxfId="55"/>
+    <tableColumn id="3" xr3:uid="{A0C72322-3C63-446F-A7B0-E45538411191}" uniqueName="3" name="Column3" queryTableFieldId="3" dataDxfId="54"/>
   </tableColumns>
   <tableStyleInfo name="TableStyleMedium7" showFirstColumn="0" showLastColumn="0" showRowStripes="1" showColumnStripes="0"/>
 </table>
@@ -5164,9 +5175,9 @@
 <table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="12" xr:uid="{BF5A7D5F-42BD-4927-9517-2459449E72C6}" name="Table012__Page_7" displayName="Table012__Page_7" ref="A17:C19" tableType="queryTable" totalsRowShown="0">
   <autoFilter ref="A17:C19" xr:uid="{BF5A7D5F-42BD-4927-9517-2459449E72C6}"/>
   <tableColumns count="3">
-    <tableColumn id="1" xr3:uid="{92B56AD9-FE6F-4702-B777-811CB1B6E64F}" uniqueName="1" name="Column1" queryTableFieldId="1" dataDxfId="54"/>
-    <tableColumn id="2" xr3:uid="{C37743D7-7886-43A1-BB26-C0F3914426C9}" uniqueName="2" name="Column2" queryTableFieldId="2" dataDxfId="53"/>
-    <tableColumn id="3" xr3:uid="{DFF6BFBF-623A-4318-86AF-C5448FC821A5}" uniqueName="3" name="Column3" queryTableFieldId="3" dataDxfId="52"/>
+    <tableColumn id="1" xr3:uid="{92B56AD9-FE6F-4702-B777-811CB1B6E64F}" uniqueName="1" name="Column1" queryTableFieldId="1" dataDxfId="53"/>
+    <tableColumn id="2" xr3:uid="{C37743D7-7886-43A1-BB26-C0F3914426C9}" uniqueName="2" name="Column2" queryTableFieldId="2" dataDxfId="52"/>
+    <tableColumn id="3" xr3:uid="{DFF6BFBF-623A-4318-86AF-C5448FC821A5}" uniqueName="3" name="Column3" queryTableFieldId="3" dataDxfId="51"/>
   </tableColumns>
   <tableStyleInfo name="TableStyleMedium7" showFirstColumn="0" showLastColumn="0" showRowStripes="1" showColumnStripes="0"/>
 </table>
@@ -5176,11 +5187,11 @@
 <table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="13" xr:uid="{4DAA9679-BE71-4F3A-B608-132984AF6DF1}" name="Table013__Page_8" displayName="Table013__Page_8" ref="A1:E16" tableType="queryTable" totalsRowShown="0">
   <autoFilter ref="A1:E16" xr:uid="{4DAA9679-BE71-4F3A-B608-132984AF6DF1}"/>
   <tableColumns count="5">
-    <tableColumn id="1" xr3:uid="{811DEB23-A3B8-4E1E-AF98-CBD4FE9515C8}" uniqueName="1" name="Column1" queryTableFieldId="1" dataDxfId="51"/>
-    <tableColumn id="2" xr3:uid="{D1233A63-9D37-45F3-9DC7-52977AC06ADC}" uniqueName="2" name="Column2" queryTableFieldId="2" dataDxfId="50"/>
-    <tableColumn id="3" xr3:uid="{400191B1-4CF8-4D78-82E7-FED7CD6730E6}" uniqueName="3" name="Column3" queryTableFieldId="3" dataDxfId="49"/>
-    <tableColumn id="4" xr3:uid="{3D829CC4-4292-4CD0-80B8-3490D4014AC9}" uniqueName="4" name="Column4" queryTableFieldId="4" dataDxfId="48"/>
-    <tableColumn id="5" xr3:uid="{9BC50CF1-EF44-42B4-9129-E887F74428C9}" uniqueName="5" name="Column5" queryTableFieldId="5" dataDxfId="47"/>
+    <tableColumn id="1" xr3:uid="{811DEB23-A3B8-4E1E-AF98-CBD4FE9515C8}" uniqueName="1" name="Column1" queryTableFieldId="1" dataDxfId="50"/>
+    <tableColumn id="2" xr3:uid="{D1233A63-9D37-45F3-9DC7-52977AC06ADC}" uniqueName="2" name="Column2" queryTableFieldId="2" dataDxfId="49"/>
+    <tableColumn id="3" xr3:uid="{400191B1-4CF8-4D78-82E7-FED7CD6730E6}" uniqueName="3" name="Column3" queryTableFieldId="3" dataDxfId="48"/>
+    <tableColumn id="4" xr3:uid="{3D829CC4-4292-4CD0-80B8-3490D4014AC9}" uniqueName="4" name="Column4" queryTableFieldId="4" dataDxfId="47"/>
+    <tableColumn id="5" xr3:uid="{9BC50CF1-EF44-42B4-9129-E887F74428C9}" uniqueName="5" name="Column5" queryTableFieldId="5" dataDxfId="46"/>
   </tableColumns>
   <tableStyleInfo name="TableStyleMedium7" showFirstColumn="0" showLastColumn="0" showRowStripes="1" showColumnStripes="0"/>
 </table>
@@ -5190,11 +5201,11 @@
 <table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="14" xr:uid="{9D3195A8-F1BD-4429-B95A-60FCF241B775}" name="Table014__Page_8" displayName="Table014__Page_8" ref="A18:E21" tableType="queryTable" totalsRowShown="0">
   <autoFilter ref="A18:E21" xr:uid="{9D3195A8-F1BD-4429-B95A-60FCF241B775}"/>
   <tableColumns count="5">
-    <tableColumn id="1" xr3:uid="{98A6121C-2EC1-48CA-8A40-28DAFD66423E}" uniqueName="1" name="Column1" queryTableFieldId="1" dataDxfId="46"/>
-    <tableColumn id="2" xr3:uid="{6B521FB3-E639-4556-B8C5-473A63201BC1}" uniqueName="2" name="Column2" queryTableFieldId="2" dataDxfId="45"/>
-    <tableColumn id="3" xr3:uid="{3D07F9E9-4DA3-41C6-98A7-BC28F0C8BFB5}" uniqueName="3" name="Column3" queryTableFieldId="3" dataDxfId="44"/>
-    <tableColumn id="4" xr3:uid="{89F1E0D5-9B1D-4170-BB1D-3FBA7855FC27}" uniqueName="4" name="Column4" queryTableFieldId="4" dataDxfId="43"/>
-    <tableColumn id="5" xr3:uid="{68E29A0D-4E20-4E2A-A030-157EF3C69E97}" uniqueName="5" name="Column5" queryTableFieldId="5" dataDxfId="42"/>
+    <tableColumn id="1" xr3:uid="{98A6121C-2EC1-48CA-8A40-28DAFD66423E}" uniqueName="1" name="Column1" queryTableFieldId="1" dataDxfId="45"/>
+    <tableColumn id="2" xr3:uid="{6B521FB3-E639-4556-B8C5-473A63201BC1}" uniqueName="2" name="Column2" queryTableFieldId="2" dataDxfId="44"/>
+    <tableColumn id="3" xr3:uid="{3D07F9E9-4DA3-41C6-98A7-BC28F0C8BFB5}" uniqueName="3" name="Column3" queryTableFieldId="3" dataDxfId="43"/>
+    <tableColumn id="4" xr3:uid="{89F1E0D5-9B1D-4170-BB1D-3FBA7855FC27}" uniqueName="4" name="Column4" queryTableFieldId="4" dataDxfId="42"/>
+    <tableColumn id="5" xr3:uid="{68E29A0D-4E20-4E2A-A030-157EF3C69E97}" uniqueName="5" name="Column5" queryTableFieldId="5" dataDxfId="41"/>
   </tableColumns>
   <tableStyleInfo name="TableStyleMedium7" showFirstColumn="0" showLastColumn="0" showRowStripes="1" showColumnStripes="0"/>
 </table>
@@ -5204,12 +5215,12 @@
 <table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="15" xr:uid="{F2B12C92-B774-477F-98C9-509526BBDEE5}" name="Table015__Page_9" displayName="Table015__Page_9" ref="A1:F16" tableType="queryTable" totalsRowShown="0">
   <autoFilter ref="A1:F16" xr:uid="{F2B12C92-B774-477F-98C9-509526BBDEE5}"/>
   <tableColumns count="6">
-    <tableColumn id="1" xr3:uid="{B9D47F1B-922B-4B02-855C-93AF62167342}" uniqueName="1" name="Column1" queryTableFieldId="1" dataDxfId="41"/>
-    <tableColumn id="2" xr3:uid="{9915D8BD-1C99-4D36-BE7E-9EBEAD6D7B12}" uniqueName="2" name="Column2" queryTableFieldId="2" dataDxfId="40"/>
-    <tableColumn id="3" xr3:uid="{D353D58B-6A1D-4079-A9EC-77376B67A375}" uniqueName="3" name="Column3" queryTableFieldId="3" dataDxfId="39"/>
-    <tableColumn id="4" xr3:uid="{ACF53426-7425-4D38-9673-B3197A3F9292}" uniqueName="4" name="Column4" queryTableFieldId="4" dataDxfId="38"/>
-    <tableColumn id="5" xr3:uid="{673A9374-D6DA-46D7-AAD2-6F2220F4ED8C}" uniqueName="5" name="Column5" queryTableFieldId="5" dataDxfId="37"/>
-    <tableColumn id="6" xr3:uid="{37C428F9-0692-44D1-B8CF-2CBC7901020B}" uniqueName="6" name="Column6" queryTableFieldId="6" dataDxfId="36"/>
+    <tableColumn id="1" xr3:uid="{B9D47F1B-922B-4B02-855C-93AF62167342}" uniqueName="1" name="Column1" queryTableFieldId="1" dataDxfId="40"/>
+    <tableColumn id="2" xr3:uid="{9915D8BD-1C99-4D36-BE7E-9EBEAD6D7B12}" uniqueName="2" name="Column2" queryTableFieldId="2" dataDxfId="39"/>
+    <tableColumn id="3" xr3:uid="{D353D58B-6A1D-4079-A9EC-77376B67A375}" uniqueName="3" name="Column3" queryTableFieldId="3" dataDxfId="38"/>
+    <tableColumn id="4" xr3:uid="{ACF53426-7425-4D38-9673-B3197A3F9292}" uniqueName="4" name="Column4" queryTableFieldId="4" dataDxfId="37"/>
+    <tableColumn id="5" xr3:uid="{673A9374-D6DA-46D7-AAD2-6F2220F4ED8C}" uniqueName="5" name="Column5" queryTableFieldId="5" dataDxfId="36"/>
+    <tableColumn id="6" xr3:uid="{37C428F9-0692-44D1-B8CF-2CBC7901020B}" uniqueName="6" name="Column6" queryTableFieldId="6" dataDxfId="35"/>
   </tableColumns>
   <tableStyleInfo name="TableStyleMedium7" showFirstColumn="0" showLastColumn="0" showRowStripes="1" showColumnStripes="0"/>
 </table>
@@ -5219,12 +5230,12 @@
 <table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="16" xr:uid="{3C596C1A-3A31-47DF-B534-2A3593167FFF}" name="Table016__Page_9" displayName="Table016__Page_9" ref="A18:F20" tableType="queryTable" totalsRowShown="0">
   <autoFilter ref="A18:F20" xr:uid="{3C596C1A-3A31-47DF-B534-2A3593167FFF}"/>
   <tableColumns count="6">
-    <tableColumn id="1" xr3:uid="{48EBD4D1-26EB-449F-8D09-DF1A8D9D96A3}" uniqueName="1" name="Column1" queryTableFieldId="1" dataDxfId="35"/>
-    <tableColumn id="2" xr3:uid="{671AE648-452F-44F1-9A65-8468F7B19950}" uniqueName="2" name="Column2" queryTableFieldId="2" dataDxfId="34"/>
-    <tableColumn id="3" xr3:uid="{C3287937-E8A8-4D80-A27C-D2A5C0E44D68}" uniqueName="3" name="Column3" queryTableFieldId="3" dataDxfId="33"/>
-    <tableColumn id="4" xr3:uid="{49CAB777-0355-40CC-9F2D-C41408ED9E98}" uniqueName="4" name="Column4" queryTableFieldId="4" dataDxfId="32"/>
-    <tableColumn id="5" xr3:uid="{A19C49CB-F2CF-4D60-B082-761FE4F0ABC5}" uniqueName="5" name="Column5" queryTableFieldId="5" dataDxfId="31"/>
-    <tableColumn id="6" xr3:uid="{801427E9-2562-451E-AE45-ACF6DAAAFFFB}" uniqueName="6" name="Column6" queryTableFieldId="6" dataDxfId="30"/>
+    <tableColumn id="1" xr3:uid="{48EBD4D1-26EB-449F-8D09-DF1A8D9D96A3}" uniqueName="1" name="Column1" queryTableFieldId="1" dataDxfId="34"/>
+    <tableColumn id="2" xr3:uid="{671AE648-452F-44F1-9A65-8468F7B19950}" uniqueName="2" name="Column2" queryTableFieldId="2" dataDxfId="33"/>
+    <tableColumn id="3" xr3:uid="{C3287937-E8A8-4D80-A27C-D2A5C0E44D68}" uniqueName="3" name="Column3" queryTableFieldId="3" dataDxfId="32"/>
+    <tableColumn id="4" xr3:uid="{49CAB777-0355-40CC-9F2D-C41408ED9E98}" uniqueName="4" name="Column4" queryTableFieldId="4" dataDxfId="31"/>
+    <tableColumn id="5" xr3:uid="{A19C49CB-F2CF-4D60-B082-761FE4F0ABC5}" uniqueName="5" name="Column5" queryTableFieldId="5" dataDxfId="30"/>
+    <tableColumn id="6" xr3:uid="{801427E9-2562-451E-AE45-ACF6DAAAFFFB}" uniqueName="6" name="Column6" queryTableFieldId="6" dataDxfId="29"/>
   </tableColumns>
   <tableStyleInfo name="TableStyleMedium7" showFirstColumn="0" showLastColumn="0" showRowStripes="1" showColumnStripes="0"/>
 </table>
@@ -5234,11 +5245,11 @@
 <table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="17" xr:uid="{510F87AB-8378-4FE2-9EBF-7361BA7DB6B8}" name="Table017__Page_10" displayName="Table017__Page_10" ref="A1:E15" tableType="queryTable" totalsRowShown="0">
   <autoFilter ref="A1:E15" xr:uid="{510F87AB-8378-4FE2-9EBF-7361BA7DB6B8}"/>
   <tableColumns count="5">
-    <tableColumn id="1" xr3:uid="{626476ED-551C-48ED-A0F5-9CB680097EF0}" uniqueName="1" name="Column1" queryTableFieldId="1" dataDxfId="29"/>
-    <tableColumn id="2" xr3:uid="{9215A7DD-9718-48E5-BA20-B6B9989DD0D2}" uniqueName="2" name="Column2" queryTableFieldId="2" dataDxfId="28"/>
-    <tableColumn id="3" xr3:uid="{AE2AC56F-3587-4342-A60B-0B4A30905DD3}" uniqueName="3" name="Column3" queryTableFieldId="3" dataDxfId="27"/>
-    <tableColumn id="4" xr3:uid="{F7BE237D-2C3F-4C27-92EF-2601ABCBA887}" uniqueName="4" name="Column4" queryTableFieldId="4" dataDxfId="26"/>
-    <tableColumn id="5" xr3:uid="{7950C4F9-8FA4-4C6E-B03A-A0235ECC51FF}" uniqueName="5" name="Column5" queryTableFieldId="5" dataDxfId="25"/>
+    <tableColumn id="1" xr3:uid="{626476ED-551C-48ED-A0F5-9CB680097EF0}" uniqueName="1" name="Column1" queryTableFieldId="1" dataDxfId="28"/>
+    <tableColumn id="2" xr3:uid="{9215A7DD-9718-48E5-BA20-B6B9989DD0D2}" uniqueName="2" name="Column2" queryTableFieldId="2" dataDxfId="27"/>
+    <tableColumn id="3" xr3:uid="{AE2AC56F-3587-4342-A60B-0B4A30905DD3}" uniqueName="3" name="Column3" queryTableFieldId="3" dataDxfId="26"/>
+    <tableColumn id="4" xr3:uid="{F7BE237D-2C3F-4C27-92EF-2601ABCBA887}" uniqueName="4" name="Column4" queryTableFieldId="4" dataDxfId="25"/>
+    <tableColumn id="5" xr3:uid="{7950C4F9-8FA4-4C6E-B03A-A0235ECC51FF}" uniqueName="5" name="Column5" queryTableFieldId="5" dataDxfId="24"/>
   </tableColumns>
   <tableStyleInfo name="TableStyleMedium7" showFirstColumn="0" showLastColumn="0" showRowStripes="1" showColumnStripes="0"/>
 </table>
@@ -5248,11 +5259,11 @@
 <table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="18" xr:uid="{14CF879A-74C7-4F0C-8E76-F1430C9579CD}" name="Table018__Page_10" displayName="Table018__Page_10" ref="A17:E19" tableType="queryTable" totalsRowShown="0">
   <autoFilter ref="A17:E19" xr:uid="{14CF879A-74C7-4F0C-8E76-F1430C9579CD}"/>
   <tableColumns count="5">
-    <tableColumn id="1" xr3:uid="{210B1486-2DC9-4D94-98AC-6BEB874B7545}" uniqueName="1" name="Column1" queryTableFieldId="1" dataDxfId="24"/>
-    <tableColumn id="2" xr3:uid="{BB67F395-3AAE-4514-BCCE-DE32693EB37D}" uniqueName="2" name="Column2" queryTableFieldId="2" dataDxfId="23"/>
-    <tableColumn id="3" xr3:uid="{230B22CA-5CA3-4E2D-92CC-C75BC5831FF2}" uniqueName="3" name="Column3" queryTableFieldId="3" dataDxfId="22"/>
-    <tableColumn id="4" xr3:uid="{42788CA6-A70D-442A-9072-79E0D19F0B28}" uniqueName="4" name="Column4" queryTableFieldId="4" dataDxfId="21"/>
-    <tableColumn id="5" xr3:uid="{E37C1038-7442-4E7D-BB43-162AD6FA4195}" uniqueName="5" name="Column5" queryTableFieldId="5" dataDxfId="20"/>
+    <tableColumn id="1" xr3:uid="{210B1486-2DC9-4D94-98AC-6BEB874B7545}" uniqueName="1" name="Column1" queryTableFieldId="1" dataDxfId="23"/>
+    <tableColumn id="2" xr3:uid="{BB67F395-3AAE-4514-BCCE-DE32693EB37D}" uniqueName="2" name="Column2" queryTableFieldId="2" dataDxfId="22"/>
+    <tableColumn id="3" xr3:uid="{230B22CA-5CA3-4E2D-92CC-C75BC5831FF2}" uniqueName="3" name="Column3" queryTableFieldId="3" dataDxfId="21"/>
+    <tableColumn id="4" xr3:uid="{42788CA6-A70D-442A-9072-79E0D19F0B28}" uniqueName="4" name="Column4" queryTableFieldId="4" dataDxfId="20"/>
+    <tableColumn id="5" xr3:uid="{E37C1038-7442-4E7D-BB43-162AD6FA4195}" uniqueName="5" name="Column5" queryTableFieldId="5" dataDxfId="19"/>
   </tableColumns>
   <tableStyleInfo name="TableStyleMedium7" showFirstColumn="0" showLastColumn="0" showRowStripes="1" showColumnStripes="0"/>
 </table>
@@ -5262,13 +5273,13 @@
 <table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="1" xr:uid="{8D8C9D73-217D-4974-B35A-0740746DA27F}" name="Table001__Page_2" displayName="Table001__Page_2" ref="A1:G16" tableType="queryTable" totalsRowShown="0">
   <autoFilter ref="A1:G16" xr:uid="{8D8C9D73-217D-4974-B35A-0740746DA27F}"/>
   <tableColumns count="7">
-    <tableColumn id="1" xr3:uid="{A26CE965-72B2-472B-B9FF-D68F7847F3C5}" uniqueName="1" name="Column1" queryTableFieldId="1" dataDxfId="141"/>
-    <tableColumn id="2" xr3:uid="{375BF78E-5806-424A-B7BD-C63C40843BE9}" uniqueName="2" name="Column2" queryTableFieldId="2" dataDxfId="140"/>
-    <tableColumn id="3" xr3:uid="{CD1FFC74-B097-42B5-B1FA-08D3BD4531B9}" uniqueName="3" name="Column3" queryTableFieldId="3" dataDxfId="139"/>
-    <tableColumn id="4" xr3:uid="{EA6F5C08-47B3-4BE3-8F9B-3167F2B34338}" uniqueName="4" name="Column4" queryTableFieldId="4" dataDxfId="138"/>
-    <tableColumn id="5" xr3:uid="{67D1B145-6151-4A54-9C79-A6B0381CDA09}" uniqueName="5" name="Column5" queryTableFieldId="5" dataDxfId="137"/>
-    <tableColumn id="6" xr3:uid="{E8D8899E-ED32-4A2F-B13D-18F4C289A59B}" uniqueName="6" name="Column6" queryTableFieldId="6" dataDxfId="136"/>
-    <tableColumn id="7" xr3:uid="{CD1BCBB0-10DE-4DDA-903D-C14D16829749}" uniqueName="7" name="Column7" queryTableFieldId="7" dataDxfId="135"/>
+    <tableColumn id="1" xr3:uid="{A26CE965-72B2-472B-B9FF-D68F7847F3C5}" uniqueName="1" name="Column1" queryTableFieldId="1" dataDxfId="140"/>
+    <tableColumn id="2" xr3:uid="{375BF78E-5806-424A-B7BD-C63C40843BE9}" uniqueName="2" name="Column2" queryTableFieldId="2" dataDxfId="139"/>
+    <tableColumn id="3" xr3:uid="{CD1FFC74-B097-42B5-B1FA-08D3BD4531B9}" uniqueName="3" name="Column3" queryTableFieldId="3" dataDxfId="138"/>
+    <tableColumn id="4" xr3:uid="{EA6F5C08-47B3-4BE3-8F9B-3167F2B34338}" uniqueName="4" name="Column4" queryTableFieldId="4" dataDxfId="137"/>
+    <tableColumn id="5" xr3:uid="{67D1B145-6151-4A54-9C79-A6B0381CDA09}" uniqueName="5" name="Column5" queryTableFieldId="5" dataDxfId="136"/>
+    <tableColumn id="6" xr3:uid="{E8D8899E-ED32-4A2F-B13D-18F4C289A59B}" uniqueName="6" name="Column6" queryTableFieldId="6" dataDxfId="135"/>
+    <tableColumn id="7" xr3:uid="{CD1BCBB0-10DE-4DDA-903D-C14D16829749}" uniqueName="7" name="Column7" queryTableFieldId="7" dataDxfId="134"/>
   </tableColumns>
   <tableStyleInfo name="TableStyleMedium7" showFirstColumn="0" showLastColumn="0" showRowStripes="1" showColumnStripes="0"/>
 </table>
@@ -5278,11 +5289,11 @@
 <table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="19" xr:uid="{A8D65B7F-C1B3-4E37-BFF7-03252131F371}" name="Table019__Page_11" displayName="Table019__Page_11" ref="A1:E16" tableType="queryTable" totalsRowShown="0">
   <autoFilter ref="A1:E16" xr:uid="{A8D65B7F-C1B3-4E37-BFF7-03252131F371}"/>
   <tableColumns count="5">
-    <tableColumn id="1" xr3:uid="{60EAA1C9-E43C-458C-A33C-365CF023541D}" uniqueName="1" name="Column1" queryTableFieldId="1" dataDxfId="19"/>
-    <tableColumn id="2" xr3:uid="{BF4ECEAF-8998-4833-A444-7DD2840947AB}" uniqueName="2" name="Column2" queryTableFieldId="2" dataDxfId="18"/>
-    <tableColumn id="3" xr3:uid="{A77E13C5-CB25-43C0-9678-51A378FA64FC}" uniqueName="3" name="Column3" queryTableFieldId="3" dataDxfId="17"/>
-    <tableColumn id="4" xr3:uid="{46713ABC-AA6E-45DD-9BBE-03C863D6B1D1}" uniqueName="4" name="Column4" queryTableFieldId="4" dataDxfId="16"/>
-    <tableColumn id="5" xr3:uid="{85365AB6-280F-40C4-AB42-3455547D61F1}" uniqueName="5" name="Column5" queryTableFieldId="5" dataDxfId="15"/>
+    <tableColumn id="1" xr3:uid="{60EAA1C9-E43C-458C-A33C-365CF023541D}" uniqueName="1" name="Column1" queryTableFieldId="1" dataDxfId="18"/>
+    <tableColumn id="2" xr3:uid="{BF4ECEAF-8998-4833-A444-7DD2840947AB}" uniqueName="2" name="Column2" queryTableFieldId="2" dataDxfId="17"/>
+    <tableColumn id="3" xr3:uid="{A77E13C5-CB25-43C0-9678-51A378FA64FC}" uniqueName="3" name="Column3" queryTableFieldId="3" dataDxfId="16"/>
+    <tableColumn id="4" xr3:uid="{46713ABC-AA6E-45DD-9BBE-03C863D6B1D1}" uniqueName="4" name="Column4" queryTableFieldId="4" dataDxfId="15"/>
+    <tableColumn id="5" xr3:uid="{85365AB6-280F-40C4-AB42-3455547D61F1}" uniqueName="5" name="Column5" queryTableFieldId="5" dataDxfId="14"/>
   </tableColumns>
   <tableStyleInfo name="TableStyleMedium7" showFirstColumn="0" showLastColumn="0" showRowStripes="1" showColumnStripes="0"/>
 </table>
@@ -5292,11 +5303,11 @@
 <table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="21" xr:uid="{0B4290D5-7CEE-4DDC-B997-690EEF6D9589}" name="Table020__Page_11" displayName="Table020__Page_11" ref="A18:E20" tableType="queryTable" totalsRowShown="0">
   <autoFilter ref="A18:E20" xr:uid="{0B4290D5-7CEE-4DDC-B997-690EEF6D9589}"/>
   <tableColumns count="5">
-    <tableColumn id="1" xr3:uid="{344C3D84-8C5A-4C60-ADD3-4EE73F83858B}" uniqueName="1" name="Column1" queryTableFieldId="1" dataDxfId="14"/>
-    <tableColumn id="2" xr3:uid="{3470DF86-5A38-429A-95CF-F5FF5E59449C}" uniqueName="2" name="Column2" queryTableFieldId="2" dataDxfId="13"/>
-    <tableColumn id="3" xr3:uid="{BC1BD851-46F6-4634-95EE-ED117E75EBB6}" uniqueName="3" name="Column3" queryTableFieldId="3" dataDxfId="12"/>
-    <tableColumn id="4" xr3:uid="{FF5D3D34-BBDB-4113-8340-C737255ED1BD}" uniqueName="4" name="Column4" queryTableFieldId="4" dataDxfId="11"/>
-    <tableColumn id="5" xr3:uid="{F05FA152-C9D6-4773-B0A5-5B18B60C7102}" uniqueName="5" name="Column5" queryTableFieldId="5" dataDxfId="10"/>
+    <tableColumn id="1" xr3:uid="{344C3D84-8C5A-4C60-ADD3-4EE73F83858B}" uniqueName="1" name="Column1" queryTableFieldId="1" dataDxfId="13"/>
+    <tableColumn id="2" xr3:uid="{3470DF86-5A38-429A-95CF-F5FF5E59449C}" uniqueName="2" name="Column2" queryTableFieldId="2" dataDxfId="12"/>
+    <tableColumn id="3" xr3:uid="{BC1BD851-46F6-4634-95EE-ED117E75EBB6}" uniqueName="3" name="Column3" queryTableFieldId="3" dataDxfId="11"/>
+    <tableColumn id="4" xr3:uid="{FF5D3D34-BBDB-4113-8340-C737255ED1BD}" uniqueName="4" name="Column4" queryTableFieldId="4" dataDxfId="10"/>
+    <tableColumn id="5" xr3:uid="{F05FA152-C9D6-4773-B0A5-5B18B60C7102}" uniqueName="5" name="Column5" queryTableFieldId="5" dataDxfId="9"/>
   </tableColumns>
   <tableStyleInfo name="TableStyleMedium7" showFirstColumn="0" showLastColumn="0" showRowStripes="1" showColumnStripes="0"/>
 </table>
@@ -5306,13 +5317,13 @@
 <table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="2" xr:uid="{D4474760-F3B7-4070-AE77-2962D090A5AB}" name="Table002__Page_2" displayName="Table002__Page_2" ref="A19:G21" tableType="queryTable" totalsRowShown="0">
   <autoFilter ref="A19:G21" xr:uid="{D4474760-F3B7-4070-AE77-2962D090A5AB}"/>
   <tableColumns count="7">
-    <tableColumn id="1" xr3:uid="{8A3681DA-5FE9-4564-BCAB-75CCDF2C3A51}" uniqueName="1" name="Column1" queryTableFieldId="1" dataDxfId="134"/>
-    <tableColumn id="2" xr3:uid="{44D6563C-A88C-4FEE-9427-B5252DF8FA5D}" uniqueName="2" name="Column6" queryTableFieldId="2" dataDxfId="133"/>
-    <tableColumn id="3" xr3:uid="{2514D758-49E4-4E3E-A628-2B2D894F398E}" uniqueName="3" name="Column2" queryTableFieldId="3" dataDxfId="132"/>
-    <tableColumn id="4" xr3:uid="{062470EA-CB73-435C-8DF3-28DE262C8D69}" uniqueName="4" name="Column3" queryTableFieldId="4" dataDxfId="131"/>
-    <tableColumn id="5" xr3:uid="{CDE500EE-B268-43D9-A30D-9E6CC1608CD0}" uniqueName="5" name="Column4" queryTableFieldId="5" dataDxfId="130"/>
-    <tableColumn id="6" xr3:uid="{699F51E2-9A1B-4953-91BE-8D6434D76B20}" uniqueName="6" name="Column5" queryTableFieldId="6" dataDxfId="129"/>
-    <tableColumn id="7" xr3:uid="{C62D0670-E212-49FF-BA61-22C41F21B60E}" uniqueName="7" name="Column62" queryTableFieldId="7" dataDxfId="128"/>
+    <tableColumn id="1" xr3:uid="{8A3681DA-5FE9-4564-BCAB-75CCDF2C3A51}" uniqueName="1" name="Column1" queryTableFieldId="1" dataDxfId="133"/>
+    <tableColumn id="2" xr3:uid="{44D6563C-A88C-4FEE-9427-B5252DF8FA5D}" uniqueName="2" name="Column6" queryTableFieldId="2" dataDxfId="132"/>
+    <tableColumn id="3" xr3:uid="{2514D758-49E4-4E3E-A628-2B2D894F398E}" uniqueName="3" name="Column2" queryTableFieldId="3" dataDxfId="131"/>
+    <tableColumn id="4" xr3:uid="{062470EA-CB73-435C-8DF3-28DE262C8D69}" uniqueName="4" name="Column3" queryTableFieldId="4" dataDxfId="130"/>
+    <tableColumn id="5" xr3:uid="{CDE500EE-B268-43D9-A30D-9E6CC1608CD0}" uniqueName="5" name="Column4" queryTableFieldId="5" dataDxfId="129"/>
+    <tableColumn id="6" xr3:uid="{699F51E2-9A1B-4953-91BE-8D6434D76B20}" uniqueName="6" name="Column5" queryTableFieldId="6" dataDxfId="128"/>
+    <tableColumn id="7" xr3:uid="{C62D0670-E212-49FF-BA61-22C41F21B60E}" uniqueName="7" name="Column62" queryTableFieldId="7" dataDxfId="127"/>
   </tableColumns>
   <tableStyleInfo name="TableStyleMedium7" showFirstColumn="0" showLastColumn="0" showRowStripes="1" showColumnStripes="0"/>
 </table>
@@ -5322,14 +5333,14 @@
 <table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="3" xr:uid="{EE92A61D-8549-4453-B707-7BA76D39611E}" name="Table003__Page_3" displayName="Table003__Page_3" ref="A1:H16" tableType="queryTable" totalsRowShown="0">
   <autoFilter ref="A1:H16" xr:uid="{EE92A61D-8549-4453-B707-7BA76D39611E}"/>
   <tableColumns count="8">
-    <tableColumn id="1" xr3:uid="{5E78ED26-3040-4033-A95F-3AC09118D17C}" uniqueName="1" name="Column1" queryTableFieldId="1" dataDxfId="127"/>
-    <tableColumn id="2" xr3:uid="{52F60F93-88D4-4F60-A15A-4B2113E53BE2}" uniqueName="2" name="Column2" queryTableFieldId="2" dataDxfId="126"/>
-    <tableColumn id="3" xr3:uid="{2A66B2A9-165C-4995-937F-8E0D8B01B3D8}" uniqueName="3" name="Column3" queryTableFieldId="3" dataDxfId="125"/>
-    <tableColumn id="4" xr3:uid="{937ED0C3-8277-4EC6-BFD2-C6699696538D}" uniqueName="4" name="Column4" queryTableFieldId="4" dataDxfId="124"/>
-    <tableColumn id="5" xr3:uid="{37EAAABA-4FEF-4D28-B237-360AD0A7194A}" uniqueName="5" name="Column5" queryTableFieldId="5" dataDxfId="123"/>
-    <tableColumn id="6" xr3:uid="{6E7D50A0-6329-4797-9F9A-628D251C7CA5}" uniqueName="6" name="Column6" queryTableFieldId="6" dataDxfId="122"/>
-    <tableColumn id="7" xr3:uid="{F8F31C01-9522-488B-915F-110987168D09}" uniqueName="7" name="Column7" queryTableFieldId="7" dataDxfId="121"/>
-    <tableColumn id="8" xr3:uid="{FFD35FDD-AAE7-4F54-8AF3-197380BC0AEB}" uniqueName="8" name="Column8" queryTableFieldId="8" dataDxfId="120"/>
+    <tableColumn id="1" xr3:uid="{5E78ED26-3040-4033-A95F-3AC09118D17C}" uniqueName="1" name="Column1" queryTableFieldId="1" dataDxfId="126"/>
+    <tableColumn id="2" xr3:uid="{52F60F93-88D4-4F60-A15A-4B2113E53BE2}" uniqueName="2" name="Column2" queryTableFieldId="2" dataDxfId="125"/>
+    <tableColumn id="3" xr3:uid="{2A66B2A9-165C-4995-937F-8E0D8B01B3D8}" uniqueName="3" name="Column3" queryTableFieldId="3" dataDxfId="124"/>
+    <tableColumn id="4" xr3:uid="{937ED0C3-8277-4EC6-BFD2-C6699696538D}" uniqueName="4" name="Column4" queryTableFieldId="4" dataDxfId="123"/>
+    <tableColumn id="5" xr3:uid="{37EAAABA-4FEF-4D28-B237-360AD0A7194A}" uniqueName="5" name="Column5" queryTableFieldId="5" dataDxfId="122"/>
+    <tableColumn id="6" xr3:uid="{6E7D50A0-6329-4797-9F9A-628D251C7CA5}" uniqueName="6" name="Column6" queryTableFieldId="6" dataDxfId="121"/>
+    <tableColumn id="7" xr3:uid="{F8F31C01-9522-488B-915F-110987168D09}" uniqueName="7" name="Column7" queryTableFieldId="7" dataDxfId="120"/>
+    <tableColumn id="8" xr3:uid="{FFD35FDD-AAE7-4F54-8AF3-197380BC0AEB}" uniqueName="8" name="Column8" queryTableFieldId="8" dataDxfId="119"/>
   </tableColumns>
   <tableStyleInfo name="TableStyleMedium7" showFirstColumn="0" showLastColumn="0" showRowStripes="1" showColumnStripes="0"/>
 </table>
@@ -5339,14 +5350,14 @@
 <table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="4" xr:uid="{1C7E55B7-7D73-418F-9229-407F52A253A6}" name="Table004__Page_3" displayName="Table004__Page_3" ref="A18:H20" tableType="queryTable" totalsRowShown="0">
   <autoFilter ref="A18:H20" xr:uid="{1C7E55B7-7D73-418F-9229-407F52A253A6}"/>
   <tableColumns count="8">
-    <tableColumn id="1" xr3:uid="{A8A6FCCE-AE43-4EDA-82DC-831809E03401}" uniqueName="1" name="Column1" queryTableFieldId="1" dataDxfId="119"/>
-    <tableColumn id="2" xr3:uid="{0231594E-DA9E-47DE-A01C-22488210A4CF}" uniqueName="2" name="Column2" queryTableFieldId="2" dataDxfId="118"/>
-    <tableColumn id="3" xr3:uid="{7A06306A-69AF-482D-910F-86D0EF88F740}" uniqueName="3" name="Column3" queryTableFieldId="3" dataDxfId="117"/>
-    <tableColumn id="4" xr3:uid="{E96F3603-E9D2-4710-BDE5-6FE3E6A378D8}" uniqueName="4" name="Column4" queryTableFieldId="4" dataDxfId="116"/>
-    <tableColumn id="5" xr3:uid="{37151140-CC9F-4EBB-B58D-F87E1081314A}" uniqueName="5" name="Column5" queryTableFieldId="5" dataDxfId="115"/>
-    <tableColumn id="6" xr3:uid="{F0AAEEC2-014D-412A-B58D-24C71FEC9A66}" uniqueName="6" name="Column6" queryTableFieldId="6" dataDxfId="114"/>
-    <tableColumn id="7" xr3:uid="{A4B4F3F0-B14D-498F-B185-AA3E2BAE729A}" uniqueName="7" name="Column7" queryTableFieldId="7" dataDxfId="113"/>
-    <tableColumn id="8" xr3:uid="{0C517BB9-44A4-4BBA-AA88-B86BB679F208}" uniqueName="8" name="Column8" queryTableFieldId="8" dataDxfId="112"/>
+    <tableColumn id="1" xr3:uid="{A8A6FCCE-AE43-4EDA-82DC-831809E03401}" uniqueName="1" name="Column1" queryTableFieldId="1" dataDxfId="118"/>
+    <tableColumn id="2" xr3:uid="{0231594E-DA9E-47DE-A01C-22488210A4CF}" uniqueName="2" name="Column2" queryTableFieldId="2" dataDxfId="117"/>
+    <tableColumn id="3" xr3:uid="{7A06306A-69AF-482D-910F-86D0EF88F740}" uniqueName="3" name="Column3" queryTableFieldId="3" dataDxfId="116"/>
+    <tableColumn id="4" xr3:uid="{E96F3603-E9D2-4710-BDE5-6FE3E6A378D8}" uniqueName="4" name="Column4" queryTableFieldId="4" dataDxfId="115"/>
+    <tableColumn id="5" xr3:uid="{37151140-CC9F-4EBB-B58D-F87E1081314A}" uniqueName="5" name="Column5" queryTableFieldId="5" dataDxfId="114"/>
+    <tableColumn id="6" xr3:uid="{F0AAEEC2-014D-412A-B58D-24C71FEC9A66}" uniqueName="6" name="Column6" queryTableFieldId="6" dataDxfId="113"/>
+    <tableColumn id="7" xr3:uid="{A4B4F3F0-B14D-498F-B185-AA3E2BAE729A}" uniqueName="7" name="Column7" queryTableFieldId="7" dataDxfId="112"/>
+    <tableColumn id="8" xr3:uid="{0C517BB9-44A4-4BBA-AA88-B86BB679F208}" uniqueName="8" name="Column8" queryTableFieldId="8" dataDxfId="111"/>
   </tableColumns>
   <tableStyleInfo name="TableStyleMedium7" showFirstColumn="0" showLastColumn="0" showRowStripes="1" showColumnStripes="0"/>
 </table>
@@ -5356,12 +5367,12 @@
 <table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="5" xr:uid="{2EB30D60-3074-4922-8217-6B97953C0F87}" name="Table005__Page_4" displayName="Table005__Page_4" ref="A1:F16" tableType="queryTable" totalsRowShown="0">
   <autoFilter ref="A1:F16" xr:uid="{2EB30D60-3074-4922-8217-6B97953C0F87}"/>
   <tableColumns count="6">
-    <tableColumn id="1" xr3:uid="{AB42FEA9-5A85-4A69-B46D-444C53C4B4EF}" uniqueName="1" name="Column1" queryTableFieldId="1" dataDxfId="111"/>
-    <tableColumn id="2" xr3:uid="{0D7919B1-FB5E-4192-8675-3D57B39D9AB0}" uniqueName="2" name="Column2" queryTableFieldId="2" dataDxfId="110"/>
-    <tableColumn id="3" xr3:uid="{94F12F3D-88BF-4BEB-85E7-FF6313F6B88E}" uniqueName="3" name="Column3" queryTableFieldId="3" dataDxfId="109"/>
-    <tableColumn id="4" xr3:uid="{2B04EEA3-DC55-4C69-860F-9571D35E352D}" uniqueName="4" name="Column4" queryTableFieldId="4" dataDxfId="108"/>
-    <tableColumn id="5" xr3:uid="{461C5084-182B-40CC-B479-24798E48D0F4}" uniqueName="5" name="Column5" queryTableFieldId="5" dataDxfId="107"/>
-    <tableColumn id="6" xr3:uid="{258F7EB6-7345-43CA-BF8A-5E088D06FF8F}" uniqueName="6" name="Column6" queryTableFieldId="6" dataDxfId="106"/>
+    <tableColumn id="1" xr3:uid="{AB42FEA9-5A85-4A69-B46D-444C53C4B4EF}" uniqueName="1" name="Column1" queryTableFieldId="1" dataDxfId="110"/>
+    <tableColumn id="2" xr3:uid="{0D7919B1-FB5E-4192-8675-3D57B39D9AB0}" uniqueName="2" name="Column2" queryTableFieldId="2" dataDxfId="109"/>
+    <tableColumn id="3" xr3:uid="{94F12F3D-88BF-4BEB-85E7-FF6313F6B88E}" uniqueName="3" name="Column3" queryTableFieldId="3" dataDxfId="108"/>
+    <tableColumn id="4" xr3:uid="{2B04EEA3-DC55-4C69-860F-9571D35E352D}" uniqueName="4" name="Column4" queryTableFieldId="4" dataDxfId="107"/>
+    <tableColumn id="5" xr3:uid="{461C5084-182B-40CC-B479-24798E48D0F4}" uniqueName="5" name="Column5" queryTableFieldId="5" dataDxfId="106"/>
+    <tableColumn id="6" xr3:uid="{258F7EB6-7345-43CA-BF8A-5E088D06FF8F}" uniqueName="6" name="Column6" queryTableFieldId="6" dataDxfId="105"/>
   </tableColumns>
   <tableStyleInfo name="TableStyleMedium7" showFirstColumn="0" showLastColumn="0" showRowStripes="1" showColumnStripes="0"/>
 </table>
@@ -5371,12 +5382,12 @@
 <table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="6" xr:uid="{BA3E356C-A98F-4646-B7E8-7B0C3904E2A4}" name="Table006__Page_4" displayName="Table006__Page_4" ref="A18:F20" tableType="queryTable" totalsRowShown="0">
   <autoFilter ref="A18:F20" xr:uid="{BA3E356C-A98F-4646-B7E8-7B0C3904E2A4}"/>
   <tableColumns count="6">
-    <tableColumn id="1" xr3:uid="{55987721-40E8-4E11-9B6F-67EE503D78F4}" uniqueName="1" name="Column1" queryTableFieldId="1" dataDxfId="105"/>
-    <tableColumn id="2" xr3:uid="{15260D47-39CC-4501-9656-F8DBE6AD3AB1}" uniqueName="2" name="Column2" queryTableFieldId="2" dataDxfId="104"/>
-    <tableColumn id="3" xr3:uid="{06C8B30C-3DD3-49E6-8BE6-C8A9D39F2FC4}" uniqueName="3" name="Column3" queryTableFieldId="3" dataDxfId="103"/>
-    <tableColumn id="4" xr3:uid="{40A070F6-4BDB-49A7-9394-4D63F3A9E318}" uniqueName="4" name="Column4" queryTableFieldId="4" dataDxfId="102"/>
-    <tableColumn id="5" xr3:uid="{C5E0BAEF-796C-4C71-ACA7-889E63543C2D}" uniqueName="5" name="Column5" queryTableFieldId="5" dataDxfId="101"/>
-    <tableColumn id="6" xr3:uid="{1BA75280-A961-41F1-B113-5935891BA00A}" uniqueName="6" name="Column6" queryTableFieldId="6" dataDxfId="100"/>
+    <tableColumn id="1" xr3:uid="{55987721-40E8-4E11-9B6F-67EE503D78F4}" uniqueName="1" name="Column1" queryTableFieldId="1" dataDxfId="104"/>
+    <tableColumn id="2" xr3:uid="{15260D47-39CC-4501-9656-F8DBE6AD3AB1}" uniqueName="2" name="Column2" queryTableFieldId="2" dataDxfId="103"/>
+    <tableColumn id="3" xr3:uid="{06C8B30C-3DD3-49E6-8BE6-C8A9D39F2FC4}" uniqueName="3" name="Column3" queryTableFieldId="3" dataDxfId="102"/>
+    <tableColumn id="4" xr3:uid="{40A070F6-4BDB-49A7-9394-4D63F3A9E318}" uniqueName="4" name="Column4" queryTableFieldId="4" dataDxfId="101"/>
+    <tableColumn id="5" xr3:uid="{C5E0BAEF-796C-4C71-ACA7-889E63543C2D}" uniqueName="5" name="Column5" queryTableFieldId="5" dataDxfId="100"/>
+    <tableColumn id="6" xr3:uid="{1BA75280-A961-41F1-B113-5935891BA00A}" uniqueName="6" name="Column6" queryTableFieldId="6" dataDxfId="99"/>
   </tableColumns>
   <tableStyleInfo name="TableStyleMedium7" showFirstColumn="0" showLastColumn="0" showRowStripes="1" showColumnStripes="0"/>
 </table>
@@ -5386,18 +5397,18 @@
 <table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="7" xr:uid="{6040FF08-DFFC-4D6C-87C0-7C33D5281777}" name="Table007__Page_5" displayName="Table007__Page_5" ref="A1:L16" tableType="queryTable" totalsRowShown="0">
   <autoFilter ref="A1:L16" xr:uid="{6040FF08-DFFC-4D6C-87C0-7C33D5281777}"/>
   <tableColumns count="12">
-    <tableColumn id="1" xr3:uid="{9561388E-64AE-4A76-863E-A0B2091E2F9F}" uniqueName="1" name="Column1" queryTableFieldId="1" dataDxfId="99"/>
-    <tableColumn id="2" xr3:uid="{151810A9-7DD3-4FD0-91D6-6608DF85A8CF}" uniqueName="2" name="Column2" queryTableFieldId="2" dataDxfId="98"/>
-    <tableColumn id="3" xr3:uid="{94D629BF-F745-493D-8F74-FA7EEFDEAA84}" uniqueName="3" name="Column3" queryTableFieldId="3" dataDxfId="97"/>
-    <tableColumn id="4" xr3:uid="{AE87299A-170F-4661-BD08-B108394E2F7C}" uniqueName="4" name="Column4" queryTableFieldId="4" dataDxfId="96"/>
-    <tableColumn id="5" xr3:uid="{708CB468-5E3F-4D0C-B6BD-C2C44C7191EC}" uniqueName="5" name="Column5" queryTableFieldId="5" dataDxfId="95"/>
-    <tableColumn id="6" xr3:uid="{5D4BD3CB-C344-4155-B3C1-ECC49F86CED1}" uniqueName="6" name="Column6" queryTableFieldId="6" dataDxfId="94"/>
-    <tableColumn id="7" xr3:uid="{61DF1122-5C54-47A3-98F9-27CA1B50CA9D}" uniqueName="7" name="Column7" queryTableFieldId="7" dataDxfId="93"/>
-    <tableColumn id="8" xr3:uid="{130590EE-DDCB-43DB-A020-385B521DA018}" uniqueName="8" name="Column8" queryTableFieldId="8" dataDxfId="92"/>
-    <tableColumn id="9" xr3:uid="{06B903F7-5E22-476D-A116-655599D2C518}" uniqueName="9" name="Column9" queryTableFieldId="9" dataDxfId="91"/>
-    <tableColumn id="10" xr3:uid="{CED96D55-8B0D-492D-B0EC-F3E56EFB2649}" uniqueName="10" name="Column10" queryTableFieldId="10" dataDxfId="90"/>
-    <tableColumn id="11" xr3:uid="{346823E9-F305-4F11-941F-1C42A8AB0C99}" uniqueName="11" name="Column11" queryTableFieldId="11" dataDxfId="89"/>
-    <tableColumn id="12" xr3:uid="{7B421AA8-C9DB-4E35-A456-DF0F56050B79}" uniqueName="12" name="Column12" queryTableFieldId="12" dataDxfId="88"/>
+    <tableColumn id="1" xr3:uid="{9561388E-64AE-4A76-863E-A0B2091E2F9F}" uniqueName="1" name="Column1" queryTableFieldId="1" dataDxfId="98"/>
+    <tableColumn id="2" xr3:uid="{151810A9-7DD3-4FD0-91D6-6608DF85A8CF}" uniqueName="2" name="Column2" queryTableFieldId="2" dataDxfId="97"/>
+    <tableColumn id="3" xr3:uid="{94D629BF-F745-493D-8F74-FA7EEFDEAA84}" uniqueName="3" name="Column3" queryTableFieldId="3" dataDxfId="96"/>
+    <tableColumn id="4" xr3:uid="{AE87299A-170F-4661-BD08-B108394E2F7C}" uniqueName="4" name="Column4" queryTableFieldId="4" dataDxfId="95"/>
+    <tableColumn id="5" xr3:uid="{708CB468-5E3F-4D0C-B6BD-C2C44C7191EC}" uniqueName="5" name="Column5" queryTableFieldId="5" dataDxfId="94"/>
+    <tableColumn id="6" xr3:uid="{5D4BD3CB-C344-4155-B3C1-ECC49F86CED1}" uniqueName="6" name="Column6" queryTableFieldId="6" dataDxfId="93"/>
+    <tableColumn id="7" xr3:uid="{61DF1122-5C54-47A3-98F9-27CA1B50CA9D}" uniqueName="7" name="Column7" queryTableFieldId="7" dataDxfId="92"/>
+    <tableColumn id="8" xr3:uid="{130590EE-DDCB-43DB-A020-385B521DA018}" uniqueName="8" name="Column8" queryTableFieldId="8" dataDxfId="91"/>
+    <tableColumn id="9" xr3:uid="{06B903F7-5E22-476D-A116-655599D2C518}" uniqueName="9" name="Column9" queryTableFieldId="9" dataDxfId="90"/>
+    <tableColumn id="10" xr3:uid="{CED96D55-8B0D-492D-B0EC-F3E56EFB2649}" uniqueName="10" name="Column10" queryTableFieldId="10" dataDxfId="89"/>
+    <tableColumn id="11" xr3:uid="{346823E9-F305-4F11-941F-1C42A8AB0C99}" uniqueName="11" name="Column11" queryTableFieldId="11" dataDxfId="88"/>
+    <tableColumn id="12" xr3:uid="{7B421AA8-C9DB-4E35-A456-DF0F56050B79}" uniqueName="12" name="Column12" queryTableFieldId="12" dataDxfId="87"/>
   </tableColumns>
   <tableStyleInfo name="TableStyleMedium7" showFirstColumn="0" showLastColumn="0" showRowStripes="1" showColumnStripes="0"/>
 </table>
@@ -5407,18 +5418,18 @@
 <table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="8" xr:uid="{DBF54861-4823-4965-9BF8-BF4D83A85FD1}" name="Table008__Page_5" displayName="Table008__Page_5" ref="A18:L20" tableType="queryTable" totalsRowShown="0">
   <autoFilter ref="A18:L20" xr:uid="{DBF54861-4823-4965-9BF8-BF4D83A85FD1}"/>
   <tableColumns count="12">
-    <tableColumn id="1" xr3:uid="{01D3C90B-BA67-46B4-BD1D-5C53486CAE57}" uniqueName="1" name="Column1" queryTableFieldId="1" dataDxfId="87"/>
-    <tableColumn id="2" xr3:uid="{166854EB-0B50-4420-BB3F-7A5A2C9FB7F7}" uniqueName="2" name="Column2" queryTableFieldId="2" dataDxfId="86"/>
-    <tableColumn id="3" xr3:uid="{638857E5-1EB4-4FBE-9FFE-2951F2F4ABD0}" uniqueName="3" name="Column3" queryTableFieldId="3" dataDxfId="85"/>
-    <tableColumn id="4" xr3:uid="{F4EFE2EF-AC84-40F8-BE68-0B6B520F8EA8}" uniqueName="4" name="Column4" queryTableFieldId="4" dataDxfId="84"/>
-    <tableColumn id="5" xr3:uid="{38D026D2-A47E-46EA-BA10-AF890A55BF2B}" uniqueName="5" name="Column5" queryTableFieldId="5" dataDxfId="83"/>
-    <tableColumn id="6" xr3:uid="{025C6DA2-37A6-491F-904E-DDE12948D35B}" uniqueName="6" name="Column6" queryTableFieldId="6" dataDxfId="82"/>
-    <tableColumn id="7" xr3:uid="{AC28B573-67B7-4468-A6A2-F648D17079B6}" uniqueName="7" name="Column7" queryTableFieldId="7" dataDxfId="81"/>
-    <tableColumn id="8" xr3:uid="{F6F06554-210B-472F-95F2-8E89D931E4C1}" uniqueName="8" name="Column8" queryTableFieldId="8" dataDxfId="80"/>
-    <tableColumn id="9" xr3:uid="{F0A8F323-36C1-4290-980B-8F6F5DC6A41E}" uniqueName="9" name="Column9" queryTableFieldId="9" dataDxfId="79"/>
-    <tableColumn id="10" xr3:uid="{25D60007-5007-4174-85F5-572E3C29FE33}" uniqueName="10" name="Column10" queryTableFieldId="10" dataDxfId="78"/>
-    <tableColumn id="11" xr3:uid="{2071EB9B-B14E-4EF0-9B86-0D5FDA96828D}" uniqueName="11" name="Column11" queryTableFieldId="11" dataDxfId="77"/>
-    <tableColumn id="12" xr3:uid="{1660C180-EE6B-48E8-9880-55F02CC623C4}" uniqueName="12" name="Column12" queryTableFieldId="12" dataDxfId="76"/>
+    <tableColumn id="1" xr3:uid="{01D3C90B-BA67-46B4-BD1D-5C53486CAE57}" uniqueName="1" name="Column1" queryTableFieldId="1" dataDxfId="86"/>
+    <tableColumn id="2" xr3:uid="{166854EB-0B50-4420-BB3F-7A5A2C9FB7F7}" uniqueName="2" name="Column2" queryTableFieldId="2" dataDxfId="85"/>
+    <tableColumn id="3" xr3:uid="{638857E5-1EB4-4FBE-9FFE-2951F2F4ABD0}" uniqueName="3" name="Column3" queryTableFieldId="3" dataDxfId="84"/>
+    <tableColumn id="4" xr3:uid="{F4EFE2EF-AC84-40F8-BE68-0B6B520F8EA8}" uniqueName="4" name="Column4" queryTableFieldId="4" dataDxfId="83"/>
+    <tableColumn id="5" xr3:uid="{38D026D2-A47E-46EA-BA10-AF890A55BF2B}" uniqueName="5" name="Column5" queryTableFieldId="5" dataDxfId="82"/>
+    <tableColumn id="6" xr3:uid="{025C6DA2-37A6-491F-904E-DDE12948D35B}" uniqueName="6" name="Column6" queryTableFieldId="6" dataDxfId="81"/>
+    <tableColumn id="7" xr3:uid="{AC28B573-67B7-4468-A6A2-F648D17079B6}" uniqueName="7" name="Column7" queryTableFieldId="7" dataDxfId="80"/>
+    <tableColumn id="8" xr3:uid="{F6F06554-210B-472F-95F2-8E89D931E4C1}" uniqueName="8" name="Column8" queryTableFieldId="8" dataDxfId="79"/>
+    <tableColumn id="9" xr3:uid="{F0A8F323-36C1-4290-980B-8F6F5DC6A41E}" uniqueName="9" name="Column9" queryTableFieldId="9" dataDxfId="78"/>
+    <tableColumn id="10" xr3:uid="{25D60007-5007-4174-85F5-572E3C29FE33}" uniqueName="10" name="Column10" queryTableFieldId="10" dataDxfId="77"/>
+    <tableColumn id="11" xr3:uid="{2071EB9B-B14E-4EF0-9B86-0D5FDA96828D}" uniqueName="11" name="Column11" queryTableFieldId="11" dataDxfId="76"/>
+    <tableColumn id="12" xr3:uid="{1660C180-EE6B-48E8-9880-55F02CC623C4}" uniqueName="12" name="Column12" queryTableFieldId="12" dataDxfId="75"/>
   </tableColumns>
   <tableStyleInfo name="TableStyleMedium7" showFirstColumn="0" showLastColumn="0" showRowStripes="1" showColumnStripes="0"/>
 </table>
@@ -5721,42 +5732,42 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{3B05C9E0-A64E-40AC-B9F4-C919ED5906CC}">
-  <dimension ref="A1:I69"/>
-  <sheetFormatPr defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
+  <dimension ref="A1:I70"/>
+  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
-    <col min="1" max="1" width="51.453125" bestFit="1" customWidth="1"/>
-    <col min="2" max="2" width="36.54296875" bestFit="1" customWidth="1"/>
-    <col min="3" max="3" width="17.1796875" bestFit="1" customWidth="1"/>
-    <col min="4" max="4" width="16.08984375" bestFit="1" customWidth="1"/>
-    <col min="5" max="6" width="17.36328125" customWidth="1"/>
-    <col min="7" max="7" width="10.90625" customWidth="1"/>
-    <col min="8" max="8" width="14.453125" bestFit="1" customWidth="1"/>
-    <col min="9" max="9" width="13.6328125" bestFit="1" customWidth="1"/>
-    <col min="10" max="10" width="14.453125" bestFit="1" customWidth="1"/>
-    <col min="11" max="11" width="18.1796875" bestFit="1" customWidth="1"/>
-    <col min="12" max="12" width="17.453125" bestFit="1" customWidth="1"/>
-    <col min="13" max="14" width="13.36328125" bestFit="1" customWidth="1"/>
-    <col min="15" max="15" width="26.6328125" bestFit="1" customWidth="1"/>
+    <col min="1" max="1" width="51.42578125" bestFit="1" customWidth="1"/>
+    <col min="2" max="2" width="36.5703125" bestFit="1" customWidth="1"/>
+    <col min="3" max="3" width="17.140625" bestFit="1" customWidth="1"/>
+    <col min="4" max="4" width="16.140625" bestFit="1" customWidth="1"/>
+    <col min="5" max="6" width="17.42578125" customWidth="1"/>
+    <col min="7" max="7" width="10.85546875" customWidth="1"/>
+    <col min="8" max="8" width="14.42578125" bestFit="1" customWidth="1"/>
+    <col min="9" max="9" width="14.28515625" bestFit="1" customWidth="1"/>
+    <col min="10" max="10" width="14.42578125" bestFit="1" customWidth="1"/>
+    <col min="11" max="11" width="18.140625" bestFit="1" customWidth="1"/>
+    <col min="12" max="12" width="17.42578125" bestFit="1" customWidth="1"/>
+    <col min="13" max="14" width="13.42578125" bestFit="1" customWidth="1"/>
+    <col min="15" max="15" width="26.5703125" bestFit="1" customWidth="1"/>
     <col min="16" max="16" width="8" bestFit="1" customWidth="1"/>
-    <col min="17" max="17" width="10.36328125" bestFit="1" customWidth="1"/>
-    <col min="18" max="18" width="25.7265625" bestFit="1" customWidth="1"/>
+    <col min="17" max="17" width="10.42578125" bestFit="1" customWidth="1"/>
+    <col min="18" max="18" width="25.7109375" bestFit="1" customWidth="1"/>
     <col min="19" max="19" width="20" bestFit="1" customWidth="1"/>
-    <col min="20" max="20" width="37.08984375" bestFit="1" customWidth="1"/>
-    <col min="21" max="21" width="33.6328125" bestFit="1" customWidth="1"/>
-    <col min="22" max="22" width="15.36328125" bestFit="1" customWidth="1"/>
-    <col min="23" max="23" width="22.1796875" bestFit="1" customWidth="1"/>
-    <col min="24" max="24" width="30.08984375" bestFit="1" customWidth="1"/>
-    <col min="25" max="25" width="26.36328125" bestFit="1" customWidth="1"/>
-    <col min="26" max="26" width="28.36328125" bestFit="1" customWidth="1"/>
-    <col min="27" max="27" width="21.08984375" bestFit="1" customWidth="1"/>
-    <col min="28" max="28" width="11.6328125" bestFit="1" customWidth="1"/>
-    <col min="29" max="29" width="25.90625" bestFit="1" customWidth="1"/>
-    <col min="30" max="30" width="34.08984375" bestFit="1" customWidth="1"/>
-    <col min="31" max="31" width="22.08984375" bestFit="1" customWidth="1"/>
-    <col min="32" max="32" width="10.7265625" bestFit="1" customWidth="1"/>
+    <col min="20" max="20" width="37.140625" bestFit="1" customWidth="1"/>
+    <col min="21" max="21" width="33.5703125" bestFit="1" customWidth="1"/>
+    <col min="22" max="22" width="15.42578125" bestFit="1" customWidth="1"/>
+    <col min="23" max="23" width="22.140625" bestFit="1" customWidth="1"/>
+    <col min="24" max="24" width="30.140625" bestFit="1" customWidth="1"/>
+    <col min="25" max="25" width="26.42578125" bestFit="1" customWidth="1"/>
+    <col min="26" max="26" width="28.42578125" bestFit="1" customWidth="1"/>
+    <col min="27" max="27" width="21.140625" bestFit="1" customWidth="1"/>
+    <col min="28" max="28" width="11.5703125" bestFit="1" customWidth="1"/>
+    <col min="29" max="29" width="25.85546875" bestFit="1" customWidth="1"/>
+    <col min="30" max="30" width="34.140625" bestFit="1" customWidth="1"/>
+    <col min="31" max="31" width="22.140625" bestFit="1" customWidth="1"/>
+    <col min="32" max="32" width="10.7109375" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:9" x14ac:dyDescent="0.35">
+    <row r="1" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A1" s="13" t="s">
         <v>551</v>
       </c>
@@ -5785,7 +5796,7 @@
         <v>585</v>
       </c>
     </row>
-    <row r="2" spans="1:9" x14ac:dyDescent="0.35">
+    <row r="2" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A2" s="10" t="s">
         <v>580</v>
       </c>
@@ -5817,7 +5828,7 @@
         <v>21000000.000000004</v>
       </c>
     </row>
-    <row r="3" spans="1:9" x14ac:dyDescent="0.35">
+    <row r="3" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A3" s="10" t="s">
         <v>555</v>
       </c>
@@ -5849,7 +5860,7 @@
         <v>21000000.000000004</v>
       </c>
     </row>
-    <row r="4" spans="1:9" x14ac:dyDescent="0.35">
+    <row r="4" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A4" s="10" t="s">
         <v>500</v>
       </c>
@@ -5881,7 +5892,7 @@
         <v>21000000.000000004</v>
       </c>
     </row>
-    <row r="5" spans="1:9" x14ac:dyDescent="0.35">
+    <row r="5" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A5" s="10" t="s">
         <v>501</v>
       </c>
@@ -5913,7 +5924,7 @@
         <v>21000000.000000004</v>
       </c>
     </row>
-    <row r="6" spans="1:9" x14ac:dyDescent="0.35">
+    <row r="6" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A6" s="10" t="s">
         <v>502</v>
       </c>
@@ -5945,7 +5956,7 @@
         <v>24999999.999999996</v>
       </c>
     </row>
-    <row r="7" spans="1:9" x14ac:dyDescent="0.35">
+    <row r="7" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A7" s="10" t="s">
         <v>515</v>
       </c>
@@ -5977,7 +5988,7 @@
         <v>23249999.999999996</v>
       </c>
     </row>
-    <row r="8" spans="1:9" x14ac:dyDescent="0.35">
+    <row r="8" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A8" s="10" t="s">
         <v>516</v>
       </c>
@@ -6009,7 +6020,7 @@
         <v>24700000.000000004</v>
       </c>
     </row>
-    <row r="9" spans="1:9" x14ac:dyDescent="0.35">
+    <row r="9" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A9" s="10" t="s">
         <v>547</v>
       </c>
@@ -6041,7 +6052,7 @@
         <v>32999999.999999996</v>
       </c>
     </row>
-    <row r="10" spans="1:9" x14ac:dyDescent="0.35">
+    <row r="10" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A10" s="10" t="s">
         <v>514</v>
       </c>
@@ -6073,7 +6084,7 @@
         <v>35000000</v>
       </c>
     </row>
-    <row r="11" spans="1:9" x14ac:dyDescent="0.35">
+    <row r="11" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A11" s="10" t="s">
         <v>496</v>
       </c>
@@ -6105,7 +6116,7 @@
         <v>35000000</v>
       </c>
     </row>
-    <row r="12" spans="1:9" x14ac:dyDescent="0.35">
+    <row r="12" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A12" s="10" t="s">
         <v>497</v>
       </c>
@@ -6137,7 +6148,7 @@
         <v>38000000</v>
       </c>
     </row>
-    <row r="13" spans="1:9" x14ac:dyDescent="0.35">
+    <row r="13" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A13" s="10" t="s">
         <v>517</v>
       </c>
@@ -6169,7 +6180,7 @@
         <v>23000000</v>
       </c>
     </row>
-    <row r="14" spans="1:9" x14ac:dyDescent="0.35">
+    <row r="14" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A14" s="10" t="s">
         <v>518</v>
       </c>
@@ -6201,7 +6212,7 @@
         <v>20000000</v>
       </c>
     </row>
-    <row r="15" spans="1:9" x14ac:dyDescent="0.35">
+    <row r="15" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A15" s="10" t="s">
         <v>519</v>
       </c>
@@ -6233,7 +6244,7 @@
         <v>13000000</v>
       </c>
     </row>
-    <row r="16" spans="1:9" x14ac:dyDescent="0.35">
+    <row r="16" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A16" s="10" t="s">
         <v>610</v>
       </c>
@@ -6265,7 +6276,7 @@
         <v>13000000</v>
       </c>
     </row>
-    <row r="17" spans="1:9" x14ac:dyDescent="0.35">
+    <row r="17" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A17" s="10" t="s">
         <v>612</v>
       </c>
@@ -6297,7 +6308,7 @@
         <v>20000000</v>
       </c>
     </row>
-    <row r="18" spans="1:9" x14ac:dyDescent="0.35">
+    <row r="18" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A18" s="10" t="s">
         <v>617</v>
       </c>
@@ -6329,7 +6340,7 @@
         <v>23000000</v>
       </c>
     </row>
-    <row r="19" spans="1:9" x14ac:dyDescent="0.35">
+    <row r="19" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A19" s="10" t="s">
         <v>503</v>
       </c>
@@ -6361,7 +6372,7 @@
         <v>29000000</v>
       </c>
     </row>
-    <row r="20" spans="1:9" x14ac:dyDescent="0.35">
+    <row r="20" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A20" s="10" t="s">
         <v>586</v>
       </c>
@@ -6393,7 +6404,7 @@
         <v>26000000</v>
       </c>
     </row>
-    <row r="21" spans="1:9" x14ac:dyDescent="0.35">
+    <row r="21" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A21" s="10" t="s">
         <v>504</v>
       </c>
@@ -6425,7 +6436,7 @@
         <v>30000000</v>
       </c>
     </row>
-    <row r="22" spans="1:9" x14ac:dyDescent="0.35">
+    <row r="22" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A22" s="10" t="s">
         <v>588</v>
       </c>
@@ -6457,7 +6468,7 @@
         <v>29000000</v>
       </c>
     </row>
-    <row r="23" spans="1:9" x14ac:dyDescent="0.35">
+    <row r="23" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A23" s="10" t="s">
         <v>587</v>
       </c>
@@ -6489,7 +6500,7 @@
         <v>29000000</v>
       </c>
     </row>
-    <row r="24" spans="1:9" x14ac:dyDescent="0.35">
+    <row r="24" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A24" s="10" t="s">
         <v>505</v>
       </c>
@@ -6521,7 +6532,7 @@
         <v>34000000</v>
       </c>
     </row>
-    <row r="25" spans="1:9" x14ac:dyDescent="0.35">
+    <row r="25" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A25" s="10" t="s">
         <v>558</v>
       </c>
@@ -6553,7 +6564,7 @@
         <v>37000000</v>
       </c>
     </row>
-    <row r="26" spans="1:9" x14ac:dyDescent="0.35">
+    <row r="26" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A26" s="10" t="s">
         <v>506</v>
       </c>
@@ -6585,7 +6596,7 @@
         <v>37000000</v>
       </c>
     </row>
-    <row r="27" spans="1:9" x14ac:dyDescent="0.35">
+    <row r="27" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A27" s="10" t="s">
         <v>561</v>
       </c>
@@ -6617,7 +6628,7 @@
         <v>37000000</v>
       </c>
     </row>
-    <row r="28" spans="1:9" x14ac:dyDescent="0.35">
+    <row r="28" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A28" s="10" t="s">
         <v>557</v>
       </c>
@@ -6649,7 +6660,7 @@
         <v>37000000</v>
       </c>
     </row>
-    <row r="29" spans="1:9" x14ac:dyDescent="0.35">
+    <row r="29" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A29" s="10" t="s">
         <v>582</v>
       </c>
@@ -6681,7 +6692,7 @@
         <v>37000000</v>
       </c>
     </row>
-    <row r="30" spans="1:9" x14ac:dyDescent="0.35">
+    <row r="30" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A30" s="10" t="s">
         <v>523</v>
       </c>
@@ -6713,7 +6724,7 @@
         <v>12700000.000000002</v>
       </c>
     </row>
-    <row r="31" spans="1:9" x14ac:dyDescent="0.35">
+    <row r="31" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A31" s="10" t="s">
         <v>560</v>
       </c>
@@ -6745,7 +6756,7 @@
         <v>12700000.000000002</v>
       </c>
     </row>
-    <row r="32" spans="1:9" x14ac:dyDescent="0.35">
+    <row r="32" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A32" s="10" t="s">
         <v>524</v>
       </c>
@@ -6777,7 +6788,7 @@
         <v>16000000</v>
       </c>
     </row>
-    <row r="33" spans="1:9" x14ac:dyDescent="0.35">
+    <row r="33" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A33" s="10" t="s">
         <v>498</v>
       </c>
@@ -6809,7 +6820,7 @@
         <v>14700000</v>
       </c>
     </row>
-    <row r="34" spans="1:9" x14ac:dyDescent="0.35">
+    <row r="34" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A34" s="10" t="s">
         <v>525</v>
       </c>
@@ -6841,7 +6852,7 @@
         <v>18300000</v>
       </c>
     </row>
-    <row r="35" spans="1:9" x14ac:dyDescent="0.35">
+    <row r="35" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A35" s="10" t="s">
         <v>527</v>
       </c>
@@ -6873,7 +6884,7 @@
         <v>20900000</v>
       </c>
     </row>
-    <row r="36" spans="1:9" x14ac:dyDescent="0.35">
+    <row r="36" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A36" s="10" t="s">
         <v>528</v>
       </c>
@@ -6905,7 +6916,7 @@
         <v>22000000</v>
       </c>
     </row>
-    <row r="37" spans="1:9" x14ac:dyDescent="0.35">
+    <row r="37" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A37" s="10" t="s">
         <v>499</v>
       </c>
@@ -6937,7 +6948,7 @@
         <v>20500000.000000004</v>
       </c>
     </row>
-    <row r="38" spans="1:9" x14ac:dyDescent="0.35">
+    <row r="38" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A38" s="10" t="s">
         <v>616</v>
       </c>
@@ -6969,7 +6980,7 @@
         <v>22400000</v>
       </c>
     </row>
-    <row r="39" spans="1:9" x14ac:dyDescent="0.35">
+    <row r="39" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A39" s="11" t="s">
         <v>522</v>
       </c>
@@ -7001,7 +7012,7 @@
         <v>25600000</v>
       </c>
     </row>
-    <row r="40" spans="1:9" x14ac:dyDescent="0.35">
+    <row r="40" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A40" s="22" t="s">
         <v>149</v>
       </c>
@@ -7033,7 +7044,7 @@
         <v>22400000</v>
       </c>
     </row>
-    <row r="41" spans="1:9" x14ac:dyDescent="0.35">
+    <row r="41" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A41" s="10" t="s">
         <v>607</v>
       </c>
@@ -7065,7 +7076,7 @@
         <v>31600000</v>
       </c>
     </row>
-    <row r="42" spans="1:9" x14ac:dyDescent="0.35">
+    <row r="42" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A42" s="10" t="s">
         <v>599</v>
       </c>
@@ -7097,7 +7108,7 @@
         <v>36400000</v>
       </c>
     </row>
-    <row r="43" spans="1:9" x14ac:dyDescent="0.35">
+    <row r="43" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A43" s="10" t="s">
         <v>618</v>
       </c>
@@ -7129,7 +7140,7 @@
         <v>32700000</v>
       </c>
     </row>
-    <row r="44" spans="1:9" x14ac:dyDescent="0.35">
+    <row r="44" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A44" s="10" t="s">
         <v>602</v>
       </c>
@@ -7161,7 +7172,7 @@
         <v>36400000</v>
       </c>
     </row>
-    <row r="45" spans="1:9" x14ac:dyDescent="0.35">
+    <row r="45" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A45" s="10" t="s">
         <v>526</v>
       </c>
@@ -7193,7 +7204,7 @@
         <v>12499999.999999998</v>
       </c>
     </row>
-    <row r="46" spans="1:9" x14ac:dyDescent="0.35">
+    <row r="46" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A46" s="16" t="s">
         <v>521</v>
       </c>
@@ -7225,7 +7236,7 @@
         <v>13500000</v>
       </c>
     </row>
-    <row r="47" spans="1:9" x14ac:dyDescent="0.35">
+    <row r="47" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A47" s="4" t="s">
         <v>529</v>
       </c>
@@ -7257,7 +7268,7 @@
         <v>12200000</v>
       </c>
     </row>
-    <row r="48" spans="1:9" x14ac:dyDescent="0.35">
+    <row r="48" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A48" s="4" t="s">
         <v>608</v>
       </c>
@@ -7289,7 +7300,7 @@
         <v>8000000</v>
       </c>
     </row>
-    <row r="49" spans="1:9" x14ac:dyDescent="0.35">
+    <row r="49" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A49" s="4" t="s">
         <v>520</v>
       </c>
@@ -7321,7 +7332,7 @@
         <v>8000000</v>
       </c>
     </row>
-    <row r="50" spans="1:9" x14ac:dyDescent="0.35">
+    <row r="50" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A50" s="17" t="s">
         <v>593</v>
       </c>
@@ -7353,7 +7364,7 @@
         <v>20000000</v>
       </c>
     </row>
-    <row r="51" spans="1:9" x14ac:dyDescent="0.35">
+    <row r="51" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A51" s="4" t="s">
         <v>603</v>
       </c>
@@ -7385,7 +7396,7 @@
         <v>20000000</v>
       </c>
     </row>
-    <row r="52" spans="1:9" x14ac:dyDescent="0.35">
+    <row r="52" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A52" s="17" t="s">
         <v>595</v>
       </c>
@@ -7417,7 +7428,7 @@
         <v>25000000</v>
       </c>
     </row>
-    <row r="53" spans="1:9" x14ac:dyDescent="0.35">
+    <row r="53" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A53" s="4" t="s">
         <v>606</v>
       </c>
@@ -7449,7 +7460,7 @@
         <v>25000000</v>
       </c>
     </row>
-    <row r="54" spans="1:9" x14ac:dyDescent="0.35">
+    <row r="54" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A54" s="17" t="s">
         <v>594</v>
       </c>
@@ -7481,7 +7492,7 @@
         <v>20000000</v>
       </c>
     </row>
-    <row r="55" spans="1:9" x14ac:dyDescent="0.35">
+    <row r="55" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A55" s="16" t="s">
         <v>605</v>
       </c>
@@ -7513,7 +7524,7 @@
         <v>20000000</v>
       </c>
     </row>
-    <row r="56" spans="1:9" x14ac:dyDescent="0.35">
+    <row r="56" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A56" s="16" t="s">
         <v>596</v>
       </c>
@@ -7545,7 +7556,7 @@
         <v>25000000</v>
       </c>
     </row>
-    <row r="57" spans="1:9" x14ac:dyDescent="0.35">
+    <row r="57" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A57" s="4" t="s">
         <v>604</v>
       </c>
@@ -7577,7 +7588,7 @@
         <v>25000000</v>
       </c>
     </row>
-    <row r="58" spans="1:9" x14ac:dyDescent="0.35">
+    <row r="58" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A58" s="16" t="s">
         <v>619</v>
       </c>
@@ -7609,7 +7620,7 @@
         <v>25000000</v>
       </c>
     </row>
-    <row r="59" spans="1:9" x14ac:dyDescent="0.35">
+    <row r="59" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A59" s="16" t="s">
         <v>620</v>
       </c>
@@ -7641,7 +7652,7 @@
         <v>35000000</v>
       </c>
     </row>
-    <row r="60" spans="1:9" x14ac:dyDescent="0.35">
+    <row r="60" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A60" s="16" t="s">
         <v>621</v>
       </c>
@@ -7673,7 +7684,7 @@
         <v>25000000</v>
       </c>
     </row>
-    <row r="61" spans="1:9" x14ac:dyDescent="0.35">
+    <row r="61" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A61" s="16" t="s">
         <v>622</v>
       </c>
@@ -7705,7 +7716,7 @@
         <v>35000000</v>
       </c>
     </row>
-    <row r="62" spans="1:9" x14ac:dyDescent="0.35">
+    <row r="62" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A62" s="16" t="s">
         <v>628</v>
       </c>
@@ -7737,7 +7748,7 @@
         <v>25000000</v>
       </c>
     </row>
-    <row r="63" spans="1:9" x14ac:dyDescent="0.35">
+    <row r="63" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A63" s="16" t="s">
         <v>627</v>
       </c>
@@ -7769,7 +7780,7 @@
         <v>35000000</v>
       </c>
     </row>
-    <row r="64" spans="1:9" x14ac:dyDescent="0.35">
+    <row r="64" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A64" s="16" t="s">
         <v>630</v>
       </c>
@@ -7801,7 +7812,7 @@
         <v>25000000</v>
       </c>
     </row>
-    <row r="65" spans="1:9" x14ac:dyDescent="0.35">
+    <row r="65" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A65" s="16" t="s">
         <v>629</v>
       </c>
@@ -7833,11 +7844,11 @@
         <v>35000000</v>
       </c>
     </row>
-    <row r="66" spans="1:9" x14ac:dyDescent="0.35">
+    <row r="66" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A66" s="16" t="s">
         <v>631</v>
       </c>
-      <c r="B66" s="25" t="s">
+      <c r="B66" s="17" t="s">
         <v>615</v>
       </c>
       <c r="C66" s="18">
@@ -7861,12 +7872,12 @@
       <c r="H66" s="17" t="s">
         <v>566</v>
       </c>
-      <c r="I66" s="26">
+      <c r="I66" s="19">
         <v>23000000</v>
       </c>
     </row>
-    <row r="67" spans="1:9" x14ac:dyDescent="0.35">
-      <c r="A67" s="27" t="s">
+    <row r="67" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="A67" s="16" t="s">
         <v>632</v>
       </c>
       <c r="B67" s="4" t="s">
@@ -7897,8 +7908,8 @@
         <v>13000000</v>
       </c>
     </row>
-    <row r="68" spans="1:9" x14ac:dyDescent="0.35">
-      <c r="A68" s="27" t="s">
+    <row r="68" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="A68" s="16" t="s">
         <v>633</v>
       </c>
       <c r="B68" s="4" t="s">
@@ -7929,34 +7940,88 @@
         <v>20000000</v>
       </c>
     </row>
-    <row r="69" spans="1:9" x14ac:dyDescent="0.35">
-      <c r="A69" s="27"/>
-      <c r="B69" s="25"/>
-      <c r="C69" s="18"/>
-      <c r="D69" s="18"/>
-      <c r="E69" s="18"/>
-      <c r="F69" s="18"/>
-      <c r="G69" s="17"/>
-      <c r="H69" s="17"/>
-      <c r="I69" s="26"/>
+    <row r="69" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="A69" s="16" t="s">
+        <v>634</v>
+      </c>
+      <c r="B69" s="17" t="s">
+        <v>636</v>
+      </c>
+      <c r="C69" s="18">
+        <v>155000000</v>
+      </c>
+      <c r="D69" s="5">
+        <f t="shared" ref="D69:D70" si="19">I69/1.12</f>
+        <v>5357142.8571428563</v>
+      </c>
+      <c r="E69" s="5">
+        <f t="shared" ref="E69:E70" si="20">D69*90%</f>
+        <v>4821428.5714285709</v>
+      </c>
+      <c r="F69" s="5">
+        <f t="shared" ref="F69:F70" si="21">D69*70%</f>
+        <v>3749999.9999999991</v>
+      </c>
+      <c r="G69" s="3">
+        <v>269</v>
+      </c>
+      <c r="H69" s="17" t="s">
+        <v>638</v>
+      </c>
+      <c r="I69" s="19">
+        <v>6000000</v>
+      </c>
+    </row>
+    <row r="70" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="A70" s="16" t="s">
+        <v>635</v>
+      </c>
+      <c r="B70" s="17" t="s">
+        <v>637</v>
+      </c>
+      <c r="C70" s="18">
+        <v>175000000</v>
+      </c>
+      <c r="D70" s="5">
+        <f t="shared" si="19"/>
+        <v>5357142.8571428563</v>
+      </c>
+      <c r="E70" s="5">
+        <f t="shared" si="20"/>
+        <v>4821428.5714285709</v>
+      </c>
+      <c r="F70" s="5">
+        <f t="shared" si="21"/>
+        <v>3749999.9999999991</v>
+      </c>
+      <c r="G70" s="3">
+        <v>270</v>
+      </c>
+      <c r="H70" s="17" t="s">
+        <v>639</v>
+      </c>
+      <c r="I70" s="19">
+        <v>6000000</v>
+      </c>
     </row>
   </sheetData>
+  <phoneticPr fontId="4" type="noConversion"/>
   <conditionalFormatting sqref="A1:A1048576">
-    <cfRule type="duplicateValues" dxfId="9" priority="2"/>
+    <cfRule type="duplicateValues" dxfId="8" priority="2"/>
   </conditionalFormatting>
   <conditionalFormatting sqref="A33:A41 A43:A46 A2:A31">
-    <cfRule type="duplicateValues" dxfId="8" priority="14"/>
+    <cfRule type="duplicateValues" dxfId="7" priority="14"/>
   </conditionalFormatting>
   <conditionalFormatting sqref="A33:A46 A2:A31">
-    <cfRule type="duplicateValues" dxfId="7" priority="18"/>
+    <cfRule type="duplicateValues" dxfId="6" priority="18"/>
   </conditionalFormatting>
   <conditionalFormatting sqref="H43:H46">
-    <cfRule type="duplicateValues" dxfId="6" priority="7"/>
-    <cfRule type="duplicateValues" dxfId="5" priority="8"/>
+    <cfRule type="duplicateValues" dxfId="5" priority="7"/>
+    <cfRule type="duplicateValues" dxfId="4" priority="8"/>
   </conditionalFormatting>
   <conditionalFormatting sqref="H51:H54">
-    <cfRule type="duplicateValues" dxfId="4" priority="3"/>
-    <cfRule type="duplicateValues" dxfId="3" priority="4"/>
+    <cfRule type="duplicateValues" dxfId="3" priority="3"/>
+    <cfRule type="duplicateValues" dxfId="2" priority="4"/>
   </conditionalFormatting>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <pageSetup paperSize="9" orientation="portrait" horizontalDpi="0" verticalDpi="0" r:id="rId1"/>
@@ -7969,16 +8034,16 @@
 <file path=xl/worksheets/sheet10.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{7F6E2486-F456-4872-8871-82688E1562A6}">
   <dimension ref="A1:F20"/>
-  <sheetFormatPr defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
+  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
-    <col min="1" max="1" width="12.6328125" bestFit="1" customWidth="1"/>
-    <col min="2" max="2" width="16.36328125" bestFit="1" customWidth="1"/>
-    <col min="3" max="3" width="31.90625" bestFit="1" customWidth="1"/>
+    <col min="1" max="1" width="12.5703125" bestFit="1" customWidth="1"/>
+    <col min="2" max="2" width="16.42578125" bestFit="1" customWidth="1"/>
+    <col min="3" max="3" width="31.85546875" bestFit="1" customWidth="1"/>
     <col min="4" max="5" width="32" bestFit="1" customWidth="1"/>
-    <col min="6" max="6" width="31.1796875" bestFit="1" customWidth="1"/>
+    <col min="6" max="6" width="31.140625" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:6" x14ac:dyDescent="0.35">
+    <row r="1" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A1" t="s">
         <v>0</v>
       </c>
@@ -7998,12 +8063,12 @@
         <v>5</v>
       </c>
     </row>
-    <row r="2" spans="1:6" x14ac:dyDescent="0.35">
+    <row r="2" spans="1:6" x14ac:dyDescent="0.25">
       <c r="C2" t="s">
         <v>82</v>
       </c>
     </row>
-    <row r="3" spans="1:6" x14ac:dyDescent="0.35">
+    <row r="3" spans="1:6" x14ac:dyDescent="0.25">
       <c r="B3" t="s">
         <v>8</v>
       </c>
@@ -8020,7 +8085,7 @@
         <v>389</v>
       </c>
     </row>
-    <row r="4" spans="1:6" x14ac:dyDescent="0.35">
+    <row r="4" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A4" t="s">
         <v>14</v>
       </c>
@@ -8040,7 +8105,7 @@
         <v>393</v>
       </c>
     </row>
-    <row r="5" spans="1:6" x14ac:dyDescent="0.35">
+    <row r="5" spans="1:6" x14ac:dyDescent="0.25">
       <c r="B5" t="s">
         <v>152</v>
       </c>
@@ -8057,7 +8122,7 @@
         <v>397</v>
       </c>
     </row>
-    <row r="6" spans="1:6" x14ac:dyDescent="0.35">
+    <row r="6" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A6" t="s">
         <v>27</v>
       </c>
@@ -8077,7 +8142,7 @@
         <v>401</v>
       </c>
     </row>
-    <row r="7" spans="1:6" x14ac:dyDescent="0.35">
+    <row r="7" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A7" t="s">
         <v>34</v>
       </c>
@@ -8097,7 +8162,7 @@
         <v>405</v>
       </c>
     </row>
-    <row r="8" spans="1:6" x14ac:dyDescent="0.35">
+    <row r="8" spans="1:6" x14ac:dyDescent="0.25">
       <c r="B8" t="s">
         <v>41</v>
       </c>
@@ -8114,7 +8179,7 @@
         <v>409</v>
       </c>
     </row>
-    <row r="9" spans="1:6" x14ac:dyDescent="0.35">
+    <row r="9" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A9" t="s">
         <v>47</v>
       </c>
@@ -8134,7 +8199,7 @@
         <v>413</v>
       </c>
     </row>
-    <row r="10" spans="1:6" x14ac:dyDescent="0.35">
+    <row r="10" spans="1:6" x14ac:dyDescent="0.25">
       <c r="B10" t="s">
         <v>123</v>
       </c>
@@ -8151,7 +8216,7 @@
         <v>409</v>
       </c>
     </row>
-    <row r="11" spans="1:6" x14ac:dyDescent="0.35">
+    <row r="11" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A11" t="s">
         <v>321</v>
       </c>
@@ -8171,7 +8236,7 @@
         <v>450000000</v>
       </c>
     </row>
-    <row r="12" spans="1:6" x14ac:dyDescent="0.35">
+    <row r="12" spans="1:6" x14ac:dyDescent="0.25">
       <c r="B12" t="s">
         <v>61</v>
       </c>
@@ -8188,7 +8253,7 @@
         <v>451000000</v>
       </c>
     </row>
-    <row r="13" spans="1:6" x14ac:dyDescent="0.35">
+    <row r="13" spans="1:6" x14ac:dyDescent="0.25">
       <c r="B13" t="s">
         <v>62</v>
       </c>
@@ -8205,7 +8270,7 @@
         <v>450000000</v>
       </c>
     </row>
-    <row r="14" spans="1:6" x14ac:dyDescent="0.35">
+    <row r="14" spans="1:6" x14ac:dyDescent="0.25">
       <c r="B14" t="s">
         <v>63</v>
       </c>
@@ -8222,7 +8287,7 @@
         <v>448800000</v>
       </c>
     </row>
-    <row r="15" spans="1:6" x14ac:dyDescent="0.35">
+    <row r="15" spans="1:6" x14ac:dyDescent="0.25">
       <c r="B15" t="s">
         <v>64</v>
       </c>
@@ -8239,7 +8304,7 @@
         <v>448800000</v>
       </c>
     </row>
-    <row r="16" spans="1:6" x14ac:dyDescent="0.35">
+    <row r="16" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A16" t="s">
         <v>65</v>
       </c>
@@ -8259,7 +8324,7 @@
         <v>466900000</v>
       </c>
     </row>
-    <row r="18" spans="1:6" x14ac:dyDescent="0.35">
+    <row r="18" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A18" t="s">
         <v>0</v>
       </c>
@@ -8279,7 +8344,7 @@
         <v>5</v>
       </c>
     </row>
-    <row r="19" spans="1:6" x14ac:dyDescent="0.35">
+    <row r="19" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A19" t="s">
         <v>135</v>
       </c>
@@ -8299,7 +8364,7 @@
         <v>423</v>
       </c>
     </row>
-    <row r="20" spans="1:6" x14ac:dyDescent="0.35">
+    <row r="20" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A20" t="s">
         <v>76</v>
       </c>
@@ -8328,15 +8393,15 @@
 <file path=xl/worksheets/sheet11.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{F98971A8-4205-45A8-A1C1-D9D164D2942F}">
   <dimension ref="A1:E19"/>
-  <sheetFormatPr defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
+  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
-    <col min="1" max="1" width="12.6328125" bestFit="1" customWidth="1"/>
-    <col min="2" max="2" width="16.36328125" bestFit="1" customWidth="1"/>
-    <col min="3" max="3" width="15.7265625" bestFit="1" customWidth="1"/>
-    <col min="4" max="5" width="15.08984375" bestFit="1" customWidth="1"/>
+    <col min="1" max="1" width="12.5703125" bestFit="1" customWidth="1"/>
+    <col min="2" max="2" width="16.42578125" bestFit="1" customWidth="1"/>
+    <col min="3" max="3" width="15.7109375" bestFit="1" customWidth="1"/>
+    <col min="4" max="5" width="15.140625" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="1" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A1" t="s">
         <v>0</v>
       </c>
@@ -8353,7 +8418,7 @@
         <v>4</v>
       </c>
     </row>
-    <row r="2" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="2" spans="1:5" x14ac:dyDescent="0.25">
       <c r="B2" t="s">
         <v>8</v>
       </c>
@@ -8361,7 +8426,7 @@
         <v>424</v>
       </c>
     </row>
-    <row r="3" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="3" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A3" t="s">
         <v>14</v>
       </c>
@@ -8378,7 +8443,7 @@
         <v>427</v>
       </c>
     </row>
-    <row r="4" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="4" spans="1:5" x14ac:dyDescent="0.25">
       <c r="B4" t="s">
         <v>152</v>
       </c>
@@ -8392,7 +8457,7 @@
         <v>430</v>
       </c>
     </row>
-    <row r="5" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="5" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A5" t="s">
         <v>27</v>
       </c>
@@ -8409,7 +8474,7 @@
         <v>433</v>
       </c>
     </row>
-    <row r="6" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="6" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A6" t="s">
         <v>34</v>
       </c>
@@ -8426,7 +8491,7 @@
         <v>436</v>
       </c>
     </row>
-    <row r="7" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="7" spans="1:5" x14ac:dyDescent="0.25">
       <c r="B7" t="s">
         <v>41</v>
       </c>
@@ -8440,7 +8505,7 @@
         <v>438</v>
       </c>
     </row>
-    <row r="8" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="8" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A8" t="s">
         <v>115</v>
       </c>
@@ -8457,7 +8522,7 @@
         <v>441</v>
       </c>
     </row>
-    <row r="9" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="9" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A9" t="s">
         <v>122</v>
       </c>
@@ -8474,7 +8539,7 @@
         <v>438</v>
       </c>
     </row>
-    <row r="10" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="10" spans="1:5" x14ac:dyDescent="0.25">
       <c r="B10" t="s">
         <v>56</v>
       </c>
@@ -8488,7 +8553,7 @@
         <v>444</v>
       </c>
     </row>
-    <row r="11" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="11" spans="1:5" x14ac:dyDescent="0.25">
       <c r="B11" t="s">
         <v>61</v>
       </c>
@@ -8502,7 +8567,7 @@
         <v>444</v>
       </c>
     </row>
-    <row r="12" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="12" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A12" t="s">
         <v>55</v>
       </c>
@@ -8519,7 +8584,7 @@
         <v>444</v>
       </c>
     </row>
-    <row r="13" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="13" spans="1:5" x14ac:dyDescent="0.25">
       <c r="B13" t="s">
         <v>63</v>
       </c>
@@ -8533,7 +8598,7 @@
         <v>444</v>
       </c>
     </row>
-    <row r="14" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="14" spans="1:5" x14ac:dyDescent="0.25">
       <c r="B14" t="s">
         <v>64</v>
       </c>
@@ -8547,7 +8612,7 @@
         <v>444</v>
       </c>
     </row>
-    <row r="15" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="15" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A15" t="s">
         <v>65</v>
       </c>
@@ -8564,7 +8629,7 @@
         <v>447</v>
       </c>
     </row>
-    <row r="17" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="17" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A17" t="s">
         <v>0</v>
       </c>
@@ -8581,7 +8646,7 @@
         <v>4</v>
       </c>
     </row>
-    <row r="18" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="18" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A18" t="s">
         <v>135</v>
       </c>
@@ -8598,7 +8663,7 @@
         <v>450</v>
       </c>
     </row>
-    <row r="19" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="19" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A19" t="s">
         <v>76</v>
       </c>
@@ -8624,15 +8689,15 @@
 <file path=xl/worksheets/sheet12.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{516E8F5E-7978-4DDA-9413-77E8ECD441FC}">
   <dimension ref="A1:E20"/>
-  <sheetFormatPr defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
+  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
-    <col min="1" max="1" width="12.6328125" bestFit="1" customWidth="1"/>
-    <col min="2" max="2" width="16.36328125" bestFit="1" customWidth="1"/>
-    <col min="3" max="3" width="31.1796875" bestFit="1" customWidth="1"/>
-    <col min="4" max="5" width="32.1796875" bestFit="1" customWidth="1"/>
+    <col min="1" max="1" width="12.5703125" bestFit="1" customWidth="1"/>
+    <col min="2" max="2" width="16.42578125" bestFit="1" customWidth="1"/>
+    <col min="3" max="3" width="31.140625" bestFit="1" customWidth="1"/>
+    <col min="4" max="5" width="32.140625" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="1" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A1" t="s">
         <v>0</v>
       </c>
@@ -8649,12 +8714,12 @@
         <v>4</v>
       </c>
     </row>
-    <row r="2" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="2" spans="1:5" x14ac:dyDescent="0.25">
       <c r="C2" t="s">
         <v>82</v>
       </c>
     </row>
-    <row r="3" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="3" spans="1:5" x14ac:dyDescent="0.25">
       <c r="B3" t="s">
         <v>8</v>
       </c>
@@ -8668,7 +8733,7 @@
         <v>455</v>
       </c>
     </row>
-    <row r="4" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="4" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A4" t="s">
         <v>14</v>
       </c>
@@ -8685,7 +8750,7 @@
         <v>458</v>
       </c>
     </row>
-    <row r="5" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="5" spans="1:5" x14ac:dyDescent="0.25">
       <c r="B5" t="s">
         <v>152</v>
       </c>
@@ -8699,7 +8764,7 @@
         <v>461</v>
       </c>
     </row>
-    <row r="6" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="6" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A6" t="s">
         <v>27</v>
       </c>
@@ -8716,7 +8781,7 @@
         <v>464</v>
       </c>
     </row>
-    <row r="7" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="7" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A7" t="s">
         <v>465</v>
       </c>
@@ -8733,7 +8798,7 @@
         <v>468</v>
       </c>
     </row>
-    <row r="8" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="8" spans="1:5" x14ac:dyDescent="0.25">
       <c r="B8" t="s">
         <v>41</v>
       </c>
@@ -8747,7 +8812,7 @@
         <v>471</v>
       </c>
     </row>
-    <row r="9" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="9" spans="1:5" x14ac:dyDescent="0.25">
       <c r="B9" t="s">
         <v>48</v>
       </c>
@@ -8761,7 +8826,7 @@
         <v>468</v>
       </c>
     </row>
-    <row r="10" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="10" spans="1:5" x14ac:dyDescent="0.25">
       <c r="B10" t="s">
         <v>54</v>
       </c>
@@ -8775,7 +8840,7 @@
         <v>471</v>
       </c>
     </row>
-    <row r="11" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="11" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A11" t="s">
         <v>472</v>
       </c>
@@ -8792,7 +8857,7 @@
         <v>475</v>
       </c>
     </row>
-    <row r="12" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="12" spans="1:5" x14ac:dyDescent="0.25">
       <c r="B12" t="s">
         <v>61</v>
       </c>
@@ -8806,7 +8871,7 @@
         <v>475</v>
       </c>
     </row>
-    <row r="13" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="13" spans="1:5" x14ac:dyDescent="0.25">
       <c r="B13" t="s">
         <v>62</v>
       </c>
@@ -8820,7 +8885,7 @@
         <v>475</v>
       </c>
     </row>
-    <row r="14" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="14" spans="1:5" x14ac:dyDescent="0.25">
       <c r="B14" t="s">
         <v>63</v>
       </c>
@@ -8834,7 +8899,7 @@
         <v>475</v>
       </c>
     </row>
-    <row r="15" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="15" spans="1:5" x14ac:dyDescent="0.25">
       <c r="B15" t="s">
         <v>64</v>
       </c>
@@ -8848,7 +8913,7 @@
         <v>475</v>
       </c>
     </row>
-    <row r="16" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="16" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A16" t="s">
         <v>65</v>
       </c>
@@ -8865,7 +8930,7 @@
         <v>478</v>
       </c>
     </row>
-    <row r="18" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="18" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A18" t="s">
         <v>0</v>
       </c>
@@ -8882,7 +8947,7 @@
         <v>4</v>
       </c>
     </row>
-    <row r="19" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="19" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A19" t="s">
         <v>135</v>
       </c>
@@ -8899,7 +8964,7 @@
         <v>481</v>
       </c>
     </row>
-    <row r="20" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="20" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A20" t="s">
         <v>76</v>
       </c>
@@ -8925,18 +8990,18 @@
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{669692EE-8762-4650-B2E9-8C0B02D25245}">
   <dimension ref="A1:H34"/>
-  <sheetFormatPr defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
+  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
-    <col min="1" max="1" width="51.453125" bestFit="1" customWidth="1"/>
-    <col min="2" max="2" width="36.54296875" bestFit="1" customWidth="1"/>
-    <col min="3" max="3" width="14.6328125" bestFit="1" customWidth="1"/>
-    <col min="4" max="4" width="12.6328125" bestFit="1" customWidth="1"/>
-    <col min="5" max="6" width="16.08984375" bestFit="1" customWidth="1"/>
+    <col min="1" max="1" width="51.42578125" bestFit="1" customWidth="1"/>
+    <col min="2" max="2" width="36.5703125" bestFit="1" customWidth="1"/>
+    <col min="3" max="3" width="14.5703125" bestFit="1" customWidth="1"/>
+    <col min="4" max="4" width="12.5703125" bestFit="1" customWidth="1"/>
+    <col min="5" max="6" width="16.140625" bestFit="1" customWidth="1"/>
     <col min="7" max="7" width="9" bestFit="1" customWidth="1"/>
-    <col min="8" max="8" width="14.453125" bestFit="1" customWidth="1"/>
+    <col min="8" max="8" width="14.42578125" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:8" x14ac:dyDescent="0.35">
+    <row r="1" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A1" s="4" t="s">
         <v>551</v>
       </c>
@@ -8962,7 +9027,7 @@
         <v>564</v>
       </c>
     </row>
-    <row r="2" spans="1:8" x14ac:dyDescent="0.35">
+    <row r="2" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A2" s="4" t="s">
         <v>514</v>
       </c>
@@ -8992,7 +9057,7 @@
         <v>565</v>
       </c>
     </row>
-    <row r="3" spans="1:8" x14ac:dyDescent="0.35">
+    <row r="3" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A3" s="4" t="s">
         <v>547</v>
       </c>
@@ -9022,7 +9087,7 @@
         <v>565</v>
       </c>
     </row>
-    <row r="4" spans="1:8" x14ac:dyDescent="0.35">
+    <row r="4" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A4" s="4" t="s">
         <v>515</v>
       </c>
@@ -9052,7 +9117,7 @@
         <v>565</v>
       </c>
     </row>
-    <row r="5" spans="1:8" x14ac:dyDescent="0.35">
+    <row r="5" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A5" s="4" t="s">
         <v>516</v>
       </c>
@@ -9082,7 +9147,7 @@
         <v>565</v>
       </c>
     </row>
-    <row r="6" spans="1:8" x14ac:dyDescent="0.35">
+    <row r="6" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A6" s="4" t="s">
         <v>496</v>
       </c>
@@ -9112,7 +9177,7 @@
         <v>565</v>
       </c>
     </row>
-    <row r="7" spans="1:8" x14ac:dyDescent="0.35">
+    <row r="7" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A7" s="4" t="s">
         <v>497</v>
       </c>
@@ -9142,7 +9207,7 @@
         <v>565</v>
       </c>
     </row>
-    <row r="8" spans="1:8" x14ac:dyDescent="0.35">
+    <row r="8" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A8" s="4" t="s">
         <v>517</v>
       </c>
@@ -9172,7 +9237,7 @@
         <v>566</v>
       </c>
     </row>
-    <row r="9" spans="1:8" x14ac:dyDescent="0.35">
+    <row r="9" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A9" s="4" t="s">
         <v>518</v>
       </c>
@@ -9202,7 +9267,7 @@
         <v>566</v>
       </c>
     </row>
-    <row r="10" spans="1:8" x14ac:dyDescent="0.35">
+    <row r="10" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A10" s="4" t="s">
         <v>519</v>
       </c>
@@ -9232,7 +9297,7 @@
         <v>566</v>
       </c>
     </row>
-    <row r="11" spans="1:8" x14ac:dyDescent="0.35">
+    <row r="11" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A11" s="4" t="s">
         <v>523</v>
       </c>
@@ -9262,7 +9327,7 @@
         <v>568</v>
       </c>
     </row>
-    <row r="12" spans="1:8" x14ac:dyDescent="0.35">
+    <row r="12" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A12" s="4" t="s">
         <v>524</v>
       </c>
@@ -9292,7 +9357,7 @@
         <v>573</v>
       </c>
     </row>
-    <row r="13" spans="1:8" x14ac:dyDescent="0.35">
+    <row r="13" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A13" s="4" t="s">
         <v>498</v>
       </c>
@@ -9322,7 +9387,7 @@
         <v>573</v>
       </c>
     </row>
-    <row r="14" spans="1:8" x14ac:dyDescent="0.35">
+    <row r="14" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A14" s="4" t="s">
         <v>527</v>
       </c>
@@ -9352,7 +9417,7 @@
         <v>567</v>
       </c>
     </row>
-    <row r="15" spans="1:8" x14ac:dyDescent="0.35">
+    <row r="15" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A15" s="4" t="s">
         <v>528</v>
       </c>
@@ -9382,7 +9447,7 @@
         <v>567</v>
       </c>
     </row>
-    <row r="16" spans="1:8" x14ac:dyDescent="0.35">
+    <row r="16" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A16" s="4" t="s">
         <v>525</v>
       </c>
@@ -9412,7 +9477,7 @@
         <v>567</v>
       </c>
     </row>
-    <row r="17" spans="1:8" x14ac:dyDescent="0.35">
+    <row r="17" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A17" s="4" t="s">
         <v>499</v>
       </c>
@@ -9442,7 +9507,7 @@
         <v>567</v>
       </c>
     </row>
-    <row r="18" spans="1:8" x14ac:dyDescent="0.35">
+    <row r="18" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A18" s="4" t="s">
         <v>555</v>
       </c>
@@ -9472,7 +9537,7 @@
         <v>574</v>
       </c>
     </row>
-    <row r="19" spans="1:8" x14ac:dyDescent="0.35">
+    <row r="19" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A19" s="4" t="s">
         <v>500</v>
       </c>
@@ -9502,7 +9567,7 @@
         <v>569</v>
       </c>
     </row>
-    <row r="20" spans="1:8" x14ac:dyDescent="0.35">
+    <row r="20" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A20" s="4" t="s">
         <v>501</v>
       </c>
@@ -9532,7 +9597,7 @@
         <v>575</v>
       </c>
     </row>
-    <row r="21" spans="1:8" x14ac:dyDescent="0.35">
+    <row r="21" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A21" s="4" t="s">
         <v>502</v>
       </c>
@@ -9562,7 +9627,7 @@
         <v>570</v>
       </c>
     </row>
-    <row r="22" spans="1:8" x14ac:dyDescent="0.35">
+    <row r="22" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A22" s="4" t="s">
         <v>503</v>
       </c>
@@ -9592,7 +9657,7 @@
         <v>576</v>
       </c>
     </row>
-    <row r="23" spans="1:8" x14ac:dyDescent="0.35">
+    <row r="23" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A23" s="4" t="s">
         <v>504</v>
       </c>
@@ -9622,7 +9687,7 @@
         <v>577</v>
       </c>
     </row>
-    <row r="24" spans="1:8" x14ac:dyDescent="0.35">
+    <row r="24" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A24" s="4" t="s">
         <v>505</v>
       </c>
@@ -9652,7 +9717,7 @@
         <v>578</v>
       </c>
     </row>
-    <row r="25" spans="1:8" x14ac:dyDescent="0.35">
+    <row r="25" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A25" s="4" t="s">
         <v>557</v>
       </c>
@@ -9682,7 +9747,7 @@
         <v>571</v>
       </c>
     </row>
-    <row r="26" spans="1:8" x14ac:dyDescent="0.35">
+    <row r="26" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A26" s="4" t="s">
         <v>558</v>
       </c>
@@ -9712,7 +9777,7 @@
         <v>571</v>
       </c>
     </row>
-    <row r="27" spans="1:8" x14ac:dyDescent="0.35">
+    <row r="27" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A27" s="4" t="s">
         <v>506</v>
       </c>
@@ -9742,7 +9807,7 @@
         <v>571</v>
       </c>
     </row>
-    <row r="28" spans="1:8" x14ac:dyDescent="0.35">
+    <row r="28" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A28" s="4" t="s">
         <v>529</v>
       </c>
@@ -9772,7 +9837,7 @@
         <v>572</v>
       </c>
     </row>
-    <row r="29" spans="1:8" x14ac:dyDescent="0.35">
+    <row r="29" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A29" s="4" t="s">
         <v>520</v>
       </c>
@@ -9802,7 +9867,7 @@
         <v>572</v>
       </c>
     </row>
-    <row r="30" spans="1:8" x14ac:dyDescent="0.35">
+    <row r="30" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A30" s="4" t="s">
         <v>521</v>
       </c>
@@ -9832,7 +9897,7 @@
         <v>579</v>
       </c>
     </row>
-    <row r="31" spans="1:8" x14ac:dyDescent="0.35">
+    <row r="31" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A31" s="4" t="s">
         <v>526</v>
       </c>
@@ -9862,7 +9927,7 @@
         <v>579</v>
       </c>
     </row>
-    <row r="32" spans="1:8" x14ac:dyDescent="0.35">
+    <row r="32" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A32" s="4" t="s">
         <v>560</v>
       </c>
@@ -9892,7 +9957,7 @@
         <v>568</v>
       </c>
     </row>
-    <row r="33" spans="1:8" x14ac:dyDescent="0.35">
+    <row r="33" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A33" s="4" t="s">
         <v>561</v>
       </c>
@@ -9922,7 +9987,7 @@
         <v>571</v>
       </c>
     </row>
-    <row r="34" spans="1:8" x14ac:dyDescent="0.35">
+    <row r="34" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A34" s="6" t="s">
         <v>522</v>
       </c>
@@ -9954,10 +10019,10 @@
     </row>
   </sheetData>
   <conditionalFormatting sqref="A2:A33">
-    <cfRule type="duplicateValues" dxfId="2" priority="1"/>
+    <cfRule type="duplicateValues" dxfId="1" priority="1"/>
   </conditionalFormatting>
   <conditionalFormatting sqref="A2:A34">
-    <cfRule type="duplicateValues" dxfId="1" priority="2"/>
+    <cfRule type="duplicateValues" dxfId="0" priority="2"/>
   </conditionalFormatting>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>
@@ -9966,16 +10031,16 @@
 <file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{91056C88-91FB-4BF3-9450-351335B49911}">
   <dimension ref="A1:G21"/>
-  <sheetFormatPr defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
+  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="1" max="1" width="13" bestFit="1" customWidth="1"/>
-    <col min="2" max="2" width="21.36328125" bestFit="1" customWidth="1"/>
-    <col min="3" max="4" width="24.36328125" bestFit="1" customWidth="1"/>
-    <col min="5" max="5" width="23.7265625" bestFit="1" customWidth="1"/>
-    <col min="6" max="7" width="24.36328125" bestFit="1" customWidth="1"/>
+    <col min="2" max="2" width="21.42578125" bestFit="1" customWidth="1"/>
+    <col min="3" max="4" width="24.42578125" bestFit="1" customWidth="1"/>
+    <col min="5" max="5" width="23.7109375" bestFit="1" customWidth="1"/>
+    <col min="6" max="7" width="24.42578125" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:7" x14ac:dyDescent="0.35">
+    <row r="1" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A1" t="s">
         <v>0</v>
       </c>
@@ -9998,12 +10063,12 @@
         <v>6</v>
       </c>
     </row>
-    <row r="2" spans="1:7" x14ac:dyDescent="0.35">
+    <row r="2" spans="1:7" x14ac:dyDescent="0.25">
       <c r="C2" t="s">
         <v>7</v>
       </c>
     </row>
-    <row r="3" spans="1:7" x14ac:dyDescent="0.35">
+    <row r="3" spans="1:7" x14ac:dyDescent="0.25">
       <c r="B3" t="s">
         <v>8</v>
       </c>
@@ -10023,7 +10088,7 @@
         <v>13</v>
       </c>
     </row>
-    <row r="4" spans="1:7" x14ac:dyDescent="0.35">
+    <row r="4" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A4" t="s">
         <v>14</v>
       </c>
@@ -10046,7 +10111,7 @@
         <v>20</v>
       </c>
     </row>
-    <row r="5" spans="1:7" x14ac:dyDescent="0.35">
+    <row r="5" spans="1:7" x14ac:dyDescent="0.25">
       <c r="B5" t="s">
         <v>21</v>
       </c>
@@ -10066,7 +10131,7 @@
         <v>26</v>
       </c>
     </row>
-    <row r="6" spans="1:7" x14ac:dyDescent="0.35">
+    <row r="6" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A6" t="s">
         <v>27</v>
       </c>
@@ -10089,7 +10154,7 @@
         <v>33</v>
       </c>
     </row>
-    <row r="7" spans="1:7" x14ac:dyDescent="0.35">
+    <row r="7" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A7" t="s">
         <v>34</v>
       </c>
@@ -10112,7 +10177,7 @@
         <v>40</v>
       </c>
     </row>
-    <row r="8" spans="1:7" x14ac:dyDescent="0.35">
+    <row r="8" spans="1:7" x14ac:dyDescent="0.25">
       <c r="B8" t="s">
         <v>41</v>
       </c>
@@ -10132,7 +10197,7 @@
         <v>46</v>
       </c>
     </row>
-    <row r="9" spans="1:7" x14ac:dyDescent="0.35">
+    <row r="9" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A9" t="s">
         <v>47</v>
       </c>
@@ -10155,7 +10220,7 @@
         <v>53</v>
       </c>
     </row>
-    <row r="10" spans="1:7" x14ac:dyDescent="0.35">
+    <row r="10" spans="1:7" x14ac:dyDescent="0.25">
       <c r="B10" t="s">
         <v>54</v>
       </c>
@@ -10175,7 +10240,7 @@
         <v>46</v>
       </c>
     </row>
-    <row r="11" spans="1:7" x14ac:dyDescent="0.35">
+    <row r="11" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A11" t="s">
         <v>55</v>
       </c>
@@ -10198,7 +10263,7 @@
         <v>45</v>
       </c>
     </row>
-    <row r="12" spans="1:7" x14ac:dyDescent="0.35">
+    <row r="12" spans="1:7" x14ac:dyDescent="0.25">
       <c r="B12" t="s">
         <v>61</v>
       </c>
@@ -10218,7 +10283,7 @@
         <v>45</v>
       </c>
     </row>
-    <row r="13" spans="1:7" x14ac:dyDescent="0.35">
+    <row r="13" spans="1:7" x14ac:dyDescent="0.25">
       <c r="B13" t="s">
         <v>62</v>
       </c>
@@ -10238,7 +10303,7 @@
         <v>45</v>
       </c>
     </row>
-    <row r="14" spans="1:7" x14ac:dyDescent="0.35">
+    <row r="14" spans="1:7" x14ac:dyDescent="0.25">
       <c r="B14" t="s">
         <v>63</v>
       </c>
@@ -10258,7 +10323,7 @@
         <v>45</v>
       </c>
     </row>
-    <row r="15" spans="1:7" x14ac:dyDescent="0.35">
+    <row r="15" spans="1:7" x14ac:dyDescent="0.25">
       <c r="B15" t="s">
         <v>64</v>
       </c>
@@ -10278,7 +10343,7 @@
         <v>45</v>
       </c>
     </row>
-    <row r="16" spans="1:7" x14ac:dyDescent="0.35">
+    <row r="16" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A16" t="s">
         <v>65</v>
       </c>
@@ -10301,7 +10366,7 @@
         <v>71</v>
       </c>
     </row>
-    <row r="19" spans="1:7" x14ac:dyDescent="0.35">
+    <row r="19" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A19" t="s">
         <v>0</v>
       </c>
@@ -10324,7 +10389,7 @@
         <v>554</v>
       </c>
     </row>
-    <row r="20" spans="1:7" x14ac:dyDescent="0.35">
+    <row r="20" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A20" t="s">
         <v>72</v>
       </c>
@@ -10344,7 +10409,7 @@
         <v>75</v>
       </c>
     </row>
-    <row r="21" spans="1:7" x14ac:dyDescent="0.35">
+    <row r="21" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A21" t="s">
         <v>76</v>
       </c>
@@ -10376,19 +10441,19 @@
 <file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{0BBF25D8-DE3B-40F5-A8DF-270BBD1A35C9}">
   <dimension ref="A1:H20"/>
-  <sheetFormatPr defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
+  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
-    <col min="1" max="1" width="12.6328125" bestFit="1" customWidth="1"/>
-    <col min="2" max="2" width="16.36328125" bestFit="1" customWidth="1"/>
-    <col min="3" max="3" width="26.08984375" bestFit="1" customWidth="1"/>
-    <col min="4" max="4" width="28.7265625" bestFit="1" customWidth="1"/>
+    <col min="1" max="1" width="12.5703125" bestFit="1" customWidth="1"/>
+    <col min="2" max="2" width="16.42578125" bestFit="1" customWidth="1"/>
+    <col min="3" max="3" width="26.140625" bestFit="1" customWidth="1"/>
+    <col min="4" max="4" width="28.7109375" bestFit="1" customWidth="1"/>
     <col min="5" max="5" width="33" bestFit="1" customWidth="1"/>
-    <col min="6" max="6" width="31.26953125" bestFit="1" customWidth="1"/>
-    <col min="7" max="7" width="29.54296875" bestFit="1" customWidth="1"/>
-    <col min="8" max="8" width="30.1796875" bestFit="1" customWidth="1"/>
+    <col min="6" max="6" width="31.28515625" bestFit="1" customWidth="1"/>
+    <col min="7" max="7" width="29.5703125" bestFit="1" customWidth="1"/>
+    <col min="8" max="8" width="30.140625" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:8" x14ac:dyDescent="0.35">
+    <row r="1" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A1" t="s">
         <v>0</v>
       </c>
@@ -10414,12 +10479,12 @@
         <v>81</v>
       </c>
     </row>
-    <row r="2" spans="1:8" x14ac:dyDescent="0.35">
+    <row r="2" spans="1:8" x14ac:dyDescent="0.25">
       <c r="D2" t="s">
         <v>82</v>
       </c>
     </row>
-    <row r="3" spans="1:8" x14ac:dyDescent="0.35">
+    <row r="3" spans="1:8" x14ac:dyDescent="0.25">
       <c r="B3" t="s">
         <v>8</v>
       </c>
@@ -10442,7 +10507,7 @@
         <v>83</v>
       </c>
     </row>
-    <row r="4" spans="1:8" x14ac:dyDescent="0.35">
+    <row r="4" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A4" t="s">
         <v>14</v>
       </c>
@@ -10468,7 +10533,7 @@
         <v>89</v>
       </c>
     </row>
-    <row r="5" spans="1:8" x14ac:dyDescent="0.35">
+    <row r="5" spans="1:8" x14ac:dyDescent="0.25">
       <c r="B5" t="s">
         <v>90</v>
       </c>
@@ -10491,7 +10556,7 @@
         <v>95</v>
       </c>
     </row>
-    <row r="6" spans="1:8" x14ac:dyDescent="0.35">
+    <row r="6" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A6" t="s">
         <v>27</v>
       </c>
@@ -10517,7 +10582,7 @@
         <v>101</v>
       </c>
     </row>
-    <row r="7" spans="1:8" x14ac:dyDescent="0.35">
+    <row r="7" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A7" t="s">
         <v>34</v>
       </c>
@@ -10543,7 +10608,7 @@
         <v>108</v>
       </c>
     </row>
-    <row r="8" spans="1:8" x14ac:dyDescent="0.35">
+    <row r="8" spans="1:8" x14ac:dyDescent="0.25">
       <c r="B8" t="s">
         <v>41</v>
       </c>
@@ -10566,7 +10631,7 @@
         <v>114</v>
       </c>
     </row>
-    <row r="9" spans="1:8" x14ac:dyDescent="0.35">
+    <row r="9" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A9" t="s">
         <v>115</v>
       </c>
@@ -10592,7 +10657,7 @@
         <v>121</v>
       </c>
     </row>
-    <row r="10" spans="1:8" x14ac:dyDescent="0.35">
+    <row r="10" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A10" t="s">
         <v>122</v>
       </c>
@@ -10618,7 +10683,7 @@
         <v>114</v>
       </c>
     </row>
-    <row r="11" spans="1:8" x14ac:dyDescent="0.35">
+    <row r="11" spans="1:8" x14ac:dyDescent="0.25">
       <c r="B11" t="s">
         <v>56</v>
       </c>
@@ -10641,7 +10706,7 @@
         <v>128</v>
       </c>
     </row>
-    <row r="12" spans="1:8" x14ac:dyDescent="0.35">
+    <row r="12" spans="1:8" x14ac:dyDescent="0.25">
       <c r="B12" t="s">
         <v>61</v>
       </c>
@@ -10664,7 +10729,7 @@
         <v>128</v>
       </c>
     </row>
-    <row r="13" spans="1:8" x14ac:dyDescent="0.35">
+    <row r="13" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A13" t="s">
         <v>55</v>
       </c>
@@ -10690,7 +10755,7 @@
         <v>128</v>
       </c>
     </row>
-    <row r="14" spans="1:8" x14ac:dyDescent="0.35">
+    <row r="14" spans="1:8" x14ac:dyDescent="0.25">
       <c r="B14" t="s">
         <v>63</v>
       </c>
@@ -10713,7 +10778,7 @@
         <v>128</v>
       </c>
     </row>
-    <row r="15" spans="1:8" x14ac:dyDescent="0.35">
+    <row r="15" spans="1:8" x14ac:dyDescent="0.25">
       <c r="B15" t="s">
         <v>64</v>
       </c>
@@ -10736,7 +10801,7 @@
         <v>128</v>
       </c>
     </row>
-    <row r="16" spans="1:8" x14ac:dyDescent="0.35">
+    <row r="16" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A16" t="s">
         <v>65</v>
       </c>
@@ -10762,7 +10827,7 @@
         <v>134</v>
       </c>
     </row>
-    <row r="18" spans="1:8" x14ac:dyDescent="0.35">
+    <row r="18" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A18" t="s">
         <v>0</v>
       </c>
@@ -10788,7 +10853,7 @@
         <v>81</v>
       </c>
     </row>
-    <row r="19" spans="1:8" x14ac:dyDescent="0.35">
+    <row r="19" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A19" t="s">
         <v>135</v>
       </c>
@@ -10814,7 +10879,7 @@
         <v>141</v>
       </c>
     </row>
-    <row r="20" spans="1:8" x14ac:dyDescent="0.35">
+    <row r="20" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A20" t="s">
         <v>76</v>
       </c>
@@ -10849,17 +10914,17 @@
 <file path=xl/worksheets/sheet5.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{19FA074E-AB8F-493A-A8F2-7BB84CEBBA91}">
   <dimension ref="A1:F20"/>
-  <sheetFormatPr defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
+  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
-    <col min="1" max="1" width="12.6328125" bestFit="1" customWidth="1"/>
-    <col min="2" max="2" width="16.36328125" bestFit="1" customWidth="1"/>
-    <col min="3" max="3" width="18.81640625" bestFit="1" customWidth="1"/>
-    <col min="4" max="4" width="20.36328125" bestFit="1" customWidth="1"/>
-    <col min="5" max="5" width="18.54296875" bestFit="1" customWidth="1"/>
-    <col min="6" max="6" width="19.54296875" bestFit="1" customWidth="1"/>
+    <col min="1" max="1" width="12.5703125" bestFit="1" customWidth="1"/>
+    <col min="2" max="2" width="16.42578125" bestFit="1" customWidth="1"/>
+    <col min="3" max="3" width="18.85546875" bestFit="1" customWidth="1"/>
+    <col min="4" max="4" width="20.42578125" bestFit="1" customWidth="1"/>
+    <col min="5" max="5" width="18.5703125" bestFit="1" customWidth="1"/>
+    <col min="6" max="6" width="19.5703125" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:6" x14ac:dyDescent="0.35">
+    <row r="1" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A1" t="s">
         <v>0</v>
       </c>
@@ -10879,12 +10944,12 @@
         <v>5</v>
       </c>
     </row>
-    <row r="2" spans="1:6" x14ac:dyDescent="0.35">
+    <row r="2" spans="1:6" x14ac:dyDescent="0.25">
       <c r="C2" t="s">
         <v>82</v>
       </c>
     </row>
-    <row r="3" spans="1:6" x14ac:dyDescent="0.35">
+    <row r="3" spans="1:6" x14ac:dyDescent="0.25">
       <c r="B3" t="s">
         <v>8</v>
       </c>
@@ -10901,7 +10966,7 @@
         <v>12</v>
       </c>
     </row>
-    <row r="4" spans="1:6" x14ac:dyDescent="0.35">
+    <row r="4" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A4" t="s">
         <v>14</v>
       </c>
@@ -10921,7 +10986,7 @@
         <v>151</v>
       </c>
     </row>
-    <row r="5" spans="1:6" x14ac:dyDescent="0.35">
+    <row r="5" spans="1:6" x14ac:dyDescent="0.25">
       <c r="B5" t="s">
         <v>152</v>
       </c>
@@ -10938,7 +11003,7 @@
         <v>156</v>
       </c>
     </row>
-    <row r="6" spans="1:6" x14ac:dyDescent="0.35">
+    <row r="6" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A6" t="s">
         <v>27</v>
       </c>
@@ -10958,7 +11023,7 @@
         <v>160</v>
       </c>
     </row>
-    <row r="7" spans="1:6" x14ac:dyDescent="0.35">
+    <row r="7" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A7" t="s">
         <v>34</v>
       </c>
@@ -10978,7 +11043,7 @@
         <v>164</v>
       </c>
     </row>
-    <row r="8" spans="1:6" x14ac:dyDescent="0.35">
+    <row r="8" spans="1:6" x14ac:dyDescent="0.25">
       <c r="B8" t="s">
         <v>41</v>
       </c>
@@ -10995,7 +11060,7 @@
         <v>168</v>
       </c>
     </row>
-    <row r="9" spans="1:6" x14ac:dyDescent="0.35">
+    <row r="9" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A9" t="s">
         <v>115</v>
       </c>
@@ -11015,7 +11080,7 @@
         <v>170</v>
       </c>
     </row>
-    <row r="10" spans="1:6" x14ac:dyDescent="0.35">
+    <row r="10" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A10" t="s">
         <v>122</v>
       </c>
@@ -11035,7 +11100,7 @@
         <v>168</v>
       </c>
     </row>
-    <row r="11" spans="1:6" x14ac:dyDescent="0.35">
+    <row r="11" spans="1:6" x14ac:dyDescent="0.25">
       <c r="B11" t="s">
         <v>56</v>
       </c>
@@ -11052,7 +11117,7 @@
         <v>172</v>
       </c>
     </row>
-    <row r="12" spans="1:6" x14ac:dyDescent="0.35">
+    <row r="12" spans="1:6" x14ac:dyDescent="0.25">
       <c r="B12" t="s">
         <v>61</v>
       </c>
@@ -11069,7 +11134,7 @@
         <v>172</v>
       </c>
     </row>
-    <row r="13" spans="1:6" x14ac:dyDescent="0.35">
+    <row r="13" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A13" t="s">
         <v>55</v>
       </c>
@@ -11089,7 +11154,7 @@
         <v>172</v>
       </c>
     </row>
-    <row r="14" spans="1:6" x14ac:dyDescent="0.35">
+    <row r="14" spans="1:6" x14ac:dyDescent="0.25">
       <c r="B14" t="s">
         <v>63</v>
       </c>
@@ -11106,7 +11171,7 @@
         <v>172</v>
       </c>
     </row>
-    <row r="15" spans="1:6" x14ac:dyDescent="0.35">
+    <row r="15" spans="1:6" x14ac:dyDescent="0.25">
       <c r="B15" t="s">
         <v>64</v>
       </c>
@@ -11123,7 +11188,7 @@
         <v>172</v>
       </c>
     </row>
-    <row r="16" spans="1:6" x14ac:dyDescent="0.35">
+    <row r="16" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A16" t="s">
         <v>65</v>
       </c>
@@ -11143,7 +11208,7 @@
         <v>176</v>
       </c>
     </row>
-    <row r="18" spans="1:6" x14ac:dyDescent="0.35">
+    <row r="18" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A18" t="s">
         <v>0</v>
       </c>
@@ -11163,7 +11228,7 @@
         <v>5</v>
       </c>
     </row>
-    <row r="19" spans="1:6" x14ac:dyDescent="0.35">
+    <row r="19" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A19" t="s">
         <v>135</v>
       </c>
@@ -11183,7 +11248,7 @@
         <v>151</v>
       </c>
     </row>
-    <row r="20" spans="1:6" x14ac:dyDescent="0.35">
+    <row r="20" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A20" t="s">
         <v>76</v>
       </c>
@@ -11212,23 +11277,23 @@
 <file path=xl/worksheets/sheet6.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{1FB12C43-352D-4DE0-BEE7-738405355D14}">
   <dimension ref="A1:L20"/>
-  <sheetFormatPr defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
+  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
-    <col min="1" max="1" width="12.6328125" bestFit="1" customWidth="1"/>
-    <col min="2" max="2" width="16.36328125" bestFit="1" customWidth="1"/>
-    <col min="3" max="3" width="22.453125" bestFit="1" customWidth="1"/>
-    <col min="4" max="4" width="26.81640625" bestFit="1" customWidth="1"/>
-    <col min="5" max="5" width="27.453125" bestFit="1" customWidth="1"/>
-    <col min="6" max="6" width="25.1796875" bestFit="1" customWidth="1"/>
-    <col min="7" max="7" width="22.6328125" bestFit="1" customWidth="1"/>
+    <col min="1" max="1" width="12.5703125" bestFit="1" customWidth="1"/>
+    <col min="2" max="2" width="16.42578125" bestFit="1" customWidth="1"/>
+    <col min="3" max="3" width="22.42578125" bestFit="1" customWidth="1"/>
+    <col min="4" max="4" width="26.85546875" bestFit="1" customWidth="1"/>
+    <col min="5" max="5" width="27.42578125" bestFit="1" customWidth="1"/>
+    <col min="6" max="6" width="25.140625" bestFit="1" customWidth="1"/>
+    <col min="7" max="7" width="22.5703125" bestFit="1" customWidth="1"/>
     <col min="8" max="8" width="27" bestFit="1" customWidth="1"/>
-    <col min="9" max="9" width="31.54296875" bestFit="1" customWidth="1"/>
-    <col min="10" max="10" width="29.26953125" bestFit="1" customWidth="1"/>
-    <col min="11" max="11" width="30.7265625" bestFit="1" customWidth="1"/>
-    <col min="12" max="12" width="28.36328125" bestFit="1" customWidth="1"/>
+    <col min="9" max="9" width="31.5703125" bestFit="1" customWidth="1"/>
+    <col min="10" max="10" width="29.28515625" bestFit="1" customWidth="1"/>
+    <col min="11" max="11" width="30.7109375" bestFit="1" customWidth="1"/>
+    <col min="12" max="12" width="28.42578125" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:12" x14ac:dyDescent="0.35">
+    <row r="1" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A1" t="s">
         <v>0</v>
       </c>
@@ -11266,12 +11331,12 @@
         <v>185</v>
       </c>
     </row>
-    <row r="2" spans="1:12" x14ac:dyDescent="0.35">
+    <row r="2" spans="1:12" x14ac:dyDescent="0.25">
       <c r="F2" t="s">
         <v>82</v>
       </c>
     </row>
-    <row r="3" spans="1:12" x14ac:dyDescent="0.35">
+    <row r="3" spans="1:12" x14ac:dyDescent="0.25">
       <c r="B3" t="s">
         <v>8</v>
       </c>
@@ -11306,7 +11371,7 @@
         <v>189</v>
       </c>
     </row>
-    <row r="4" spans="1:12" x14ac:dyDescent="0.35">
+    <row r="4" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A4" t="s">
         <v>14</v>
       </c>
@@ -11344,7 +11409,7 @@
         <v>494</v>
       </c>
     </row>
-    <row r="5" spans="1:12" x14ac:dyDescent="0.35">
+    <row r="5" spans="1:12" x14ac:dyDescent="0.25">
       <c r="B5" t="s">
         <v>152</v>
       </c>
@@ -11379,7 +11444,7 @@
         <v>201</v>
       </c>
     </row>
-    <row r="6" spans="1:12" x14ac:dyDescent="0.35">
+    <row r="6" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A6" t="s">
         <v>27</v>
       </c>
@@ -11417,7 +11482,7 @@
         <v>211</v>
       </c>
     </row>
-    <row r="7" spans="1:12" x14ac:dyDescent="0.35">
+    <row r="7" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A7" t="s">
         <v>34</v>
       </c>
@@ -11455,7 +11520,7 @@
         <v>221</v>
       </c>
     </row>
-    <row r="8" spans="1:12" x14ac:dyDescent="0.35">
+    <row r="8" spans="1:12" x14ac:dyDescent="0.25">
       <c r="B8" t="s">
         <v>41</v>
       </c>
@@ -11490,7 +11555,7 @@
         <v>231</v>
       </c>
     </row>
-    <row r="9" spans="1:12" x14ac:dyDescent="0.35">
+    <row r="9" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A9" t="s">
         <v>115</v>
       </c>
@@ -11528,7 +11593,7 @@
         <v>238</v>
       </c>
     </row>
-    <row r="10" spans="1:12" x14ac:dyDescent="0.35">
+    <row r="10" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A10" t="s">
         <v>122</v>
       </c>
@@ -11566,7 +11631,7 @@
         <v>231</v>
       </c>
     </row>
-    <row r="11" spans="1:12" x14ac:dyDescent="0.35">
+    <row r="11" spans="1:12" x14ac:dyDescent="0.25">
       <c r="B11" t="s">
         <v>56</v>
       </c>
@@ -11601,7 +11666,7 @@
         <v>245</v>
       </c>
     </row>
-    <row r="12" spans="1:12" x14ac:dyDescent="0.35">
+    <row r="12" spans="1:12" x14ac:dyDescent="0.25">
       <c r="B12" t="s">
         <v>61</v>
       </c>
@@ -11636,7 +11701,7 @@
         <v>245</v>
       </c>
     </row>
-    <row r="13" spans="1:12" x14ac:dyDescent="0.35">
+    <row r="13" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A13" t="s">
         <v>55</v>
       </c>
@@ -11674,7 +11739,7 @@
         <v>245</v>
       </c>
     </row>
-    <row r="14" spans="1:12" x14ac:dyDescent="0.35">
+    <row r="14" spans="1:12" x14ac:dyDescent="0.25">
       <c r="B14" t="s">
         <v>63</v>
       </c>
@@ -11709,7 +11774,7 @@
         <v>245</v>
       </c>
     </row>
-    <row r="15" spans="1:12" x14ac:dyDescent="0.35">
+    <row r="15" spans="1:12" x14ac:dyDescent="0.25">
       <c r="B15" t="s">
         <v>64</v>
       </c>
@@ -11744,7 +11809,7 @@
         <v>245</v>
       </c>
     </row>
-    <row r="16" spans="1:12" x14ac:dyDescent="0.35">
+    <row r="16" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A16" t="s">
         <v>65</v>
       </c>
@@ -11782,7 +11847,7 @@
         <v>254</v>
       </c>
     </row>
-    <row r="18" spans="1:12" x14ac:dyDescent="0.35">
+    <row r="18" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A18" t="s">
         <v>0</v>
       </c>
@@ -11820,7 +11885,7 @@
         <v>185</v>
       </c>
     </row>
-    <row r="19" spans="1:12" x14ac:dyDescent="0.35">
+    <row r="19" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A19" t="s">
         <v>135</v>
       </c>
@@ -11858,7 +11923,7 @@
         <v>264</v>
       </c>
     </row>
-    <row r="20" spans="1:12" x14ac:dyDescent="0.35">
+    <row r="20" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A20" t="s">
         <v>76</v>
       </c>
@@ -11905,19 +11970,19 @@
 <file path=xl/worksheets/sheet7.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{6200D3EF-F83A-49B0-BAF0-4EF918D3F281}">
   <dimension ref="A1:I20"/>
-  <sheetFormatPr defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
+  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
-    <col min="1" max="1" width="12.6328125" bestFit="1" customWidth="1"/>
-    <col min="2" max="2" width="16.36328125" bestFit="1" customWidth="1"/>
-    <col min="3" max="3" width="27.08984375" bestFit="1" customWidth="1"/>
-    <col min="4" max="4" width="34.26953125" bestFit="1" customWidth="1"/>
+    <col min="1" max="1" width="12.5703125" bestFit="1" customWidth="1"/>
+    <col min="2" max="2" width="16.42578125" bestFit="1" customWidth="1"/>
+    <col min="3" max="3" width="27.140625" bestFit="1" customWidth="1"/>
+    <col min="4" max="4" width="34.28515625" bestFit="1" customWidth="1"/>
     <col min="5" max="5" width="23" bestFit="1" customWidth="1"/>
-    <col min="6" max="6" width="25.1796875" bestFit="1" customWidth="1"/>
-    <col min="7" max="7" width="30.90625" bestFit="1" customWidth="1"/>
-    <col min="8" max="9" width="38.36328125" bestFit="1" customWidth="1"/>
+    <col min="6" max="6" width="25.140625" bestFit="1" customWidth="1"/>
+    <col min="7" max="7" width="30.85546875" bestFit="1" customWidth="1"/>
+    <col min="8" max="9" width="38.42578125" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:9" x14ac:dyDescent="0.35">
+    <row r="1" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A1" t="s">
         <v>0</v>
       </c>
@@ -11946,12 +12011,12 @@
         <v>182</v>
       </c>
     </row>
-    <row r="2" spans="1:9" x14ac:dyDescent="0.35">
+    <row r="2" spans="1:9" x14ac:dyDescent="0.25">
       <c r="D2" t="s">
         <v>271</v>
       </c>
     </row>
-    <row r="3" spans="1:9" x14ac:dyDescent="0.35">
+    <row r="3" spans="1:9" x14ac:dyDescent="0.25">
       <c r="B3" t="s">
         <v>8</v>
       </c>
@@ -11977,7 +12042,7 @@
         <v>278</v>
       </c>
     </row>
-    <row r="4" spans="1:9" x14ac:dyDescent="0.35">
+    <row r="4" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A4" t="s">
         <v>14</v>
       </c>
@@ -12006,7 +12071,7 @@
         <v>285</v>
       </c>
     </row>
-    <row r="5" spans="1:9" x14ac:dyDescent="0.35">
+    <row r="5" spans="1:9" x14ac:dyDescent="0.25">
       <c r="B5" t="s">
         <v>152</v>
       </c>
@@ -12032,7 +12097,7 @@
         <v>292</v>
       </c>
     </row>
-    <row r="6" spans="1:9" x14ac:dyDescent="0.35">
+    <row r="6" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A6" t="s">
         <v>27</v>
       </c>
@@ -12061,7 +12126,7 @@
         <v>299</v>
       </c>
     </row>
-    <row r="7" spans="1:9" x14ac:dyDescent="0.35">
+    <row r="7" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A7" t="s">
         <v>34</v>
       </c>
@@ -12090,7 +12155,7 @@
         <v>306</v>
       </c>
     </row>
-    <row r="8" spans="1:9" x14ac:dyDescent="0.35">
+    <row r="8" spans="1:9" x14ac:dyDescent="0.25">
       <c r="B8" t="s">
         <v>41</v>
       </c>
@@ -12116,7 +12181,7 @@
         <v>313</v>
       </c>
     </row>
-    <row r="9" spans="1:9" x14ac:dyDescent="0.35">
+    <row r="9" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A9" t="s">
         <v>47</v>
       </c>
@@ -12145,7 +12210,7 @@
         <v>320</v>
       </c>
     </row>
-    <row r="10" spans="1:9" x14ac:dyDescent="0.35">
+    <row r="10" spans="1:9" x14ac:dyDescent="0.25">
       <c r="B10" t="s">
         <v>123</v>
       </c>
@@ -12171,7 +12236,7 @@
         <v>313</v>
       </c>
     </row>
-    <row r="11" spans="1:9" x14ac:dyDescent="0.35">
+    <row r="11" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A11" t="s">
         <v>321</v>
       </c>
@@ -12200,7 +12265,7 @@
         <v>328</v>
       </c>
     </row>
-    <row r="12" spans="1:9" x14ac:dyDescent="0.35">
+    <row r="12" spans="1:9" x14ac:dyDescent="0.25">
       <c r="B12" t="s">
         <v>61</v>
       </c>
@@ -12226,7 +12291,7 @@
         <v>328</v>
       </c>
     </row>
-    <row r="13" spans="1:9" x14ac:dyDescent="0.35">
+    <row r="13" spans="1:9" x14ac:dyDescent="0.25">
       <c r="B13" t="s">
         <v>62</v>
       </c>
@@ -12252,7 +12317,7 @@
         <v>328</v>
       </c>
     </row>
-    <row r="14" spans="1:9" x14ac:dyDescent="0.35">
+    <row r="14" spans="1:9" x14ac:dyDescent="0.25">
       <c r="B14" t="s">
         <v>63</v>
       </c>
@@ -12278,7 +12343,7 @@
         <v>328</v>
       </c>
     </row>
-    <row r="15" spans="1:9" x14ac:dyDescent="0.35">
+    <row r="15" spans="1:9" x14ac:dyDescent="0.25">
       <c r="B15" t="s">
         <v>64</v>
       </c>
@@ -12304,7 +12369,7 @@
         <v>328</v>
       </c>
     </row>
-    <row r="16" spans="1:9" x14ac:dyDescent="0.35">
+    <row r="16" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A16" t="s">
         <v>65</v>
       </c>
@@ -12333,7 +12398,7 @@
         <v>335</v>
       </c>
     </row>
-    <row r="18" spans="1:9" x14ac:dyDescent="0.35">
+    <row r="18" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A18" t="s">
         <v>0</v>
       </c>
@@ -12362,7 +12427,7 @@
         <v>182</v>
       </c>
     </row>
-    <row r="19" spans="1:9" x14ac:dyDescent="0.35">
+    <row r="19" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A19" t="s">
         <v>135</v>
       </c>
@@ -12391,7 +12456,7 @@
         <v>336</v>
       </c>
     </row>
-    <row r="20" spans="1:9" x14ac:dyDescent="0.35">
+    <row r="20" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A20" t="s">
         <v>76</v>
       </c>
@@ -12429,14 +12494,14 @@
 <file path=xl/worksheets/sheet8.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{B22E4AE0-A502-421C-ABBD-9E881E10F770}">
   <dimension ref="A1:C19"/>
-  <sheetFormatPr defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
+  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
-    <col min="1" max="1" width="12.6328125" bestFit="1" customWidth="1"/>
-    <col min="2" max="2" width="16.36328125" bestFit="1" customWidth="1"/>
-    <col min="3" max="3" width="30.6328125" bestFit="1" customWidth="1"/>
+    <col min="1" max="1" width="12.5703125" bestFit="1" customWidth="1"/>
+    <col min="2" max="2" width="16.42578125" bestFit="1" customWidth="1"/>
+    <col min="3" max="3" width="30.5703125" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:3" x14ac:dyDescent="0.35">
+    <row r="1" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A1" t="s">
         <v>0</v>
       </c>
@@ -12447,7 +12512,7 @@
         <v>2</v>
       </c>
     </row>
-    <row r="2" spans="1:3" x14ac:dyDescent="0.35">
+    <row r="2" spans="1:3" x14ac:dyDescent="0.25">
       <c r="B2" t="s">
         <v>8</v>
       </c>
@@ -12455,7 +12520,7 @@
         <v>344</v>
       </c>
     </row>
-    <row r="3" spans="1:3" x14ac:dyDescent="0.35">
+    <row r="3" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A3" t="s">
         <v>14</v>
       </c>
@@ -12466,7 +12531,7 @@
         <v>345</v>
       </c>
     </row>
-    <row r="4" spans="1:3" x14ac:dyDescent="0.35">
+    <row r="4" spans="1:3" x14ac:dyDescent="0.25">
       <c r="B4" t="s">
         <v>152</v>
       </c>
@@ -12474,7 +12539,7 @@
         <v>346</v>
       </c>
     </row>
-    <row r="5" spans="1:3" x14ac:dyDescent="0.35">
+    <row r="5" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A5" t="s">
         <v>27</v>
       </c>
@@ -12485,7 +12550,7 @@
         <v>347</v>
       </c>
     </row>
-    <row r="6" spans="1:3" x14ac:dyDescent="0.35">
+    <row r="6" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A6" t="s">
         <v>34</v>
       </c>
@@ -12496,7 +12561,7 @@
         <v>348</v>
       </c>
     </row>
-    <row r="7" spans="1:3" x14ac:dyDescent="0.35">
+    <row r="7" spans="1:3" x14ac:dyDescent="0.25">
       <c r="B7" t="s">
         <v>41</v>
       </c>
@@ -12504,7 +12569,7 @@
         <v>349</v>
       </c>
     </row>
-    <row r="8" spans="1:3" x14ac:dyDescent="0.35">
+    <row r="8" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A8" t="s">
         <v>47</v>
       </c>
@@ -12515,7 +12580,7 @@
         <v>348</v>
       </c>
     </row>
-    <row r="9" spans="1:3" x14ac:dyDescent="0.35">
+    <row r="9" spans="1:3" x14ac:dyDescent="0.25">
       <c r="B9" t="s">
         <v>123</v>
       </c>
@@ -12523,7 +12588,7 @@
         <v>349</v>
       </c>
     </row>
-    <row r="10" spans="1:3" x14ac:dyDescent="0.35">
+    <row r="10" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A10" t="s">
         <v>321</v>
       </c>
@@ -12534,7 +12599,7 @@
         <v>350</v>
       </c>
     </row>
-    <row r="11" spans="1:3" x14ac:dyDescent="0.35">
+    <row r="11" spans="1:3" x14ac:dyDescent="0.25">
       <c r="B11" t="s">
         <v>61</v>
       </c>
@@ -12542,7 +12607,7 @@
         <v>350</v>
       </c>
     </row>
-    <row r="12" spans="1:3" x14ac:dyDescent="0.35">
+    <row r="12" spans="1:3" x14ac:dyDescent="0.25">
       <c r="B12" t="s">
         <v>62</v>
       </c>
@@ -12550,7 +12615,7 @@
         <v>350</v>
       </c>
     </row>
-    <row r="13" spans="1:3" x14ac:dyDescent="0.35">
+    <row r="13" spans="1:3" x14ac:dyDescent="0.25">
       <c r="B13" t="s">
         <v>63</v>
       </c>
@@ -12558,7 +12623,7 @@
         <v>350</v>
       </c>
     </row>
-    <row r="14" spans="1:3" x14ac:dyDescent="0.35">
+    <row r="14" spans="1:3" x14ac:dyDescent="0.25">
       <c r="B14" t="s">
         <v>64</v>
       </c>
@@ -12566,7 +12631,7 @@
         <v>350</v>
       </c>
     </row>
-    <row r="15" spans="1:3" x14ac:dyDescent="0.35">
+    <row r="15" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A15" t="s">
         <v>65</v>
       </c>
@@ -12577,7 +12642,7 @@
         <v>351</v>
       </c>
     </row>
-    <row r="17" spans="1:3" x14ac:dyDescent="0.35">
+    <row r="17" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A17" t="s">
         <v>0</v>
       </c>
@@ -12588,7 +12653,7 @@
         <v>2</v>
       </c>
     </row>
-    <row r="18" spans="1:3" x14ac:dyDescent="0.35">
+    <row r="18" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A18" t="s">
         <v>135</v>
       </c>
@@ -12599,7 +12664,7 @@
         <v>345</v>
       </c>
     </row>
-    <row r="19" spans="1:3" x14ac:dyDescent="0.35">
+    <row r="19" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A19" t="s">
         <v>76</v>
       </c>
@@ -12619,16 +12684,16 @@
 <file path=xl/worksheets/sheet9.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{E5F91B12-5D52-447E-877C-7C65848770FC}">
   <dimension ref="A1:E21"/>
-  <sheetFormatPr defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
+  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
-    <col min="1" max="1" width="12.6328125" bestFit="1" customWidth="1"/>
-    <col min="2" max="2" width="16.36328125" bestFit="1" customWidth="1"/>
-    <col min="3" max="3" width="22.1796875" bestFit="1" customWidth="1"/>
-    <col min="4" max="4" width="15.90625" bestFit="1" customWidth="1"/>
-    <col min="5" max="5" width="28.08984375" bestFit="1" customWidth="1"/>
+    <col min="1" max="1" width="12.5703125" bestFit="1" customWidth="1"/>
+    <col min="2" max="2" width="16.42578125" bestFit="1" customWidth="1"/>
+    <col min="3" max="3" width="22.140625" bestFit="1" customWidth="1"/>
+    <col min="4" max="4" width="15.85546875" bestFit="1" customWidth="1"/>
+    <col min="5" max="5" width="28.140625" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="1" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A1" t="s">
         <v>0</v>
       </c>
@@ -12645,7 +12710,7 @@
         <v>4</v>
       </c>
     </row>
-    <row r="2" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="2" spans="1:5" x14ac:dyDescent="0.25">
       <c r="B2" t="s">
         <v>8</v>
       </c>
@@ -12653,12 +12718,12 @@
         <v>82</v>
       </c>
     </row>
-    <row r="3" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="3" spans="1:5" x14ac:dyDescent="0.25">
       <c r="C3" t="s">
         <v>353</v>
       </c>
     </row>
-    <row r="4" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="4" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A4" t="s">
         <v>14</v>
       </c>
@@ -12675,7 +12740,7 @@
         <v>356</v>
       </c>
     </row>
-    <row r="5" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="5" spans="1:5" x14ac:dyDescent="0.25">
       <c r="B5" t="s">
         <v>21</v>
       </c>
@@ -12689,7 +12754,7 @@
         <v>359</v>
       </c>
     </row>
-    <row r="6" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="6" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A6" t="s">
         <v>27</v>
       </c>
@@ -12706,7 +12771,7 @@
         <v>362</v>
       </c>
     </row>
-    <row r="7" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="7" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A7" t="s">
         <v>34</v>
       </c>
@@ -12723,7 +12788,7 @@
         <v>365</v>
       </c>
     </row>
-    <row r="8" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="8" spans="1:5" x14ac:dyDescent="0.25">
       <c r="B8" t="s">
         <v>41</v>
       </c>
@@ -12737,7 +12802,7 @@
         <v>368</v>
       </c>
     </row>
-    <row r="9" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="9" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A9" t="s">
         <v>47</v>
       </c>
@@ -12754,7 +12819,7 @@
         <v>371</v>
       </c>
     </row>
-    <row r="10" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="10" spans="1:5" x14ac:dyDescent="0.25">
       <c r="B10" t="s">
         <v>123</v>
       </c>
@@ -12768,7 +12833,7 @@
         <v>368</v>
       </c>
     </row>
-    <row r="11" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="11" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A11" t="s">
         <v>321</v>
       </c>
@@ -12785,7 +12850,7 @@
         <v>374</v>
       </c>
     </row>
-    <row r="12" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="12" spans="1:5" x14ac:dyDescent="0.25">
       <c r="B12" t="s">
         <v>61</v>
       </c>
@@ -12799,7 +12864,7 @@
         <v>374</v>
       </c>
     </row>
-    <row r="13" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="13" spans="1:5" x14ac:dyDescent="0.25">
       <c r="B13" t="s">
         <v>62</v>
       </c>
@@ -12813,7 +12878,7 @@
         <v>374</v>
       </c>
     </row>
-    <row r="14" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="14" spans="1:5" x14ac:dyDescent="0.25">
       <c r="B14" t="s">
         <v>63</v>
       </c>
@@ -12827,7 +12892,7 @@
         <v>374</v>
       </c>
     </row>
-    <row r="15" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="15" spans="1:5" x14ac:dyDescent="0.25">
       <c r="B15" t="s">
         <v>64</v>
       </c>
@@ -12841,7 +12906,7 @@
         <v>374</v>
       </c>
     </row>
-    <row r="16" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="16" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A16" t="s">
         <v>65</v>
       </c>
@@ -12858,7 +12923,7 @@
         <v>376</v>
       </c>
     </row>
-    <row r="18" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="18" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A18" t="s">
         <v>0</v>
       </c>
@@ -12875,7 +12940,7 @@
         <v>4</v>
       </c>
     </row>
-    <row r="19" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="19" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A19" t="s">
         <v>135</v>
       </c>
@@ -12892,7 +12957,7 @@
         <v>379</v>
       </c>
     </row>
-    <row r="20" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="20" spans="1:5" x14ac:dyDescent="0.25">
       <c r="C20" t="s">
         <v>380</v>
       </c>
@@ -12903,7 +12968,7 @@
         <v>382</v>
       </c>
     </row>
-    <row r="21" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="21" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A21" t="s">
         <v>76</v>
       </c>

</xml_diff>

<commit_message>
UPDATE: Added new pricelist for new units
</commit_message>
<xml_diff>
--- a/gp-app-1.0/Pricelist Car.xlsx
+++ b/gp-app-1.0/Pricelist Car.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="30228"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="27029"/>
   <workbookPr hidePivotFieldList="1" defaultThemeVersion="166925"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="G:\Other computers\My Laptop\Work\gp-app\gp-app-1.0\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\Work\gp-app\gp-app-1.0\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{29A2033F-A2F0-4A1F-A376-25BE6D563462}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{391995BF-E4CA-4326-ADE8-70EFB6FB3E44}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="16440" tabRatio="861" xr2:uid="{C4C7316A-D95F-426A-ADF9-AD32FA680374}"/>
+    <workbookView xWindow="-110" yWindow="-110" windowWidth="19420" windowHeight="11020" tabRatio="861" xr2:uid="{C4C7316A-D95F-426A-ADF9-AD32FA680374}"/>
   </bookViews>
   <sheets>
     <sheet name="Pricelist" sheetId="11" r:id="rId1"/>
@@ -490,7 +490,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1423" uniqueCount="640">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1450" uniqueCount="651">
   <si>
     <t>Column1</t>
   </si>
@@ -2490,6 +2490,39 @@
   </si>
   <si>
     <t>AIRA EV LV2</t>
+  </si>
+  <si>
+    <t>DARION EV CE 540 KM</t>
+  </si>
+  <si>
+    <t>DARION EV CE 480 KM</t>
+  </si>
+  <si>
+    <t>DARION EV EX 540 KM</t>
+  </si>
+  <si>
+    <t>DARION PHEV EX</t>
+  </si>
+  <si>
+    <t>DARION PHEV CE</t>
+  </si>
+  <si>
+    <t>E260REV50ZW333LV0Y2A</t>
+  </si>
+  <si>
+    <t>E260REV50ZW333LV1Y2A</t>
+  </si>
+  <si>
+    <t>100 E2C (4x2) A/T LV1</t>
+  </si>
+  <si>
+    <t>100 E2D (4x2) A/T LV2</t>
+  </si>
+  <si>
+    <t>New Cloud Lite</t>
+  </si>
+  <si>
+    <t>New Cloud Pro</t>
   </si>
 </sst>
 </file>
@@ -2497,7 +2530,7 @@
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
   <numFmts count="1">
-    <numFmt numFmtId="164" formatCode="_-* #,##0.00_-;\-* #,##0.00_-;_-* &quot;-&quot;??_-;_-@_-"/>
+    <numFmt numFmtId="43" formatCode="_-* #,##0.00_-;\-* #,##0.00_-;_-* &quot;-&quot;??_-;_-@_-"/>
   </numFmts>
   <fonts count="5" x14ac:knownFonts="1">
     <font>
@@ -2684,10 +2717,10 @@
   <cellStyleXfs count="4">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0"/>
-    <xf numFmtId="164" fontId="2" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
+    <xf numFmtId="43" fontId="2" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="25">
+  <cellXfs count="30">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="2" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
     <xf numFmtId="3" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
@@ -2695,7 +2728,7 @@
       <alignment horizontal="center" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyBorder="1"/>
-    <xf numFmtId="164" fontId="0" fillId="0" borderId="1" xfId="2" applyFont="1" applyBorder="1"/>
+    <xf numFmtId="43" fontId="0" fillId="0" borderId="1" xfId="2" applyFont="1" applyBorder="1"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left"/>
     </xf>
@@ -2703,19 +2736,19 @@
       <alignment horizontal="center"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="2" xfId="0" applyBorder="1"/>
-    <xf numFmtId="164" fontId="0" fillId="0" borderId="1" xfId="2" applyFont="1" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="43" fontId="0" fillId="0" borderId="1" xfId="2" applyFont="1" applyFill="1" applyBorder="1"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="3" xfId="0" applyBorder="1"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="3" xfId="0" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left"/>
     </xf>
-    <xf numFmtId="164" fontId="0" fillId="0" borderId="4" xfId="0" applyNumberFormat="1" applyBorder="1"/>
+    <xf numFmtId="43" fontId="0" fillId="0" borderId="4" xfId="0" applyNumberFormat="1" applyBorder="1"/>
     <xf numFmtId="0" fontId="3" fillId="0" borderId="5" xfId="0" applyFont="1" applyBorder="1"/>
     <xf numFmtId="0" fontId="3" fillId="0" borderId="6" xfId="0" applyFont="1" applyBorder="1"/>
     <xf numFmtId="0" fontId="3" fillId="0" borderId="7" xfId="0" applyFont="1" applyBorder="1"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="8" xfId="0" applyBorder="1"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="9" xfId="0" applyBorder="1"/>
-    <xf numFmtId="164" fontId="0" fillId="0" borderId="9" xfId="2" applyFont="1" applyFill="1" applyBorder="1"/>
-    <xf numFmtId="164" fontId="0" fillId="0" borderId="10" xfId="0" applyNumberFormat="1" applyBorder="1"/>
+    <xf numFmtId="43" fontId="0" fillId="0" borderId="9" xfId="2" applyFont="1" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="43" fontId="0" fillId="0" borderId="10" xfId="0" applyNumberFormat="1" applyBorder="1"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
@@ -2725,10 +2758,15 @@
     <xf numFmtId="0" fontId="0" fillId="0" borderId="3" xfId="0" applyBorder="1" applyAlignment="1">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="164" fontId="0" fillId="0" borderId="9" xfId="2" applyFont="1" applyBorder="1"/>
+    <xf numFmtId="43" fontId="0" fillId="0" borderId="9" xfId="2" applyFont="1" applyBorder="1"/>
     <xf numFmtId="0" fontId="2" fillId="2" borderId="9" xfId="3" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="3" xfId="0" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="43" fontId="0" fillId="0" borderId="4" xfId="0" applyNumberFormat="1" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="8" xfId="0" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="9" xfId="0" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="43" fontId="0" fillId="0" borderId="10" xfId="0" applyNumberFormat="1" applyFill="1" applyBorder="1"/>
   </cellXfs>
   <cellStyles count="4">
     <cellStyle name="Comma" xfId="2" builtinId="3"/>
@@ -2736,7 +2774,7 @@
     <cellStyle name="Normal 2" xfId="1" xr:uid="{DA2601EE-1999-4BF8-AF5E-538A4398209C}"/>
     <cellStyle name="Normal 2 2" xfId="3" xr:uid="{8C240942-BC33-4996-847D-14CFBB46F4A3}"/>
   </cellStyles>
-  <dxfs count="154">
+  <dxfs count="156">
     <dxf>
       <font>
         <color rgb="FF9C0006"/>
@@ -2828,6 +2866,26 @@
       </fill>
     </dxf>
     <dxf>
+      <font>
+        <color rgb="FF9C0006"/>
+      </font>
+      <fill>
+        <patternFill>
+          <bgColor rgb="FFFFC7CE"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <font>
+        <color rgb="FF9C0006"/>
+      </font>
+      <fill>
+        <patternFill>
+          <bgColor rgb="FFFFC7CE"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
       <numFmt numFmtId="0" formatCode="General"/>
     </dxf>
     <dxf>
@@ -3224,7 +3282,7 @@
       <numFmt numFmtId="0" formatCode="General"/>
     </dxf>
     <dxf>
-      <numFmt numFmtId="164" formatCode="_-* #,##0.00_-;\-* #,##0.00_-;_-* &quot;-&quot;??_-;_-@_-"/>
+      <numFmt numFmtId="35" formatCode="_-* #,##0.00_-;\-* #,##0.00_-;_-* &quot;-&quot;??_-;_-@_-"/>
       <fill>
         <patternFill patternType="none">
           <fgColor indexed="64"/>
@@ -5103,21 +5161,21 @@
 </file>
 
 <file path=xl/tables/table1.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="20" xr:uid="{DF067A72-54A6-48F4-972D-2DE4603D61A4}" name="Table20" displayName="Table20" ref="A1:I70" totalsRowShown="0" headerRowDxfId="153" headerRowBorderDxfId="152" tableBorderDxfId="151" totalsRowBorderDxfId="150">
-  <autoFilter ref="A1:I70" xr:uid="{DF067A72-54A6-48F4-972D-2DE4603D61A4}"/>
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="20" xr:uid="{DF067A72-54A6-48F4-972D-2DE4603D61A4}" name="Table20" displayName="Table20" ref="A1:I79" totalsRowShown="0" headerRowDxfId="155" headerRowBorderDxfId="154" tableBorderDxfId="153" totalsRowBorderDxfId="152">
+  <autoFilter ref="A1:I79" xr:uid="{DF067A72-54A6-48F4-972D-2DE4603D61A4}"/>
   <sortState xmlns:xlrd2="http://schemas.microsoft.com/office/spreadsheetml/2017/richdata2" ref="A2:I57">
     <sortCondition ref="H1:H57"/>
   </sortState>
   <tableColumns count="9">
-    <tableColumn id="1" xr3:uid="{0E6335F2-6B6A-436C-92FA-B48E61551308}" name="Merek/Type" dataDxfId="149"/>
-    <tableColumn id="2" xr3:uid="{5A4965DA-398A-4134-90BD-9CE4D8355880}" name="Tipe" dataDxfId="148"/>
-    <tableColumn id="3" xr3:uid="{010303D1-E0A2-4DE6-8E87-64ACC3102E09}" name="Harga OTR Awal" dataDxfId="147" dataCellStyle="Comma"/>
-    <tableColumn id="4" xr3:uid="{91C798B0-7964-436A-84A5-7687993F376F}" name="Dealer Margin" dataDxfId="146" dataCellStyle="Comma"/>
-    <tableColumn id="5" xr3:uid="{CD936623-36F3-4BAA-A615-AF79A61C51E8}" name="Dealer Margin 9 %" dataDxfId="145" dataCellStyle="Comma"/>
-    <tableColumn id="6" xr3:uid="{A36173E8-D9B2-4F38-A572-F5D32CDADEB8}" name="Dealer Margin 7 %" dataDxfId="144" dataCellStyle="Comma"/>
-    <tableColumn id="7" xr3:uid="{7A11B7F5-7683-492A-A8B5-D96984323DDD}" name="Code Unit" dataDxfId="143"/>
-    <tableColumn id="8" xr3:uid="{AF243BB3-2044-4D1E-9F0D-A1EC0D2C15CF}" name="Merk/Type" dataDxfId="142"/>
-    <tableColumn id="9" xr3:uid="{9E0E2E6A-108F-4ACE-959D-9EB0F753BD73}" name="Full Margin" dataDxfId="141"/>
+    <tableColumn id="1" xr3:uid="{0E6335F2-6B6A-436C-92FA-B48E61551308}" name="Merek/Type" dataDxfId="151"/>
+    <tableColumn id="2" xr3:uid="{5A4965DA-398A-4134-90BD-9CE4D8355880}" name="Tipe" dataDxfId="150"/>
+    <tableColumn id="3" xr3:uid="{010303D1-E0A2-4DE6-8E87-64ACC3102E09}" name="Harga OTR Awal" dataDxfId="149" dataCellStyle="Comma"/>
+    <tableColumn id="4" xr3:uid="{91C798B0-7964-436A-84A5-7687993F376F}" name="Dealer Margin" dataDxfId="148" dataCellStyle="Comma"/>
+    <tableColumn id="5" xr3:uid="{CD936623-36F3-4BAA-A615-AF79A61C51E8}" name="Dealer Margin 9 %" dataDxfId="147" dataCellStyle="Comma"/>
+    <tableColumn id="6" xr3:uid="{A36173E8-D9B2-4F38-A572-F5D32CDADEB8}" name="Dealer Margin 7 %" dataDxfId="146" dataCellStyle="Comma"/>
+    <tableColumn id="7" xr3:uid="{7A11B7F5-7683-492A-A8B5-D96984323DDD}" name="Code Unit" dataDxfId="145"/>
+    <tableColumn id="8" xr3:uid="{AF243BB3-2044-4D1E-9F0D-A1EC0D2C15CF}" name="Merk/Type" dataDxfId="144"/>
+    <tableColumn id="9" xr3:uid="{9E0E2E6A-108F-4ACE-959D-9EB0F753BD73}" name="Full Margin" dataDxfId="143"/>
   </tableColumns>
   <tableStyleInfo name="TableStyleMedium2" showFirstColumn="0" showLastColumn="0" showRowStripes="1" showColumnStripes="0"/>
 </table>
@@ -5127,15 +5185,15 @@
 <table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="9" xr:uid="{630D8221-A5B4-4162-BEFC-7BB63825B861}" name="Table009__Page_6" displayName="Table009__Page_6" ref="A1:I16" tableType="queryTable" totalsRowShown="0">
   <autoFilter ref="A1:I16" xr:uid="{630D8221-A5B4-4162-BEFC-7BB63825B861}"/>
   <tableColumns count="9">
-    <tableColumn id="1" xr3:uid="{5980B244-73E4-43AF-B863-305E8B039C33}" uniqueName="1" name="Column1" queryTableFieldId="1" dataDxfId="74"/>
-    <tableColumn id="2" xr3:uid="{549208EE-7E07-4F0F-ACFD-9606CC8F6B50}" uniqueName="2" name="Column2" queryTableFieldId="2" dataDxfId="73"/>
-    <tableColumn id="3" xr3:uid="{086F7B88-A201-47FD-B9A0-0C976108E144}" uniqueName="3" name="Column3" queryTableFieldId="3" dataDxfId="72"/>
-    <tableColumn id="4" xr3:uid="{CC912184-CE02-4DC9-8815-71C4295C86DF}" uniqueName="4" name="Column4" queryTableFieldId="4" dataDxfId="71"/>
-    <tableColumn id="5" xr3:uid="{8F3F2202-7C07-4D43-B483-871C9E242208}" uniqueName="5" name="Column5" queryTableFieldId="5" dataDxfId="70"/>
-    <tableColumn id="6" xr3:uid="{6D2190D6-B434-4BB9-95B1-A29148C453AF}" uniqueName="6" name="Column6" queryTableFieldId="6" dataDxfId="69"/>
-    <tableColumn id="7" xr3:uid="{A33DE0AF-7DA7-4623-87E7-DBA2BF4E404A}" uniqueName="7" name="Column7" queryTableFieldId="7" dataDxfId="68"/>
-    <tableColumn id="8" xr3:uid="{CD689B59-BA44-4F67-9FF9-E08337BE66FD}" uniqueName="8" name="Column8" queryTableFieldId="8" dataDxfId="67"/>
-    <tableColumn id="9" xr3:uid="{744F224A-BA1E-4758-B291-8D5C8D341610}" uniqueName="9" name="Column9" queryTableFieldId="9" dataDxfId="66"/>
+    <tableColumn id="1" xr3:uid="{5980B244-73E4-43AF-B863-305E8B039C33}" uniqueName="1" name="Column1" queryTableFieldId="1" dataDxfId="76"/>
+    <tableColumn id="2" xr3:uid="{549208EE-7E07-4F0F-ACFD-9606CC8F6B50}" uniqueName="2" name="Column2" queryTableFieldId="2" dataDxfId="75"/>
+    <tableColumn id="3" xr3:uid="{086F7B88-A201-47FD-B9A0-0C976108E144}" uniqueName="3" name="Column3" queryTableFieldId="3" dataDxfId="74"/>
+    <tableColumn id="4" xr3:uid="{CC912184-CE02-4DC9-8815-71C4295C86DF}" uniqueName="4" name="Column4" queryTableFieldId="4" dataDxfId="73"/>
+    <tableColumn id="5" xr3:uid="{8F3F2202-7C07-4D43-B483-871C9E242208}" uniqueName="5" name="Column5" queryTableFieldId="5" dataDxfId="72"/>
+    <tableColumn id="6" xr3:uid="{6D2190D6-B434-4BB9-95B1-A29148C453AF}" uniqueName="6" name="Column6" queryTableFieldId="6" dataDxfId="71"/>
+    <tableColumn id="7" xr3:uid="{A33DE0AF-7DA7-4623-87E7-DBA2BF4E404A}" uniqueName="7" name="Column7" queryTableFieldId="7" dataDxfId="70"/>
+    <tableColumn id="8" xr3:uid="{CD689B59-BA44-4F67-9FF9-E08337BE66FD}" uniqueName="8" name="Column8" queryTableFieldId="8" dataDxfId="69"/>
+    <tableColumn id="9" xr3:uid="{744F224A-BA1E-4758-B291-8D5C8D341610}" uniqueName="9" name="Column9" queryTableFieldId="9" dataDxfId="68"/>
   </tableColumns>
   <tableStyleInfo name="TableStyleMedium7" showFirstColumn="0" showLastColumn="0" showRowStripes="1" showColumnStripes="0"/>
 </table>
@@ -5145,15 +5203,15 @@
 <table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="10" xr:uid="{116BBD7B-F856-4C44-8F1F-EA66756E3A0B}" name="Table010__Page_6" displayName="Table010__Page_6" ref="A18:I20" tableType="queryTable" totalsRowShown="0">
   <autoFilter ref="A18:I20" xr:uid="{116BBD7B-F856-4C44-8F1F-EA66756E3A0B}"/>
   <tableColumns count="9">
-    <tableColumn id="1" xr3:uid="{D02866AC-7C8C-4041-B0D6-297717EA2BCA}" uniqueName="1" name="Column1" queryTableFieldId="1" dataDxfId="65"/>
-    <tableColumn id="2" xr3:uid="{F9BA0334-AC0F-4599-91DD-1D3B53530BA2}" uniqueName="2" name="Column2" queryTableFieldId="2" dataDxfId="64"/>
-    <tableColumn id="3" xr3:uid="{2E40CB08-FF90-4211-A5F6-3255AA5CEAED}" uniqueName="3" name="Column3" queryTableFieldId="3" dataDxfId="63"/>
-    <tableColumn id="4" xr3:uid="{951E49DE-3DB8-41C0-8F36-6E5A1649659D}" uniqueName="4" name="Column4" queryTableFieldId="4" dataDxfId="62"/>
-    <tableColumn id="5" xr3:uid="{D7FC7D23-AA29-4FAE-8DF4-B23A11020D8C}" uniqueName="5" name="Column5" queryTableFieldId="5" dataDxfId="61"/>
-    <tableColumn id="6" xr3:uid="{85DA6C7C-BC56-4316-BB56-3D2CA86DF4B0}" uniqueName="6" name="Column6" queryTableFieldId="6" dataDxfId="60"/>
-    <tableColumn id="7" xr3:uid="{47F39228-8CCC-4319-9964-568280350AF4}" uniqueName="7" name="Column7" queryTableFieldId="7" dataDxfId="59"/>
-    <tableColumn id="8" xr3:uid="{781188CD-5AC0-41B9-8575-2EACD4BA90A4}" uniqueName="8" name="Column8" queryTableFieldId="8" dataDxfId="58"/>
-    <tableColumn id="9" xr3:uid="{A2DFBEC8-960F-4613-A8B8-821CF42818AC}" uniqueName="9" name="Column9" queryTableFieldId="9" dataDxfId="57"/>
+    <tableColumn id="1" xr3:uid="{D02866AC-7C8C-4041-B0D6-297717EA2BCA}" uniqueName="1" name="Column1" queryTableFieldId="1" dataDxfId="67"/>
+    <tableColumn id="2" xr3:uid="{F9BA0334-AC0F-4599-91DD-1D3B53530BA2}" uniqueName="2" name="Column2" queryTableFieldId="2" dataDxfId="66"/>
+    <tableColumn id="3" xr3:uid="{2E40CB08-FF90-4211-A5F6-3255AA5CEAED}" uniqueName="3" name="Column3" queryTableFieldId="3" dataDxfId="65"/>
+    <tableColumn id="4" xr3:uid="{951E49DE-3DB8-41C0-8F36-6E5A1649659D}" uniqueName="4" name="Column4" queryTableFieldId="4" dataDxfId="64"/>
+    <tableColumn id="5" xr3:uid="{D7FC7D23-AA29-4FAE-8DF4-B23A11020D8C}" uniqueName="5" name="Column5" queryTableFieldId="5" dataDxfId="63"/>
+    <tableColumn id="6" xr3:uid="{85DA6C7C-BC56-4316-BB56-3D2CA86DF4B0}" uniqueName="6" name="Column6" queryTableFieldId="6" dataDxfId="62"/>
+    <tableColumn id="7" xr3:uid="{47F39228-8CCC-4319-9964-568280350AF4}" uniqueName="7" name="Column7" queryTableFieldId="7" dataDxfId="61"/>
+    <tableColumn id="8" xr3:uid="{781188CD-5AC0-41B9-8575-2EACD4BA90A4}" uniqueName="8" name="Column8" queryTableFieldId="8" dataDxfId="60"/>
+    <tableColumn id="9" xr3:uid="{A2DFBEC8-960F-4613-A8B8-821CF42818AC}" uniqueName="9" name="Column9" queryTableFieldId="9" dataDxfId="59"/>
   </tableColumns>
   <tableStyleInfo name="TableStyleMedium7" showFirstColumn="0" showLastColumn="0" showRowStripes="1" showColumnStripes="0"/>
 </table>
@@ -5163,9 +5221,9 @@
 <table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="11" xr:uid="{D5A80464-2F5E-4F81-BC09-642A89962C82}" name="Table011__Page_7" displayName="Table011__Page_7" ref="A1:C15" tableType="queryTable" totalsRowShown="0">
   <autoFilter ref="A1:C15" xr:uid="{D5A80464-2F5E-4F81-BC09-642A89962C82}"/>
   <tableColumns count="3">
-    <tableColumn id="1" xr3:uid="{384F6B08-E7B1-4ECD-BC7E-1F8C8FC9CD11}" uniqueName="1" name="Column1" queryTableFieldId="1" dataDxfId="56"/>
-    <tableColumn id="2" xr3:uid="{BD116665-54B3-487B-82AD-7E260403FB1A}" uniqueName="2" name="Column2" queryTableFieldId="2" dataDxfId="55"/>
-    <tableColumn id="3" xr3:uid="{A0C72322-3C63-446F-A7B0-E45538411191}" uniqueName="3" name="Column3" queryTableFieldId="3" dataDxfId="54"/>
+    <tableColumn id="1" xr3:uid="{384F6B08-E7B1-4ECD-BC7E-1F8C8FC9CD11}" uniqueName="1" name="Column1" queryTableFieldId="1" dataDxfId="58"/>
+    <tableColumn id="2" xr3:uid="{BD116665-54B3-487B-82AD-7E260403FB1A}" uniqueName="2" name="Column2" queryTableFieldId="2" dataDxfId="57"/>
+    <tableColumn id="3" xr3:uid="{A0C72322-3C63-446F-A7B0-E45538411191}" uniqueName="3" name="Column3" queryTableFieldId="3" dataDxfId="56"/>
   </tableColumns>
   <tableStyleInfo name="TableStyleMedium7" showFirstColumn="0" showLastColumn="0" showRowStripes="1" showColumnStripes="0"/>
 </table>
@@ -5175,9 +5233,9 @@
 <table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="12" xr:uid="{BF5A7D5F-42BD-4927-9517-2459449E72C6}" name="Table012__Page_7" displayName="Table012__Page_7" ref="A17:C19" tableType="queryTable" totalsRowShown="0">
   <autoFilter ref="A17:C19" xr:uid="{BF5A7D5F-42BD-4927-9517-2459449E72C6}"/>
   <tableColumns count="3">
-    <tableColumn id="1" xr3:uid="{92B56AD9-FE6F-4702-B777-811CB1B6E64F}" uniqueName="1" name="Column1" queryTableFieldId="1" dataDxfId="53"/>
-    <tableColumn id="2" xr3:uid="{C37743D7-7886-43A1-BB26-C0F3914426C9}" uniqueName="2" name="Column2" queryTableFieldId="2" dataDxfId="52"/>
-    <tableColumn id="3" xr3:uid="{DFF6BFBF-623A-4318-86AF-C5448FC821A5}" uniqueName="3" name="Column3" queryTableFieldId="3" dataDxfId="51"/>
+    <tableColumn id="1" xr3:uid="{92B56AD9-FE6F-4702-B777-811CB1B6E64F}" uniqueName="1" name="Column1" queryTableFieldId="1" dataDxfId="55"/>
+    <tableColumn id="2" xr3:uid="{C37743D7-7886-43A1-BB26-C0F3914426C9}" uniqueName="2" name="Column2" queryTableFieldId="2" dataDxfId="54"/>
+    <tableColumn id="3" xr3:uid="{DFF6BFBF-623A-4318-86AF-C5448FC821A5}" uniqueName="3" name="Column3" queryTableFieldId="3" dataDxfId="53"/>
   </tableColumns>
   <tableStyleInfo name="TableStyleMedium7" showFirstColumn="0" showLastColumn="0" showRowStripes="1" showColumnStripes="0"/>
 </table>
@@ -5187,11 +5245,11 @@
 <table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="13" xr:uid="{4DAA9679-BE71-4F3A-B608-132984AF6DF1}" name="Table013__Page_8" displayName="Table013__Page_8" ref="A1:E16" tableType="queryTable" totalsRowShown="0">
   <autoFilter ref="A1:E16" xr:uid="{4DAA9679-BE71-4F3A-B608-132984AF6DF1}"/>
   <tableColumns count="5">
-    <tableColumn id="1" xr3:uid="{811DEB23-A3B8-4E1E-AF98-CBD4FE9515C8}" uniqueName="1" name="Column1" queryTableFieldId="1" dataDxfId="50"/>
-    <tableColumn id="2" xr3:uid="{D1233A63-9D37-45F3-9DC7-52977AC06ADC}" uniqueName="2" name="Column2" queryTableFieldId="2" dataDxfId="49"/>
-    <tableColumn id="3" xr3:uid="{400191B1-4CF8-4D78-82E7-FED7CD6730E6}" uniqueName="3" name="Column3" queryTableFieldId="3" dataDxfId="48"/>
-    <tableColumn id="4" xr3:uid="{3D829CC4-4292-4CD0-80B8-3490D4014AC9}" uniqueName="4" name="Column4" queryTableFieldId="4" dataDxfId="47"/>
-    <tableColumn id="5" xr3:uid="{9BC50CF1-EF44-42B4-9129-E887F74428C9}" uniqueName="5" name="Column5" queryTableFieldId="5" dataDxfId="46"/>
+    <tableColumn id="1" xr3:uid="{811DEB23-A3B8-4E1E-AF98-CBD4FE9515C8}" uniqueName="1" name="Column1" queryTableFieldId="1" dataDxfId="52"/>
+    <tableColumn id="2" xr3:uid="{D1233A63-9D37-45F3-9DC7-52977AC06ADC}" uniqueName="2" name="Column2" queryTableFieldId="2" dataDxfId="51"/>
+    <tableColumn id="3" xr3:uid="{400191B1-4CF8-4D78-82E7-FED7CD6730E6}" uniqueName="3" name="Column3" queryTableFieldId="3" dataDxfId="50"/>
+    <tableColumn id="4" xr3:uid="{3D829CC4-4292-4CD0-80B8-3490D4014AC9}" uniqueName="4" name="Column4" queryTableFieldId="4" dataDxfId="49"/>
+    <tableColumn id="5" xr3:uid="{9BC50CF1-EF44-42B4-9129-E887F74428C9}" uniqueName="5" name="Column5" queryTableFieldId="5" dataDxfId="48"/>
   </tableColumns>
   <tableStyleInfo name="TableStyleMedium7" showFirstColumn="0" showLastColumn="0" showRowStripes="1" showColumnStripes="0"/>
 </table>
@@ -5201,11 +5259,11 @@
 <table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="14" xr:uid="{9D3195A8-F1BD-4429-B95A-60FCF241B775}" name="Table014__Page_8" displayName="Table014__Page_8" ref="A18:E21" tableType="queryTable" totalsRowShown="0">
   <autoFilter ref="A18:E21" xr:uid="{9D3195A8-F1BD-4429-B95A-60FCF241B775}"/>
   <tableColumns count="5">
-    <tableColumn id="1" xr3:uid="{98A6121C-2EC1-48CA-8A40-28DAFD66423E}" uniqueName="1" name="Column1" queryTableFieldId="1" dataDxfId="45"/>
-    <tableColumn id="2" xr3:uid="{6B521FB3-E639-4556-B8C5-473A63201BC1}" uniqueName="2" name="Column2" queryTableFieldId="2" dataDxfId="44"/>
-    <tableColumn id="3" xr3:uid="{3D07F9E9-4DA3-41C6-98A7-BC28F0C8BFB5}" uniqueName="3" name="Column3" queryTableFieldId="3" dataDxfId="43"/>
-    <tableColumn id="4" xr3:uid="{89F1E0D5-9B1D-4170-BB1D-3FBA7855FC27}" uniqueName="4" name="Column4" queryTableFieldId="4" dataDxfId="42"/>
-    <tableColumn id="5" xr3:uid="{68E29A0D-4E20-4E2A-A030-157EF3C69E97}" uniqueName="5" name="Column5" queryTableFieldId="5" dataDxfId="41"/>
+    <tableColumn id="1" xr3:uid="{98A6121C-2EC1-48CA-8A40-28DAFD66423E}" uniqueName="1" name="Column1" queryTableFieldId="1" dataDxfId="47"/>
+    <tableColumn id="2" xr3:uid="{6B521FB3-E639-4556-B8C5-473A63201BC1}" uniqueName="2" name="Column2" queryTableFieldId="2" dataDxfId="46"/>
+    <tableColumn id="3" xr3:uid="{3D07F9E9-4DA3-41C6-98A7-BC28F0C8BFB5}" uniqueName="3" name="Column3" queryTableFieldId="3" dataDxfId="45"/>
+    <tableColumn id="4" xr3:uid="{89F1E0D5-9B1D-4170-BB1D-3FBA7855FC27}" uniqueName="4" name="Column4" queryTableFieldId="4" dataDxfId="44"/>
+    <tableColumn id="5" xr3:uid="{68E29A0D-4E20-4E2A-A030-157EF3C69E97}" uniqueName="5" name="Column5" queryTableFieldId="5" dataDxfId="43"/>
   </tableColumns>
   <tableStyleInfo name="TableStyleMedium7" showFirstColumn="0" showLastColumn="0" showRowStripes="1" showColumnStripes="0"/>
 </table>
@@ -5215,12 +5273,12 @@
 <table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="15" xr:uid="{F2B12C92-B774-477F-98C9-509526BBDEE5}" name="Table015__Page_9" displayName="Table015__Page_9" ref="A1:F16" tableType="queryTable" totalsRowShown="0">
   <autoFilter ref="A1:F16" xr:uid="{F2B12C92-B774-477F-98C9-509526BBDEE5}"/>
   <tableColumns count="6">
-    <tableColumn id="1" xr3:uid="{B9D47F1B-922B-4B02-855C-93AF62167342}" uniqueName="1" name="Column1" queryTableFieldId="1" dataDxfId="40"/>
-    <tableColumn id="2" xr3:uid="{9915D8BD-1C99-4D36-BE7E-9EBEAD6D7B12}" uniqueName="2" name="Column2" queryTableFieldId="2" dataDxfId="39"/>
-    <tableColumn id="3" xr3:uid="{D353D58B-6A1D-4079-A9EC-77376B67A375}" uniqueName="3" name="Column3" queryTableFieldId="3" dataDxfId="38"/>
-    <tableColumn id="4" xr3:uid="{ACF53426-7425-4D38-9673-B3197A3F9292}" uniqueName="4" name="Column4" queryTableFieldId="4" dataDxfId="37"/>
-    <tableColumn id="5" xr3:uid="{673A9374-D6DA-46D7-AAD2-6F2220F4ED8C}" uniqueName="5" name="Column5" queryTableFieldId="5" dataDxfId="36"/>
-    <tableColumn id="6" xr3:uid="{37C428F9-0692-44D1-B8CF-2CBC7901020B}" uniqueName="6" name="Column6" queryTableFieldId="6" dataDxfId="35"/>
+    <tableColumn id="1" xr3:uid="{B9D47F1B-922B-4B02-855C-93AF62167342}" uniqueName="1" name="Column1" queryTableFieldId="1" dataDxfId="42"/>
+    <tableColumn id="2" xr3:uid="{9915D8BD-1C99-4D36-BE7E-9EBEAD6D7B12}" uniqueName="2" name="Column2" queryTableFieldId="2" dataDxfId="41"/>
+    <tableColumn id="3" xr3:uid="{D353D58B-6A1D-4079-A9EC-77376B67A375}" uniqueName="3" name="Column3" queryTableFieldId="3" dataDxfId="40"/>
+    <tableColumn id="4" xr3:uid="{ACF53426-7425-4D38-9673-B3197A3F9292}" uniqueName="4" name="Column4" queryTableFieldId="4" dataDxfId="39"/>
+    <tableColumn id="5" xr3:uid="{673A9374-D6DA-46D7-AAD2-6F2220F4ED8C}" uniqueName="5" name="Column5" queryTableFieldId="5" dataDxfId="38"/>
+    <tableColumn id="6" xr3:uid="{37C428F9-0692-44D1-B8CF-2CBC7901020B}" uniqueName="6" name="Column6" queryTableFieldId="6" dataDxfId="37"/>
   </tableColumns>
   <tableStyleInfo name="TableStyleMedium7" showFirstColumn="0" showLastColumn="0" showRowStripes="1" showColumnStripes="0"/>
 </table>
@@ -5230,12 +5288,12 @@
 <table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="16" xr:uid="{3C596C1A-3A31-47DF-B534-2A3593167FFF}" name="Table016__Page_9" displayName="Table016__Page_9" ref="A18:F20" tableType="queryTable" totalsRowShown="0">
   <autoFilter ref="A18:F20" xr:uid="{3C596C1A-3A31-47DF-B534-2A3593167FFF}"/>
   <tableColumns count="6">
-    <tableColumn id="1" xr3:uid="{48EBD4D1-26EB-449F-8D09-DF1A8D9D96A3}" uniqueName="1" name="Column1" queryTableFieldId="1" dataDxfId="34"/>
-    <tableColumn id="2" xr3:uid="{671AE648-452F-44F1-9A65-8468F7B19950}" uniqueName="2" name="Column2" queryTableFieldId="2" dataDxfId="33"/>
-    <tableColumn id="3" xr3:uid="{C3287937-E8A8-4D80-A27C-D2A5C0E44D68}" uniqueName="3" name="Column3" queryTableFieldId="3" dataDxfId="32"/>
-    <tableColumn id="4" xr3:uid="{49CAB777-0355-40CC-9F2D-C41408ED9E98}" uniqueName="4" name="Column4" queryTableFieldId="4" dataDxfId="31"/>
-    <tableColumn id="5" xr3:uid="{A19C49CB-F2CF-4D60-B082-761FE4F0ABC5}" uniqueName="5" name="Column5" queryTableFieldId="5" dataDxfId="30"/>
-    <tableColumn id="6" xr3:uid="{801427E9-2562-451E-AE45-ACF6DAAAFFFB}" uniqueName="6" name="Column6" queryTableFieldId="6" dataDxfId="29"/>
+    <tableColumn id="1" xr3:uid="{48EBD4D1-26EB-449F-8D09-DF1A8D9D96A3}" uniqueName="1" name="Column1" queryTableFieldId="1" dataDxfId="36"/>
+    <tableColumn id="2" xr3:uid="{671AE648-452F-44F1-9A65-8468F7B19950}" uniqueName="2" name="Column2" queryTableFieldId="2" dataDxfId="35"/>
+    <tableColumn id="3" xr3:uid="{C3287937-E8A8-4D80-A27C-D2A5C0E44D68}" uniqueName="3" name="Column3" queryTableFieldId="3" dataDxfId="34"/>
+    <tableColumn id="4" xr3:uid="{49CAB777-0355-40CC-9F2D-C41408ED9E98}" uniqueName="4" name="Column4" queryTableFieldId="4" dataDxfId="33"/>
+    <tableColumn id="5" xr3:uid="{A19C49CB-F2CF-4D60-B082-761FE4F0ABC5}" uniqueName="5" name="Column5" queryTableFieldId="5" dataDxfId="32"/>
+    <tableColumn id="6" xr3:uid="{801427E9-2562-451E-AE45-ACF6DAAAFFFB}" uniqueName="6" name="Column6" queryTableFieldId="6" dataDxfId="31"/>
   </tableColumns>
   <tableStyleInfo name="TableStyleMedium7" showFirstColumn="0" showLastColumn="0" showRowStripes="1" showColumnStripes="0"/>
 </table>
@@ -5245,11 +5303,11 @@
 <table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="17" xr:uid="{510F87AB-8378-4FE2-9EBF-7361BA7DB6B8}" name="Table017__Page_10" displayName="Table017__Page_10" ref="A1:E15" tableType="queryTable" totalsRowShown="0">
   <autoFilter ref="A1:E15" xr:uid="{510F87AB-8378-4FE2-9EBF-7361BA7DB6B8}"/>
   <tableColumns count="5">
-    <tableColumn id="1" xr3:uid="{626476ED-551C-48ED-A0F5-9CB680097EF0}" uniqueName="1" name="Column1" queryTableFieldId="1" dataDxfId="28"/>
-    <tableColumn id="2" xr3:uid="{9215A7DD-9718-48E5-BA20-B6B9989DD0D2}" uniqueName="2" name="Column2" queryTableFieldId="2" dataDxfId="27"/>
-    <tableColumn id="3" xr3:uid="{AE2AC56F-3587-4342-A60B-0B4A30905DD3}" uniqueName="3" name="Column3" queryTableFieldId="3" dataDxfId="26"/>
-    <tableColumn id="4" xr3:uid="{F7BE237D-2C3F-4C27-92EF-2601ABCBA887}" uniqueName="4" name="Column4" queryTableFieldId="4" dataDxfId="25"/>
-    <tableColumn id="5" xr3:uid="{7950C4F9-8FA4-4C6E-B03A-A0235ECC51FF}" uniqueName="5" name="Column5" queryTableFieldId="5" dataDxfId="24"/>
+    <tableColumn id="1" xr3:uid="{626476ED-551C-48ED-A0F5-9CB680097EF0}" uniqueName="1" name="Column1" queryTableFieldId="1" dataDxfId="30"/>
+    <tableColumn id="2" xr3:uid="{9215A7DD-9718-48E5-BA20-B6B9989DD0D2}" uniqueName="2" name="Column2" queryTableFieldId="2" dataDxfId="29"/>
+    <tableColumn id="3" xr3:uid="{AE2AC56F-3587-4342-A60B-0B4A30905DD3}" uniqueName="3" name="Column3" queryTableFieldId="3" dataDxfId="28"/>
+    <tableColumn id="4" xr3:uid="{F7BE237D-2C3F-4C27-92EF-2601ABCBA887}" uniqueName="4" name="Column4" queryTableFieldId="4" dataDxfId="27"/>
+    <tableColumn id="5" xr3:uid="{7950C4F9-8FA4-4C6E-B03A-A0235ECC51FF}" uniqueName="5" name="Column5" queryTableFieldId="5" dataDxfId="26"/>
   </tableColumns>
   <tableStyleInfo name="TableStyleMedium7" showFirstColumn="0" showLastColumn="0" showRowStripes="1" showColumnStripes="0"/>
 </table>
@@ -5259,11 +5317,11 @@
 <table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="18" xr:uid="{14CF879A-74C7-4F0C-8E76-F1430C9579CD}" name="Table018__Page_10" displayName="Table018__Page_10" ref="A17:E19" tableType="queryTable" totalsRowShown="0">
   <autoFilter ref="A17:E19" xr:uid="{14CF879A-74C7-4F0C-8E76-F1430C9579CD}"/>
   <tableColumns count="5">
-    <tableColumn id="1" xr3:uid="{210B1486-2DC9-4D94-98AC-6BEB874B7545}" uniqueName="1" name="Column1" queryTableFieldId="1" dataDxfId="23"/>
-    <tableColumn id="2" xr3:uid="{BB67F395-3AAE-4514-BCCE-DE32693EB37D}" uniqueName="2" name="Column2" queryTableFieldId="2" dataDxfId="22"/>
-    <tableColumn id="3" xr3:uid="{230B22CA-5CA3-4E2D-92CC-C75BC5831FF2}" uniqueName="3" name="Column3" queryTableFieldId="3" dataDxfId="21"/>
-    <tableColumn id="4" xr3:uid="{42788CA6-A70D-442A-9072-79E0D19F0B28}" uniqueName="4" name="Column4" queryTableFieldId="4" dataDxfId="20"/>
-    <tableColumn id="5" xr3:uid="{E37C1038-7442-4E7D-BB43-162AD6FA4195}" uniqueName="5" name="Column5" queryTableFieldId="5" dataDxfId="19"/>
+    <tableColumn id="1" xr3:uid="{210B1486-2DC9-4D94-98AC-6BEB874B7545}" uniqueName="1" name="Column1" queryTableFieldId="1" dataDxfId="25"/>
+    <tableColumn id="2" xr3:uid="{BB67F395-3AAE-4514-BCCE-DE32693EB37D}" uniqueName="2" name="Column2" queryTableFieldId="2" dataDxfId="24"/>
+    <tableColumn id="3" xr3:uid="{230B22CA-5CA3-4E2D-92CC-C75BC5831FF2}" uniqueName="3" name="Column3" queryTableFieldId="3" dataDxfId="23"/>
+    <tableColumn id="4" xr3:uid="{42788CA6-A70D-442A-9072-79E0D19F0B28}" uniqueName="4" name="Column4" queryTableFieldId="4" dataDxfId="22"/>
+    <tableColumn id="5" xr3:uid="{E37C1038-7442-4E7D-BB43-162AD6FA4195}" uniqueName="5" name="Column5" queryTableFieldId="5" dataDxfId="21"/>
   </tableColumns>
   <tableStyleInfo name="TableStyleMedium7" showFirstColumn="0" showLastColumn="0" showRowStripes="1" showColumnStripes="0"/>
 </table>
@@ -5273,13 +5331,13 @@
 <table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="1" xr:uid="{8D8C9D73-217D-4974-B35A-0740746DA27F}" name="Table001__Page_2" displayName="Table001__Page_2" ref="A1:G16" tableType="queryTable" totalsRowShown="0">
   <autoFilter ref="A1:G16" xr:uid="{8D8C9D73-217D-4974-B35A-0740746DA27F}"/>
   <tableColumns count="7">
-    <tableColumn id="1" xr3:uid="{A26CE965-72B2-472B-B9FF-D68F7847F3C5}" uniqueName="1" name="Column1" queryTableFieldId="1" dataDxfId="140"/>
-    <tableColumn id="2" xr3:uid="{375BF78E-5806-424A-B7BD-C63C40843BE9}" uniqueName="2" name="Column2" queryTableFieldId="2" dataDxfId="139"/>
-    <tableColumn id="3" xr3:uid="{CD1FFC74-B097-42B5-B1FA-08D3BD4531B9}" uniqueName="3" name="Column3" queryTableFieldId="3" dataDxfId="138"/>
-    <tableColumn id="4" xr3:uid="{EA6F5C08-47B3-4BE3-8F9B-3167F2B34338}" uniqueName="4" name="Column4" queryTableFieldId="4" dataDxfId="137"/>
-    <tableColumn id="5" xr3:uid="{67D1B145-6151-4A54-9C79-A6B0381CDA09}" uniqueName="5" name="Column5" queryTableFieldId="5" dataDxfId="136"/>
-    <tableColumn id="6" xr3:uid="{E8D8899E-ED32-4A2F-B13D-18F4C289A59B}" uniqueName="6" name="Column6" queryTableFieldId="6" dataDxfId="135"/>
-    <tableColumn id="7" xr3:uid="{CD1BCBB0-10DE-4DDA-903D-C14D16829749}" uniqueName="7" name="Column7" queryTableFieldId="7" dataDxfId="134"/>
+    <tableColumn id="1" xr3:uid="{A26CE965-72B2-472B-B9FF-D68F7847F3C5}" uniqueName="1" name="Column1" queryTableFieldId="1" dataDxfId="142"/>
+    <tableColumn id="2" xr3:uid="{375BF78E-5806-424A-B7BD-C63C40843BE9}" uniqueName="2" name="Column2" queryTableFieldId="2" dataDxfId="141"/>
+    <tableColumn id="3" xr3:uid="{CD1FFC74-B097-42B5-B1FA-08D3BD4531B9}" uniqueName="3" name="Column3" queryTableFieldId="3" dataDxfId="140"/>
+    <tableColumn id="4" xr3:uid="{EA6F5C08-47B3-4BE3-8F9B-3167F2B34338}" uniqueName="4" name="Column4" queryTableFieldId="4" dataDxfId="139"/>
+    <tableColumn id="5" xr3:uid="{67D1B145-6151-4A54-9C79-A6B0381CDA09}" uniqueName="5" name="Column5" queryTableFieldId="5" dataDxfId="138"/>
+    <tableColumn id="6" xr3:uid="{E8D8899E-ED32-4A2F-B13D-18F4C289A59B}" uniqueName="6" name="Column6" queryTableFieldId="6" dataDxfId="137"/>
+    <tableColumn id="7" xr3:uid="{CD1BCBB0-10DE-4DDA-903D-C14D16829749}" uniqueName="7" name="Column7" queryTableFieldId="7" dataDxfId="136"/>
   </tableColumns>
   <tableStyleInfo name="TableStyleMedium7" showFirstColumn="0" showLastColumn="0" showRowStripes="1" showColumnStripes="0"/>
 </table>
@@ -5289,11 +5347,11 @@
 <table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="19" xr:uid="{A8D65B7F-C1B3-4E37-BFF7-03252131F371}" name="Table019__Page_11" displayName="Table019__Page_11" ref="A1:E16" tableType="queryTable" totalsRowShown="0">
   <autoFilter ref="A1:E16" xr:uid="{A8D65B7F-C1B3-4E37-BFF7-03252131F371}"/>
   <tableColumns count="5">
-    <tableColumn id="1" xr3:uid="{60EAA1C9-E43C-458C-A33C-365CF023541D}" uniqueName="1" name="Column1" queryTableFieldId="1" dataDxfId="18"/>
-    <tableColumn id="2" xr3:uid="{BF4ECEAF-8998-4833-A444-7DD2840947AB}" uniqueName="2" name="Column2" queryTableFieldId="2" dataDxfId="17"/>
-    <tableColumn id="3" xr3:uid="{A77E13C5-CB25-43C0-9678-51A378FA64FC}" uniqueName="3" name="Column3" queryTableFieldId="3" dataDxfId="16"/>
-    <tableColumn id="4" xr3:uid="{46713ABC-AA6E-45DD-9BBE-03C863D6B1D1}" uniqueName="4" name="Column4" queryTableFieldId="4" dataDxfId="15"/>
-    <tableColumn id="5" xr3:uid="{85365AB6-280F-40C4-AB42-3455547D61F1}" uniqueName="5" name="Column5" queryTableFieldId="5" dataDxfId="14"/>
+    <tableColumn id="1" xr3:uid="{60EAA1C9-E43C-458C-A33C-365CF023541D}" uniqueName="1" name="Column1" queryTableFieldId="1" dataDxfId="20"/>
+    <tableColumn id="2" xr3:uid="{BF4ECEAF-8998-4833-A444-7DD2840947AB}" uniqueName="2" name="Column2" queryTableFieldId="2" dataDxfId="19"/>
+    <tableColumn id="3" xr3:uid="{A77E13C5-CB25-43C0-9678-51A378FA64FC}" uniqueName="3" name="Column3" queryTableFieldId="3" dataDxfId="18"/>
+    <tableColumn id="4" xr3:uid="{46713ABC-AA6E-45DD-9BBE-03C863D6B1D1}" uniqueName="4" name="Column4" queryTableFieldId="4" dataDxfId="17"/>
+    <tableColumn id="5" xr3:uid="{85365AB6-280F-40C4-AB42-3455547D61F1}" uniqueName="5" name="Column5" queryTableFieldId="5" dataDxfId="16"/>
   </tableColumns>
   <tableStyleInfo name="TableStyleMedium7" showFirstColumn="0" showLastColumn="0" showRowStripes="1" showColumnStripes="0"/>
 </table>
@@ -5303,11 +5361,11 @@
 <table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="21" xr:uid="{0B4290D5-7CEE-4DDC-B997-690EEF6D9589}" name="Table020__Page_11" displayName="Table020__Page_11" ref="A18:E20" tableType="queryTable" totalsRowShown="0">
   <autoFilter ref="A18:E20" xr:uid="{0B4290D5-7CEE-4DDC-B997-690EEF6D9589}"/>
   <tableColumns count="5">
-    <tableColumn id="1" xr3:uid="{344C3D84-8C5A-4C60-ADD3-4EE73F83858B}" uniqueName="1" name="Column1" queryTableFieldId="1" dataDxfId="13"/>
-    <tableColumn id="2" xr3:uid="{3470DF86-5A38-429A-95CF-F5FF5E59449C}" uniqueName="2" name="Column2" queryTableFieldId="2" dataDxfId="12"/>
-    <tableColumn id="3" xr3:uid="{BC1BD851-46F6-4634-95EE-ED117E75EBB6}" uniqueName="3" name="Column3" queryTableFieldId="3" dataDxfId="11"/>
-    <tableColumn id="4" xr3:uid="{FF5D3D34-BBDB-4113-8340-C737255ED1BD}" uniqueName="4" name="Column4" queryTableFieldId="4" dataDxfId="10"/>
-    <tableColumn id="5" xr3:uid="{F05FA152-C9D6-4773-B0A5-5B18B60C7102}" uniqueName="5" name="Column5" queryTableFieldId="5" dataDxfId="9"/>
+    <tableColumn id="1" xr3:uid="{344C3D84-8C5A-4C60-ADD3-4EE73F83858B}" uniqueName="1" name="Column1" queryTableFieldId="1" dataDxfId="15"/>
+    <tableColumn id="2" xr3:uid="{3470DF86-5A38-429A-95CF-F5FF5E59449C}" uniqueName="2" name="Column2" queryTableFieldId="2" dataDxfId="14"/>
+    <tableColumn id="3" xr3:uid="{BC1BD851-46F6-4634-95EE-ED117E75EBB6}" uniqueName="3" name="Column3" queryTableFieldId="3" dataDxfId="13"/>
+    <tableColumn id="4" xr3:uid="{FF5D3D34-BBDB-4113-8340-C737255ED1BD}" uniqueName="4" name="Column4" queryTableFieldId="4" dataDxfId="12"/>
+    <tableColumn id="5" xr3:uid="{F05FA152-C9D6-4773-B0A5-5B18B60C7102}" uniqueName="5" name="Column5" queryTableFieldId="5" dataDxfId="11"/>
   </tableColumns>
   <tableStyleInfo name="TableStyleMedium7" showFirstColumn="0" showLastColumn="0" showRowStripes="1" showColumnStripes="0"/>
 </table>
@@ -5317,13 +5375,13 @@
 <table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="2" xr:uid="{D4474760-F3B7-4070-AE77-2962D090A5AB}" name="Table002__Page_2" displayName="Table002__Page_2" ref="A19:G21" tableType="queryTable" totalsRowShown="0">
   <autoFilter ref="A19:G21" xr:uid="{D4474760-F3B7-4070-AE77-2962D090A5AB}"/>
   <tableColumns count="7">
-    <tableColumn id="1" xr3:uid="{8A3681DA-5FE9-4564-BCAB-75CCDF2C3A51}" uniqueName="1" name="Column1" queryTableFieldId="1" dataDxfId="133"/>
-    <tableColumn id="2" xr3:uid="{44D6563C-A88C-4FEE-9427-B5252DF8FA5D}" uniqueName="2" name="Column6" queryTableFieldId="2" dataDxfId="132"/>
-    <tableColumn id="3" xr3:uid="{2514D758-49E4-4E3E-A628-2B2D894F398E}" uniqueName="3" name="Column2" queryTableFieldId="3" dataDxfId="131"/>
-    <tableColumn id="4" xr3:uid="{062470EA-CB73-435C-8DF3-28DE262C8D69}" uniqueName="4" name="Column3" queryTableFieldId="4" dataDxfId="130"/>
-    <tableColumn id="5" xr3:uid="{CDE500EE-B268-43D9-A30D-9E6CC1608CD0}" uniqueName="5" name="Column4" queryTableFieldId="5" dataDxfId="129"/>
-    <tableColumn id="6" xr3:uid="{699F51E2-9A1B-4953-91BE-8D6434D76B20}" uniqueName="6" name="Column5" queryTableFieldId="6" dataDxfId="128"/>
-    <tableColumn id="7" xr3:uid="{C62D0670-E212-49FF-BA61-22C41F21B60E}" uniqueName="7" name="Column62" queryTableFieldId="7" dataDxfId="127"/>
+    <tableColumn id="1" xr3:uid="{8A3681DA-5FE9-4564-BCAB-75CCDF2C3A51}" uniqueName="1" name="Column1" queryTableFieldId="1" dataDxfId="135"/>
+    <tableColumn id="2" xr3:uid="{44D6563C-A88C-4FEE-9427-B5252DF8FA5D}" uniqueName="2" name="Column6" queryTableFieldId="2" dataDxfId="134"/>
+    <tableColumn id="3" xr3:uid="{2514D758-49E4-4E3E-A628-2B2D894F398E}" uniqueName="3" name="Column2" queryTableFieldId="3" dataDxfId="133"/>
+    <tableColumn id="4" xr3:uid="{062470EA-CB73-435C-8DF3-28DE262C8D69}" uniqueName="4" name="Column3" queryTableFieldId="4" dataDxfId="132"/>
+    <tableColumn id="5" xr3:uid="{CDE500EE-B268-43D9-A30D-9E6CC1608CD0}" uniqueName="5" name="Column4" queryTableFieldId="5" dataDxfId="131"/>
+    <tableColumn id="6" xr3:uid="{699F51E2-9A1B-4953-91BE-8D6434D76B20}" uniqueName="6" name="Column5" queryTableFieldId="6" dataDxfId="130"/>
+    <tableColumn id="7" xr3:uid="{C62D0670-E212-49FF-BA61-22C41F21B60E}" uniqueName="7" name="Column62" queryTableFieldId="7" dataDxfId="129"/>
   </tableColumns>
   <tableStyleInfo name="TableStyleMedium7" showFirstColumn="0" showLastColumn="0" showRowStripes="1" showColumnStripes="0"/>
 </table>
@@ -5333,14 +5391,14 @@
 <table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="3" xr:uid="{EE92A61D-8549-4453-B707-7BA76D39611E}" name="Table003__Page_3" displayName="Table003__Page_3" ref="A1:H16" tableType="queryTable" totalsRowShown="0">
   <autoFilter ref="A1:H16" xr:uid="{EE92A61D-8549-4453-B707-7BA76D39611E}"/>
   <tableColumns count="8">
-    <tableColumn id="1" xr3:uid="{5E78ED26-3040-4033-A95F-3AC09118D17C}" uniqueName="1" name="Column1" queryTableFieldId="1" dataDxfId="126"/>
-    <tableColumn id="2" xr3:uid="{52F60F93-88D4-4F60-A15A-4B2113E53BE2}" uniqueName="2" name="Column2" queryTableFieldId="2" dataDxfId="125"/>
-    <tableColumn id="3" xr3:uid="{2A66B2A9-165C-4995-937F-8E0D8B01B3D8}" uniqueName="3" name="Column3" queryTableFieldId="3" dataDxfId="124"/>
-    <tableColumn id="4" xr3:uid="{937ED0C3-8277-4EC6-BFD2-C6699696538D}" uniqueName="4" name="Column4" queryTableFieldId="4" dataDxfId="123"/>
-    <tableColumn id="5" xr3:uid="{37EAAABA-4FEF-4D28-B237-360AD0A7194A}" uniqueName="5" name="Column5" queryTableFieldId="5" dataDxfId="122"/>
-    <tableColumn id="6" xr3:uid="{6E7D50A0-6329-4797-9F9A-628D251C7CA5}" uniqueName="6" name="Column6" queryTableFieldId="6" dataDxfId="121"/>
-    <tableColumn id="7" xr3:uid="{F8F31C01-9522-488B-915F-110987168D09}" uniqueName="7" name="Column7" queryTableFieldId="7" dataDxfId="120"/>
-    <tableColumn id="8" xr3:uid="{FFD35FDD-AAE7-4F54-8AF3-197380BC0AEB}" uniqueName="8" name="Column8" queryTableFieldId="8" dataDxfId="119"/>
+    <tableColumn id="1" xr3:uid="{5E78ED26-3040-4033-A95F-3AC09118D17C}" uniqueName="1" name="Column1" queryTableFieldId="1" dataDxfId="128"/>
+    <tableColumn id="2" xr3:uid="{52F60F93-88D4-4F60-A15A-4B2113E53BE2}" uniqueName="2" name="Column2" queryTableFieldId="2" dataDxfId="127"/>
+    <tableColumn id="3" xr3:uid="{2A66B2A9-165C-4995-937F-8E0D8B01B3D8}" uniqueName="3" name="Column3" queryTableFieldId="3" dataDxfId="126"/>
+    <tableColumn id="4" xr3:uid="{937ED0C3-8277-4EC6-BFD2-C6699696538D}" uniqueName="4" name="Column4" queryTableFieldId="4" dataDxfId="125"/>
+    <tableColumn id="5" xr3:uid="{37EAAABA-4FEF-4D28-B237-360AD0A7194A}" uniqueName="5" name="Column5" queryTableFieldId="5" dataDxfId="124"/>
+    <tableColumn id="6" xr3:uid="{6E7D50A0-6329-4797-9F9A-628D251C7CA5}" uniqueName="6" name="Column6" queryTableFieldId="6" dataDxfId="123"/>
+    <tableColumn id="7" xr3:uid="{F8F31C01-9522-488B-915F-110987168D09}" uniqueName="7" name="Column7" queryTableFieldId="7" dataDxfId="122"/>
+    <tableColumn id="8" xr3:uid="{FFD35FDD-AAE7-4F54-8AF3-197380BC0AEB}" uniqueName="8" name="Column8" queryTableFieldId="8" dataDxfId="121"/>
   </tableColumns>
   <tableStyleInfo name="TableStyleMedium7" showFirstColumn="0" showLastColumn="0" showRowStripes="1" showColumnStripes="0"/>
 </table>
@@ -5350,14 +5408,14 @@
 <table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="4" xr:uid="{1C7E55B7-7D73-418F-9229-407F52A253A6}" name="Table004__Page_3" displayName="Table004__Page_3" ref="A18:H20" tableType="queryTable" totalsRowShown="0">
   <autoFilter ref="A18:H20" xr:uid="{1C7E55B7-7D73-418F-9229-407F52A253A6}"/>
   <tableColumns count="8">
-    <tableColumn id="1" xr3:uid="{A8A6FCCE-AE43-4EDA-82DC-831809E03401}" uniqueName="1" name="Column1" queryTableFieldId="1" dataDxfId="118"/>
-    <tableColumn id="2" xr3:uid="{0231594E-DA9E-47DE-A01C-22488210A4CF}" uniqueName="2" name="Column2" queryTableFieldId="2" dataDxfId="117"/>
-    <tableColumn id="3" xr3:uid="{7A06306A-69AF-482D-910F-86D0EF88F740}" uniqueName="3" name="Column3" queryTableFieldId="3" dataDxfId="116"/>
-    <tableColumn id="4" xr3:uid="{E96F3603-E9D2-4710-BDE5-6FE3E6A378D8}" uniqueName="4" name="Column4" queryTableFieldId="4" dataDxfId="115"/>
-    <tableColumn id="5" xr3:uid="{37151140-CC9F-4EBB-B58D-F87E1081314A}" uniqueName="5" name="Column5" queryTableFieldId="5" dataDxfId="114"/>
-    <tableColumn id="6" xr3:uid="{F0AAEEC2-014D-412A-B58D-24C71FEC9A66}" uniqueName="6" name="Column6" queryTableFieldId="6" dataDxfId="113"/>
-    <tableColumn id="7" xr3:uid="{A4B4F3F0-B14D-498F-B185-AA3E2BAE729A}" uniqueName="7" name="Column7" queryTableFieldId="7" dataDxfId="112"/>
-    <tableColumn id="8" xr3:uid="{0C517BB9-44A4-4BBA-AA88-B86BB679F208}" uniqueName="8" name="Column8" queryTableFieldId="8" dataDxfId="111"/>
+    <tableColumn id="1" xr3:uid="{A8A6FCCE-AE43-4EDA-82DC-831809E03401}" uniqueName="1" name="Column1" queryTableFieldId="1" dataDxfId="120"/>
+    <tableColumn id="2" xr3:uid="{0231594E-DA9E-47DE-A01C-22488210A4CF}" uniqueName="2" name="Column2" queryTableFieldId="2" dataDxfId="119"/>
+    <tableColumn id="3" xr3:uid="{7A06306A-69AF-482D-910F-86D0EF88F740}" uniqueName="3" name="Column3" queryTableFieldId="3" dataDxfId="118"/>
+    <tableColumn id="4" xr3:uid="{E96F3603-E9D2-4710-BDE5-6FE3E6A378D8}" uniqueName="4" name="Column4" queryTableFieldId="4" dataDxfId="117"/>
+    <tableColumn id="5" xr3:uid="{37151140-CC9F-4EBB-B58D-F87E1081314A}" uniqueName="5" name="Column5" queryTableFieldId="5" dataDxfId="116"/>
+    <tableColumn id="6" xr3:uid="{F0AAEEC2-014D-412A-B58D-24C71FEC9A66}" uniqueName="6" name="Column6" queryTableFieldId="6" dataDxfId="115"/>
+    <tableColumn id="7" xr3:uid="{A4B4F3F0-B14D-498F-B185-AA3E2BAE729A}" uniqueName="7" name="Column7" queryTableFieldId="7" dataDxfId="114"/>
+    <tableColumn id="8" xr3:uid="{0C517BB9-44A4-4BBA-AA88-B86BB679F208}" uniqueName="8" name="Column8" queryTableFieldId="8" dataDxfId="113"/>
   </tableColumns>
   <tableStyleInfo name="TableStyleMedium7" showFirstColumn="0" showLastColumn="0" showRowStripes="1" showColumnStripes="0"/>
 </table>
@@ -5367,12 +5425,12 @@
 <table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="5" xr:uid="{2EB30D60-3074-4922-8217-6B97953C0F87}" name="Table005__Page_4" displayName="Table005__Page_4" ref="A1:F16" tableType="queryTable" totalsRowShown="0">
   <autoFilter ref="A1:F16" xr:uid="{2EB30D60-3074-4922-8217-6B97953C0F87}"/>
   <tableColumns count="6">
-    <tableColumn id="1" xr3:uid="{AB42FEA9-5A85-4A69-B46D-444C53C4B4EF}" uniqueName="1" name="Column1" queryTableFieldId="1" dataDxfId="110"/>
-    <tableColumn id="2" xr3:uid="{0D7919B1-FB5E-4192-8675-3D57B39D9AB0}" uniqueName="2" name="Column2" queryTableFieldId="2" dataDxfId="109"/>
-    <tableColumn id="3" xr3:uid="{94F12F3D-88BF-4BEB-85E7-FF6313F6B88E}" uniqueName="3" name="Column3" queryTableFieldId="3" dataDxfId="108"/>
-    <tableColumn id="4" xr3:uid="{2B04EEA3-DC55-4C69-860F-9571D35E352D}" uniqueName="4" name="Column4" queryTableFieldId="4" dataDxfId="107"/>
-    <tableColumn id="5" xr3:uid="{461C5084-182B-40CC-B479-24798E48D0F4}" uniqueName="5" name="Column5" queryTableFieldId="5" dataDxfId="106"/>
-    <tableColumn id="6" xr3:uid="{258F7EB6-7345-43CA-BF8A-5E088D06FF8F}" uniqueName="6" name="Column6" queryTableFieldId="6" dataDxfId="105"/>
+    <tableColumn id="1" xr3:uid="{AB42FEA9-5A85-4A69-B46D-444C53C4B4EF}" uniqueName="1" name="Column1" queryTableFieldId="1" dataDxfId="112"/>
+    <tableColumn id="2" xr3:uid="{0D7919B1-FB5E-4192-8675-3D57B39D9AB0}" uniqueName="2" name="Column2" queryTableFieldId="2" dataDxfId="111"/>
+    <tableColumn id="3" xr3:uid="{94F12F3D-88BF-4BEB-85E7-FF6313F6B88E}" uniqueName="3" name="Column3" queryTableFieldId="3" dataDxfId="110"/>
+    <tableColumn id="4" xr3:uid="{2B04EEA3-DC55-4C69-860F-9571D35E352D}" uniqueName="4" name="Column4" queryTableFieldId="4" dataDxfId="109"/>
+    <tableColumn id="5" xr3:uid="{461C5084-182B-40CC-B479-24798E48D0F4}" uniqueName="5" name="Column5" queryTableFieldId="5" dataDxfId="108"/>
+    <tableColumn id="6" xr3:uid="{258F7EB6-7345-43CA-BF8A-5E088D06FF8F}" uniqueName="6" name="Column6" queryTableFieldId="6" dataDxfId="107"/>
   </tableColumns>
   <tableStyleInfo name="TableStyleMedium7" showFirstColumn="0" showLastColumn="0" showRowStripes="1" showColumnStripes="0"/>
 </table>
@@ -5382,12 +5440,12 @@
 <table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="6" xr:uid="{BA3E356C-A98F-4646-B7E8-7B0C3904E2A4}" name="Table006__Page_4" displayName="Table006__Page_4" ref="A18:F20" tableType="queryTable" totalsRowShown="0">
   <autoFilter ref="A18:F20" xr:uid="{BA3E356C-A98F-4646-B7E8-7B0C3904E2A4}"/>
   <tableColumns count="6">
-    <tableColumn id="1" xr3:uid="{55987721-40E8-4E11-9B6F-67EE503D78F4}" uniqueName="1" name="Column1" queryTableFieldId="1" dataDxfId="104"/>
-    <tableColumn id="2" xr3:uid="{15260D47-39CC-4501-9656-F8DBE6AD3AB1}" uniqueName="2" name="Column2" queryTableFieldId="2" dataDxfId="103"/>
-    <tableColumn id="3" xr3:uid="{06C8B30C-3DD3-49E6-8BE6-C8A9D39F2FC4}" uniqueName="3" name="Column3" queryTableFieldId="3" dataDxfId="102"/>
-    <tableColumn id="4" xr3:uid="{40A070F6-4BDB-49A7-9394-4D63F3A9E318}" uniqueName="4" name="Column4" queryTableFieldId="4" dataDxfId="101"/>
-    <tableColumn id="5" xr3:uid="{C5E0BAEF-796C-4C71-ACA7-889E63543C2D}" uniqueName="5" name="Column5" queryTableFieldId="5" dataDxfId="100"/>
-    <tableColumn id="6" xr3:uid="{1BA75280-A961-41F1-B113-5935891BA00A}" uniqueName="6" name="Column6" queryTableFieldId="6" dataDxfId="99"/>
+    <tableColumn id="1" xr3:uid="{55987721-40E8-4E11-9B6F-67EE503D78F4}" uniqueName="1" name="Column1" queryTableFieldId="1" dataDxfId="106"/>
+    <tableColumn id="2" xr3:uid="{15260D47-39CC-4501-9656-F8DBE6AD3AB1}" uniqueName="2" name="Column2" queryTableFieldId="2" dataDxfId="105"/>
+    <tableColumn id="3" xr3:uid="{06C8B30C-3DD3-49E6-8BE6-C8A9D39F2FC4}" uniqueName="3" name="Column3" queryTableFieldId="3" dataDxfId="104"/>
+    <tableColumn id="4" xr3:uid="{40A070F6-4BDB-49A7-9394-4D63F3A9E318}" uniqueName="4" name="Column4" queryTableFieldId="4" dataDxfId="103"/>
+    <tableColumn id="5" xr3:uid="{C5E0BAEF-796C-4C71-ACA7-889E63543C2D}" uniqueName="5" name="Column5" queryTableFieldId="5" dataDxfId="102"/>
+    <tableColumn id="6" xr3:uid="{1BA75280-A961-41F1-B113-5935891BA00A}" uniqueName="6" name="Column6" queryTableFieldId="6" dataDxfId="101"/>
   </tableColumns>
   <tableStyleInfo name="TableStyleMedium7" showFirstColumn="0" showLastColumn="0" showRowStripes="1" showColumnStripes="0"/>
 </table>
@@ -5397,18 +5455,18 @@
 <table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="7" xr:uid="{6040FF08-DFFC-4D6C-87C0-7C33D5281777}" name="Table007__Page_5" displayName="Table007__Page_5" ref="A1:L16" tableType="queryTable" totalsRowShown="0">
   <autoFilter ref="A1:L16" xr:uid="{6040FF08-DFFC-4D6C-87C0-7C33D5281777}"/>
   <tableColumns count="12">
-    <tableColumn id="1" xr3:uid="{9561388E-64AE-4A76-863E-A0B2091E2F9F}" uniqueName="1" name="Column1" queryTableFieldId="1" dataDxfId="98"/>
-    <tableColumn id="2" xr3:uid="{151810A9-7DD3-4FD0-91D6-6608DF85A8CF}" uniqueName="2" name="Column2" queryTableFieldId="2" dataDxfId="97"/>
-    <tableColumn id="3" xr3:uid="{94D629BF-F745-493D-8F74-FA7EEFDEAA84}" uniqueName="3" name="Column3" queryTableFieldId="3" dataDxfId="96"/>
-    <tableColumn id="4" xr3:uid="{AE87299A-170F-4661-BD08-B108394E2F7C}" uniqueName="4" name="Column4" queryTableFieldId="4" dataDxfId="95"/>
-    <tableColumn id="5" xr3:uid="{708CB468-5E3F-4D0C-B6BD-C2C44C7191EC}" uniqueName="5" name="Column5" queryTableFieldId="5" dataDxfId="94"/>
-    <tableColumn id="6" xr3:uid="{5D4BD3CB-C344-4155-B3C1-ECC49F86CED1}" uniqueName="6" name="Column6" queryTableFieldId="6" dataDxfId="93"/>
-    <tableColumn id="7" xr3:uid="{61DF1122-5C54-47A3-98F9-27CA1B50CA9D}" uniqueName="7" name="Column7" queryTableFieldId="7" dataDxfId="92"/>
-    <tableColumn id="8" xr3:uid="{130590EE-DDCB-43DB-A020-385B521DA018}" uniqueName="8" name="Column8" queryTableFieldId="8" dataDxfId="91"/>
-    <tableColumn id="9" xr3:uid="{06B903F7-5E22-476D-A116-655599D2C518}" uniqueName="9" name="Column9" queryTableFieldId="9" dataDxfId="90"/>
-    <tableColumn id="10" xr3:uid="{CED96D55-8B0D-492D-B0EC-F3E56EFB2649}" uniqueName="10" name="Column10" queryTableFieldId="10" dataDxfId="89"/>
-    <tableColumn id="11" xr3:uid="{346823E9-F305-4F11-941F-1C42A8AB0C99}" uniqueName="11" name="Column11" queryTableFieldId="11" dataDxfId="88"/>
-    <tableColumn id="12" xr3:uid="{7B421AA8-C9DB-4E35-A456-DF0F56050B79}" uniqueName="12" name="Column12" queryTableFieldId="12" dataDxfId="87"/>
+    <tableColumn id="1" xr3:uid="{9561388E-64AE-4A76-863E-A0B2091E2F9F}" uniqueName="1" name="Column1" queryTableFieldId="1" dataDxfId="100"/>
+    <tableColumn id="2" xr3:uid="{151810A9-7DD3-4FD0-91D6-6608DF85A8CF}" uniqueName="2" name="Column2" queryTableFieldId="2" dataDxfId="99"/>
+    <tableColumn id="3" xr3:uid="{94D629BF-F745-493D-8F74-FA7EEFDEAA84}" uniqueName="3" name="Column3" queryTableFieldId="3" dataDxfId="98"/>
+    <tableColumn id="4" xr3:uid="{AE87299A-170F-4661-BD08-B108394E2F7C}" uniqueName="4" name="Column4" queryTableFieldId="4" dataDxfId="97"/>
+    <tableColumn id="5" xr3:uid="{708CB468-5E3F-4D0C-B6BD-C2C44C7191EC}" uniqueName="5" name="Column5" queryTableFieldId="5" dataDxfId="96"/>
+    <tableColumn id="6" xr3:uid="{5D4BD3CB-C344-4155-B3C1-ECC49F86CED1}" uniqueName="6" name="Column6" queryTableFieldId="6" dataDxfId="95"/>
+    <tableColumn id="7" xr3:uid="{61DF1122-5C54-47A3-98F9-27CA1B50CA9D}" uniqueName="7" name="Column7" queryTableFieldId="7" dataDxfId="94"/>
+    <tableColumn id="8" xr3:uid="{130590EE-DDCB-43DB-A020-385B521DA018}" uniqueName="8" name="Column8" queryTableFieldId="8" dataDxfId="93"/>
+    <tableColumn id="9" xr3:uid="{06B903F7-5E22-476D-A116-655599D2C518}" uniqueName="9" name="Column9" queryTableFieldId="9" dataDxfId="92"/>
+    <tableColumn id="10" xr3:uid="{CED96D55-8B0D-492D-B0EC-F3E56EFB2649}" uniqueName="10" name="Column10" queryTableFieldId="10" dataDxfId="91"/>
+    <tableColumn id="11" xr3:uid="{346823E9-F305-4F11-941F-1C42A8AB0C99}" uniqueName="11" name="Column11" queryTableFieldId="11" dataDxfId="90"/>
+    <tableColumn id="12" xr3:uid="{7B421AA8-C9DB-4E35-A456-DF0F56050B79}" uniqueName="12" name="Column12" queryTableFieldId="12" dataDxfId="89"/>
   </tableColumns>
   <tableStyleInfo name="TableStyleMedium7" showFirstColumn="0" showLastColumn="0" showRowStripes="1" showColumnStripes="0"/>
 </table>
@@ -5418,18 +5476,18 @@
 <table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="8" xr:uid="{DBF54861-4823-4965-9BF8-BF4D83A85FD1}" name="Table008__Page_5" displayName="Table008__Page_5" ref="A18:L20" tableType="queryTable" totalsRowShown="0">
   <autoFilter ref="A18:L20" xr:uid="{DBF54861-4823-4965-9BF8-BF4D83A85FD1}"/>
   <tableColumns count="12">
-    <tableColumn id="1" xr3:uid="{01D3C90B-BA67-46B4-BD1D-5C53486CAE57}" uniqueName="1" name="Column1" queryTableFieldId="1" dataDxfId="86"/>
-    <tableColumn id="2" xr3:uid="{166854EB-0B50-4420-BB3F-7A5A2C9FB7F7}" uniqueName="2" name="Column2" queryTableFieldId="2" dataDxfId="85"/>
-    <tableColumn id="3" xr3:uid="{638857E5-1EB4-4FBE-9FFE-2951F2F4ABD0}" uniqueName="3" name="Column3" queryTableFieldId="3" dataDxfId="84"/>
-    <tableColumn id="4" xr3:uid="{F4EFE2EF-AC84-40F8-BE68-0B6B520F8EA8}" uniqueName="4" name="Column4" queryTableFieldId="4" dataDxfId="83"/>
-    <tableColumn id="5" xr3:uid="{38D026D2-A47E-46EA-BA10-AF890A55BF2B}" uniqueName="5" name="Column5" queryTableFieldId="5" dataDxfId="82"/>
-    <tableColumn id="6" xr3:uid="{025C6DA2-37A6-491F-904E-DDE12948D35B}" uniqueName="6" name="Column6" queryTableFieldId="6" dataDxfId="81"/>
-    <tableColumn id="7" xr3:uid="{AC28B573-67B7-4468-A6A2-F648D17079B6}" uniqueName="7" name="Column7" queryTableFieldId="7" dataDxfId="80"/>
-    <tableColumn id="8" xr3:uid="{F6F06554-210B-472F-95F2-8E89D931E4C1}" uniqueName="8" name="Column8" queryTableFieldId="8" dataDxfId="79"/>
-    <tableColumn id="9" xr3:uid="{F0A8F323-36C1-4290-980B-8F6F5DC6A41E}" uniqueName="9" name="Column9" queryTableFieldId="9" dataDxfId="78"/>
-    <tableColumn id="10" xr3:uid="{25D60007-5007-4174-85F5-572E3C29FE33}" uniqueName="10" name="Column10" queryTableFieldId="10" dataDxfId="77"/>
-    <tableColumn id="11" xr3:uid="{2071EB9B-B14E-4EF0-9B86-0D5FDA96828D}" uniqueName="11" name="Column11" queryTableFieldId="11" dataDxfId="76"/>
-    <tableColumn id="12" xr3:uid="{1660C180-EE6B-48E8-9880-55F02CC623C4}" uniqueName="12" name="Column12" queryTableFieldId="12" dataDxfId="75"/>
+    <tableColumn id="1" xr3:uid="{01D3C90B-BA67-46B4-BD1D-5C53486CAE57}" uniqueName="1" name="Column1" queryTableFieldId="1" dataDxfId="88"/>
+    <tableColumn id="2" xr3:uid="{166854EB-0B50-4420-BB3F-7A5A2C9FB7F7}" uniqueName="2" name="Column2" queryTableFieldId="2" dataDxfId="87"/>
+    <tableColumn id="3" xr3:uid="{638857E5-1EB4-4FBE-9FFE-2951F2F4ABD0}" uniqueName="3" name="Column3" queryTableFieldId="3" dataDxfId="86"/>
+    <tableColumn id="4" xr3:uid="{F4EFE2EF-AC84-40F8-BE68-0B6B520F8EA8}" uniqueName="4" name="Column4" queryTableFieldId="4" dataDxfId="85"/>
+    <tableColumn id="5" xr3:uid="{38D026D2-A47E-46EA-BA10-AF890A55BF2B}" uniqueName="5" name="Column5" queryTableFieldId="5" dataDxfId="84"/>
+    <tableColumn id="6" xr3:uid="{025C6DA2-37A6-491F-904E-DDE12948D35B}" uniqueName="6" name="Column6" queryTableFieldId="6" dataDxfId="83"/>
+    <tableColumn id="7" xr3:uid="{AC28B573-67B7-4468-A6A2-F648D17079B6}" uniqueName="7" name="Column7" queryTableFieldId="7" dataDxfId="82"/>
+    <tableColumn id="8" xr3:uid="{F6F06554-210B-472F-95F2-8E89D931E4C1}" uniqueName="8" name="Column8" queryTableFieldId="8" dataDxfId="81"/>
+    <tableColumn id="9" xr3:uid="{F0A8F323-36C1-4290-980B-8F6F5DC6A41E}" uniqueName="9" name="Column9" queryTableFieldId="9" dataDxfId="80"/>
+    <tableColumn id="10" xr3:uid="{25D60007-5007-4174-85F5-572E3C29FE33}" uniqueName="10" name="Column10" queryTableFieldId="10" dataDxfId="79"/>
+    <tableColumn id="11" xr3:uid="{2071EB9B-B14E-4EF0-9B86-0D5FDA96828D}" uniqueName="11" name="Column11" queryTableFieldId="11" dataDxfId="78"/>
+    <tableColumn id="12" xr3:uid="{1660C180-EE6B-48E8-9880-55F02CC623C4}" uniqueName="12" name="Column12" queryTableFieldId="12" dataDxfId="77"/>
   </tableColumns>
   <tableStyleInfo name="TableStyleMedium7" showFirstColumn="0" showLastColumn="0" showRowStripes="1" showColumnStripes="0"/>
 </table>
@@ -5732,42 +5790,42 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{3B05C9E0-A64E-40AC-B9F4-C919ED5906CC}">
-  <dimension ref="A1:I70"/>
-  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
+  <dimension ref="A1:I79"/>
+  <sheetFormatPr defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
   <cols>
-    <col min="1" max="1" width="51.42578125" bestFit="1" customWidth="1"/>
-    <col min="2" max="2" width="36.5703125" bestFit="1" customWidth="1"/>
-    <col min="3" max="3" width="17.140625" bestFit="1" customWidth="1"/>
-    <col min="4" max="4" width="16.140625" bestFit="1" customWidth="1"/>
-    <col min="5" max="6" width="17.42578125" customWidth="1"/>
-    <col min="7" max="7" width="10.85546875" customWidth="1"/>
-    <col min="8" max="8" width="14.42578125" bestFit="1" customWidth="1"/>
-    <col min="9" max="9" width="14.28515625" bestFit="1" customWidth="1"/>
-    <col min="10" max="10" width="14.42578125" bestFit="1" customWidth="1"/>
-    <col min="11" max="11" width="18.140625" bestFit="1" customWidth="1"/>
-    <col min="12" max="12" width="17.42578125" bestFit="1" customWidth="1"/>
-    <col min="13" max="14" width="13.42578125" bestFit="1" customWidth="1"/>
-    <col min="15" max="15" width="26.5703125" bestFit="1" customWidth="1"/>
+    <col min="1" max="1" width="51.453125" bestFit="1" customWidth="1"/>
+    <col min="2" max="2" width="36.54296875" bestFit="1" customWidth="1"/>
+    <col min="3" max="3" width="17.1796875" bestFit="1" customWidth="1"/>
+    <col min="4" max="4" width="16.1796875" bestFit="1" customWidth="1"/>
+    <col min="5" max="6" width="17.453125" customWidth="1"/>
+    <col min="7" max="7" width="10.81640625" customWidth="1"/>
+    <col min="8" max="8" width="14.453125" bestFit="1" customWidth="1"/>
+    <col min="9" max="9" width="14.26953125" bestFit="1" customWidth="1"/>
+    <col min="10" max="10" width="14.453125" bestFit="1" customWidth="1"/>
+    <col min="11" max="11" width="18.1796875" bestFit="1" customWidth="1"/>
+    <col min="12" max="12" width="17.453125" bestFit="1" customWidth="1"/>
+    <col min="13" max="14" width="13.453125" bestFit="1" customWidth="1"/>
+    <col min="15" max="15" width="26.54296875" bestFit="1" customWidth="1"/>
     <col min="16" max="16" width="8" bestFit="1" customWidth="1"/>
-    <col min="17" max="17" width="10.42578125" bestFit="1" customWidth="1"/>
-    <col min="18" max="18" width="25.7109375" bestFit="1" customWidth="1"/>
+    <col min="17" max="17" width="10.453125" bestFit="1" customWidth="1"/>
+    <col min="18" max="18" width="25.7265625" bestFit="1" customWidth="1"/>
     <col min="19" max="19" width="20" bestFit="1" customWidth="1"/>
-    <col min="20" max="20" width="37.140625" bestFit="1" customWidth="1"/>
-    <col min="21" max="21" width="33.5703125" bestFit="1" customWidth="1"/>
-    <col min="22" max="22" width="15.42578125" bestFit="1" customWidth="1"/>
-    <col min="23" max="23" width="22.140625" bestFit="1" customWidth="1"/>
-    <col min="24" max="24" width="30.140625" bestFit="1" customWidth="1"/>
-    <col min="25" max="25" width="26.42578125" bestFit="1" customWidth="1"/>
-    <col min="26" max="26" width="28.42578125" bestFit="1" customWidth="1"/>
-    <col min="27" max="27" width="21.140625" bestFit="1" customWidth="1"/>
-    <col min="28" max="28" width="11.5703125" bestFit="1" customWidth="1"/>
-    <col min="29" max="29" width="25.85546875" bestFit="1" customWidth="1"/>
-    <col min="30" max="30" width="34.140625" bestFit="1" customWidth="1"/>
-    <col min="31" max="31" width="22.140625" bestFit="1" customWidth="1"/>
-    <col min="32" max="32" width="10.7109375" bestFit="1" customWidth="1"/>
+    <col min="20" max="20" width="37.1796875" bestFit="1" customWidth="1"/>
+    <col min="21" max="21" width="33.54296875" bestFit="1" customWidth="1"/>
+    <col min="22" max="22" width="15.453125" bestFit="1" customWidth="1"/>
+    <col min="23" max="23" width="22.1796875" bestFit="1" customWidth="1"/>
+    <col min="24" max="24" width="30.1796875" bestFit="1" customWidth="1"/>
+    <col min="25" max="25" width="26.453125" bestFit="1" customWidth="1"/>
+    <col min="26" max="26" width="28.453125" bestFit="1" customWidth="1"/>
+    <col min="27" max="27" width="21.1796875" bestFit="1" customWidth="1"/>
+    <col min="28" max="28" width="11.54296875" bestFit="1" customWidth="1"/>
+    <col min="29" max="29" width="25.81640625" bestFit="1" customWidth="1"/>
+    <col min="30" max="30" width="34.1796875" bestFit="1" customWidth="1"/>
+    <col min="31" max="31" width="22.1796875" bestFit="1" customWidth="1"/>
+    <col min="32" max="32" width="10.7265625" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:9" x14ac:dyDescent="0.25">
+    <row r="1" spans="1:9" x14ac:dyDescent="0.35">
       <c r="A1" s="13" t="s">
         <v>551</v>
       </c>
@@ -5796,7 +5854,7 @@
         <v>585</v>
       </c>
     </row>
-    <row r="2" spans="1:9" x14ac:dyDescent="0.25">
+    <row r="2" spans="1:9" x14ac:dyDescent="0.35">
       <c r="A2" s="10" t="s">
         <v>580</v>
       </c>
@@ -5828,7 +5886,7 @@
         <v>21000000.000000004</v>
       </c>
     </row>
-    <row r="3" spans="1:9" x14ac:dyDescent="0.25">
+    <row r="3" spans="1:9" x14ac:dyDescent="0.35">
       <c r="A3" s="10" t="s">
         <v>555</v>
       </c>
@@ -5860,7 +5918,7 @@
         <v>21000000.000000004</v>
       </c>
     </row>
-    <row r="4" spans="1:9" x14ac:dyDescent="0.25">
+    <row r="4" spans="1:9" x14ac:dyDescent="0.35">
       <c r="A4" s="10" t="s">
         <v>500</v>
       </c>
@@ -5892,7 +5950,7 @@
         <v>21000000.000000004</v>
       </c>
     </row>
-    <row r="5" spans="1:9" x14ac:dyDescent="0.25">
+    <row r="5" spans="1:9" x14ac:dyDescent="0.35">
       <c r="A5" s="10" t="s">
         <v>501</v>
       </c>
@@ -5924,7 +5982,7 @@
         <v>21000000.000000004</v>
       </c>
     </row>
-    <row r="6" spans="1:9" x14ac:dyDescent="0.25">
+    <row r="6" spans="1:9" x14ac:dyDescent="0.35">
       <c r="A6" s="10" t="s">
         <v>502</v>
       </c>
@@ -5956,7 +6014,7 @@
         <v>24999999.999999996</v>
       </c>
     </row>
-    <row r="7" spans="1:9" x14ac:dyDescent="0.25">
+    <row r="7" spans="1:9" x14ac:dyDescent="0.35">
       <c r="A7" s="10" t="s">
         <v>515</v>
       </c>
@@ -5988,7 +6046,7 @@
         <v>23249999.999999996</v>
       </c>
     </row>
-    <row r="8" spans="1:9" x14ac:dyDescent="0.25">
+    <row r="8" spans="1:9" x14ac:dyDescent="0.35">
       <c r="A8" s="10" t="s">
         <v>516</v>
       </c>
@@ -6020,7 +6078,7 @@
         <v>24700000.000000004</v>
       </c>
     </row>
-    <row r="9" spans="1:9" x14ac:dyDescent="0.25">
+    <row r="9" spans="1:9" x14ac:dyDescent="0.35">
       <c r="A9" s="10" t="s">
         <v>547</v>
       </c>
@@ -6052,7 +6110,7 @@
         <v>32999999.999999996</v>
       </c>
     </row>
-    <row r="10" spans="1:9" x14ac:dyDescent="0.25">
+    <row r="10" spans="1:9" x14ac:dyDescent="0.35">
       <c r="A10" s="10" t="s">
         <v>514</v>
       </c>
@@ -6084,7 +6142,7 @@
         <v>35000000</v>
       </c>
     </row>
-    <row r="11" spans="1:9" x14ac:dyDescent="0.25">
+    <row r="11" spans="1:9" x14ac:dyDescent="0.35">
       <c r="A11" s="10" t="s">
         <v>496</v>
       </c>
@@ -6116,7 +6174,7 @@
         <v>35000000</v>
       </c>
     </row>
-    <row r="12" spans="1:9" x14ac:dyDescent="0.25">
+    <row r="12" spans="1:9" x14ac:dyDescent="0.35">
       <c r="A12" s="10" t="s">
         <v>497</v>
       </c>
@@ -6148,7 +6206,7 @@
         <v>38000000</v>
       </c>
     </row>
-    <row r="13" spans="1:9" x14ac:dyDescent="0.25">
+    <row r="13" spans="1:9" x14ac:dyDescent="0.35">
       <c r="A13" s="10" t="s">
         <v>517</v>
       </c>
@@ -6180,7 +6238,7 @@
         <v>23000000</v>
       </c>
     </row>
-    <row r="14" spans="1:9" x14ac:dyDescent="0.25">
+    <row r="14" spans="1:9" x14ac:dyDescent="0.35">
       <c r="A14" s="10" t="s">
         <v>518</v>
       </c>
@@ -6212,7 +6270,7 @@
         <v>20000000</v>
       </c>
     </row>
-    <row r="15" spans="1:9" x14ac:dyDescent="0.25">
+    <row r="15" spans="1:9" x14ac:dyDescent="0.35">
       <c r="A15" s="10" t="s">
         <v>519</v>
       </c>
@@ -6244,7 +6302,7 @@
         <v>13000000</v>
       </c>
     </row>
-    <row r="16" spans="1:9" x14ac:dyDescent="0.25">
+    <row r="16" spans="1:9" x14ac:dyDescent="0.35">
       <c r="A16" s="10" t="s">
         <v>610</v>
       </c>
@@ -6276,7 +6334,7 @@
         <v>13000000</v>
       </c>
     </row>
-    <row r="17" spans="1:9" x14ac:dyDescent="0.25">
+    <row r="17" spans="1:9" x14ac:dyDescent="0.35">
       <c r="A17" s="10" t="s">
         <v>612</v>
       </c>
@@ -6308,7 +6366,7 @@
         <v>20000000</v>
       </c>
     </row>
-    <row r="18" spans="1:9" x14ac:dyDescent="0.25">
+    <row r="18" spans="1:9" x14ac:dyDescent="0.35">
       <c r="A18" s="10" t="s">
         <v>617</v>
       </c>
@@ -6340,7 +6398,7 @@
         <v>23000000</v>
       </c>
     </row>
-    <row r="19" spans="1:9" x14ac:dyDescent="0.25">
+    <row r="19" spans="1:9" x14ac:dyDescent="0.35">
       <c r="A19" s="10" t="s">
         <v>503</v>
       </c>
@@ -6372,7 +6430,7 @@
         <v>29000000</v>
       </c>
     </row>
-    <row r="20" spans="1:9" x14ac:dyDescent="0.25">
+    <row r="20" spans="1:9" x14ac:dyDescent="0.35">
       <c r="A20" s="10" t="s">
         <v>586</v>
       </c>
@@ -6404,7 +6462,7 @@
         <v>26000000</v>
       </c>
     </row>
-    <row r="21" spans="1:9" x14ac:dyDescent="0.25">
+    <row r="21" spans="1:9" x14ac:dyDescent="0.35">
       <c r="A21" s="10" t="s">
         <v>504</v>
       </c>
@@ -6436,7 +6494,7 @@
         <v>30000000</v>
       </c>
     </row>
-    <row r="22" spans="1:9" x14ac:dyDescent="0.25">
+    <row r="22" spans="1:9" x14ac:dyDescent="0.35">
       <c r="A22" s="10" t="s">
         <v>588</v>
       </c>
@@ -6468,7 +6526,7 @@
         <v>29000000</v>
       </c>
     </row>
-    <row r="23" spans="1:9" x14ac:dyDescent="0.25">
+    <row r="23" spans="1:9" x14ac:dyDescent="0.35">
       <c r="A23" s="10" t="s">
         <v>587</v>
       </c>
@@ -6500,7 +6558,7 @@
         <v>29000000</v>
       </c>
     </row>
-    <row r="24" spans="1:9" x14ac:dyDescent="0.25">
+    <row r="24" spans="1:9" x14ac:dyDescent="0.35">
       <c r="A24" s="10" t="s">
         <v>505</v>
       </c>
@@ -6532,7 +6590,7 @@
         <v>34000000</v>
       </c>
     </row>
-    <row r="25" spans="1:9" x14ac:dyDescent="0.25">
+    <row r="25" spans="1:9" x14ac:dyDescent="0.35">
       <c r="A25" s="10" t="s">
         <v>558</v>
       </c>
@@ -6564,7 +6622,7 @@
         <v>37000000</v>
       </c>
     </row>
-    <row r="26" spans="1:9" x14ac:dyDescent="0.25">
+    <row r="26" spans="1:9" x14ac:dyDescent="0.35">
       <c r="A26" s="10" t="s">
         <v>506</v>
       </c>
@@ -6596,7 +6654,7 @@
         <v>37000000</v>
       </c>
     </row>
-    <row r="27" spans="1:9" x14ac:dyDescent="0.25">
+    <row r="27" spans="1:9" x14ac:dyDescent="0.35">
       <c r="A27" s="10" t="s">
         <v>561</v>
       </c>
@@ -6628,7 +6686,7 @@
         <v>37000000</v>
       </c>
     </row>
-    <row r="28" spans="1:9" x14ac:dyDescent="0.25">
+    <row r="28" spans="1:9" x14ac:dyDescent="0.35">
       <c r="A28" s="10" t="s">
         <v>557</v>
       </c>
@@ -6660,7 +6718,7 @@
         <v>37000000</v>
       </c>
     </row>
-    <row r="29" spans="1:9" x14ac:dyDescent="0.25">
+    <row r="29" spans="1:9" x14ac:dyDescent="0.35">
       <c r="A29" s="10" t="s">
         <v>582</v>
       </c>
@@ -6692,7 +6750,7 @@
         <v>37000000</v>
       </c>
     </row>
-    <row r="30" spans="1:9" x14ac:dyDescent="0.25">
+    <row r="30" spans="1:9" x14ac:dyDescent="0.35">
       <c r="A30" s="10" t="s">
         <v>523</v>
       </c>
@@ -6724,7 +6782,7 @@
         <v>12700000.000000002</v>
       </c>
     </row>
-    <row r="31" spans="1:9" x14ac:dyDescent="0.25">
+    <row r="31" spans="1:9" x14ac:dyDescent="0.35">
       <c r="A31" s="10" t="s">
         <v>560</v>
       </c>
@@ -6756,7 +6814,7 @@
         <v>12700000.000000002</v>
       </c>
     </row>
-    <row r="32" spans="1:9" x14ac:dyDescent="0.25">
+    <row r="32" spans="1:9" x14ac:dyDescent="0.35">
       <c r="A32" s="10" t="s">
         <v>524</v>
       </c>
@@ -6788,7 +6846,7 @@
         <v>16000000</v>
       </c>
     </row>
-    <row r="33" spans="1:9" x14ac:dyDescent="0.25">
+    <row r="33" spans="1:9" x14ac:dyDescent="0.35">
       <c r="A33" s="10" t="s">
         <v>498</v>
       </c>
@@ -6820,7 +6878,7 @@
         <v>14700000</v>
       </c>
     </row>
-    <row r="34" spans="1:9" x14ac:dyDescent="0.25">
+    <row r="34" spans="1:9" x14ac:dyDescent="0.35">
       <c r="A34" s="10" t="s">
         <v>525</v>
       </c>
@@ -6852,7 +6910,7 @@
         <v>18300000</v>
       </c>
     </row>
-    <row r="35" spans="1:9" x14ac:dyDescent="0.25">
+    <row r="35" spans="1:9" x14ac:dyDescent="0.35">
       <c r="A35" s="10" t="s">
         <v>527</v>
       </c>
@@ -6884,7 +6942,7 @@
         <v>20900000</v>
       </c>
     </row>
-    <row r="36" spans="1:9" x14ac:dyDescent="0.25">
+    <row r="36" spans="1:9" x14ac:dyDescent="0.35">
       <c r="A36" s="10" t="s">
         <v>528</v>
       </c>
@@ -6916,7 +6974,7 @@
         <v>22000000</v>
       </c>
     </row>
-    <row r="37" spans="1:9" x14ac:dyDescent="0.25">
+    <row r="37" spans="1:9" x14ac:dyDescent="0.35">
       <c r="A37" s="10" t="s">
         <v>499</v>
       </c>
@@ -6948,7 +7006,7 @@
         <v>20500000.000000004</v>
       </c>
     </row>
-    <row r="38" spans="1:9" x14ac:dyDescent="0.25">
+    <row r="38" spans="1:9" x14ac:dyDescent="0.35">
       <c r="A38" s="10" t="s">
         <v>616</v>
       </c>
@@ -6980,7 +7038,7 @@
         <v>22400000</v>
       </c>
     </row>
-    <row r="39" spans="1:9" x14ac:dyDescent="0.25">
+    <row r="39" spans="1:9" x14ac:dyDescent="0.35">
       <c r="A39" s="11" t="s">
         <v>522</v>
       </c>
@@ -7012,7 +7070,7 @@
         <v>25600000</v>
       </c>
     </row>
-    <row r="40" spans="1:9" x14ac:dyDescent="0.25">
+    <row r="40" spans="1:9" x14ac:dyDescent="0.35">
       <c r="A40" s="22" t="s">
         <v>149</v>
       </c>
@@ -7044,7 +7102,7 @@
         <v>22400000</v>
       </c>
     </row>
-    <row r="41" spans="1:9" x14ac:dyDescent="0.25">
+    <row r="41" spans="1:9" x14ac:dyDescent="0.35">
       <c r="A41" s="10" t="s">
         <v>607</v>
       </c>
@@ -7076,7 +7134,7 @@
         <v>31600000</v>
       </c>
     </row>
-    <row r="42" spans="1:9" x14ac:dyDescent="0.25">
+    <row r="42" spans="1:9" x14ac:dyDescent="0.35">
       <c r="A42" s="10" t="s">
         <v>599</v>
       </c>
@@ -7108,7 +7166,7 @@
         <v>36400000</v>
       </c>
     </row>
-    <row r="43" spans="1:9" x14ac:dyDescent="0.25">
+    <row r="43" spans="1:9" x14ac:dyDescent="0.35">
       <c r="A43" s="10" t="s">
         <v>618</v>
       </c>
@@ -7140,7 +7198,7 @@
         <v>32700000</v>
       </c>
     </row>
-    <row r="44" spans="1:9" x14ac:dyDescent="0.25">
+    <row r="44" spans="1:9" x14ac:dyDescent="0.35">
       <c r="A44" s="10" t="s">
         <v>602</v>
       </c>
@@ -7172,7 +7230,7 @@
         <v>36400000</v>
       </c>
     </row>
-    <row r="45" spans="1:9" x14ac:dyDescent="0.25">
+    <row r="45" spans="1:9" x14ac:dyDescent="0.35">
       <c r="A45" s="10" t="s">
         <v>526</v>
       </c>
@@ -7204,7 +7262,7 @@
         <v>12499999.999999998</v>
       </c>
     </row>
-    <row r="46" spans="1:9" x14ac:dyDescent="0.25">
+    <row r="46" spans="1:9" x14ac:dyDescent="0.35">
       <c r="A46" s="16" t="s">
         <v>521</v>
       </c>
@@ -7236,7 +7294,7 @@
         <v>13500000</v>
       </c>
     </row>
-    <row r="47" spans="1:9" x14ac:dyDescent="0.25">
+    <row r="47" spans="1:9" x14ac:dyDescent="0.35">
       <c r="A47" s="4" t="s">
         <v>529</v>
       </c>
@@ -7268,7 +7326,7 @@
         <v>12200000</v>
       </c>
     </row>
-    <row r="48" spans="1:9" x14ac:dyDescent="0.25">
+    <row r="48" spans="1:9" x14ac:dyDescent="0.35">
       <c r="A48" s="4" t="s">
         <v>608</v>
       </c>
@@ -7300,7 +7358,7 @@
         <v>8000000</v>
       </c>
     </row>
-    <row r="49" spans="1:9" x14ac:dyDescent="0.25">
+    <row r="49" spans="1:9" x14ac:dyDescent="0.35">
       <c r="A49" s="4" t="s">
         <v>520</v>
       </c>
@@ -7332,7 +7390,7 @@
         <v>8000000</v>
       </c>
     </row>
-    <row r="50" spans="1:9" x14ac:dyDescent="0.25">
+    <row r="50" spans="1:9" x14ac:dyDescent="0.35">
       <c r="A50" s="17" t="s">
         <v>593</v>
       </c>
@@ -7364,7 +7422,7 @@
         <v>20000000</v>
       </c>
     </row>
-    <row r="51" spans="1:9" x14ac:dyDescent="0.25">
+    <row r="51" spans="1:9" x14ac:dyDescent="0.35">
       <c r="A51" s="4" t="s">
         <v>603</v>
       </c>
@@ -7396,7 +7454,7 @@
         <v>20000000</v>
       </c>
     </row>
-    <row r="52" spans="1:9" x14ac:dyDescent="0.25">
+    <row r="52" spans="1:9" x14ac:dyDescent="0.35">
       <c r="A52" s="17" t="s">
         <v>595</v>
       </c>
@@ -7428,7 +7486,7 @@
         <v>25000000</v>
       </c>
     </row>
-    <row r="53" spans="1:9" x14ac:dyDescent="0.25">
+    <row r="53" spans="1:9" x14ac:dyDescent="0.35">
       <c r="A53" s="4" t="s">
         <v>606</v>
       </c>
@@ -7460,7 +7518,7 @@
         <v>25000000</v>
       </c>
     </row>
-    <row r="54" spans="1:9" x14ac:dyDescent="0.25">
+    <row r="54" spans="1:9" x14ac:dyDescent="0.35">
       <c r="A54" s="17" t="s">
         <v>594</v>
       </c>
@@ -7492,7 +7550,7 @@
         <v>20000000</v>
       </c>
     </row>
-    <row r="55" spans="1:9" x14ac:dyDescent="0.25">
+    <row r="55" spans="1:9" x14ac:dyDescent="0.35">
       <c r="A55" s="16" t="s">
         <v>605</v>
       </c>
@@ -7524,7 +7582,7 @@
         <v>20000000</v>
       </c>
     </row>
-    <row r="56" spans="1:9" x14ac:dyDescent="0.25">
+    <row r="56" spans="1:9" x14ac:dyDescent="0.35">
       <c r="A56" s="16" t="s">
         <v>596</v>
       </c>
@@ -7556,7 +7614,7 @@
         <v>25000000</v>
       </c>
     </row>
-    <row r="57" spans="1:9" x14ac:dyDescent="0.25">
+    <row r="57" spans="1:9" x14ac:dyDescent="0.35">
       <c r="A57" s="4" t="s">
         <v>604</v>
       </c>
@@ -7588,7 +7646,7 @@
         <v>25000000</v>
       </c>
     </row>
-    <row r="58" spans="1:9" x14ac:dyDescent="0.25">
+    <row r="58" spans="1:9" x14ac:dyDescent="0.35">
       <c r="A58" s="16" t="s">
         <v>619</v>
       </c>
@@ -7620,7 +7678,7 @@
         <v>25000000</v>
       </c>
     </row>
-    <row r="59" spans="1:9" x14ac:dyDescent="0.25">
+    <row r="59" spans="1:9" x14ac:dyDescent="0.35">
       <c r="A59" s="16" t="s">
         <v>620</v>
       </c>
@@ -7652,7 +7710,7 @@
         <v>35000000</v>
       </c>
     </row>
-    <row r="60" spans="1:9" x14ac:dyDescent="0.25">
+    <row r="60" spans="1:9" x14ac:dyDescent="0.35">
       <c r="A60" s="16" t="s">
         <v>621</v>
       </c>
@@ -7684,7 +7742,7 @@
         <v>25000000</v>
       </c>
     </row>
-    <row r="61" spans="1:9" x14ac:dyDescent="0.25">
+    <row r="61" spans="1:9" x14ac:dyDescent="0.35">
       <c r="A61" s="16" t="s">
         <v>622</v>
       </c>
@@ -7716,7 +7774,7 @@
         <v>35000000</v>
       </c>
     </row>
-    <row r="62" spans="1:9" x14ac:dyDescent="0.25">
+    <row r="62" spans="1:9" x14ac:dyDescent="0.35">
       <c r="A62" s="16" t="s">
         <v>628</v>
       </c>
@@ -7748,7 +7806,7 @@
         <v>25000000</v>
       </c>
     </row>
-    <row r="63" spans="1:9" x14ac:dyDescent="0.25">
+    <row r="63" spans="1:9" x14ac:dyDescent="0.35">
       <c r="A63" s="16" t="s">
         <v>627</v>
       </c>
@@ -7780,7 +7838,7 @@
         <v>35000000</v>
       </c>
     </row>
-    <row r="64" spans="1:9" x14ac:dyDescent="0.25">
+    <row r="64" spans="1:9" x14ac:dyDescent="0.35">
       <c r="A64" s="16" t="s">
         <v>630</v>
       </c>
@@ -7812,7 +7870,7 @@
         <v>25000000</v>
       </c>
     </row>
-    <row r="65" spans="1:9" x14ac:dyDescent="0.25">
+    <row r="65" spans="1:9" x14ac:dyDescent="0.35">
       <c r="A65" s="16" t="s">
         <v>629</v>
       </c>
@@ -7844,7 +7902,7 @@
         <v>35000000</v>
       </c>
     </row>
-    <row r="66" spans="1:9" x14ac:dyDescent="0.25">
+    <row r="66" spans="1:9" x14ac:dyDescent="0.35">
       <c r="A66" s="16" t="s">
         <v>631</v>
       </c>
@@ -7876,7 +7934,7 @@
         <v>23000000</v>
       </c>
     </row>
-    <row r="67" spans="1:9" x14ac:dyDescent="0.25">
+    <row r="67" spans="1:9" x14ac:dyDescent="0.35">
       <c r="A67" s="16" t="s">
         <v>632</v>
       </c>
@@ -7908,7 +7966,7 @@
         <v>13000000</v>
       </c>
     </row>
-    <row r="68" spans="1:9" x14ac:dyDescent="0.25">
+    <row r="68" spans="1:9" x14ac:dyDescent="0.35">
       <c r="A68" s="16" t="s">
         <v>633</v>
       </c>
@@ -7940,7 +7998,7 @@
         <v>20000000</v>
       </c>
     </row>
-    <row r="69" spans="1:9" x14ac:dyDescent="0.25">
+    <row r="69" spans="1:9" x14ac:dyDescent="0.35">
       <c r="A69" s="16" t="s">
         <v>634</v>
       </c>
@@ -7951,15 +8009,15 @@
         <v>155000000</v>
       </c>
       <c r="D69" s="5">
-        <f t="shared" ref="D69:D70" si="19">I69/1.12</f>
+        <f t="shared" ref="D69:D71" si="19">I69/1.12</f>
         <v>5357142.8571428563</v>
       </c>
       <c r="E69" s="5">
-        <f t="shared" ref="E69:E70" si="20">D69*90%</f>
+        <f t="shared" ref="E69:E71" si="20">D69*90%</f>
         <v>4821428.5714285709</v>
       </c>
       <c r="F69" s="5">
-        <f t="shared" ref="F69:F70" si="21">D69*70%</f>
+        <f t="shared" ref="F69:F71" si="21">D69*70%</f>
         <v>3749999.9999999991</v>
       </c>
       <c r="G69" s="3">
@@ -7972,7 +8030,7 @@
         <v>6000000</v>
       </c>
     </row>
-    <row r="70" spans="1:9" x14ac:dyDescent="0.25">
+    <row r="70" spans="1:9" x14ac:dyDescent="0.35">
       <c r="A70" s="16" t="s">
         <v>635</v>
       </c>
@@ -8004,24 +8062,316 @@
         <v>6000000</v>
       </c>
     </row>
+    <row r="71" spans="1:9" x14ac:dyDescent="0.35">
+      <c r="A71" s="16" t="s">
+        <v>641</v>
+      </c>
+      <c r="B71" s="4" t="s">
+        <v>597</v>
+      </c>
+      <c r="C71" s="9">
+        <v>389000000</v>
+      </c>
+      <c r="D71" s="9">
+        <f t="shared" si="19"/>
+        <v>27499999.999999996</v>
+      </c>
+      <c r="E71" s="9">
+        <f t="shared" si="20"/>
+        <v>24749999.999999996</v>
+      </c>
+      <c r="F71" s="9">
+        <f t="shared" si="21"/>
+        <v>19249999.999999996</v>
+      </c>
+      <c r="G71" s="20">
+        <v>271</v>
+      </c>
+      <c r="H71" s="4" t="s">
+        <v>597</v>
+      </c>
+      <c r="I71" s="12">
+        <v>30800000</v>
+      </c>
+    </row>
+    <row r="72" spans="1:9" x14ac:dyDescent="0.35">
+      <c r="A72" s="16" t="s">
+        <v>640</v>
+      </c>
+      <c r="B72" s="4" t="s">
+        <v>597</v>
+      </c>
+      <c r="C72" s="9">
+        <v>399000000</v>
+      </c>
+      <c r="D72" s="9">
+        <f t="shared" ref="D72:D75" si="22">I72/1.12</f>
+        <v>28214285.714285713</v>
+      </c>
+      <c r="E72" s="9">
+        <f t="shared" ref="E72:E75" si="23">D72*90%</f>
+        <v>25392857.142857142</v>
+      </c>
+      <c r="F72" s="9">
+        <f t="shared" ref="F72:F75" si="24">D72*70%</f>
+        <v>19749999.999999996</v>
+      </c>
+      <c r="G72" s="20">
+        <v>258</v>
+      </c>
+      <c r="H72" s="4" t="s">
+        <v>597</v>
+      </c>
+      <c r="I72" s="12">
+        <v>31600000</v>
+      </c>
+    </row>
+    <row r="73" spans="1:9" x14ac:dyDescent="0.35">
+      <c r="A73" s="16" t="s">
+        <v>642</v>
+      </c>
+      <c r="B73" s="4" t="s">
+        <v>598</v>
+      </c>
+      <c r="C73" s="9">
+        <v>459000000</v>
+      </c>
+      <c r="D73" s="9">
+        <f t="shared" si="22"/>
+        <v>32499999.999999996</v>
+      </c>
+      <c r="E73" s="9">
+        <f t="shared" si="23"/>
+        <v>29249999.999999996</v>
+      </c>
+      <c r="F73" s="9">
+        <f t="shared" si="24"/>
+        <v>22749999.999999996</v>
+      </c>
+      <c r="G73" s="20">
+        <v>259</v>
+      </c>
+      <c r="H73" s="4" t="s">
+        <v>598</v>
+      </c>
+      <c r="I73" s="12">
+        <v>36400000</v>
+      </c>
+    </row>
+    <row r="74" spans="1:9" x14ac:dyDescent="0.35">
+      <c r="A74" s="16" t="s">
+        <v>644</v>
+      </c>
+      <c r="B74" s="4" t="s">
+        <v>600</v>
+      </c>
+      <c r="C74" s="9">
+        <v>449000000</v>
+      </c>
+      <c r="D74" s="9">
+        <f t="shared" si="22"/>
+        <v>29196428.571428567</v>
+      </c>
+      <c r="E74" s="9">
+        <f t="shared" si="23"/>
+        <v>26276785.714285713</v>
+      </c>
+      <c r="F74" s="9">
+        <f t="shared" si="24"/>
+        <v>20437499.999999996</v>
+      </c>
+      <c r="G74" s="20">
+        <v>260</v>
+      </c>
+      <c r="H74" s="10" t="s">
+        <v>600</v>
+      </c>
+      <c r="I74" s="12">
+        <v>32700000</v>
+      </c>
+    </row>
+    <row r="75" spans="1:9" x14ac:dyDescent="0.35">
+      <c r="A75" s="16" t="s">
+        <v>643</v>
+      </c>
+      <c r="B75" s="4" t="s">
+        <v>601</v>
+      </c>
+      <c r="C75" s="9">
+        <v>499000000</v>
+      </c>
+      <c r="D75" s="9">
+        <f t="shared" si="22"/>
+        <v>32499999.999999996</v>
+      </c>
+      <c r="E75" s="9">
+        <f t="shared" si="23"/>
+        <v>29249999.999999996</v>
+      </c>
+      <c r="F75" s="9">
+        <f t="shared" si="24"/>
+        <v>22749999.999999996</v>
+      </c>
+      <c r="G75" s="20">
+        <v>261</v>
+      </c>
+      <c r="H75" s="10" t="s">
+        <v>601</v>
+      </c>
+      <c r="I75" s="12">
+        <v>36400000</v>
+      </c>
+    </row>
+    <row r="76" spans="1:9" x14ac:dyDescent="0.35">
+      <c r="A76" s="25" t="s">
+        <v>645</v>
+      </c>
+      <c r="B76" s="4" t="s">
+        <v>583</v>
+      </c>
+      <c r="C76" s="9">
+        <v>289000000</v>
+      </c>
+      <c r="D76" s="9">
+        <f t="shared" ref="D76:D77" si="25">I76/1.12</f>
+        <v>13392857.142857142</v>
+      </c>
+      <c r="E76" s="9">
+        <f t="shared" ref="E76:E77" si="26">D76*90%</f>
+        <v>12053571.428571427</v>
+      </c>
+      <c r="F76" s="9">
+        <f t="shared" ref="F76:F77" si="27">D76*70%</f>
+        <v>9374999.9999999981</v>
+      </c>
+      <c r="G76" s="20">
+        <v>272</v>
+      </c>
+      <c r="H76" s="4" t="s">
+        <v>576</v>
+      </c>
+      <c r="I76" s="26">
+        <v>15000000</v>
+      </c>
+    </row>
+    <row r="77" spans="1:9" x14ac:dyDescent="0.35">
+      <c r="A77" s="25" t="s">
+        <v>646</v>
+      </c>
+      <c r="B77" s="4" t="s">
+        <v>584</v>
+      </c>
+      <c r="C77" s="18">
+        <v>319000000</v>
+      </c>
+      <c r="D77" s="9">
+        <f t="shared" si="25"/>
+        <v>13392857.142857142</v>
+      </c>
+      <c r="E77" s="9">
+        <f t="shared" si="26"/>
+        <v>12053571.428571427</v>
+      </c>
+      <c r="F77" s="9">
+        <f t="shared" si="27"/>
+        <v>9374999.9999999981</v>
+      </c>
+      <c r="G77" s="20">
+        <v>273</v>
+      </c>
+      <c r="H77" s="4" t="s">
+        <v>577</v>
+      </c>
+      <c r="I77" s="26">
+        <v>15000000</v>
+      </c>
+    </row>
+    <row r="78" spans="1:9" x14ac:dyDescent="0.35">
+      <c r="A78" s="27" t="s">
+        <v>647</v>
+      </c>
+      <c r="B78" s="28" t="s">
+        <v>649</v>
+      </c>
+      <c r="C78" s="18">
+        <v>299000000</v>
+      </c>
+      <c r="D78" s="9">
+        <f t="shared" ref="D78:D79" si="28">I78/1.12</f>
+        <v>17857142.857142854</v>
+      </c>
+      <c r="E78" s="9">
+        <f t="shared" ref="E78:E79" si="29">D78*90%</f>
+        <v>16071428.571428569</v>
+      </c>
+      <c r="F78" s="9">
+        <f t="shared" ref="F78:F79" si="30">D78*70%</f>
+        <v>12499999.999999998</v>
+      </c>
+      <c r="G78" s="20">
+        <v>274</v>
+      </c>
+      <c r="H78" s="4" t="s">
+        <v>581</v>
+      </c>
+      <c r="I78" s="29">
+        <v>20000000</v>
+      </c>
+    </row>
+    <row r="79" spans="1:9" x14ac:dyDescent="0.35">
+      <c r="A79" s="27" t="s">
+        <v>648</v>
+      </c>
+      <c r="B79" s="28" t="s">
+        <v>650</v>
+      </c>
+      <c r="C79" s="18">
+        <v>339000000</v>
+      </c>
+      <c r="D79" s="9">
+        <f t="shared" si="28"/>
+        <v>22321428.571428571</v>
+      </c>
+      <c r="E79" s="9">
+        <f t="shared" si="29"/>
+        <v>20089285.714285713</v>
+      </c>
+      <c r="F79" s="9">
+        <f t="shared" si="30"/>
+        <v>15624999.999999998</v>
+      </c>
+      <c r="G79" s="20">
+        <v>275</v>
+      </c>
+      <c r="H79" s="4" t="s">
+        <v>571</v>
+      </c>
+      <c r="I79" s="29">
+        <v>25000000</v>
+      </c>
+    </row>
   </sheetData>
   <phoneticPr fontId="4" type="noConversion"/>
   <conditionalFormatting sqref="A1:A1048576">
-    <cfRule type="duplicateValues" dxfId="8" priority="2"/>
+    <cfRule type="duplicateValues" dxfId="10" priority="4"/>
   </conditionalFormatting>
   <conditionalFormatting sqref="A33:A41 A43:A46 A2:A31">
-    <cfRule type="duplicateValues" dxfId="7" priority="14"/>
+    <cfRule type="duplicateValues" dxfId="9" priority="16"/>
   </conditionalFormatting>
   <conditionalFormatting sqref="A33:A46 A2:A31">
-    <cfRule type="duplicateValues" dxfId="6" priority="18"/>
+    <cfRule type="duplicateValues" dxfId="8" priority="20"/>
   </conditionalFormatting>
   <conditionalFormatting sqref="H43:H46">
-    <cfRule type="duplicateValues" dxfId="5" priority="7"/>
-    <cfRule type="duplicateValues" dxfId="4" priority="8"/>
+    <cfRule type="duplicateValues" dxfId="7" priority="9"/>
+    <cfRule type="duplicateValues" dxfId="6" priority="10"/>
   </conditionalFormatting>
   <conditionalFormatting sqref="H51:H54">
-    <cfRule type="duplicateValues" dxfId="3" priority="3"/>
-    <cfRule type="duplicateValues" dxfId="2" priority="4"/>
+    <cfRule type="duplicateValues" dxfId="5" priority="5"/>
+    <cfRule type="duplicateValues" dxfId="4" priority="6"/>
+  </conditionalFormatting>
+  <conditionalFormatting sqref="H74:H75">
+    <cfRule type="duplicateValues" dxfId="3" priority="1"/>
+    <cfRule type="duplicateValues" dxfId="2" priority="2"/>
   </conditionalFormatting>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <pageSetup paperSize="9" orientation="portrait" horizontalDpi="0" verticalDpi="0" r:id="rId1"/>
@@ -8034,16 +8384,16 @@
 <file path=xl/worksheets/sheet10.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{7F6E2486-F456-4872-8871-82688E1562A6}">
   <dimension ref="A1:F20"/>
-  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
+  <sheetFormatPr defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
   <cols>
-    <col min="1" max="1" width="12.5703125" bestFit="1" customWidth="1"/>
-    <col min="2" max="2" width="16.42578125" bestFit="1" customWidth="1"/>
-    <col min="3" max="3" width="31.85546875" bestFit="1" customWidth="1"/>
+    <col min="1" max="1" width="12.54296875" bestFit="1" customWidth="1"/>
+    <col min="2" max="2" width="16.453125" bestFit="1" customWidth="1"/>
+    <col min="3" max="3" width="31.81640625" bestFit="1" customWidth="1"/>
     <col min="4" max="5" width="32" bestFit="1" customWidth="1"/>
-    <col min="6" max="6" width="31.140625" bestFit="1" customWidth="1"/>
+    <col min="6" max="6" width="31.1796875" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="1" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A1" t="s">
         <v>0</v>
       </c>
@@ -8063,12 +8413,12 @@
         <v>5</v>
       </c>
     </row>
-    <row r="2" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="2" spans="1:6" x14ac:dyDescent="0.35">
       <c r="C2" t="s">
         <v>82</v>
       </c>
     </row>
-    <row r="3" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="3" spans="1:6" x14ac:dyDescent="0.35">
       <c r="B3" t="s">
         <v>8</v>
       </c>
@@ -8085,7 +8435,7 @@
         <v>389</v>
       </c>
     </row>
-    <row r="4" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="4" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A4" t="s">
         <v>14</v>
       </c>
@@ -8105,7 +8455,7 @@
         <v>393</v>
       </c>
     </row>
-    <row r="5" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="5" spans="1:6" x14ac:dyDescent="0.35">
       <c r="B5" t="s">
         <v>152</v>
       </c>
@@ -8122,7 +8472,7 @@
         <v>397</v>
       </c>
     </row>
-    <row r="6" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="6" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A6" t="s">
         <v>27</v>
       </c>
@@ -8142,7 +8492,7 @@
         <v>401</v>
       </c>
     </row>
-    <row r="7" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="7" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A7" t="s">
         <v>34</v>
       </c>
@@ -8162,7 +8512,7 @@
         <v>405</v>
       </c>
     </row>
-    <row r="8" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="8" spans="1:6" x14ac:dyDescent="0.35">
       <c r="B8" t="s">
         <v>41</v>
       </c>
@@ -8179,7 +8529,7 @@
         <v>409</v>
       </c>
     </row>
-    <row r="9" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="9" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A9" t="s">
         <v>47</v>
       </c>
@@ -8199,7 +8549,7 @@
         <v>413</v>
       </c>
     </row>
-    <row r="10" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="10" spans="1:6" x14ac:dyDescent="0.35">
       <c r="B10" t="s">
         <v>123</v>
       </c>
@@ -8216,7 +8566,7 @@
         <v>409</v>
       </c>
     </row>
-    <row r="11" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="11" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A11" t="s">
         <v>321</v>
       </c>
@@ -8236,7 +8586,7 @@
         <v>450000000</v>
       </c>
     </row>
-    <row r="12" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="12" spans="1:6" x14ac:dyDescent="0.35">
       <c r="B12" t="s">
         <v>61</v>
       </c>
@@ -8253,7 +8603,7 @@
         <v>451000000</v>
       </c>
     </row>
-    <row r="13" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="13" spans="1:6" x14ac:dyDescent="0.35">
       <c r="B13" t="s">
         <v>62</v>
       </c>
@@ -8270,7 +8620,7 @@
         <v>450000000</v>
       </c>
     </row>
-    <row r="14" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="14" spans="1:6" x14ac:dyDescent="0.35">
       <c r="B14" t="s">
         <v>63</v>
       </c>
@@ -8287,7 +8637,7 @@
         <v>448800000</v>
       </c>
     </row>
-    <row r="15" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="15" spans="1:6" x14ac:dyDescent="0.35">
       <c r="B15" t="s">
         <v>64</v>
       </c>
@@ -8304,7 +8654,7 @@
         <v>448800000</v>
       </c>
     </row>
-    <row r="16" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="16" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A16" t="s">
         <v>65</v>
       </c>
@@ -8324,7 +8674,7 @@
         <v>466900000</v>
       </c>
     </row>
-    <row r="18" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="18" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A18" t="s">
         <v>0</v>
       </c>
@@ -8344,7 +8694,7 @@
         <v>5</v>
       </c>
     </row>
-    <row r="19" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="19" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A19" t="s">
         <v>135</v>
       </c>
@@ -8364,7 +8714,7 @@
         <v>423</v>
       </c>
     </row>
-    <row r="20" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="20" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A20" t="s">
         <v>76</v>
       </c>
@@ -8393,15 +8743,15 @@
 <file path=xl/worksheets/sheet11.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{F98971A8-4205-45A8-A1C1-D9D164D2942F}">
   <dimension ref="A1:E19"/>
-  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
+  <sheetFormatPr defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
   <cols>
-    <col min="1" max="1" width="12.5703125" bestFit="1" customWidth="1"/>
-    <col min="2" max="2" width="16.42578125" bestFit="1" customWidth="1"/>
-    <col min="3" max="3" width="15.7109375" bestFit="1" customWidth="1"/>
-    <col min="4" max="5" width="15.140625" bestFit="1" customWidth="1"/>
+    <col min="1" max="1" width="12.54296875" bestFit="1" customWidth="1"/>
+    <col min="2" max="2" width="16.453125" bestFit="1" customWidth="1"/>
+    <col min="3" max="3" width="15.7265625" bestFit="1" customWidth="1"/>
+    <col min="4" max="5" width="15.1796875" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="1" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A1" t="s">
         <v>0</v>
       </c>
@@ -8418,7 +8768,7 @@
         <v>4</v>
       </c>
     </row>
-    <row r="2" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="2" spans="1:5" x14ac:dyDescent="0.35">
       <c r="B2" t="s">
         <v>8</v>
       </c>
@@ -8426,7 +8776,7 @@
         <v>424</v>
       </c>
     </row>
-    <row r="3" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="3" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A3" t="s">
         <v>14</v>
       </c>
@@ -8443,7 +8793,7 @@
         <v>427</v>
       </c>
     </row>
-    <row r="4" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="4" spans="1:5" x14ac:dyDescent="0.35">
       <c r="B4" t="s">
         <v>152</v>
       </c>
@@ -8457,7 +8807,7 @@
         <v>430</v>
       </c>
     </row>
-    <row r="5" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="5" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A5" t="s">
         <v>27</v>
       </c>
@@ -8474,7 +8824,7 @@
         <v>433</v>
       </c>
     </row>
-    <row r="6" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="6" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A6" t="s">
         <v>34</v>
       </c>
@@ -8491,7 +8841,7 @@
         <v>436</v>
       </c>
     </row>
-    <row r="7" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="7" spans="1:5" x14ac:dyDescent="0.35">
       <c r="B7" t="s">
         <v>41</v>
       </c>
@@ -8505,7 +8855,7 @@
         <v>438</v>
       </c>
     </row>
-    <row r="8" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="8" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A8" t="s">
         <v>115</v>
       </c>
@@ -8522,7 +8872,7 @@
         <v>441</v>
       </c>
     </row>
-    <row r="9" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="9" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A9" t="s">
         <v>122</v>
       </c>
@@ -8539,7 +8889,7 @@
         <v>438</v>
       </c>
     </row>
-    <row r="10" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="10" spans="1:5" x14ac:dyDescent="0.35">
       <c r="B10" t="s">
         <v>56</v>
       </c>
@@ -8553,7 +8903,7 @@
         <v>444</v>
       </c>
     </row>
-    <row r="11" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="11" spans="1:5" x14ac:dyDescent="0.35">
       <c r="B11" t="s">
         <v>61</v>
       </c>
@@ -8567,7 +8917,7 @@
         <v>444</v>
       </c>
     </row>
-    <row r="12" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="12" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A12" t="s">
         <v>55</v>
       </c>
@@ -8584,7 +8934,7 @@
         <v>444</v>
       </c>
     </row>
-    <row r="13" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="13" spans="1:5" x14ac:dyDescent="0.35">
       <c r="B13" t="s">
         <v>63</v>
       </c>
@@ -8598,7 +8948,7 @@
         <v>444</v>
       </c>
     </row>
-    <row r="14" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="14" spans="1:5" x14ac:dyDescent="0.35">
       <c r="B14" t="s">
         <v>64</v>
       </c>
@@ -8612,7 +8962,7 @@
         <v>444</v>
       </c>
     </row>
-    <row r="15" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="15" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A15" t="s">
         <v>65</v>
       </c>
@@ -8629,7 +8979,7 @@
         <v>447</v>
       </c>
     </row>
-    <row r="17" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="17" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A17" t="s">
         <v>0</v>
       </c>
@@ -8646,7 +8996,7 @@
         <v>4</v>
       </c>
     </row>
-    <row r="18" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="18" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A18" t="s">
         <v>135</v>
       </c>
@@ -8663,7 +9013,7 @@
         <v>450</v>
       </c>
     </row>
-    <row r="19" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="19" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A19" t="s">
         <v>76</v>
       </c>
@@ -8689,15 +9039,15 @@
 <file path=xl/worksheets/sheet12.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{516E8F5E-7978-4DDA-9413-77E8ECD441FC}">
   <dimension ref="A1:E20"/>
-  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
+  <sheetFormatPr defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
   <cols>
-    <col min="1" max="1" width="12.5703125" bestFit="1" customWidth="1"/>
-    <col min="2" max="2" width="16.42578125" bestFit="1" customWidth="1"/>
-    <col min="3" max="3" width="31.140625" bestFit="1" customWidth="1"/>
-    <col min="4" max="5" width="32.140625" bestFit="1" customWidth="1"/>
+    <col min="1" max="1" width="12.54296875" bestFit="1" customWidth="1"/>
+    <col min="2" max="2" width="16.453125" bestFit="1" customWidth="1"/>
+    <col min="3" max="3" width="31.1796875" bestFit="1" customWidth="1"/>
+    <col min="4" max="5" width="32.1796875" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="1" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A1" t="s">
         <v>0</v>
       </c>
@@ -8714,12 +9064,12 @@
         <v>4</v>
       </c>
     </row>
-    <row r="2" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="2" spans="1:5" x14ac:dyDescent="0.35">
       <c r="C2" t="s">
         <v>82</v>
       </c>
     </row>
-    <row r="3" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="3" spans="1:5" x14ac:dyDescent="0.35">
       <c r="B3" t="s">
         <v>8</v>
       </c>
@@ -8733,7 +9083,7 @@
         <v>455</v>
       </c>
     </row>
-    <row r="4" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="4" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A4" t="s">
         <v>14</v>
       </c>
@@ -8750,7 +9100,7 @@
         <v>458</v>
       </c>
     </row>
-    <row r="5" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="5" spans="1:5" x14ac:dyDescent="0.35">
       <c r="B5" t="s">
         <v>152</v>
       </c>
@@ -8764,7 +9114,7 @@
         <v>461</v>
       </c>
     </row>
-    <row r="6" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="6" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A6" t="s">
         <v>27</v>
       </c>
@@ -8781,7 +9131,7 @@
         <v>464</v>
       </c>
     </row>
-    <row r="7" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="7" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A7" t="s">
         <v>465</v>
       </c>
@@ -8798,7 +9148,7 @@
         <v>468</v>
       </c>
     </row>
-    <row r="8" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="8" spans="1:5" x14ac:dyDescent="0.35">
       <c r="B8" t="s">
         <v>41</v>
       </c>
@@ -8812,7 +9162,7 @@
         <v>471</v>
       </c>
     </row>
-    <row r="9" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="9" spans="1:5" x14ac:dyDescent="0.35">
       <c r="B9" t="s">
         <v>48</v>
       </c>
@@ -8826,7 +9176,7 @@
         <v>468</v>
       </c>
     </row>
-    <row r="10" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="10" spans="1:5" x14ac:dyDescent="0.35">
       <c r="B10" t="s">
         <v>54</v>
       </c>
@@ -8840,7 +9190,7 @@
         <v>471</v>
       </c>
     </row>
-    <row r="11" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="11" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A11" t="s">
         <v>472</v>
       </c>
@@ -8857,7 +9207,7 @@
         <v>475</v>
       </c>
     </row>
-    <row r="12" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="12" spans="1:5" x14ac:dyDescent="0.35">
       <c r="B12" t="s">
         <v>61</v>
       </c>
@@ -8871,7 +9221,7 @@
         <v>475</v>
       </c>
     </row>
-    <row r="13" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="13" spans="1:5" x14ac:dyDescent="0.35">
       <c r="B13" t="s">
         <v>62</v>
       </c>
@@ -8885,7 +9235,7 @@
         <v>475</v>
       </c>
     </row>
-    <row r="14" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="14" spans="1:5" x14ac:dyDescent="0.35">
       <c r="B14" t="s">
         <v>63</v>
       </c>
@@ -8899,7 +9249,7 @@
         <v>475</v>
       </c>
     </row>
-    <row r="15" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="15" spans="1:5" x14ac:dyDescent="0.35">
       <c r="B15" t="s">
         <v>64</v>
       </c>
@@ -8913,7 +9263,7 @@
         <v>475</v>
       </c>
     </row>
-    <row r="16" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="16" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A16" t="s">
         <v>65</v>
       </c>
@@ -8930,7 +9280,7 @@
         <v>478</v>
       </c>
     </row>
-    <row r="18" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="18" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A18" t="s">
         <v>0</v>
       </c>
@@ -8947,7 +9297,7 @@
         <v>4</v>
       </c>
     </row>
-    <row r="19" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="19" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A19" t="s">
         <v>135</v>
       </c>
@@ -8964,7 +9314,7 @@
         <v>481</v>
       </c>
     </row>
-    <row r="20" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="20" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A20" t="s">
         <v>76</v>
       </c>
@@ -8990,18 +9340,18 @@
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{669692EE-8762-4650-B2E9-8C0B02D25245}">
   <dimension ref="A1:H34"/>
-  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
+  <sheetFormatPr defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
   <cols>
-    <col min="1" max="1" width="51.42578125" bestFit="1" customWidth="1"/>
-    <col min="2" max="2" width="36.5703125" bestFit="1" customWidth="1"/>
-    <col min="3" max="3" width="14.5703125" bestFit="1" customWidth="1"/>
-    <col min="4" max="4" width="12.5703125" bestFit="1" customWidth="1"/>
-    <col min="5" max="6" width="16.140625" bestFit="1" customWidth="1"/>
+    <col min="1" max="1" width="51.453125" bestFit="1" customWidth="1"/>
+    <col min="2" max="2" width="36.54296875" bestFit="1" customWidth="1"/>
+    <col min="3" max="3" width="14.54296875" bestFit="1" customWidth="1"/>
+    <col min="4" max="4" width="12.54296875" bestFit="1" customWidth="1"/>
+    <col min="5" max="6" width="16.1796875" bestFit="1" customWidth="1"/>
     <col min="7" max="7" width="9" bestFit="1" customWidth="1"/>
-    <col min="8" max="8" width="14.42578125" bestFit="1" customWidth="1"/>
+    <col min="8" max="8" width="14.453125" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:8" x14ac:dyDescent="0.25">
+    <row r="1" spans="1:8" x14ac:dyDescent="0.35">
       <c r="A1" s="4" t="s">
         <v>551</v>
       </c>
@@ -9027,7 +9377,7 @@
         <v>564</v>
       </c>
     </row>
-    <row r="2" spans="1:8" x14ac:dyDescent="0.25">
+    <row r="2" spans="1:8" x14ac:dyDescent="0.35">
       <c r="A2" s="4" t="s">
         <v>514</v>
       </c>
@@ -9057,7 +9407,7 @@
         <v>565</v>
       </c>
     </row>
-    <row r="3" spans="1:8" x14ac:dyDescent="0.25">
+    <row r="3" spans="1:8" x14ac:dyDescent="0.35">
       <c r="A3" s="4" t="s">
         <v>547</v>
       </c>
@@ -9087,7 +9437,7 @@
         <v>565</v>
       </c>
     </row>
-    <row r="4" spans="1:8" x14ac:dyDescent="0.25">
+    <row r="4" spans="1:8" x14ac:dyDescent="0.35">
       <c r="A4" s="4" t="s">
         <v>515</v>
       </c>
@@ -9117,7 +9467,7 @@
         <v>565</v>
       </c>
     </row>
-    <row r="5" spans="1:8" x14ac:dyDescent="0.25">
+    <row r="5" spans="1:8" x14ac:dyDescent="0.35">
       <c r="A5" s="4" t="s">
         <v>516</v>
       </c>
@@ -9147,7 +9497,7 @@
         <v>565</v>
       </c>
     </row>
-    <row r="6" spans="1:8" x14ac:dyDescent="0.25">
+    <row r="6" spans="1:8" x14ac:dyDescent="0.35">
       <c r="A6" s="4" t="s">
         <v>496</v>
       </c>
@@ -9177,7 +9527,7 @@
         <v>565</v>
       </c>
     </row>
-    <row r="7" spans="1:8" x14ac:dyDescent="0.25">
+    <row r="7" spans="1:8" x14ac:dyDescent="0.35">
       <c r="A7" s="4" t="s">
         <v>497</v>
       </c>
@@ -9207,7 +9557,7 @@
         <v>565</v>
       </c>
     </row>
-    <row r="8" spans="1:8" x14ac:dyDescent="0.25">
+    <row r="8" spans="1:8" x14ac:dyDescent="0.35">
       <c r="A8" s="4" t="s">
         <v>517</v>
       </c>
@@ -9237,7 +9587,7 @@
         <v>566</v>
       </c>
     </row>
-    <row r="9" spans="1:8" x14ac:dyDescent="0.25">
+    <row r="9" spans="1:8" x14ac:dyDescent="0.35">
       <c r="A9" s="4" t="s">
         <v>518</v>
       </c>
@@ -9267,7 +9617,7 @@
         <v>566</v>
       </c>
     </row>
-    <row r="10" spans="1:8" x14ac:dyDescent="0.25">
+    <row r="10" spans="1:8" x14ac:dyDescent="0.35">
       <c r="A10" s="4" t="s">
         <v>519</v>
       </c>
@@ -9297,7 +9647,7 @@
         <v>566</v>
       </c>
     </row>
-    <row r="11" spans="1:8" x14ac:dyDescent="0.25">
+    <row r="11" spans="1:8" x14ac:dyDescent="0.35">
       <c r="A11" s="4" t="s">
         <v>523</v>
       </c>
@@ -9327,7 +9677,7 @@
         <v>568</v>
       </c>
     </row>
-    <row r="12" spans="1:8" x14ac:dyDescent="0.25">
+    <row r="12" spans="1:8" x14ac:dyDescent="0.35">
       <c r="A12" s="4" t="s">
         <v>524</v>
       </c>
@@ -9357,7 +9707,7 @@
         <v>573</v>
       </c>
     </row>
-    <row r="13" spans="1:8" x14ac:dyDescent="0.25">
+    <row r="13" spans="1:8" x14ac:dyDescent="0.35">
       <c r="A13" s="4" t="s">
         <v>498</v>
       </c>
@@ -9387,7 +9737,7 @@
         <v>573</v>
       </c>
     </row>
-    <row r="14" spans="1:8" x14ac:dyDescent="0.25">
+    <row r="14" spans="1:8" x14ac:dyDescent="0.35">
       <c r="A14" s="4" t="s">
         <v>527</v>
       </c>
@@ -9417,7 +9767,7 @@
         <v>567</v>
       </c>
     </row>
-    <row r="15" spans="1:8" x14ac:dyDescent="0.25">
+    <row r="15" spans="1:8" x14ac:dyDescent="0.35">
       <c r="A15" s="4" t="s">
         <v>528</v>
       </c>
@@ -9447,7 +9797,7 @@
         <v>567</v>
       </c>
     </row>
-    <row r="16" spans="1:8" x14ac:dyDescent="0.25">
+    <row r="16" spans="1:8" x14ac:dyDescent="0.35">
       <c r="A16" s="4" t="s">
         <v>525</v>
       </c>
@@ -9477,7 +9827,7 @@
         <v>567</v>
       </c>
     </row>
-    <row r="17" spans="1:8" x14ac:dyDescent="0.25">
+    <row r="17" spans="1:8" x14ac:dyDescent="0.35">
       <c r="A17" s="4" t="s">
         <v>499</v>
       </c>
@@ -9507,7 +9857,7 @@
         <v>567</v>
       </c>
     </row>
-    <row r="18" spans="1:8" x14ac:dyDescent="0.25">
+    <row r="18" spans="1:8" x14ac:dyDescent="0.35">
       <c r="A18" s="4" t="s">
         <v>555</v>
       </c>
@@ -9537,7 +9887,7 @@
         <v>574</v>
       </c>
     </row>
-    <row r="19" spans="1:8" x14ac:dyDescent="0.25">
+    <row r="19" spans="1:8" x14ac:dyDescent="0.35">
       <c r="A19" s="4" t="s">
         <v>500</v>
       </c>
@@ -9567,7 +9917,7 @@
         <v>569</v>
       </c>
     </row>
-    <row r="20" spans="1:8" x14ac:dyDescent="0.25">
+    <row r="20" spans="1:8" x14ac:dyDescent="0.35">
       <c r="A20" s="4" t="s">
         <v>501</v>
       </c>
@@ -9597,7 +9947,7 @@
         <v>575</v>
       </c>
     </row>
-    <row r="21" spans="1:8" x14ac:dyDescent="0.25">
+    <row r="21" spans="1:8" x14ac:dyDescent="0.35">
       <c r="A21" s="4" t="s">
         <v>502</v>
       </c>
@@ -9627,7 +9977,7 @@
         <v>570</v>
       </c>
     </row>
-    <row r="22" spans="1:8" x14ac:dyDescent="0.25">
+    <row r="22" spans="1:8" x14ac:dyDescent="0.35">
       <c r="A22" s="4" t="s">
         <v>503</v>
       </c>
@@ -9657,7 +10007,7 @@
         <v>576</v>
       </c>
     </row>
-    <row r="23" spans="1:8" x14ac:dyDescent="0.25">
+    <row r="23" spans="1:8" x14ac:dyDescent="0.35">
       <c r="A23" s="4" t="s">
         <v>504</v>
       </c>
@@ -9687,7 +10037,7 @@
         <v>577</v>
       </c>
     </row>
-    <row r="24" spans="1:8" x14ac:dyDescent="0.25">
+    <row r="24" spans="1:8" x14ac:dyDescent="0.35">
       <c r="A24" s="4" t="s">
         <v>505</v>
       </c>
@@ -9717,7 +10067,7 @@
         <v>578</v>
       </c>
     </row>
-    <row r="25" spans="1:8" x14ac:dyDescent="0.25">
+    <row r="25" spans="1:8" x14ac:dyDescent="0.35">
       <c r="A25" s="4" t="s">
         <v>557</v>
       </c>
@@ -9747,7 +10097,7 @@
         <v>571</v>
       </c>
     </row>
-    <row r="26" spans="1:8" x14ac:dyDescent="0.25">
+    <row r="26" spans="1:8" x14ac:dyDescent="0.35">
       <c r="A26" s="4" t="s">
         <v>558</v>
       </c>
@@ -9777,7 +10127,7 @@
         <v>571</v>
       </c>
     </row>
-    <row r="27" spans="1:8" x14ac:dyDescent="0.25">
+    <row r="27" spans="1:8" x14ac:dyDescent="0.35">
       <c r="A27" s="4" t="s">
         <v>506</v>
       </c>
@@ -9807,7 +10157,7 @@
         <v>571</v>
       </c>
     </row>
-    <row r="28" spans="1:8" x14ac:dyDescent="0.25">
+    <row r="28" spans="1:8" x14ac:dyDescent="0.35">
       <c r="A28" s="4" t="s">
         <v>529</v>
       </c>
@@ -9837,7 +10187,7 @@
         <v>572</v>
       </c>
     </row>
-    <row r="29" spans="1:8" x14ac:dyDescent="0.25">
+    <row r="29" spans="1:8" x14ac:dyDescent="0.35">
       <c r="A29" s="4" t="s">
         <v>520</v>
       </c>
@@ -9867,7 +10217,7 @@
         <v>572</v>
       </c>
     </row>
-    <row r="30" spans="1:8" x14ac:dyDescent="0.25">
+    <row r="30" spans="1:8" x14ac:dyDescent="0.35">
       <c r="A30" s="4" t="s">
         <v>521</v>
       </c>
@@ -9897,7 +10247,7 @@
         <v>579</v>
       </c>
     </row>
-    <row r="31" spans="1:8" x14ac:dyDescent="0.25">
+    <row r="31" spans="1:8" x14ac:dyDescent="0.35">
       <c r="A31" s="4" t="s">
         <v>526</v>
       </c>
@@ -9927,7 +10277,7 @@
         <v>579</v>
       </c>
     </row>
-    <row r="32" spans="1:8" x14ac:dyDescent="0.25">
+    <row r="32" spans="1:8" x14ac:dyDescent="0.35">
       <c r="A32" s="4" t="s">
         <v>560</v>
       </c>
@@ -9957,7 +10307,7 @@
         <v>568</v>
       </c>
     </row>
-    <row r="33" spans="1:8" x14ac:dyDescent="0.25">
+    <row r="33" spans="1:8" x14ac:dyDescent="0.35">
       <c r="A33" s="4" t="s">
         <v>561</v>
       </c>
@@ -9987,7 +10337,7 @@
         <v>571</v>
       </c>
     </row>
-    <row r="34" spans="1:8" x14ac:dyDescent="0.25">
+    <row r="34" spans="1:8" x14ac:dyDescent="0.35">
       <c r="A34" s="6" t="s">
         <v>522</v>
       </c>
@@ -10031,16 +10381,16 @@
 <file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{91056C88-91FB-4BF3-9450-351335B49911}">
   <dimension ref="A1:G21"/>
-  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
+  <sheetFormatPr defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
   <cols>
     <col min="1" max="1" width="13" bestFit="1" customWidth="1"/>
-    <col min="2" max="2" width="21.42578125" bestFit="1" customWidth="1"/>
-    <col min="3" max="4" width="24.42578125" bestFit="1" customWidth="1"/>
-    <col min="5" max="5" width="23.7109375" bestFit="1" customWidth="1"/>
-    <col min="6" max="7" width="24.42578125" bestFit="1" customWidth="1"/>
+    <col min="2" max="2" width="21.453125" bestFit="1" customWidth="1"/>
+    <col min="3" max="4" width="24.453125" bestFit="1" customWidth="1"/>
+    <col min="5" max="5" width="23.7265625" bestFit="1" customWidth="1"/>
+    <col min="6" max="7" width="24.453125" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="1" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A1" t="s">
         <v>0</v>
       </c>
@@ -10063,12 +10413,12 @@
         <v>6</v>
       </c>
     </row>
-    <row r="2" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="2" spans="1:7" x14ac:dyDescent="0.35">
       <c r="C2" t="s">
         <v>7</v>
       </c>
     </row>
-    <row r="3" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="3" spans="1:7" x14ac:dyDescent="0.35">
       <c r="B3" t="s">
         <v>8</v>
       </c>
@@ -10088,7 +10438,7 @@
         <v>13</v>
       </c>
     </row>
-    <row r="4" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="4" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A4" t="s">
         <v>14</v>
       </c>
@@ -10111,7 +10461,7 @@
         <v>20</v>
       </c>
     </row>
-    <row r="5" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="5" spans="1:7" x14ac:dyDescent="0.35">
       <c r="B5" t="s">
         <v>21</v>
       </c>
@@ -10131,7 +10481,7 @@
         <v>26</v>
       </c>
     </row>
-    <row r="6" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="6" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A6" t="s">
         <v>27</v>
       </c>
@@ -10154,7 +10504,7 @@
         <v>33</v>
       </c>
     </row>
-    <row r="7" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="7" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A7" t="s">
         <v>34</v>
       </c>
@@ -10177,7 +10527,7 @@
         <v>40</v>
       </c>
     </row>
-    <row r="8" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="8" spans="1:7" x14ac:dyDescent="0.35">
       <c r="B8" t="s">
         <v>41</v>
       </c>
@@ -10197,7 +10547,7 @@
         <v>46</v>
       </c>
     </row>
-    <row r="9" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="9" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A9" t="s">
         <v>47</v>
       </c>
@@ -10220,7 +10570,7 @@
         <v>53</v>
       </c>
     </row>
-    <row r="10" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="10" spans="1:7" x14ac:dyDescent="0.35">
       <c r="B10" t="s">
         <v>54</v>
       </c>
@@ -10240,7 +10590,7 @@
         <v>46</v>
       </c>
     </row>
-    <row r="11" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="11" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A11" t="s">
         <v>55</v>
       </c>
@@ -10263,7 +10613,7 @@
         <v>45</v>
       </c>
     </row>
-    <row r="12" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="12" spans="1:7" x14ac:dyDescent="0.35">
       <c r="B12" t="s">
         <v>61</v>
       </c>
@@ -10283,7 +10633,7 @@
         <v>45</v>
       </c>
     </row>
-    <row r="13" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="13" spans="1:7" x14ac:dyDescent="0.35">
       <c r="B13" t="s">
         <v>62</v>
       </c>
@@ -10303,7 +10653,7 @@
         <v>45</v>
       </c>
     </row>
-    <row r="14" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="14" spans="1:7" x14ac:dyDescent="0.35">
       <c r="B14" t="s">
         <v>63</v>
       </c>
@@ -10323,7 +10673,7 @@
         <v>45</v>
       </c>
     </row>
-    <row r="15" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="15" spans="1:7" x14ac:dyDescent="0.35">
       <c r="B15" t="s">
         <v>64</v>
       </c>
@@ -10343,7 +10693,7 @@
         <v>45</v>
       </c>
     </row>
-    <row r="16" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="16" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A16" t="s">
         <v>65</v>
       </c>
@@ -10366,7 +10716,7 @@
         <v>71</v>
       </c>
     </row>
-    <row r="19" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="19" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A19" t="s">
         <v>0</v>
       </c>
@@ -10389,7 +10739,7 @@
         <v>554</v>
       </c>
     </row>
-    <row r="20" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="20" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A20" t="s">
         <v>72</v>
       </c>
@@ -10409,7 +10759,7 @@
         <v>75</v>
       </c>
     </row>
-    <row r="21" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="21" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A21" t="s">
         <v>76</v>
       </c>
@@ -10441,19 +10791,19 @@
 <file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{0BBF25D8-DE3B-40F5-A8DF-270BBD1A35C9}">
   <dimension ref="A1:H20"/>
-  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
+  <sheetFormatPr defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
   <cols>
-    <col min="1" max="1" width="12.5703125" bestFit="1" customWidth="1"/>
-    <col min="2" max="2" width="16.42578125" bestFit="1" customWidth="1"/>
-    <col min="3" max="3" width="26.140625" bestFit="1" customWidth="1"/>
-    <col min="4" max="4" width="28.7109375" bestFit="1" customWidth="1"/>
+    <col min="1" max="1" width="12.54296875" bestFit="1" customWidth="1"/>
+    <col min="2" max="2" width="16.453125" bestFit="1" customWidth="1"/>
+    <col min="3" max="3" width="26.1796875" bestFit="1" customWidth="1"/>
+    <col min="4" max="4" width="28.7265625" bestFit="1" customWidth="1"/>
     <col min="5" max="5" width="33" bestFit="1" customWidth="1"/>
-    <col min="6" max="6" width="31.28515625" bestFit="1" customWidth="1"/>
-    <col min="7" max="7" width="29.5703125" bestFit="1" customWidth="1"/>
-    <col min="8" max="8" width="30.140625" bestFit="1" customWidth="1"/>
+    <col min="6" max="6" width="31.26953125" bestFit="1" customWidth="1"/>
+    <col min="7" max="7" width="29.54296875" bestFit="1" customWidth="1"/>
+    <col min="8" max="8" width="30.1796875" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:8" x14ac:dyDescent="0.25">
+    <row r="1" spans="1:8" x14ac:dyDescent="0.35">
       <c r="A1" t="s">
         <v>0</v>
       </c>
@@ -10479,12 +10829,12 @@
         <v>81</v>
       </c>
     </row>
-    <row r="2" spans="1:8" x14ac:dyDescent="0.25">
+    <row r="2" spans="1:8" x14ac:dyDescent="0.35">
       <c r="D2" t="s">
         <v>82</v>
       </c>
     </row>
-    <row r="3" spans="1:8" x14ac:dyDescent="0.25">
+    <row r="3" spans="1:8" x14ac:dyDescent="0.35">
       <c r="B3" t="s">
         <v>8</v>
       </c>
@@ -10507,7 +10857,7 @@
         <v>83</v>
       </c>
     </row>
-    <row r="4" spans="1:8" x14ac:dyDescent="0.25">
+    <row r="4" spans="1:8" x14ac:dyDescent="0.35">
       <c r="A4" t="s">
         <v>14</v>
       </c>
@@ -10533,7 +10883,7 @@
         <v>89</v>
       </c>
     </row>
-    <row r="5" spans="1:8" x14ac:dyDescent="0.25">
+    <row r="5" spans="1:8" x14ac:dyDescent="0.35">
       <c r="B5" t="s">
         <v>90</v>
       </c>
@@ -10556,7 +10906,7 @@
         <v>95</v>
       </c>
     </row>
-    <row r="6" spans="1:8" x14ac:dyDescent="0.25">
+    <row r="6" spans="1:8" x14ac:dyDescent="0.35">
       <c r="A6" t="s">
         <v>27</v>
       </c>
@@ -10582,7 +10932,7 @@
         <v>101</v>
       </c>
     </row>
-    <row r="7" spans="1:8" x14ac:dyDescent="0.25">
+    <row r="7" spans="1:8" x14ac:dyDescent="0.35">
       <c r="A7" t="s">
         <v>34</v>
       </c>
@@ -10608,7 +10958,7 @@
         <v>108</v>
       </c>
     </row>
-    <row r="8" spans="1:8" x14ac:dyDescent="0.25">
+    <row r="8" spans="1:8" x14ac:dyDescent="0.35">
       <c r="B8" t="s">
         <v>41</v>
       </c>
@@ -10631,7 +10981,7 @@
         <v>114</v>
       </c>
     </row>
-    <row r="9" spans="1:8" x14ac:dyDescent="0.25">
+    <row r="9" spans="1:8" x14ac:dyDescent="0.35">
       <c r="A9" t="s">
         <v>115</v>
       </c>
@@ -10657,7 +11007,7 @@
         <v>121</v>
       </c>
     </row>
-    <row r="10" spans="1:8" x14ac:dyDescent="0.25">
+    <row r="10" spans="1:8" x14ac:dyDescent="0.35">
       <c r="A10" t="s">
         <v>122</v>
       </c>
@@ -10683,7 +11033,7 @@
         <v>114</v>
       </c>
     </row>
-    <row r="11" spans="1:8" x14ac:dyDescent="0.25">
+    <row r="11" spans="1:8" x14ac:dyDescent="0.35">
       <c r="B11" t="s">
         <v>56</v>
       </c>
@@ -10706,7 +11056,7 @@
         <v>128</v>
       </c>
     </row>
-    <row r="12" spans="1:8" x14ac:dyDescent="0.25">
+    <row r="12" spans="1:8" x14ac:dyDescent="0.35">
       <c r="B12" t="s">
         <v>61</v>
       </c>
@@ -10729,7 +11079,7 @@
         <v>128</v>
       </c>
     </row>
-    <row r="13" spans="1:8" x14ac:dyDescent="0.25">
+    <row r="13" spans="1:8" x14ac:dyDescent="0.35">
       <c r="A13" t="s">
         <v>55</v>
       </c>
@@ -10755,7 +11105,7 @@
         <v>128</v>
       </c>
     </row>
-    <row r="14" spans="1:8" x14ac:dyDescent="0.25">
+    <row r="14" spans="1:8" x14ac:dyDescent="0.35">
       <c r="B14" t="s">
         <v>63</v>
       </c>
@@ -10778,7 +11128,7 @@
         <v>128</v>
       </c>
     </row>
-    <row r="15" spans="1:8" x14ac:dyDescent="0.25">
+    <row r="15" spans="1:8" x14ac:dyDescent="0.35">
       <c r="B15" t="s">
         <v>64</v>
       </c>
@@ -10801,7 +11151,7 @@
         <v>128</v>
       </c>
     </row>
-    <row r="16" spans="1:8" x14ac:dyDescent="0.25">
+    <row r="16" spans="1:8" x14ac:dyDescent="0.35">
       <c r="A16" t="s">
         <v>65</v>
       </c>
@@ -10827,7 +11177,7 @@
         <v>134</v>
       </c>
     </row>
-    <row r="18" spans="1:8" x14ac:dyDescent="0.25">
+    <row r="18" spans="1:8" x14ac:dyDescent="0.35">
       <c r="A18" t="s">
         <v>0</v>
       </c>
@@ -10853,7 +11203,7 @@
         <v>81</v>
       </c>
     </row>
-    <row r="19" spans="1:8" x14ac:dyDescent="0.25">
+    <row r="19" spans="1:8" x14ac:dyDescent="0.35">
       <c r="A19" t="s">
         <v>135</v>
       </c>
@@ -10879,7 +11229,7 @@
         <v>141</v>
       </c>
     </row>
-    <row r="20" spans="1:8" x14ac:dyDescent="0.25">
+    <row r="20" spans="1:8" x14ac:dyDescent="0.35">
       <c r="A20" t="s">
         <v>76</v>
       </c>
@@ -10914,17 +11264,17 @@
 <file path=xl/worksheets/sheet5.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{19FA074E-AB8F-493A-A8F2-7BB84CEBBA91}">
   <dimension ref="A1:F20"/>
-  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
+  <sheetFormatPr defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
   <cols>
-    <col min="1" max="1" width="12.5703125" bestFit="1" customWidth="1"/>
-    <col min="2" max="2" width="16.42578125" bestFit="1" customWidth="1"/>
-    <col min="3" max="3" width="18.85546875" bestFit="1" customWidth="1"/>
-    <col min="4" max="4" width="20.42578125" bestFit="1" customWidth="1"/>
-    <col min="5" max="5" width="18.5703125" bestFit="1" customWidth="1"/>
-    <col min="6" max="6" width="19.5703125" bestFit="1" customWidth="1"/>
+    <col min="1" max="1" width="12.54296875" bestFit="1" customWidth="1"/>
+    <col min="2" max="2" width="16.453125" bestFit="1" customWidth="1"/>
+    <col min="3" max="3" width="18.81640625" bestFit="1" customWidth="1"/>
+    <col min="4" max="4" width="20.453125" bestFit="1" customWidth="1"/>
+    <col min="5" max="5" width="18.54296875" bestFit="1" customWidth="1"/>
+    <col min="6" max="6" width="19.54296875" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="1" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A1" t="s">
         <v>0</v>
       </c>
@@ -10944,12 +11294,12 @@
         <v>5</v>
       </c>
     </row>
-    <row r="2" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="2" spans="1:6" x14ac:dyDescent="0.35">
       <c r="C2" t="s">
         <v>82</v>
       </c>
     </row>
-    <row r="3" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="3" spans="1:6" x14ac:dyDescent="0.35">
       <c r="B3" t="s">
         <v>8</v>
       </c>
@@ -10966,7 +11316,7 @@
         <v>12</v>
       </c>
     </row>
-    <row r="4" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="4" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A4" t="s">
         <v>14</v>
       </c>
@@ -10986,7 +11336,7 @@
         <v>151</v>
       </c>
     </row>
-    <row r="5" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="5" spans="1:6" x14ac:dyDescent="0.35">
       <c r="B5" t="s">
         <v>152</v>
       </c>
@@ -11003,7 +11353,7 @@
         <v>156</v>
       </c>
     </row>
-    <row r="6" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="6" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A6" t="s">
         <v>27</v>
       </c>
@@ -11023,7 +11373,7 @@
         <v>160</v>
       </c>
     </row>
-    <row r="7" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="7" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A7" t="s">
         <v>34</v>
       </c>
@@ -11043,7 +11393,7 @@
         <v>164</v>
       </c>
     </row>
-    <row r="8" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="8" spans="1:6" x14ac:dyDescent="0.35">
       <c r="B8" t="s">
         <v>41</v>
       </c>
@@ -11060,7 +11410,7 @@
         <v>168</v>
       </c>
     </row>
-    <row r="9" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="9" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A9" t="s">
         <v>115</v>
       </c>
@@ -11080,7 +11430,7 @@
         <v>170</v>
       </c>
     </row>
-    <row r="10" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="10" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A10" t="s">
         <v>122</v>
       </c>
@@ -11100,7 +11450,7 @@
         <v>168</v>
       </c>
     </row>
-    <row r="11" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="11" spans="1:6" x14ac:dyDescent="0.35">
       <c r="B11" t="s">
         <v>56</v>
       </c>
@@ -11117,7 +11467,7 @@
         <v>172</v>
       </c>
     </row>
-    <row r="12" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="12" spans="1:6" x14ac:dyDescent="0.35">
       <c r="B12" t="s">
         <v>61</v>
       </c>
@@ -11134,7 +11484,7 @@
         <v>172</v>
       </c>
     </row>
-    <row r="13" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="13" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A13" t="s">
         <v>55</v>
       </c>
@@ -11154,7 +11504,7 @@
         <v>172</v>
       </c>
     </row>
-    <row r="14" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="14" spans="1:6" x14ac:dyDescent="0.35">
       <c r="B14" t="s">
         <v>63</v>
       </c>
@@ -11171,7 +11521,7 @@
         <v>172</v>
       </c>
     </row>
-    <row r="15" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="15" spans="1:6" x14ac:dyDescent="0.35">
       <c r="B15" t="s">
         <v>64</v>
       </c>
@@ -11188,7 +11538,7 @@
         <v>172</v>
       </c>
     </row>
-    <row r="16" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="16" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A16" t="s">
         <v>65</v>
       </c>
@@ -11208,7 +11558,7 @@
         <v>176</v>
       </c>
     </row>
-    <row r="18" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="18" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A18" t="s">
         <v>0</v>
       </c>
@@ -11228,7 +11578,7 @@
         <v>5</v>
       </c>
     </row>
-    <row r="19" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="19" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A19" t="s">
         <v>135</v>
       </c>
@@ -11248,7 +11598,7 @@
         <v>151</v>
       </c>
     </row>
-    <row r="20" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="20" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A20" t="s">
         <v>76</v>
       </c>
@@ -11277,23 +11627,23 @@
 <file path=xl/worksheets/sheet6.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{1FB12C43-352D-4DE0-BEE7-738405355D14}">
   <dimension ref="A1:L20"/>
-  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
+  <sheetFormatPr defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
   <cols>
-    <col min="1" max="1" width="12.5703125" bestFit="1" customWidth="1"/>
-    <col min="2" max="2" width="16.42578125" bestFit="1" customWidth="1"/>
-    <col min="3" max="3" width="22.42578125" bestFit="1" customWidth="1"/>
-    <col min="4" max="4" width="26.85546875" bestFit="1" customWidth="1"/>
-    <col min="5" max="5" width="27.42578125" bestFit="1" customWidth="1"/>
-    <col min="6" max="6" width="25.140625" bestFit="1" customWidth="1"/>
-    <col min="7" max="7" width="22.5703125" bestFit="1" customWidth="1"/>
+    <col min="1" max="1" width="12.54296875" bestFit="1" customWidth="1"/>
+    <col min="2" max="2" width="16.453125" bestFit="1" customWidth="1"/>
+    <col min="3" max="3" width="22.453125" bestFit="1" customWidth="1"/>
+    <col min="4" max="4" width="26.81640625" bestFit="1" customWidth="1"/>
+    <col min="5" max="5" width="27.453125" bestFit="1" customWidth="1"/>
+    <col min="6" max="6" width="25.1796875" bestFit="1" customWidth="1"/>
+    <col min="7" max="7" width="22.54296875" bestFit="1" customWidth="1"/>
     <col min="8" max="8" width="27" bestFit="1" customWidth="1"/>
-    <col min="9" max="9" width="31.5703125" bestFit="1" customWidth="1"/>
-    <col min="10" max="10" width="29.28515625" bestFit="1" customWidth="1"/>
-    <col min="11" max="11" width="30.7109375" bestFit="1" customWidth="1"/>
-    <col min="12" max="12" width="28.42578125" bestFit="1" customWidth="1"/>
+    <col min="9" max="9" width="31.54296875" bestFit="1" customWidth="1"/>
+    <col min="10" max="10" width="29.26953125" bestFit="1" customWidth="1"/>
+    <col min="11" max="11" width="30.7265625" bestFit="1" customWidth="1"/>
+    <col min="12" max="12" width="28.453125" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:12" x14ac:dyDescent="0.25">
+    <row r="1" spans="1:12" x14ac:dyDescent="0.35">
       <c r="A1" t="s">
         <v>0</v>
       </c>
@@ -11331,12 +11681,12 @@
         <v>185</v>
       </c>
     </row>
-    <row r="2" spans="1:12" x14ac:dyDescent="0.25">
+    <row r="2" spans="1:12" x14ac:dyDescent="0.35">
       <c r="F2" t="s">
         <v>82</v>
       </c>
     </row>
-    <row r="3" spans="1:12" x14ac:dyDescent="0.25">
+    <row r="3" spans="1:12" x14ac:dyDescent="0.35">
       <c r="B3" t="s">
         <v>8</v>
       </c>
@@ -11371,7 +11721,7 @@
         <v>189</v>
       </c>
     </row>
-    <row r="4" spans="1:12" x14ac:dyDescent="0.25">
+    <row r="4" spans="1:12" x14ac:dyDescent="0.35">
       <c r="A4" t="s">
         <v>14</v>
       </c>
@@ -11409,7 +11759,7 @@
         <v>494</v>
       </c>
     </row>
-    <row r="5" spans="1:12" x14ac:dyDescent="0.25">
+    <row r="5" spans="1:12" x14ac:dyDescent="0.35">
       <c r="B5" t="s">
         <v>152</v>
       </c>
@@ -11444,7 +11794,7 @@
         <v>201</v>
       </c>
     </row>
-    <row r="6" spans="1:12" x14ac:dyDescent="0.25">
+    <row r="6" spans="1:12" x14ac:dyDescent="0.35">
       <c r="A6" t="s">
         <v>27</v>
       </c>
@@ -11482,7 +11832,7 @@
         <v>211</v>
       </c>
     </row>
-    <row r="7" spans="1:12" x14ac:dyDescent="0.25">
+    <row r="7" spans="1:12" x14ac:dyDescent="0.35">
       <c r="A7" t="s">
         <v>34</v>
       </c>
@@ -11520,7 +11870,7 @@
         <v>221</v>
       </c>
     </row>
-    <row r="8" spans="1:12" x14ac:dyDescent="0.25">
+    <row r="8" spans="1:12" x14ac:dyDescent="0.35">
       <c r="B8" t="s">
         <v>41</v>
       </c>
@@ -11555,7 +11905,7 @@
         <v>231</v>
       </c>
     </row>
-    <row r="9" spans="1:12" x14ac:dyDescent="0.25">
+    <row r="9" spans="1:12" x14ac:dyDescent="0.35">
       <c r="A9" t="s">
         <v>115</v>
       </c>
@@ -11593,7 +11943,7 @@
         <v>238</v>
       </c>
     </row>
-    <row r="10" spans="1:12" x14ac:dyDescent="0.25">
+    <row r="10" spans="1:12" x14ac:dyDescent="0.35">
       <c r="A10" t="s">
         <v>122</v>
       </c>
@@ -11631,7 +11981,7 @@
         <v>231</v>
       </c>
     </row>
-    <row r="11" spans="1:12" x14ac:dyDescent="0.25">
+    <row r="11" spans="1:12" x14ac:dyDescent="0.35">
       <c r="B11" t="s">
         <v>56</v>
       </c>
@@ -11666,7 +12016,7 @@
         <v>245</v>
       </c>
     </row>
-    <row r="12" spans="1:12" x14ac:dyDescent="0.25">
+    <row r="12" spans="1:12" x14ac:dyDescent="0.35">
       <c r="B12" t="s">
         <v>61</v>
       </c>
@@ -11701,7 +12051,7 @@
         <v>245</v>
       </c>
     </row>
-    <row r="13" spans="1:12" x14ac:dyDescent="0.25">
+    <row r="13" spans="1:12" x14ac:dyDescent="0.35">
       <c r="A13" t="s">
         <v>55</v>
       </c>
@@ -11739,7 +12089,7 @@
         <v>245</v>
       </c>
     </row>
-    <row r="14" spans="1:12" x14ac:dyDescent="0.25">
+    <row r="14" spans="1:12" x14ac:dyDescent="0.35">
       <c r="B14" t="s">
         <v>63</v>
       </c>
@@ -11774,7 +12124,7 @@
         <v>245</v>
       </c>
     </row>
-    <row r="15" spans="1:12" x14ac:dyDescent="0.25">
+    <row r="15" spans="1:12" x14ac:dyDescent="0.35">
       <c r="B15" t="s">
         <v>64</v>
       </c>
@@ -11809,7 +12159,7 @@
         <v>245</v>
       </c>
     </row>
-    <row r="16" spans="1:12" x14ac:dyDescent="0.25">
+    <row r="16" spans="1:12" x14ac:dyDescent="0.35">
       <c r="A16" t="s">
         <v>65</v>
       </c>
@@ -11847,7 +12197,7 @@
         <v>254</v>
       </c>
     </row>
-    <row r="18" spans="1:12" x14ac:dyDescent="0.25">
+    <row r="18" spans="1:12" x14ac:dyDescent="0.35">
       <c r="A18" t="s">
         <v>0</v>
       </c>
@@ -11885,7 +12235,7 @@
         <v>185</v>
       </c>
     </row>
-    <row r="19" spans="1:12" x14ac:dyDescent="0.25">
+    <row r="19" spans="1:12" x14ac:dyDescent="0.35">
       <c r="A19" t="s">
         <v>135</v>
       </c>
@@ -11923,7 +12273,7 @@
         <v>264</v>
       </c>
     </row>
-    <row r="20" spans="1:12" x14ac:dyDescent="0.25">
+    <row r="20" spans="1:12" x14ac:dyDescent="0.35">
       <c r="A20" t="s">
         <v>76</v>
       </c>
@@ -11970,19 +12320,19 @@
 <file path=xl/worksheets/sheet7.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{6200D3EF-F83A-49B0-BAF0-4EF918D3F281}">
   <dimension ref="A1:I20"/>
-  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
+  <sheetFormatPr defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
   <cols>
-    <col min="1" max="1" width="12.5703125" bestFit="1" customWidth="1"/>
-    <col min="2" max="2" width="16.42578125" bestFit="1" customWidth="1"/>
-    <col min="3" max="3" width="27.140625" bestFit="1" customWidth="1"/>
-    <col min="4" max="4" width="34.28515625" bestFit="1" customWidth="1"/>
+    <col min="1" max="1" width="12.54296875" bestFit="1" customWidth="1"/>
+    <col min="2" max="2" width="16.453125" bestFit="1" customWidth="1"/>
+    <col min="3" max="3" width="27.1796875" bestFit="1" customWidth="1"/>
+    <col min="4" max="4" width="34.26953125" bestFit="1" customWidth="1"/>
     <col min="5" max="5" width="23" bestFit="1" customWidth="1"/>
-    <col min="6" max="6" width="25.140625" bestFit="1" customWidth="1"/>
-    <col min="7" max="7" width="30.85546875" bestFit="1" customWidth="1"/>
-    <col min="8" max="9" width="38.42578125" bestFit="1" customWidth="1"/>
+    <col min="6" max="6" width="25.1796875" bestFit="1" customWidth="1"/>
+    <col min="7" max="7" width="30.81640625" bestFit="1" customWidth="1"/>
+    <col min="8" max="9" width="38.453125" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:9" x14ac:dyDescent="0.25">
+    <row r="1" spans="1:9" x14ac:dyDescent="0.35">
       <c r="A1" t="s">
         <v>0</v>
       </c>
@@ -12011,12 +12361,12 @@
         <v>182</v>
       </c>
     </row>
-    <row r="2" spans="1:9" x14ac:dyDescent="0.25">
+    <row r="2" spans="1:9" x14ac:dyDescent="0.35">
       <c r="D2" t="s">
         <v>271</v>
       </c>
     </row>
-    <row r="3" spans="1:9" x14ac:dyDescent="0.25">
+    <row r="3" spans="1:9" x14ac:dyDescent="0.35">
       <c r="B3" t="s">
         <v>8</v>
       </c>
@@ -12042,7 +12392,7 @@
         <v>278</v>
       </c>
     </row>
-    <row r="4" spans="1:9" x14ac:dyDescent="0.25">
+    <row r="4" spans="1:9" x14ac:dyDescent="0.35">
       <c r="A4" t="s">
         <v>14</v>
       </c>
@@ -12071,7 +12421,7 @@
         <v>285</v>
       </c>
     </row>
-    <row r="5" spans="1:9" x14ac:dyDescent="0.25">
+    <row r="5" spans="1:9" x14ac:dyDescent="0.35">
       <c r="B5" t="s">
         <v>152</v>
       </c>
@@ -12097,7 +12447,7 @@
         <v>292</v>
       </c>
     </row>
-    <row r="6" spans="1:9" x14ac:dyDescent="0.25">
+    <row r="6" spans="1:9" x14ac:dyDescent="0.35">
       <c r="A6" t="s">
         <v>27</v>
       </c>
@@ -12126,7 +12476,7 @@
         <v>299</v>
       </c>
     </row>
-    <row r="7" spans="1:9" x14ac:dyDescent="0.25">
+    <row r="7" spans="1:9" x14ac:dyDescent="0.35">
       <c r="A7" t="s">
         <v>34</v>
       </c>
@@ -12155,7 +12505,7 @@
         <v>306</v>
       </c>
     </row>
-    <row r="8" spans="1:9" x14ac:dyDescent="0.25">
+    <row r="8" spans="1:9" x14ac:dyDescent="0.35">
       <c r="B8" t="s">
         <v>41</v>
       </c>
@@ -12181,7 +12531,7 @@
         <v>313</v>
       </c>
     </row>
-    <row r="9" spans="1:9" x14ac:dyDescent="0.25">
+    <row r="9" spans="1:9" x14ac:dyDescent="0.35">
       <c r="A9" t="s">
         <v>47</v>
       </c>
@@ -12210,7 +12560,7 @@
         <v>320</v>
       </c>
     </row>
-    <row r="10" spans="1:9" x14ac:dyDescent="0.25">
+    <row r="10" spans="1:9" x14ac:dyDescent="0.35">
       <c r="B10" t="s">
         <v>123</v>
       </c>
@@ -12236,7 +12586,7 @@
         <v>313</v>
       </c>
     </row>
-    <row r="11" spans="1:9" x14ac:dyDescent="0.25">
+    <row r="11" spans="1:9" x14ac:dyDescent="0.35">
       <c r="A11" t="s">
         <v>321</v>
       </c>
@@ -12265,7 +12615,7 @@
         <v>328</v>
       </c>
     </row>
-    <row r="12" spans="1:9" x14ac:dyDescent="0.25">
+    <row r="12" spans="1:9" x14ac:dyDescent="0.35">
       <c r="B12" t="s">
         <v>61</v>
       </c>
@@ -12291,7 +12641,7 @@
         <v>328</v>
       </c>
     </row>
-    <row r="13" spans="1:9" x14ac:dyDescent="0.25">
+    <row r="13" spans="1:9" x14ac:dyDescent="0.35">
       <c r="B13" t="s">
         <v>62</v>
       </c>
@@ -12317,7 +12667,7 @@
         <v>328</v>
       </c>
     </row>
-    <row r="14" spans="1:9" x14ac:dyDescent="0.25">
+    <row r="14" spans="1:9" x14ac:dyDescent="0.35">
       <c r="B14" t="s">
         <v>63</v>
       </c>
@@ -12343,7 +12693,7 @@
         <v>328</v>
       </c>
     </row>
-    <row r="15" spans="1:9" x14ac:dyDescent="0.25">
+    <row r="15" spans="1:9" x14ac:dyDescent="0.35">
       <c r="B15" t="s">
         <v>64</v>
       </c>
@@ -12369,7 +12719,7 @@
         <v>328</v>
       </c>
     </row>
-    <row r="16" spans="1:9" x14ac:dyDescent="0.25">
+    <row r="16" spans="1:9" x14ac:dyDescent="0.35">
       <c r="A16" t="s">
         <v>65</v>
       </c>
@@ -12398,7 +12748,7 @@
         <v>335</v>
       </c>
     </row>
-    <row r="18" spans="1:9" x14ac:dyDescent="0.25">
+    <row r="18" spans="1:9" x14ac:dyDescent="0.35">
       <c r="A18" t="s">
         <v>0</v>
       </c>
@@ -12427,7 +12777,7 @@
         <v>182</v>
       </c>
     </row>
-    <row r="19" spans="1:9" x14ac:dyDescent="0.25">
+    <row r="19" spans="1:9" x14ac:dyDescent="0.35">
       <c r="A19" t="s">
         <v>135</v>
       </c>
@@ -12456,7 +12806,7 @@
         <v>336</v>
       </c>
     </row>
-    <row r="20" spans="1:9" x14ac:dyDescent="0.25">
+    <row r="20" spans="1:9" x14ac:dyDescent="0.35">
       <c r="A20" t="s">
         <v>76</v>
       </c>
@@ -12494,14 +12844,14 @@
 <file path=xl/worksheets/sheet8.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{B22E4AE0-A502-421C-ABBD-9E881E10F770}">
   <dimension ref="A1:C19"/>
-  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
+  <sheetFormatPr defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
   <cols>
-    <col min="1" max="1" width="12.5703125" bestFit="1" customWidth="1"/>
-    <col min="2" max="2" width="16.42578125" bestFit="1" customWidth="1"/>
-    <col min="3" max="3" width="30.5703125" bestFit="1" customWidth="1"/>
+    <col min="1" max="1" width="12.54296875" bestFit="1" customWidth="1"/>
+    <col min="2" max="2" width="16.453125" bestFit="1" customWidth="1"/>
+    <col min="3" max="3" width="30.54296875" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="1" spans="1:3" x14ac:dyDescent="0.35">
       <c r="A1" t="s">
         <v>0</v>
       </c>
@@ -12512,7 +12862,7 @@
         <v>2</v>
       </c>
     </row>
-    <row r="2" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="2" spans="1:3" x14ac:dyDescent="0.35">
       <c r="B2" t="s">
         <v>8</v>
       </c>
@@ -12520,7 +12870,7 @@
         <v>344</v>
       </c>
     </row>
-    <row r="3" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="3" spans="1:3" x14ac:dyDescent="0.35">
       <c r="A3" t="s">
         <v>14</v>
       </c>
@@ -12531,7 +12881,7 @@
         <v>345</v>
       </c>
     </row>
-    <row r="4" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="4" spans="1:3" x14ac:dyDescent="0.35">
       <c r="B4" t="s">
         <v>152</v>
       </c>
@@ -12539,7 +12889,7 @@
         <v>346</v>
       </c>
     </row>
-    <row r="5" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="5" spans="1:3" x14ac:dyDescent="0.35">
       <c r="A5" t="s">
         <v>27</v>
       </c>
@@ -12550,7 +12900,7 @@
         <v>347</v>
       </c>
     </row>
-    <row r="6" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="6" spans="1:3" x14ac:dyDescent="0.35">
       <c r="A6" t="s">
         <v>34</v>
       </c>
@@ -12561,7 +12911,7 @@
         <v>348</v>
       </c>
     </row>
-    <row r="7" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="7" spans="1:3" x14ac:dyDescent="0.35">
       <c r="B7" t="s">
         <v>41</v>
       </c>
@@ -12569,7 +12919,7 @@
         <v>349</v>
       </c>
     </row>
-    <row r="8" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="8" spans="1:3" x14ac:dyDescent="0.35">
       <c r="A8" t="s">
         <v>47</v>
       </c>
@@ -12580,7 +12930,7 @@
         <v>348</v>
       </c>
     </row>
-    <row r="9" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="9" spans="1:3" x14ac:dyDescent="0.35">
       <c r="B9" t="s">
         <v>123</v>
       </c>
@@ -12588,7 +12938,7 @@
         <v>349</v>
       </c>
     </row>
-    <row r="10" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="10" spans="1:3" x14ac:dyDescent="0.35">
       <c r="A10" t="s">
         <v>321</v>
       </c>
@@ -12599,7 +12949,7 @@
         <v>350</v>
       </c>
     </row>
-    <row r="11" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="11" spans="1:3" x14ac:dyDescent="0.35">
       <c r="B11" t="s">
         <v>61</v>
       </c>
@@ -12607,7 +12957,7 @@
         <v>350</v>
       </c>
     </row>
-    <row r="12" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="12" spans="1:3" x14ac:dyDescent="0.35">
       <c r="B12" t="s">
         <v>62</v>
       </c>
@@ -12615,7 +12965,7 @@
         <v>350</v>
       </c>
     </row>
-    <row r="13" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="13" spans="1:3" x14ac:dyDescent="0.35">
       <c r="B13" t="s">
         <v>63</v>
       </c>
@@ -12623,7 +12973,7 @@
         <v>350</v>
       </c>
     </row>
-    <row r="14" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="14" spans="1:3" x14ac:dyDescent="0.35">
       <c r="B14" t="s">
         <v>64</v>
       </c>
@@ -12631,7 +12981,7 @@
         <v>350</v>
       </c>
     </row>
-    <row r="15" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="15" spans="1:3" x14ac:dyDescent="0.35">
       <c r="A15" t="s">
         <v>65</v>
       </c>
@@ -12642,7 +12992,7 @@
         <v>351</v>
       </c>
     </row>
-    <row r="17" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="17" spans="1:3" x14ac:dyDescent="0.35">
       <c r="A17" t="s">
         <v>0</v>
       </c>
@@ -12653,7 +13003,7 @@
         <v>2</v>
       </c>
     </row>
-    <row r="18" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="18" spans="1:3" x14ac:dyDescent="0.35">
       <c r="A18" t="s">
         <v>135</v>
       </c>
@@ -12664,7 +13014,7 @@
         <v>345</v>
       </c>
     </row>
-    <row r="19" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="19" spans="1:3" x14ac:dyDescent="0.35">
       <c r="A19" t="s">
         <v>76</v>
       </c>
@@ -12684,16 +13034,16 @@
 <file path=xl/worksheets/sheet9.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{E5F91B12-5D52-447E-877C-7C65848770FC}">
   <dimension ref="A1:E21"/>
-  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
+  <sheetFormatPr defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
   <cols>
-    <col min="1" max="1" width="12.5703125" bestFit="1" customWidth="1"/>
-    <col min="2" max="2" width="16.42578125" bestFit="1" customWidth="1"/>
-    <col min="3" max="3" width="22.140625" bestFit="1" customWidth="1"/>
-    <col min="4" max="4" width="15.85546875" bestFit="1" customWidth="1"/>
-    <col min="5" max="5" width="28.140625" bestFit="1" customWidth="1"/>
+    <col min="1" max="1" width="12.54296875" bestFit="1" customWidth="1"/>
+    <col min="2" max="2" width="16.453125" bestFit="1" customWidth="1"/>
+    <col min="3" max="3" width="22.1796875" bestFit="1" customWidth="1"/>
+    <col min="4" max="4" width="15.81640625" bestFit="1" customWidth="1"/>
+    <col min="5" max="5" width="28.1796875" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="1" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A1" t="s">
         <v>0</v>
       </c>
@@ -12710,7 +13060,7 @@
         <v>4</v>
       </c>
     </row>
-    <row r="2" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="2" spans="1:5" x14ac:dyDescent="0.35">
       <c r="B2" t="s">
         <v>8</v>
       </c>
@@ -12718,12 +13068,12 @@
         <v>82</v>
       </c>
     </row>
-    <row r="3" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="3" spans="1:5" x14ac:dyDescent="0.35">
       <c r="C3" t="s">
         <v>353</v>
       </c>
     </row>
-    <row r="4" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="4" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A4" t="s">
         <v>14</v>
       </c>
@@ -12740,7 +13090,7 @@
         <v>356</v>
       </c>
     </row>
-    <row r="5" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="5" spans="1:5" x14ac:dyDescent="0.35">
       <c r="B5" t="s">
         <v>21</v>
       </c>
@@ -12754,7 +13104,7 @@
         <v>359</v>
       </c>
     </row>
-    <row r="6" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="6" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A6" t="s">
         <v>27</v>
       </c>
@@ -12771,7 +13121,7 @@
         <v>362</v>
       </c>
     </row>
-    <row r="7" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="7" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A7" t="s">
         <v>34</v>
       </c>
@@ -12788,7 +13138,7 @@
         <v>365</v>
       </c>
     </row>
-    <row r="8" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="8" spans="1:5" x14ac:dyDescent="0.35">
       <c r="B8" t="s">
         <v>41</v>
       </c>
@@ -12802,7 +13152,7 @@
         <v>368</v>
       </c>
     </row>
-    <row r="9" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="9" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A9" t="s">
         <v>47</v>
       </c>
@@ -12819,7 +13169,7 @@
         <v>371</v>
       </c>
     </row>
-    <row r="10" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="10" spans="1:5" x14ac:dyDescent="0.35">
       <c r="B10" t="s">
         <v>123</v>
       </c>
@@ -12833,7 +13183,7 @@
         <v>368</v>
       </c>
     </row>
-    <row r="11" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="11" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A11" t="s">
         <v>321</v>
       </c>
@@ -12850,7 +13200,7 @@
         <v>374</v>
       </c>
     </row>
-    <row r="12" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="12" spans="1:5" x14ac:dyDescent="0.35">
       <c r="B12" t="s">
         <v>61</v>
       </c>
@@ -12864,7 +13214,7 @@
         <v>374</v>
       </c>
     </row>
-    <row r="13" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="13" spans="1:5" x14ac:dyDescent="0.35">
       <c r="B13" t="s">
         <v>62</v>
       </c>
@@ -12878,7 +13228,7 @@
         <v>374</v>
       </c>
     </row>
-    <row r="14" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="14" spans="1:5" x14ac:dyDescent="0.35">
       <c r="B14" t="s">
         <v>63</v>
       </c>
@@ -12892,7 +13242,7 @@
         <v>374</v>
       </c>
     </row>
-    <row r="15" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="15" spans="1:5" x14ac:dyDescent="0.35">
       <c r="B15" t="s">
         <v>64</v>
       </c>
@@ -12906,7 +13256,7 @@
         <v>374</v>
       </c>
     </row>
-    <row r="16" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="16" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A16" t="s">
         <v>65</v>
       </c>
@@ -12923,7 +13273,7 @@
         <v>376</v>
       </c>
     </row>
-    <row r="18" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="18" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A18" t="s">
         <v>0</v>
       </c>
@@ -12940,7 +13290,7 @@
         <v>4</v>
       </c>
     </row>
-    <row r="19" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="19" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A19" t="s">
         <v>135</v>
       </c>
@@ -12957,7 +13307,7 @@
         <v>379</v>
       </c>
     </row>
-    <row r="20" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="20" spans="1:5" x14ac:dyDescent="0.35">
       <c r="C20" t="s">
         <v>380</v>
       </c>
@@ -12968,7 +13318,7 @@
         <v>382</v>
       </c>
     </row>
-    <row r="21" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="21" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A21" t="s">
         <v>76</v>
       </c>

</xml_diff>

<commit_message>
UPDATE: Added new column for 'Kupang'
</commit_message>
<xml_diff>
--- a/gp-app-1.0/Pricelist Car.xlsx
+++ b/gp-app-1.0/Pricelist Car.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\Work\gp-app\gp-app-1.0\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{391995BF-E4CA-4326-ADE8-70EFB6FB3E44}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{35F1378E-01C9-4702-8EF2-1841E6041172}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-110" yWindow="-110" windowWidth="19420" windowHeight="11020" tabRatio="861" xr2:uid="{C4C7316A-D95F-426A-ADF9-AD32FA680374}"/>
   </bookViews>
@@ -2720,7 +2720,7 @@
     <xf numFmtId="43" fontId="2" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="30">
+  <cellXfs count="25">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="2" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
     <xf numFmtId="3" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
@@ -2762,11 +2762,6 @@
     <xf numFmtId="0" fontId="2" fillId="2" borderId="9" xfId="3" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="3" xfId="0" applyFill="1" applyBorder="1"/>
-    <xf numFmtId="43" fontId="0" fillId="0" borderId="4" xfId="0" applyNumberFormat="1" applyFill="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="8" xfId="0" applyFill="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="9" xfId="0" applyFill="1" applyBorder="1"/>
-    <xf numFmtId="43" fontId="0" fillId="0" borderId="10" xfId="0" applyNumberFormat="1" applyFill="1" applyBorder="1"/>
   </cellXfs>
   <cellStyles count="4">
     <cellStyle name="Comma" xfId="2" builtinId="3"/>
@@ -5163,9 +5158,6 @@
 <file path=xl/tables/table1.xml><?xml version="1.0" encoding="utf-8"?>
 <table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="20" xr:uid="{DF067A72-54A6-48F4-972D-2DE4603D61A4}" name="Table20" displayName="Table20" ref="A1:I79" totalsRowShown="0" headerRowDxfId="155" headerRowBorderDxfId="154" tableBorderDxfId="153" totalsRowBorderDxfId="152">
   <autoFilter ref="A1:I79" xr:uid="{DF067A72-54A6-48F4-972D-2DE4603D61A4}"/>
-  <sortState xmlns:xlrd2="http://schemas.microsoft.com/office/spreadsheetml/2017/richdata2" ref="A2:I57">
-    <sortCondition ref="H1:H57"/>
-  </sortState>
   <tableColumns count="9">
     <tableColumn id="1" xr3:uid="{0E6335F2-6B6A-436C-92FA-B48E61551308}" name="Merek/Type" dataDxfId="151"/>
     <tableColumn id="2" xr3:uid="{5A4965DA-398A-4134-90BD-9CE4D8355880}" name="Tipe" dataDxfId="150"/>
@@ -7241,16 +7233,16 @@
         <v>168000000</v>
       </c>
       <c r="D45" s="5">
-        <f t="shared" si="7"/>
-        <v>11160714.285714284</v>
+        <f>I45/1.11</f>
+        <v>11261261.261261258</v>
       </c>
       <c r="E45" s="5">
         <f t="shared" si="8"/>
-        <v>10044642.857142856</v>
+        <v>10135135.135135133</v>
       </c>
       <c r="F45" s="5">
         <f t="shared" si="9"/>
-        <v>7812499.9999999981</v>
+        <v>7882882.88288288</v>
       </c>
       <c r="G45" s="3">
         <v>237</v>
@@ -7273,16 +7265,16 @@
         <v>176000000</v>
       </c>
       <c r="D46" s="5">
-        <f t="shared" si="7"/>
-        <v>12053571.428571427</v>
+        <f t="shared" ref="D46:D49" si="13">I46/1.11</f>
+        <v>12162162.162162161</v>
       </c>
       <c r="E46" s="5">
         <f t="shared" si="8"/>
-        <v>10848214.285714285</v>
+        <v>10945945.945945945</v>
       </c>
       <c r="F46" s="5">
         <f t="shared" si="9"/>
-        <v>8437499.9999999981</v>
+        <v>8513513.513513511</v>
       </c>
       <c r="G46" s="24">
         <v>238</v>
@@ -7305,16 +7297,16 @@
         <v>155700000</v>
       </c>
       <c r="D47" s="5">
-        <f t="shared" si="7"/>
-        <v>10892857.142857142</v>
+        <f t="shared" si="13"/>
+        <v>10990990.990990991</v>
       </c>
       <c r="E47" s="5">
         <f t="shared" si="8"/>
-        <v>9803571.4285714272</v>
+        <v>9891891.8918918911</v>
       </c>
       <c r="F47" s="5">
         <f t="shared" si="9"/>
-        <v>7624999.9999999991</v>
+        <v>7693693.6936936928</v>
       </c>
       <c r="G47" s="3">
         <v>201</v>
@@ -7336,17 +7328,17 @@
       <c r="C48" s="9">
         <v>167800000</v>
       </c>
-      <c r="D48" s="9">
-        <f t="shared" si="7"/>
-        <v>7142857.1428571418</v>
+      <c r="D48" s="5">
+        <f t="shared" si="13"/>
+        <v>7207207.2072072066</v>
       </c>
       <c r="E48" s="9">
         <f t="shared" si="8"/>
-        <v>6428571.4285714282</v>
+        <v>6486486.4864864862</v>
       </c>
       <c r="F48" s="9">
         <f t="shared" si="9"/>
-        <v>4999999.9999999991</v>
+        <v>5045045.0450450443</v>
       </c>
       <c r="G48" s="20">
         <v>229</v>
@@ -7369,16 +7361,16 @@
         <v>172600000</v>
       </c>
       <c r="D49" s="5">
-        <f t="shared" si="7"/>
-        <v>7142857.1428571418</v>
+        <f t="shared" si="13"/>
+        <v>7207207.2072072066</v>
       </c>
       <c r="E49" s="5">
         <f t="shared" si="8"/>
-        <v>6428571.4285714282</v>
+        <v>6486486.4864864862</v>
       </c>
       <c r="F49" s="5">
         <f t="shared" si="9"/>
-        <v>4999999.9999999991</v>
+        <v>5045045.0450450443</v>
       </c>
       <c r="G49" s="3">
         <v>230</v>
@@ -7657,15 +7649,15 @@
         <v>399000000</v>
       </c>
       <c r="D58" s="9">
-        <f t="shared" ref="D58:D65" si="13">I58/1.12</f>
+        <f t="shared" ref="D58:D65" si="14">I58/1.12</f>
         <v>22321428.571428571</v>
       </c>
       <c r="E58" s="9">
-        <f t="shared" ref="E58:E65" si="14">D58*90%</f>
+        <f t="shared" ref="E58:E65" si="15">D58*90%</f>
         <v>20089285.714285713</v>
       </c>
       <c r="F58" s="9">
-        <f t="shared" ref="F58:F65" si="15">D58*70%</f>
+        <f t="shared" ref="F58:F65" si="16">D58*70%</f>
         <v>15624999.999999998</v>
       </c>
       <c r="G58" s="21">
@@ -7689,15 +7681,15 @@
         <v>469000000</v>
       </c>
       <c r="D59" s="9">
-        <f t="shared" si="13"/>
+        <f t="shared" si="14"/>
         <v>31249999.999999996</v>
       </c>
       <c r="E59" s="9">
-        <f t="shared" si="14"/>
+        <f t="shared" si="15"/>
         <v>28124999.999999996</v>
       </c>
       <c r="F59" s="9">
-        <f t="shared" si="15"/>
+        <f t="shared" si="16"/>
         <v>21874999.999999996</v>
       </c>
       <c r="G59" s="21">
@@ -7721,15 +7713,15 @@
         <v>459000000</v>
       </c>
       <c r="D60" s="9">
-        <f t="shared" si="13"/>
+        <f t="shared" si="14"/>
         <v>22321428.571428571</v>
       </c>
       <c r="E60" s="9">
-        <f t="shared" si="14"/>
+        <f t="shared" si="15"/>
         <v>20089285.714285713</v>
       </c>
       <c r="F60" s="9">
-        <f t="shared" si="15"/>
+        <f t="shared" si="16"/>
         <v>15624999.999999998</v>
       </c>
       <c r="G60" s="21">
@@ -7753,15 +7745,15 @@
         <v>509000000</v>
       </c>
       <c r="D61" s="9">
-        <f t="shared" si="13"/>
+        <f t="shared" si="14"/>
         <v>31249999.999999996</v>
       </c>
       <c r="E61" s="9">
-        <f t="shared" si="14"/>
+        <f t="shared" si="15"/>
         <v>28124999.999999996</v>
       </c>
       <c r="F61" s="9">
-        <f t="shared" si="15"/>
+        <f t="shared" si="16"/>
         <v>21874999.999999996</v>
       </c>
       <c r="G61" s="21">
@@ -7785,15 +7777,15 @@
         <v>399000000</v>
       </c>
       <c r="D62" s="9">
-        <f t="shared" si="13"/>
+        <f t="shared" si="14"/>
         <v>22321428.571428571</v>
       </c>
       <c r="E62" s="9">
-        <f t="shared" si="14"/>
+        <f t="shared" si="15"/>
         <v>20089285.714285713</v>
       </c>
       <c r="F62" s="9">
-        <f t="shared" si="15"/>
+        <f t="shared" si="16"/>
         <v>15624999.999999998</v>
       </c>
       <c r="G62" s="21">
@@ -7817,15 +7809,15 @@
         <v>469000000</v>
       </c>
       <c r="D63" s="9">
-        <f t="shared" si="13"/>
+        <f t="shared" si="14"/>
         <v>31249999.999999996</v>
       </c>
       <c r="E63" s="9">
-        <f t="shared" si="14"/>
+        <f t="shared" si="15"/>
         <v>28124999.999999996</v>
       </c>
       <c r="F63" s="9">
-        <f t="shared" si="15"/>
+        <f t="shared" si="16"/>
         <v>21874999.999999996</v>
       </c>
       <c r="G63" s="21">
@@ -7849,15 +7841,15 @@
         <v>459000000</v>
       </c>
       <c r="D64" s="9">
-        <f t="shared" si="13"/>
+        <f t="shared" si="14"/>
         <v>22321428.571428571</v>
       </c>
       <c r="E64" s="9">
-        <f t="shared" si="14"/>
+        <f t="shared" si="15"/>
         <v>20089285.714285713</v>
       </c>
       <c r="F64" s="9">
-        <f t="shared" si="15"/>
+        <f t="shared" si="16"/>
         <v>15624999.999999998</v>
       </c>
       <c r="G64" s="21">
@@ -7881,15 +7873,15 @@
         <v>509000000</v>
       </c>
       <c r="D65" s="9">
-        <f t="shared" si="13"/>
+        <f t="shared" si="14"/>
         <v>31249999.999999996</v>
       </c>
       <c r="E65" s="9">
-        <f t="shared" si="14"/>
+        <f t="shared" si="15"/>
         <v>28124999.999999996</v>
       </c>
       <c r="F65" s="9">
-        <f t="shared" si="15"/>
+        <f t="shared" si="16"/>
         <v>21874999.999999996</v>
       </c>
       <c r="G65" s="21">
@@ -7913,15 +7905,15 @@
         <v>303000000</v>
       </c>
       <c r="D66" s="9">
-        <f t="shared" ref="D66:D68" si="16">I66/1.12</f>
+        <f t="shared" ref="D66:D68" si="17">I66/1.12</f>
         <v>20535714.285714284</v>
       </c>
       <c r="E66" s="9">
-        <f t="shared" ref="E66:E68" si="17">D66*90%</f>
+        <f t="shared" ref="E66:E68" si="18">D66*90%</f>
         <v>18482142.857142854</v>
       </c>
       <c r="F66" s="9">
-        <f t="shared" ref="F66:F68" si="18">D66*70%</f>
+        <f t="shared" ref="F66:F68" si="19">D66*70%</f>
         <v>14374999.999999998</v>
       </c>
       <c r="G66" s="3">
@@ -7945,15 +7937,15 @@
         <v>217000000</v>
       </c>
       <c r="D67" s="5">
-        <f t="shared" si="16"/>
+        <f t="shared" si="17"/>
         <v>11607142.857142856</v>
       </c>
       <c r="E67" s="5">
-        <f t="shared" si="17"/>
+        <f t="shared" si="18"/>
         <v>10446428.571428571</v>
       </c>
       <c r="F67" s="5">
-        <f t="shared" si="18"/>
+        <f t="shared" si="19"/>
         <v>8124999.9999999991</v>
       </c>
       <c r="G67" s="3">
@@ -7977,15 +7969,15 @@
         <v>263000000</v>
       </c>
       <c r="D68" s="5">
-        <f t="shared" si="16"/>
+        <f t="shared" si="17"/>
         <v>17857142.857142854</v>
       </c>
       <c r="E68" s="5">
-        <f t="shared" si="17"/>
+        <f t="shared" si="18"/>
         <v>16071428.571428569</v>
       </c>
       <c r="F68" s="5">
-        <f t="shared" si="18"/>
+        <f t="shared" si="19"/>
         <v>12499999.999999998</v>
       </c>
       <c r="G68" s="3">
@@ -8009,15 +8001,15 @@
         <v>155000000</v>
       </c>
       <c r="D69" s="5">
-        <f t="shared" ref="D69:D71" si="19">I69/1.12</f>
+        <f t="shared" ref="D69:D71" si="20">I69/1.12</f>
         <v>5357142.8571428563</v>
       </c>
       <c r="E69" s="5">
-        <f t="shared" ref="E69:E71" si="20">D69*90%</f>
+        <f t="shared" ref="E69:E71" si="21">D69*90%</f>
         <v>4821428.5714285709</v>
       </c>
       <c r="F69" s="5">
-        <f t="shared" ref="F69:F71" si="21">D69*70%</f>
+        <f t="shared" ref="F69:F71" si="22">D69*70%</f>
         <v>3749999.9999999991</v>
       </c>
       <c r="G69" s="3">
@@ -8041,15 +8033,15 @@
         <v>175000000</v>
       </c>
       <c r="D70" s="5">
-        <f t="shared" si="19"/>
+        <f t="shared" si="20"/>
         <v>5357142.8571428563</v>
       </c>
       <c r="E70" s="5">
-        <f t="shared" si="20"/>
+        <f t="shared" si="21"/>
         <v>4821428.5714285709</v>
       </c>
       <c r="F70" s="5">
-        <f t="shared" si="21"/>
+        <f t="shared" si="22"/>
         <v>3749999.9999999991</v>
       </c>
       <c r="G70" s="3">
@@ -8073,15 +8065,15 @@
         <v>389000000</v>
       </c>
       <c r="D71" s="9">
-        <f t="shared" si="19"/>
+        <f t="shared" si="20"/>
         <v>27499999.999999996</v>
       </c>
       <c r="E71" s="9">
-        <f t="shared" si="20"/>
+        <f t="shared" si="21"/>
         <v>24749999.999999996</v>
       </c>
       <c r="F71" s="9">
-        <f t="shared" si="21"/>
+        <f t="shared" si="22"/>
         <v>19249999.999999996</v>
       </c>
       <c r="G71" s="20">
@@ -8105,15 +8097,15 @@
         <v>399000000</v>
       </c>
       <c r="D72" s="9">
-        <f t="shared" ref="D72:D75" si="22">I72/1.12</f>
+        <f t="shared" ref="D72:D75" si="23">I72/1.12</f>
         <v>28214285.714285713</v>
       </c>
       <c r="E72" s="9">
-        <f t="shared" ref="E72:E75" si="23">D72*90%</f>
+        <f t="shared" ref="E72:E75" si="24">D72*90%</f>
         <v>25392857.142857142</v>
       </c>
       <c r="F72" s="9">
-        <f t="shared" ref="F72:F75" si="24">D72*70%</f>
+        <f t="shared" ref="F72:F75" si="25">D72*70%</f>
         <v>19749999.999999996</v>
       </c>
       <c r="G72" s="20">
@@ -8137,15 +8129,15 @@
         <v>459000000</v>
       </c>
       <c r="D73" s="9">
-        <f t="shared" si="22"/>
+        <f t="shared" si="23"/>
         <v>32499999.999999996</v>
       </c>
       <c r="E73" s="9">
-        <f t="shared" si="23"/>
+        <f t="shared" si="24"/>
         <v>29249999.999999996</v>
       </c>
       <c r="F73" s="9">
-        <f t="shared" si="24"/>
+        <f t="shared" si="25"/>
         <v>22749999.999999996</v>
       </c>
       <c r="G73" s="20">
@@ -8169,15 +8161,15 @@
         <v>449000000</v>
       </c>
       <c r="D74" s="9">
-        <f t="shared" si="22"/>
+        <f t="shared" si="23"/>
         <v>29196428.571428567</v>
       </c>
       <c r="E74" s="9">
-        <f t="shared" si="23"/>
+        <f t="shared" si="24"/>
         <v>26276785.714285713</v>
       </c>
       <c r="F74" s="9">
-        <f t="shared" si="24"/>
+        <f t="shared" si="25"/>
         <v>20437499.999999996</v>
       </c>
       <c r="G74" s="20">
@@ -8201,15 +8193,15 @@
         <v>499000000</v>
       </c>
       <c r="D75" s="9">
-        <f t="shared" si="22"/>
+        <f t="shared" si="23"/>
         <v>32499999.999999996</v>
       </c>
       <c r="E75" s="9">
-        <f t="shared" si="23"/>
+        <f t="shared" si="24"/>
         <v>29249999.999999996</v>
       </c>
       <c r="F75" s="9">
-        <f t="shared" si="24"/>
+        <f t="shared" si="25"/>
         <v>22749999.999999996</v>
       </c>
       <c r="G75" s="20">
@@ -8223,7 +8215,7 @@
       </c>
     </row>
     <row r="76" spans="1:9" x14ac:dyDescent="0.35">
-      <c r="A76" s="25" t="s">
+      <c r="A76" s="10" t="s">
         <v>645</v>
       </c>
       <c r="B76" s="4" t="s">
@@ -8233,15 +8225,15 @@
         <v>289000000</v>
       </c>
       <c r="D76" s="9">
-        <f t="shared" ref="D76:D77" si="25">I76/1.12</f>
+        <f t="shared" ref="D76:D77" si="26">I76/1.12</f>
         <v>13392857.142857142</v>
       </c>
       <c r="E76" s="9">
-        <f t="shared" ref="E76:E77" si="26">D76*90%</f>
+        <f t="shared" ref="E76:E77" si="27">D76*90%</f>
         <v>12053571.428571427</v>
       </c>
       <c r="F76" s="9">
-        <f t="shared" ref="F76:F77" si="27">D76*70%</f>
+        <f t="shared" ref="F76:F77" si="28">D76*70%</f>
         <v>9374999.9999999981</v>
       </c>
       <c r="G76" s="20">
@@ -8250,12 +8242,12 @@
       <c r="H76" s="4" t="s">
         <v>576</v>
       </c>
-      <c r="I76" s="26">
+      <c r="I76" s="12">
         <v>15000000</v>
       </c>
     </row>
     <row r="77" spans="1:9" x14ac:dyDescent="0.35">
-      <c r="A77" s="25" t="s">
+      <c r="A77" s="10" t="s">
         <v>646</v>
       </c>
       <c r="B77" s="4" t="s">
@@ -8265,15 +8257,15 @@
         <v>319000000</v>
       </c>
       <c r="D77" s="9">
-        <f t="shared" si="25"/>
+        <f t="shared" si="26"/>
         <v>13392857.142857142</v>
       </c>
       <c r="E77" s="9">
-        <f t="shared" si="26"/>
+        <f t="shared" si="27"/>
         <v>12053571.428571427</v>
       </c>
       <c r="F77" s="9">
-        <f t="shared" si="27"/>
+        <f t="shared" si="28"/>
         <v>9374999.9999999981</v>
       </c>
       <c r="G77" s="20">
@@ -8282,30 +8274,30 @@
       <c r="H77" s="4" t="s">
         <v>577</v>
       </c>
-      <c r="I77" s="26">
+      <c r="I77" s="12">
         <v>15000000</v>
       </c>
     </row>
     <row r="78" spans="1:9" x14ac:dyDescent="0.35">
-      <c r="A78" s="27" t="s">
+      <c r="A78" s="16" t="s">
         <v>647</v>
       </c>
-      <c r="B78" s="28" t="s">
+      <c r="B78" s="17" t="s">
         <v>649</v>
       </c>
       <c r="C78" s="18">
         <v>299000000</v>
       </c>
       <c r="D78" s="9">
-        <f t="shared" ref="D78:D79" si="28">I78/1.12</f>
+        <f t="shared" ref="D78:D79" si="29">I78/1.12</f>
         <v>17857142.857142854</v>
       </c>
       <c r="E78" s="9">
-        <f t="shared" ref="E78:E79" si="29">D78*90%</f>
+        <f t="shared" ref="E78:E79" si="30">D78*90%</f>
         <v>16071428.571428569</v>
       </c>
       <c r="F78" s="9">
-        <f t="shared" ref="F78:F79" si="30">D78*70%</f>
+        <f t="shared" ref="F78:F79" si="31">D78*70%</f>
         <v>12499999.999999998</v>
       </c>
       <c r="G78" s="20">
@@ -8314,30 +8306,30 @@
       <c r="H78" s="4" t="s">
         <v>581</v>
       </c>
-      <c r="I78" s="29">
+      <c r="I78" s="19">
         <v>20000000</v>
       </c>
     </row>
     <row r="79" spans="1:9" x14ac:dyDescent="0.35">
-      <c r="A79" s="27" t="s">
+      <c r="A79" s="16" t="s">
         <v>648</v>
       </c>
-      <c r="B79" s="28" t="s">
+      <c r="B79" s="17" t="s">
         <v>650</v>
       </c>
       <c r="C79" s="18">
         <v>339000000</v>
       </c>
       <c r="D79" s="9">
-        <f t="shared" si="28"/>
+        <f t="shared" si="29"/>
         <v>22321428.571428571</v>
       </c>
       <c r="E79" s="9">
-        <f t="shared" si="29"/>
+        <f t="shared" si="30"/>
         <v>20089285.714285713</v>
       </c>
       <c r="F79" s="9">
-        <f t="shared" si="30"/>
+        <f t="shared" si="31"/>
         <v>15624999.999999998</v>
       </c>
       <c r="G79" s="20">
@@ -8346,7 +8338,7 @@
       <c r="H79" s="4" t="s">
         <v>571</v>
       </c>
-      <c r="I79" s="29">
+      <c r="I79" s="19">
         <v>25000000</v>
       </c>
     </row>

</xml_diff>

<commit_message>
UPDATE: Added new unit to pricelist
</commit_message>
<xml_diff>
--- a/gp-app-1.0/Pricelist Car.xlsx
+++ b/gp-app-1.0/Pricelist Car.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\Work\gp-app\gp-app-1.0\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{35F1378E-01C9-4702-8EF2-1841E6041172}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{52799D07-20FD-48B2-BAE3-C136D01F2CE3}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-110" yWindow="-110" windowWidth="19420" windowHeight="11020" tabRatio="861" xr2:uid="{C4C7316A-D95F-426A-ADF9-AD32FA680374}"/>
   </bookViews>
@@ -2772,6 +2772,47 @@
   <dxfs count="156">
     <dxf>
       <font>
+        <b val="0"/>
+        <i val="0"/>
+        <strike val="0"/>
+        <condense val="0"/>
+        <extend val="0"/>
+        <outline val="0"/>
+        <shadow val="0"/>
+        <u val="none"/>
+        <vertAlign val="baseline"/>
+        <sz val="11"/>
+        <color theme="1"/>
+        <name val="Calibri"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </font>
+      <numFmt numFmtId="35" formatCode="_-* #,##0.00_-;\-* #,##0.00_-;_-* &quot;-&quot;??_-;_-@_-"/>
+      <fill>
+        <patternFill patternType="none">
+          <fgColor indexed="64"/>
+          <bgColor indexed="65"/>
+        </patternFill>
+      </fill>
+      <border diagonalUp="0" diagonalDown="0">
+        <left style="thin">
+          <color indexed="64"/>
+        </left>
+        <right style="thin">
+          <color indexed="64"/>
+        </right>
+        <top style="thin">
+          <color indexed="64"/>
+        </top>
+        <bottom style="thin">
+          <color indexed="64"/>
+        </bottom>
+        <vertical/>
+        <horizontal/>
+      </border>
+    </dxf>
+    <dxf>
+      <font>
         <color rgb="FF9C0006"/>
       </font>
       <fill>
@@ -3318,46 +3359,6 @@
       </border>
     </dxf>
     <dxf>
-      <border diagonalUp="0" diagonalDown="0">
-        <left style="thin">
-          <color indexed="64"/>
-        </left>
-        <right style="thin">
-          <color indexed="64"/>
-        </right>
-        <top style="thin">
-          <color indexed="64"/>
-        </top>
-        <bottom style="thin">
-          <color indexed="64"/>
-        </bottom>
-        <vertical/>
-        <horizontal/>
-      </border>
-    </dxf>
-    <dxf>
-      <font>
-        <b val="0"/>
-        <i val="0"/>
-        <strike val="0"/>
-        <condense val="0"/>
-        <extend val="0"/>
-        <outline val="0"/>
-        <shadow val="0"/>
-        <u val="none"/>
-        <vertAlign val="baseline"/>
-        <sz val="11"/>
-        <color theme="1"/>
-        <name val="Calibri"/>
-        <family val="2"/>
-        <scheme val="minor"/>
-      </font>
-      <fill>
-        <patternFill patternType="none">
-          <fgColor indexed="64"/>
-          <bgColor indexed="65"/>
-        </patternFill>
-      </fill>
       <border diagonalUp="0" diagonalDown="0">
         <left style="thin">
           <color indexed="64"/>
@@ -5162,12 +5163,14 @@
     <tableColumn id="1" xr3:uid="{0E6335F2-6B6A-436C-92FA-B48E61551308}" name="Merek/Type" dataDxfId="151"/>
     <tableColumn id="2" xr3:uid="{5A4965DA-398A-4134-90BD-9CE4D8355880}" name="Tipe" dataDxfId="150"/>
     <tableColumn id="3" xr3:uid="{010303D1-E0A2-4DE6-8E87-64ACC3102E09}" name="Harga OTR Awal" dataDxfId="149" dataCellStyle="Comma"/>
-    <tableColumn id="4" xr3:uid="{91C798B0-7964-436A-84A5-7687993F376F}" name="Dealer Margin" dataDxfId="148" dataCellStyle="Comma"/>
-    <tableColumn id="5" xr3:uid="{CD936623-36F3-4BAA-A615-AF79A61C51E8}" name="Dealer Margin 9 %" dataDxfId="147" dataCellStyle="Comma"/>
-    <tableColumn id="6" xr3:uid="{A36173E8-D9B2-4F38-A572-F5D32CDADEB8}" name="Dealer Margin 7 %" dataDxfId="146" dataCellStyle="Comma"/>
-    <tableColumn id="7" xr3:uid="{7A11B7F5-7683-492A-A8B5-D96984323DDD}" name="Code Unit" dataDxfId="145"/>
-    <tableColumn id="8" xr3:uid="{AF243BB3-2044-4D1E-9F0D-A1EC0D2C15CF}" name="Merk/Type" dataDxfId="144"/>
-    <tableColumn id="9" xr3:uid="{9E0E2E6A-108F-4ACE-959D-9EB0F753BD73}" name="Full Margin" dataDxfId="143"/>
+    <tableColumn id="4" xr3:uid="{91C798B0-7964-436A-84A5-7687993F376F}" name="Dealer Margin" dataDxfId="0" dataCellStyle="Comma">
+      <calculatedColumnFormula>I2/1.12</calculatedColumnFormula>
+    </tableColumn>
+    <tableColumn id="5" xr3:uid="{CD936623-36F3-4BAA-A615-AF79A61C51E8}" name="Dealer Margin 9 %" dataDxfId="148" dataCellStyle="Comma"/>
+    <tableColumn id="6" xr3:uid="{A36173E8-D9B2-4F38-A572-F5D32CDADEB8}" name="Dealer Margin 7 %" dataDxfId="147" dataCellStyle="Comma"/>
+    <tableColumn id="7" xr3:uid="{7A11B7F5-7683-492A-A8B5-D96984323DDD}" name="Code Unit" dataDxfId="146"/>
+    <tableColumn id="8" xr3:uid="{AF243BB3-2044-4D1E-9F0D-A1EC0D2C15CF}" name="Merk/Type" dataDxfId="145"/>
+    <tableColumn id="9" xr3:uid="{9E0E2E6A-108F-4ACE-959D-9EB0F753BD73}" name="Full Margin" dataDxfId="144"/>
   </tableColumns>
   <tableStyleInfo name="TableStyleMedium2" showFirstColumn="0" showLastColumn="0" showRowStripes="1" showColumnStripes="0"/>
 </table>
@@ -5177,15 +5180,15 @@
 <table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="9" xr:uid="{630D8221-A5B4-4162-BEFC-7BB63825B861}" name="Table009__Page_6" displayName="Table009__Page_6" ref="A1:I16" tableType="queryTable" totalsRowShown="0">
   <autoFilter ref="A1:I16" xr:uid="{630D8221-A5B4-4162-BEFC-7BB63825B861}"/>
   <tableColumns count="9">
-    <tableColumn id="1" xr3:uid="{5980B244-73E4-43AF-B863-305E8B039C33}" uniqueName="1" name="Column1" queryTableFieldId="1" dataDxfId="76"/>
-    <tableColumn id="2" xr3:uid="{549208EE-7E07-4F0F-ACFD-9606CC8F6B50}" uniqueName="2" name="Column2" queryTableFieldId="2" dataDxfId="75"/>
-    <tableColumn id="3" xr3:uid="{086F7B88-A201-47FD-B9A0-0C976108E144}" uniqueName="3" name="Column3" queryTableFieldId="3" dataDxfId="74"/>
-    <tableColumn id="4" xr3:uid="{CC912184-CE02-4DC9-8815-71C4295C86DF}" uniqueName="4" name="Column4" queryTableFieldId="4" dataDxfId="73"/>
-    <tableColumn id="5" xr3:uid="{8F3F2202-7C07-4D43-B483-871C9E242208}" uniqueName="5" name="Column5" queryTableFieldId="5" dataDxfId="72"/>
-    <tableColumn id="6" xr3:uid="{6D2190D6-B434-4BB9-95B1-A29148C453AF}" uniqueName="6" name="Column6" queryTableFieldId="6" dataDxfId="71"/>
-    <tableColumn id="7" xr3:uid="{A33DE0AF-7DA7-4623-87E7-DBA2BF4E404A}" uniqueName="7" name="Column7" queryTableFieldId="7" dataDxfId="70"/>
-    <tableColumn id="8" xr3:uid="{CD689B59-BA44-4F67-9FF9-E08337BE66FD}" uniqueName="8" name="Column8" queryTableFieldId="8" dataDxfId="69"/>
-    <tableColumn id="9" xr3:uid="{744F224A-BA1E-4758-B291-8D5C8D341610}" uniqueName="9" name="Column9" queryTableFieldId="9" dataDxfId="68"/>
+    <tableColumn id="1" xr3:uid="{5980B244-73E4-43AF-B863-305E8B039C33}" uniqueName="1" name="Column1" queryTableFieldId="1" dataDxfId="77"/>
+    <tableColumn id="2" xr3:uid="{549208EE-7E07-4F0F-ACFD-9606CC8F6B50}" uniqueName="2" name="Column2" queryTableFieldId="2" dataDxfId="76"/>
+    <tableColumn id="3" xr3:uid="{086F7B88-A201-47FD-B9A0-0C976108E144}" uniqueName="3" name="Column3" queryTableFieldId="3" dataDxfId="75"/>
+    <tableColumn id="4" xr3:uid="{CC912184-CE02-4DC9-8815-71C4295C86DF}" uniqueName="4" name="Column4" queryTableFieldId="4" dataDxfId="74"/>
+    <tableColumn id="5" xr3:uid="{8F3F2202-7C07-4D43-B483-871C9E242208}" uniqueName="5" name="Column5" queryTableFieldId="5" dataDxfId="73"/>
+    <tableColumn id="6" xr3:uid="{6D2190D6-B434-4BB9-95B1-A29148C453AF}" uniqueName="6" name="Column6" queryTableFieldId="6" dataDxfId="72"/>
+    <tableColumn id="7" xr3:uid="{A33DE0AF-7DA7-4623-87E7-DBA2BF4E404A}" uniqueName="7" name="Column7" queryTableFieldId="7" dataDxfId="71"/>
+    <tableColumn id="8" xr3:uid="{CD689B59-BA44-4F67-9FF9-E08337BE66FD}" uniqueName="8" name="Column8" queryTableFieldId="8" dataDxfId="70"/>
+    <tableColumn id="9" xr3:uid="{744F224A-BA1E-4758-B291-8D5C8D341610}" uniqueName="9" name="Column9" queryTableFieldId="9" dataDxfId="69"/>
   </tableColumns>
   <tableStyleInfo name="TableStyleMedium7" showFirstColumn="0" showLastColumn="0" showRowStripes="1" showColumnStripes="0"/>
 </table>
@@ -5195,15 +5198,15 @@
 <table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="10" xr:uid="{116BBD7B-F856-4C44-8F1F-EA66756E3A0B}" name="Table010__Page_6" displayName="Table010__Page_6" ref="A18:I20" tableType="queryTable" totalsRowShown="0">
   <autoFilter ref="A18:I20" xr:uid="{116BBD7B-F856-4C44-8F1F-EA66756E3A0B}"/>
   <tableColumns count="9">
-    <tableColumn id="1" xr3:uid="{D02866AC-7C8C-4041-B0D6-297717EA2BCA}" uniqueName="1" name="Column1" queryTableFieldId="1" dataDxfId="67"/>
-    <tableColumn id="2" xr3:uid="{F9BA0334-AC0F-4599-91DD-1D3B53530BA2}" uniqueName="2" name="Column2" queryTableFieldId="2" dataDxfId="66"/>
-    <tableColumn id="3" xr3:uid="{2E40CB08-FF90-4211-A5F6-3255AA5CEAED}" uniqueName="3" name="Column3" queryTableFieldId="3" dataDxfId="65"/>
-    <tableColumn id="4" xr3:uid="{951E49DE-3DB8-41C0-8F36-6E5A1649659D}" uniqueName="4" name="Column4" queryTableFieldId="4" dataDxfId="64"/>
-    <tableColumn id="5" xr3:uid="{D7FC7D23-AA29-4FAE-8DF4-B23A11020D8C}" uniqueName="5" name="Column5" queryTableFieldId="5" dataDxfId="63"/>
-    <tableColumn id="6" xr3:uid="{85DA6C7C-BC56-4316-BB56-3D2CA86DF4B0}" uniqueName="6" name="Column6" queryTableFieldId="6" dataDxfId="62"/>
-    <tableColumn id="7" xr3:uid="{47F39228-8CCC-4319-9964-568280350AF4}" uniqueName="7" name="Column7" queryTableFieldId="7" dataDxfId="61"/>
-    <tableColumn id="8" xr3:uid="{781188CD-5AC0-41B9-8575-2EACD4BA90A4}" uniqueName="8" name="Column8" queryTableFieldId="8" dataDxfId="60"/>
-    <tableColumn id="9" xr3:uid="{A2DFBEC8-960F-4613-A8B8-821CF42818AC}" uniqueName="9" name="Column9" queryTableFieldId="9" dataDxfId="59"/>
+    <tableColumn id="1" xr3:uid="{D02866AC-7C8C-4041-B0D6-297717EA2BCA}" uniqueName="1" name="Column1" queryTableFieldId="1" dataDxfId="68"/>
+    <tableColumn id="2" xr3:uid="{F9BA0334-AC0F-4599-91DD-1D3B53530BA2}" uniqueName="2" name="Column2" queryTableFieldId="2" dataDxfId="67"/>
+    <tableColumn id="3" xr3:uid="{2E40CB08-FF90-4211-A5F6-3255AA5CEAED}" uniqueName="3" name="Column3" queryTableFieldId="3" dataDxfId="66"/>
+    <tableColumn id="4" xr3:uid="{951E49DE-3DB8-41C0-8F36-6E5A1649659D}" uniqueName="4" name="Column4" queryTableFieldId="4" dataDxfId="65"/>
+    <tableColumn id="5" xr3:uid="{D7FC7D23-AA29-4FAE-8DF4-B23A11020D8C}" uniqueName="5" name="Column5" queryTableFieldId="5" dataDxfId="64"/>
+    <tableColumn id="6" xr3:uid="{85DA6C7C-BC56-4316-BB56-3D2CA86DF4B0}" uniqueName="6" name="Column6" queryTableFieldId="6" dataDxfId="63"/>
+    <tableColumn id="7" xr3:uid="{47F39228-8CCC-4319-9964-568280350AF4}" uniqueName="7" name="Column7" queryTableFieldId="7" dataDxfId="62"/>
+    <tableColumn id="8" xr3:uid="{781188CD-5AC0-41B9-8575-2EACD4BA90A4}" uniqueName="8" name="Column8" queryTableFieldId="8" dataDxfId="61"/>
+    <tableColumn id="9" xr3:uid="{A2DFBEC8-960F-4613-A8B8-821CF42818AC}" uniqueName="9" name="Column9" queryTableFieldId="9" dataDxfId="60"/>
   </tableColumns>
   <tableStyleInfo name="TableStyleMedium7" showFirstColumn="0" showLastColumn="0" showRowStripes="1" showColumnStripes="0"/>
 </table>
@@ -5213,9 +5216,9 @@
 <table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="11" xr:uid="{D5A80464-2F5E-4F81-BC09-642A89962C82}" name="Table011__Page_7" displayName="Table011__Page_7" ref="A1:C15" tableType="queryTable" totalsRowShown="0">
   <autoFilter ref="A1:C15" xr:uid="{D5A80464-2F5E-4F81-BC09-642A89962C82}"/>
   <tableColumns count="3">
-    <tableColumn id="1" xr3:uid="{384F6B08-E7B1-4ECD-BC7E-1F8C8FC9CD11}" uniqueName="1" name="Column1" queryTableFieldId="1" dataDxfId="58"/>
-    <tableColumn id="2" xr3:uid="{BD116665-54B3-487B-82AD-7E260403FB1A}" uniqueName="2" name="Column2" queryTableFieldId="2" dataDxfId="57"/>
-    <tableColumn id="3" xr3:uid="{A0C72322-3C63-446F-A7B0-E45538411191}" uniqueName="3" name="Column3" queryTableFieldId="3" dataDxfId="56"/>
+    <tableColumn id="1" xr3:uid="{384F6B08-E7B1-4ECD-BC7E-1F8C8FC9CD11}" uniqueName="1" name="Column1" queryTableFieldId="1" dataDxfId="59"/>
+    <tableColumn id="2" xr3:uid="{BD116665-54B3-487B-82AD-7E260403FB1A}" uniqueName="2" name="Column2" queryTableFieldId="2" dataDxfId="58"/>
+    <tableColumn id="3" xr3:uid="{A0C72322-3C63-446F-A7B0-E45538411191}" uniqueName="3" name="Column3" queryTableFieldId="3" dataDxfId="57"/>
   </tableColumns>
   <tableStyleInfo name="TableStyleMedium7" showFirstColumn="0" showLastColumn="0" showRowStripes="1" showColumnStripes="0"/>
 </table>
@@ -5225,9 +5228,9 @@
 <table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="12" xr:uid="{BF5A7D5F-42BD-4927-9517-2459449E72C6}" name="Table012__Page_7" displayName="Table012__Page_7" ref="A17:C19" tableType="queryTable" totalsRowShown="0">
   <autoFilter ref="A17:C19" xr:uid="{BF5A7D5F-42BD-4927-9517-2459449E72C6}"/>
   <tableColumns count="3">
-    <tableColumn id="1" xr3:uid="{92B56AD9-FE6F-4702-B777-811CB1B6E64F}" uniqueName="1" name="Column1" queryTableFieldId="1" dataDxfId="55"/>
-    <tableColumn id="2" xr3:uid="{C37743D7-7886-43A1-BB26-C0F3914426C9}" uniqueName="2" name="Column2" queryTableFieldId="2" dataDxfId="54"/>
-    <tableColumn id="3" xr3:uid="{DFF6BFBF-623A-4318-86AF-C5448FC821A5}" uniqueName="3" name="Column3" queryTableFieldId="3" dataDxfId="53"/>
+    <tableColumn id="1" xr3:uid="{92B56AD9-FE6F-4702-B777-811CB1B6E64F}" uniqueName="1" name="Column1" queryTableFieldId="1" dataDxfId="56"/>
+    <tableColumn id="2" xr3:uid="{C37743D7-7886-43A1-BB26-C0F3914426C9}" uniqueName="2" name="Column2" queryTableFieldId="2" dataDxfId="55"/>
+    <tableColumn id="3" xr3:uid="{DFF6BFBF-623A-4318-86AF-C5448FC821A5}" uniqueName="3" name="Column3" queryTableFieldId="3" dataDxfId="54"/>
   </tableColumns>
   <tableStyleInfo name="TableStyleMedium7" showFirstColumn="0" showLastColumn="0" showRowStripes="1" showColumnStripes="0"/>
 </table>
@@ -5237,11 +5240,11 @@
 <table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="13" xr:uid="{4DAA9679-BE71-4F3A-B608-132984AF6DF1}" name="Table013__Page_8" displayName="Table013__Page_8" ref="A1:E16" tableType="queryTable" totalsRowShown="0">
   <autoFilter ref="A1:E16" xr:uid="{4DAA9679-BE71-4F3A-B608-132984AF6DF1}"/>
   <tableColumns count="5">
-    <tableColumn id="1" xr3:uid="{811DEB23-A3B8-4E1E-AF98-CBD4FE9515C8}" uniqueName="1" name="Column1" queryTableFieldId="1" dataDxfId="52"/>
-    <tableColumn id="2" xr3:uid="{D1233A63-9D37-45F3-9DC7-52977AC06ADC}" uniqueName="2" name="Column2" queryTableFieldId="2" dataDxfId="51"/>
-    <tableColumn id="3" xr3:uid="{400191B1-4CF8-4D78-82E7-FED7CD6730E6}" uniqueName="3" name="Column3" queryTableFieldId="3" dataDxfId="50"/>
-    <tableColumn id="4" xr3:uid="{3D829CC4-4292-4CD0-80B8-3490D4014AC9}" uniqueName="4" name="Column4" queryTableFieldId="4" dataDxfId="49"/>
-    <tableColumn id="5" xr3:uid="{9BC50CF1-EF44-42B4-9129-E887F74428C9}" uniqueName="5" name="Column5" queryTableFieldId="5" dataDxfId="48"/>
+    <tableColumn id="1" xr3:uid="{811DEB23-A3B8-4E1E-AF98-CBD4FE9515C8}" uniqueName="1" name="Column1" queryTableFieldId="1" dataDxfId="53"/>
+    <tableColumn id="2" xr3:uid="{D1233A63-9D37-45F3-9DC7-52977AC06ADC}" uniqueName="2" name="Column2" queryTableFieldId="2" dataDxfId="52"/>
+    <tableColumn id="3" xr3:uid="{400191B1-4CF8-4D78-82E7-FED7CD6730E6}" uniqueName="3" name="Column3" queryTableFieldId="3" dataDxfId="51"/>
+    <tableColumn id="4" xr3:uid="{3D829CC4-4292-4CD0-80B8-3490D4014AC9}" uniqueName="4" name="Column4" queryTableFieldId="4" dataDxfId="50"/>
+    <tableColumn id="5" xr3:uid="{9BC50CF1-EF44-42B4-9129-E887F74428C9}" uniqueName="5" name="Column5" queryTableFieldId="5" dataDxfId="49"/>
   </tableColumns>
   <tableStyleInfo name="TableStyleMedium7" showFirstColumn="0" showLastColumn="0" showRowStripes="1" showColumnStripes="0"/>
 </table>
@@ -5251,11 +5254,11 @@
 <table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="14" xr:uid="{9D3195A8-F1BD-4429-B95A-60FCF241B775}" name="Table014__Page_8" displayName="Table014__Page_8" ref="A18:E21" tableType="queryTable" totalsRowShown="0">
   <autoFilter ref="A18:E21" xr:uid="{9D3195A8-F1BD-4429-B95A-60FCF241B775}"/>
   <tableColumns count="5">
-    <tableColumn id="1" xr3:uid="{98A6121C-2EC1-48CA-8A40-28DAFD66423E}" uniqueName="1" name="Column1" queryTableFieldId="1" dataDxfId="47"/>
-    <tableColumn id="2" xr3:uid="{6B521FB3-E639-4556-B8C5-473A63201BC1}" uniqueName="2" name="Column2" queryTableFieldId="2" dataDxfId="46"/>
-    <tableColumn id="3" xr3:uid="{3D07F9E9-4DA3-41C6-98A7-BC28F0C8BFB5}" uniqueName="3" name="Column3" queryTableFieldId="3" dataDxfId="45"/>
-    <tableColumn id="4" xr3:uid="{89F1E0D5-9B1D-4170-BB1D-3FBA7855FC27}" uniqueName="4" name="Column4" queryTableFieldId="4" dataDxfId="44"/>
-    <tableColumn id="5" xr3:uid="{68E29A0D-4E20-4E2A-A030-157EF3C69E97}" uniqueName="5" name="Column5" queryTableFieldId="5" dataDxfId="43"/>
+    <tableColumn id="1" xr3:uid="{98A6121C-2EC1-48CA-8A40-28DAFD66423E}" uniqueName="1" name="Column1" queryTableFieldId="1" dataDxfId="48"/>
+    <tableColumn id="2" xr3:uid="{6B521FB3-E639-4556-B8C5-473A63201BC1}" uniqueName="2" name="Column2" queryTableFieldId="2" dataDxfId="47"/>
+    <tableColumn id="3" xr3:uid="{3D07F9E9-4DA3-41C6-98A7-BC28F0C8BFB5}" uniqueName="3" name="Column3" queryTableFieldId="3" dataDxfId="46"/>
+    <tableColumn id="4" xr3:uid="{89F1E0D5-9B1D-4170-BB1D-3FBA7855FC27}" uniqueName="4" name="Column4" queryTableFieldId="4" dataDxfId="45"/>
+    <tableColumn id="5" xr3:uid="{68E29A0D-4E20-4E2A-A030-157EF3C69E97}" uniqueName="5" name="Column5" queryTableFieldId="5" dataDxfId="44"/>
   </tableColumns>
   <tableStyleInfo name="TableStyleMedium7" showFirstColumn="0" showLastColumn="0" showRowStripes="1" showColumnStripes="0"/>
 </table>
@@ -5265,12 +5268,12 @@
 <table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="15" xr:uid="{F2B12C92-B774-477F-98C9-509526BBDEE5}" name="Table015__Page_9" displayName="Table015__Page_9" ref="A1:F16" tableType="queryTable" totalsRowShown="0">
   <autoFilter ref="A1:F16" xr:uid="{F2B12C92-B774-477F-98C9-509526BBDEE5}"/>
   <tableColumns count="6">
-    <tableColumn id="1" xr3:uid="{B9D47F1B-922B-4B02-855C-93AF62167342}" uniqueName="1" name="Column1" queryTableFieldId="1" dataDxfId="42"/>
-    <tableColumn id="2" xr3:uid="{9915D8BD-1C99-4D36-BE7E-9EBEAD6D7B12}" uniqueName="2" name="Column2" queryTableFieldId="2" dataDxfId="41"/>
-    <tableColumn id="3" xr3:uid="{D353D58B-6A1D-4079-A9EC-77376B67A375}" uniqueName="3" name="Column3" queryTableFieldId="3" dataDxfId="40"/>
-    <tableColumn id="4" xr3:uid="{ACF53426-7425-4D38-9673-B3197A3F9292}" uniqueName="4" name="Column4" queryTableFieldId="4" dataDxfId="39"/>
-    <tableColumn id="5" xr3:uid="{673A9374-D6DA-46D7-AAD2-6F2220F4ED8C}" uniqueName="5" name="Column5" queryTableFieldId="5" dataDxfId="38"/>
-    <tableColumn id="6" xr3:uid="{37C428F9-0692-44D1-B8CF-2CBC7901020B}" uniqueName="6" name="Column6" queryTableFieldId="6" dataDxfId="37"/>
+    <tableColumn id="1" xr3:uid="{B9D47F1B-922B-4B02-855C-93AF62167342}" uniqueName="1" name="Column1" queryTableFieldId="1" dataDxfId="43"/>
+    <tableColumn id="2" xr3:uid="{9915D8BD-1C99-4D36-BE7E-9EBEAD6D7B12}" uniqueName="2" name="Column2" queryTableFieldId="2" dataDxfId="42"/>
+    <tableColumn id="3" xr3:uid="{D353D58B-6A1D-4079-A9EC-77376B67A375}" uniqueName="3" name="Column3" queryTableFieldId="3" dataDxfId="41"/>
+    <tableColumn id="4" xr3:uid="{ACF53426-7425-4D38-9673-B3197A3F9292}" uniqueName="4" name="Column4" queryTableFieldId="4" dataDxfId="40"/>
+    <tableColumn id="5" xr3:uid="{673A9374-D6DA-46D7-AAD2-6F2220F4ED8C}" uniqueName="5" name="Column5" queryTableFieldId="5" dataDxfId="39"/>
+    <tableColumn id="6" xr3:uid="{37C428F9-0692-44D1-B8CF-2CBC7901020B}" uniqueName="6" name="Column6" queryTableFieldId="6" dataDxfId="38"/>
   </tableColumns>
   <tableStyleInfo name="TableStyleMedium7" showFirstColumn="0" showLastColumn="0" showRowStripes="1" showColumnStripes="0"/>
 </table>
@@ -5280,12 +5283,12 @@
 <table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="16" xr:uid="{3C596C1A-3A31-47DF-B534-2A3593167FFF}" name="Table016__Page_9" displayName="Table016__Page_9" ref="A18:F20" tableType="queryTable" totalsRowShown="0">
   <autoFilter ref="A18:F20" xr:uid="{3C596C1A-3A31-47DF-B534-2A3593167FFF}"/>
   <tableColumns count="6">
-    <tableColumn id="1" xr3:uid="{48EBD4D1-26EB-449F-8D09-DF1A8D9D96A3}" uniqueName="1" name="Column1" queryTableFieldId="1" dataDxfId="36"/>
-    <tableColumn id="2" xr3:uid="{671AE648-452F-44F1-9A65-8468F7B19950}" uniqueName="2" name="Column2" queryTableFieldId="2" dataDxfId="35"/>
-    <tableColumn id="3" xr3:uid="{C3287937-E8A8-4D80-A27C-D2A5C0E44D68}" uniqueName="3" name="Column3" queryTableFieldId="3" dataDxfId="34"/>
-    <tableColumn id="4" xr3:uid="{49CAB777-0355-40CC-9F2D-C41408ED9E98}" uniqueName="4" name="Column4" queryTableFieldId="4" dataDxfId="33"/>
-    <tableColumn id="5" xr3:uid="{A19C49CB-F2CF-4D60-B082-761FE4F0ABC5}" uniqueName="5" name="Column5" queryTableFieldId="5" dataDxfId="32"/>
-    <tableColumn id="6" xr3:uid="{801427E9-2562-451E-AE45-ACF6DAAAFFFB}" uniqueName="6" name="Column6" queryTableFieldId="6" dataDxfId="31"/>
+    <tableColumn id="1" xr3:uid="{48EBD4D1-26EB-449F-8D09-DF1A8D9D96A3}" uniqueName="1" name="Column1" queryTableFieldId="1" dataDxfId="37"/>
+    <tableColumn id="2" xr3:uid="{671AE648-452F-44F1-9A65-8468F7B19950}" uniqueName="2" name="Column2" queryTableFieldId="2" dataDxfId="36"/>
+    <tableColumn id="3" xr3:uid="{C3287937-E8A8-4D80-A27C-D2A5C0E44D68}" uniqueName="3" name="Column3" queryTableFieldId="3" dataDxfId="35"/>
+    <tableColumn id="4" xr3:uid="{49CAB777-0355-40CC-9F2D-C41408ED9E98}" uniqueName="4" name="Column4" queryTableFieldId="4" dataDxfId="34"/>
+    <tableColumn id="5" xr3:uid="{A19C49CB-F2CF-4D60-B082-761FE4F0ABC5}" uniqueName="5" name="Column5" queryTableFieldId="5" dataDxfId="33"/>
+    <tableColumn id="6" xr3:uid="{801427E9-2562-451E-AE45-ACF6DAAAFFFB}" uniqueName="6" name="Column6" queryTableFieldId="6" dataDxfId="32"/>
   </tableColumns>
   <tableStyleInfo name="TableStyleMedium7" showFirstColumn="0" showLastColumn="0" showRowStripes="1" showColumnStripes="0"/>
 </table>
@@ -5295,11 +5298,11 @@
 <table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="17" xr:uid="{510F87AB-8378-4FE2-9EBF-7361BA7DB6B8}" name="Table017__Page_10" displayName="Table017__Page_10" ref="A1:E15" tableType="queryTable" totalsRowShown="0">
   <autoFilter ref="A1:E15" xr:uid="{510F87AB-8378-4FE2-9EBF-7361BA7DB6B8}"/>
   <tableColumns count="5">
-    <tableColumn id="1" xr3:uid="{626476ED-551C-48ED-A0F5-9CB680097EF0}" uniqueName="1" name="Column1" queryTableFieldId="1" dataDxfId="30"/>
-    <tableColumn id="2" xr3:uid="{9215A7DD-9718-48E5-BA20-B6B9989DD0D2}" uniqueName="2" name="Column2" queryTableFieldId="2" dataDxfId="29"/>
-    <tableColumn id="3" xr3:uid="{AE2AC56F-3587-4342-A60B-0B4A30905DD3}" uniqueName="3" name="Column3" queryTableFieldId="3" dataDxfId="28"/>
-    <tableColumn id="4" xr3:uid="{F7BE237D-2C3F-4C27-92EF-2601ABCBA887}" uniqueName="4" name="Column4" queryTableFieldId="4" dataDxfId="27"/>
-    <tableColumn id="5" xr3:uid="{7950C4F9-8FA4-4C6E-B03A-A0235ECC51FF}" uniqueName="5" name="Column5" queryTableFieldId="5" dataDxfId="26"/>
+    <tableColumn id="1" xr3:uid="{626476ED-551C-48ED-A0F5-9CB680097EF0}" uniqueName="1" name="Column1" queryTableFieldId="1" dataDxfId="31"/>
+    <tableColumn id="2" xr3:uid="{9215A7DD-9718-48E5-BA20-B6B9989DD0D2}" uniqueName="2" name="Column2" queryTableFieldId="2" dataDxfId="30"/>
+    <tableColumn id="3" xr3:uid="{AE2AC56F-3587-4342-A60B-0B4A30905DD3}" uniqueName="3" name="Column3" queryTableFieldId="3" dataDxfId="29"/>
+    <tableColumn id="4" xr3:uid="{F7BE237D-2C3F-4C27-92EF-2601ABCBA887}" uniqueName="4" name="Column4" queryTableFieldId="4" dataDxfId="28"/>
+    <tableColumn id="5" xr3:uid="{7950C4F9-8FA4-4C6E-B03A-A0235ECC51FF}" uniqueName="5" name="Column5" queryTableFieldId="5" dataDxfId="27"/>
   </tableColumns>
   <tableStyleInfo name="TableStyleMedium7" showFirstColumn="0" showLastColumn="0" showRowStripes="1" showColumnStripes="0"/>
 </table>
@@ -5309,11 +5312,11 @@
 <table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="18" xr:uid="{14CF879A-74C7-4F0C-8E76-F1430C9579CD}" name="Table018__Page_10" displayName="Table018__Page_10" ref="A17:E19" tableType="queryTable" totalsRowShown="0">
   <autoFilter ref="A17:E19" xr:uid="{14CF879A-74C7-4F0C-8E76-F1430C9579CD}"/>
   <tableColumns count="5">
-    <tableColumn id="1" xr3:uid="{210B1486-2DC9-4D94-98AC-6BEB874B7545}" uniqueName="1" name="Column1" queryTableFieldId="1" dataDxfId="25"/>
-    <tableColumn id="2" xr3:uid="{BB67F395-3AAE-4514-BCCE-DE32693EB37D}" uniqueName="2" name="Column2" queryTableFieldId="2" dataDxfId="24"/>
-    <tableColumn id="3" xr3:uid="{230B22CA-5CA3-4E2D-92CC-C75BC5831FF2}" uniqueName="3" name="Column3" queryTableFieldId="3" dataDxfId="23"/>
-    <tableColumn id="4" xr3:uid="{42788CA6-A70D-442A-9072-79E0D19F0B28}" uniqueName="4" name="Column4" queryTableFieldId="4" dataDxfId="22"/>
-    <tableColumn id="5" xr3:uid="{E37C1038-7442-4E7D-BB43-162AD6FA4195}" uniqueName="5" name="Column5" queryTableFieldId="5" dataDxfId="21"/>
+    <tableColumn id="1" xr3:uid="{210B1486-2DC9-4D94-98AC-6BEB874B7545}" uniqueName="1" name="Column1" queryTableFieldId="1" dataDxfId="26"/>
+    <tableColumn id="2" xr3:uid="{BB67F395-3AAE-4514-BCCE-DE32693EB37D}" uniqueName="2" name="Column2" queryTableFieldId="2" dataDxfId="25"/>
+    <tableColumn id="3" xr3:uid="{230B22CA-5CA3-4E2D-92CC-C75BC5831FF2}" uniqueName="3" name="Column3" queryTableFieldId="3" dataDxfId="24"/>
+    <tableColumn id="4" xr3:uid="{42788CA6-A70D-442A-9072-79E0D19F0B28}" uniqueName="4" name="Column4" queryTableFieldId="4" dataDxfId="23"/>
+    <tableColumn id="5" xr3:uid="{E37C1038-7442-4E7D-BB43-162AD6FA4195}" uniqueName="5" name="Column5" queryTableFieldId="5" dataDxfId="22"/>
   </tableColumns>
   <tableStyleInfo name="TableStyleMedium7" showFirstColumn="0" showLastColumn="0" showRowStripes="1" showColumnStripes="0"/>
 </table>
@@ -5323,13 +5326,13 @@
 <table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="1" xr:uid="{8D8C9D73-217D-4974-B35A-0740746DA27F}" name="Table001__Page_2" displayName="Table001__Page_2" ref="A1:G16" tableType="queryTable" totalsRowShown="0">
   <autoFilter ref="A1:G16" xr:uid="{8D8C9D73-217D-4974-B35A-0740746DA27F}"/>
   <tableColumns count="7">
-    <tableColumn id="1" xr3:uid="{A26CE965-72B2-472B-B9FF-D68F7847F3C5}" uniqueName="1" name="Column1" queryTableFieldId="1" dataDxfId="142"/>
-    <tableColumn id="2" xr3:uid="{375BF78E-5806-424A-B7BD-C63C40843BE9}" uniqueName="2" name="Column2" queryTableFieldId="2" dataDxfId="141"/>
-    <tableColumn id="3" xr3:uid="{CD1FFC74-B097-42B5-B1FA-08D3BD4531B9}" uniqueName="3" name="Column3" queryTableFieldId="3" dataDxfId="140"/>
-    <tableColumn id="4" xr3:uid="{EA6F5C08-47B3-4BE3-8F9B-3167F2B34338}" uniqueName="4" name="Column4" queryTableFieldId="4" dataDxfId="139"/>
-    <tableColumn id="5" xr3:uid="{67D1B145-6151-4A54-9C79-A6B0381CDA09}" uniqueName="5" name="Column5" queryTableFieldId="5" dataDxfId="138"/>
-    <tableColumn id="6" xr3:uid="{E8D8899E-ED32-4A2F-B13D-18F4C289A59B}" uniqueName="6" name="Column6" queryTableFieldId="6" dataDxfId="137"/>
-    <tableColumn id="7" xr3:uid="{CD1BCBB0-10DE-4DDA-903D-C14D16829749}" uniqueName="7" name="Column7" queryTableFieldId="7" dataDxfId="136"/>
+    <tableColumn id="1" xr3:uid="{A26CE965-72B2-472B-B9FF-D68F7847F3C5}" uniqueName="1" name="Column1" queryTableFieldId="1" dataDxfId="143"/>
+    <tableColumn id="2" xr3:uid="{375BF78E-5806-424A-B7BD-C63C40843BE9}" uniqueName="2" name="Column2" queryTableFieldId="2" dataDxfId="142"/>
+    <tableColumn id="3" xr3:uid="{CD1FFC74-B097-42B5-B1FA-08D3BD4531B9}" uniqueName="3" name="Column3" queryTableFieldId="3" dataDxfId="141"/>
+    <tableColumn id="4" xr3:uid="{EA6F5C08-47B3-4BE3-8F9B-3167F2B34338}" uniqueName="4" name="Column4" queryTableFieldId="4" dataDxfId="140"/>
+    <tableColumn id="5" xr3:uid="{67D1B145-6151-4A54-9C79-A6B0381CDA09}" uniqueName="5" name="Column5" queryTableFieldId="5" dataDxfId="139"/>
+    <tableColumn id="6" xr3:uid="{E8D8899E-ED32-4A2F-B13D-18F4C289A59B}" uniqueName="6" name="Column6" queryTableFieldId="6" dataDxfId="138"/>
+    <tableColumn id="7" xr3:uid="{CD1BCBB0-10DE-4DDA-903D-C14D16829749}" uniqueName="7" name="Column7" queryTableFieldId="7" dataDxfId="137"/>
   </tableColumns>
   <tableStyleInfo name="TableStyleMedium7" showFirstColumn="0" showLastColumn="0" showRowStripes="1" showColumnStripes="0"/>
 </table>
@@ -5339,11 +5342,11 @@
 <table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="19" xr:uid="{A8D65B7F-C1B3-4E37-BFF7-03252131F371}" name="Table019__Page_11" displayName="Table019__Page_11" ref="A1:E16" tableType="queryTable" totalsRowShown="0">
   <autoFilter ref="A1:E16" xr:uid="{A8D65B7F-C1B3-4E37-BFF7-03252131F371}"/>
   <tableColumns count="5">
-    <tableColumn id="1" xr3:uid="{60EAA1C9-E43C-458C-A33C-365CF023541D}" uniqueName="1" name="Column1" queryTableFieldId="1" dataDxfId="20"/>
-    <tableColumn id="2" xr3:uid="{BF4ECEAF-8998-4833-A444-7DD2840947AB}" uniqueName="2" name="Column2" queryTableFieldId="2" dataDxfId="19"/>
-    <tableColumn id="3" xr3:uid="{A77E13C5-CB25-43C0-9678-51A378FA64FC}" uniqueName="3" name="Column3" queryTableFieldId="3" dataDxfId="18"/>
-    <tableColumn id="4" xr3:uid="{46713ABC-AA6E-45DD-9BBE-03C863D6B1D1}" uniqueName="4" name="Column4" queryTableFieldId="4" dataDxfId="17"/>
-    <tableColumn id="5" xr3:uid="{85365AB6-280F-40C4-AB42-3455547D61F1}" uniqueName="5" name="Column5" queryTableFieldId="5" dataDxfId="16"/>
+    <tableColumn id="1" xr3:uid="{60EAA1C9-E43C-458C-A33C-365CF023541D}" uniqueName="1" name="Column1" queryTableFieldId="1" dataDxfId="21"/>
+    <tableColumn id="2" xr3:uid="{BF4ECEAF-8998-4833-A444-7DD2840947AB}" uniqueName="2" name="Column2" queryTableFieldId="2" dataDxfId="20"/>
+    <tableColumn id="3" xr3:uid="{A77E13C5-CB25-43C0-9678-51A378FA64FC}" uniqueName="3" name="Column3" queryTableFieldId="3" dataDxfId="19"/>
+    <tableColumn id="4" xr3:uid="{46713ABC-AA6E-45DD-9BBE-03C863D6B1D1}" uniqueName="4" name="Column4" queryTableFieldId="4" dataDxfId="18"/>
+    <tableColumn id="5" xr3:uid="{85365AB6-280F-40C4-AB42-3455547D61F1}" uniqueName="5" name="Column5" queryTableFieldId="5" dataDxfId="17"/>
   </tableColumns>
   <tableStyleInfo name="TableStyleMedium7" showFirstColumn="0" showLastColumn="0" showRowStripes="1" showColumnStripes="0"/>
 </table>
@@ -5353,11 +5356,11 @@
 <table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="21" xr:uid="{0B4290D5-7CEE-4DDC-B997-690EEF6D9589}" name="Table020__Page_11" displayName="Table020__Page_11" ref="A18:E20" tableType="queryTable" totalsRowShown="0">
   <autoFilter ref="A18:E20" xr:uid="{0B4290D5-7CEE-4DDC-B997-690EEF6D9589}"/>
   <tableColumns count="5">
-    <tableColumn id="1" xr3:uid="{344C3D84-8C5A-4C60-ADD3-4EE73F83858B}" uniqueName="1" name="Column1" queryTableFieldId="1" dataDxfId="15"/>
-    <tableColumn id="2" xr3:uid="{3470DF86-5A38-429A-95CF-F5FF5E59449C}" uniqueName="2" name="Column2" queryTableFieldId="2" dataDxfId="14"/>
-    <tableColumn id="3" xr3:uid="{BC1BD851-46F6-4634-95EE-ED117E75EBB6}" uniqueName="3" name="Column3" queryTableFieldId="3" dataDxfId="13"/>
-    <tableColumn id="4" xr3:uid="{FF5D3D34-BBDB-4113-8340-C737255ED1BD}" uniqueName="4" name="Column4" queryTableFieldId="4" dataDxfId="12"/>
-    <tableColumn id="5" xr3:uid="{F05FA152-C9D6-4773-B0A5-5B18B60C7102}" uniqueName="5" name="Column5" queryTableFieldId="5" dataDxfId="11"/>
+    <tableColumn id="1" xr3:uid="{344C3D84-8C5A-4C60-ADD3-4EE73F83858B}" uniqueName="1" name="Column1" queryTableFieldId="1" dataDxfId="16"/>
+    <tableColumn id="2" xr3:uid="{3470DF86-5A38-429A-95CF-F5FF5E59449C}" uniqueName="2" name="Column2" queryTableFieldId="2" dataDxfId="15"/>
+    <tableColumn id="3" xr3:uid="{BC1BD851-46F6-4634-95EE-ED117E75EBB6}" uniqueName="3" name="Column3" queryTableFieldId="3" dataDxfId="14"/>
+    <tableColumn id="4" xr3:uid="{FF5D3D34-BBDB-4113-8340-C737255ED1BD}" uniqueName="4" name="Column4" queryTableFieldId="4" dataDxfId="13"/>
+    <tableColumn id="5" xr3:uid="{F05FA152-C9D6-4773-B0A5-5B18B60C7102}" uniqueName="5" name="Column5" queryTableFieldId="5" dataDxfId="12"/>
   </tableColumns>
   <tableStyleInfo name="TableStyleMedium7" showFirstColumn="0" showLastColumn="0" showRowStripes="1" showColumnStripes="0"/>
 </table>
@@ -5367,13 +5370,13 @@
 <table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="2" xr:uid="{D4474760-F3B7-4070-AE77-2962D090A5AB}" name="Table002__Page_2" displayName="Table002__Page_2" ref="A19:G21" tableType="queryTable" totalsRowShown="0">
   <autoFilter ref="A19:G21" xr:uid="{D4474760-F3B7-4070-AE77-2962D090A5AB}"/>
   <tableColumns count="7">
-    <tableColumn id="1" xr3:uid="{8A3681DA-5FE9-4564-BCAB-75CCDF2C3A51}" uniqueName="1" name="Column1" queryTableFieldId="1" dataDxfId="135"/>
-    <tableColumn id="2" xr3:uid="{44D6563C-A88C-4FEE-9427-B5252DF8FA5D}" uniqueName="2" name="Column6" queryTableFieldId="2" dataDxfId="134"/>
-    <tableColumn id="3" xr3:uid="{2514D758-49E4-4E3E-A628-2B2D894F398E}" uniqueName="3" name="Column2" queryTableFieldId="3" dataDxfId="133"/>
-    <tableColumn id="4" xr3:uid="{062470EA-CB73-435C-8DF3-28DE262C8D69}" uniqueName="4" name="Column3" queryTableFieldId="4" dataDxfId="132"/>
-    <tableColumn id="5" xr3:uid="{CDE500EE-B268-43D9-A30D-9E6CC1608CD0}" uniqueName="5" name="Column4" queryTableFieldId="5" dataDxfId="131"/>
-    <tableColumn id="6" xr3:uid="{699F51E2-9A1B-4953-91BE-8D6434D76B20}" uniqueName="6" name="Column5" queryTableFieldId="6" dataDxfId="130"/>
-    <tableColumn id="7" xr3:uid="{C62D0670-E212-49FF-BA61-22C41F21B60E}" uniqueName="7" name="Column62" queryTableFieldId="7" dataDxfId="129"/>
+    <tableColumn id="1" xr3:uid="{8A3681DA-5FE9-4564-BCAB-75CCDF2C3A51}" uniqueName="1" name="Column1" queryTableFieldId="1" dataDxfId="136"/>
+    <tableColumn id="2" xr3:uid="{44D6563C-A88C-4FEE-9427-B5252DF8FA5D}" uniqueName="2" name="Column6" queryTableFieldId="2" dataDxfId="135"/>
+    <tableColumn id="3" xr3:uid="{2514D758-49E4-4E3E-A628-2B2D894F398E}" uniqueName="3" name="Column2" queryTableFieldId="3" dataDxfId="134"/>
+    <tableColumn id="4" xr3:uid="{062470EA-CB73-435C-8DF3-28DE262C8D69}" uniqueName="4" name="Column3" queryTableFieldId="4" dataDxfId="133"/>
+    <tableColumn id="5" xr3:uid="{CDE500EE-B268-43D9-A30D-9E6CC1608CD0}" uniqueName="5" name="Column4" queryTableFieldId="5" dataDxfId="132"/>
+    <tableColumn id="6" xr3:uid="{699F51E2-9A1B-4953-91BE-8D6434D76B20}" uniqueName="6" name="Column5" queryTableFieldId="6" dataDxfId="131"/>
+    <tableColumn id="7" xr3:uid="{C62D0670-E212-49FF-BA61-22C41F21B60E}" uniqueName="7" name="Column62" queryTableFieldId="7" dataDxfId="130"/>
   </tableColumns>
   <tableStyleInfo name="TableStyleMedium7" showFirstColumn="0" showLastColumn="0" showRowStripes="1" showColumnStripes="0"/>
 </table>
@@ -5383,14 +5386,14 @@
 <table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="3" xr:uid="{EE92A61D-8549-4453-B707-7BA76D39611E}" name="Table003__Page_3" displayName="Table003__Page_3" ref="A1:H16" tableType="queryTable" totalsRowShown="0">
   <autoFilter ref="A1:H16" xr:uid="{EE92A61D-8549-4453-B707-7BA76D39611E}"/>
   <tableColumns count="8">
-    <tableColumn id="1" xr3:uid="{5E78ED26-3040-4033-A95F-3AC09118D17C}" uniqueName="1" name="Column1" queryTableFieldId="1" dataDxfId="128"/>
-    <tableColumn id="2" xr3:uid="{52F60F93-88D4-4F60-A15A-4B2113E53BE2}" uniqueName="2" name="Column2" queryTableFieldId="2" dataDxfId="127"/>
-    <tableColumn id="3" xr3:uid="{2A66B2A9-165C-4995-937F-8E0D8B01B3D8}" uniqueName="3" name="Column3" queryTableFieldId="3" dataDxfId="126"/>
-    <tableColumn id="4" xr3:uid="{937ED0C3-8277-4EC6-BFD2-C6699696538D}" uniqueName="4" name="Column4" queryTableFieldId="4" dataDxfId="125"/>
-    <tableColumn id="5" xr3:uid="{37EAAABA-4FEF-4D28-B237-360AD0A7194A}" uniqueName="5" name="Column5" queryTableFieldId="5" dataDxfId="124"/>
-    <tableColumn id="6" xr3:uid="{6E7D50A0-6329-4797-9F9A-628D251C7CA5}" uniqueName="6" name="Column6" queryTableFieldId="6" dataDxfId="123"/>
-    <tableColumn id="7" xr3:uid="{F8F31C01-9522-488B-915F-110987168D09}" uniqueName="7" name="Column7" queryTableFieldId="7" dataDxfId="122"/>
-    <tableColumn id="8" xr3:uid="{FFD35FDD-AAE7-4F54-8AF3-197380BC0AEB}" uniqueName="8" name="Column8" queryTableFieldId="8" dataDxfId="121"/>
+    <tableColumn id="1" xr3:uid="{5E78ED26-3040-4033-A95F-3AC09118D17C}" uniqueName="1" name="Column1" queryTableFieldId="1" dataDxfId="129"/>
+    <tableColumn id="2" xr3:uid="{52F60F93-88D4-4F60-A15A-4B2113E53BE2}" uniqueName="2" name="Column2" queryTableFieldId="2" dataDxfId="128"/>
+    <tableColumn id="3" xr3:uid="{2A66B2A9-165C-4995-937F-8E0D8B01B3D8}" uniqueName="3" name="Column3" queryTableFieldId="3" dataDxfId="127"/>
+    <tableColumn id="4" xr3:uid="{937ED0C3-8277-4EC6-BFD2-C6699696538D}" uniqueName="4" name="Column4" queryTableFieldId="4" dataDxfId="126"/>
+    <tableColumn id="5" xr3:uid="{37EAAABA-4FEF-4D28-B237-360AD0A7194A}" uniqueName="5" name="Column5" queryTableFieldId="5" dataDxfId="125"/>
+    <tableColumn id="6" xr3:uid="{6E7D50A0-6329-4797-9F9A-628D251C7CA5}" uniqueName="6" name="Column6" queryTableFieldId="6" dataDxfId="124"/>
+    <tableColumn id="7" xr3:uid="{F8F31C01-9522-488B-915F-110987168D09}" uniqueName="7" name="Column7" queryTableFieldId="7" dataDxfId="123"/>
+    <tableColumn id="8" xr3:uid="{FFD35FDD-AAE7-4F54-8AF3-197380BC0AEB}" uniqueName="8" name="Column8" queryTableFieldId="8" dataDxfId="122"/>
   </tableColumns>
   <tableStyleInfo name="TableStyleMedium7" showFirstColumn="0" showLastColumn="0" showRowStripes="1" showColumnStripes="0"/>
 </table>
@@ -5400,14 +5403,14 @@
 <table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="4" xr:uid="{1C7E55B7-7D73-418F-9229-407F52A253A6}" name="Table004__Page_3" displayName="Table004__Page_3" ref="A18:H20" tableType="queryTable" totalsRowShown="0">
   <autoFilter ref="A18:H20" xr:uid="{1C7E55B7-7D73-418F-9229-407F52A253A6}"/>
   <tableColumns count="8">
-    <tableColumn id="1" xr3:uid="{A8A6FCCE-AE43-4EDA-82DC-831809E03401}" uniqueName="1" name="Column1" queryTableFieldId="1" dataDxfId="120"/>
-    <tableColumn id="2" xr3:uid="{0231594E-DA9E-47DE-A01C-22488210A4CF}" uniqueName="2" name="Column2" queryTableFieldId="2" dataDxfId="119"/>
-    <tableColumn id="3" xr3:uid="{7A06306A-69AF-482D-910F-86D0EF88F740}" uniqueName="3" name="Column3" queryTableFieldId="3" dataDxfId="118"/>
-    <tableColumn id="4" xr3:uid="{E96F3603-E9D2-4710-BDE5-6FE3E6A378D8}" uniqueName="4" name="Column4" queryTableFieldId="4" dataDxfId="117"/>
-    <tableColumn id="5" xr3:uid="{37151140-CC9F-4EBB-B58D-F87E1081314A}" uniqueName="5" name="Column5" queryTableFieldId="5" dataDxfId="116"/>
-    <tableColumn id="6" xr3:uid="{F0AAEEC2-014D-412A-B58D-24C71FEC9A66}" uniqueName="6" name="Column6" queryTableFieldId="6" dataDxfId="115"/>
-    <tableColumn id="7" xr3:uid="{A4B4F3F0-B14D-498F-B185-AA3E2BAE729A}" uniqueName="7" name="Column7" queryTableFieldId="7" dataDxfId="114"/>
-    <tableColumn id="8" xr3:uid="{0C517BB9-44A4-4BBA-AA88-B86BB679F208}" uniqueName="8" name="Column8" queryTableFieldId="8" dataDxfId="113"/>
+    <tableColumn id="1" xr3:uid="{A8A6FCCE-AE43-4EDA-82DC-831809E03401}" uniqueName="1" name="Column1" queryTableFieldId="1" dataDxfId="121"/>
+    <tableColumn id="2" xr3:uid="{0231594E-DA9E-47DE-A01C-22488210A4CF}" uniqueName="2" name="Column2" queryTableFieldId="2" dataDxfId="120"/>
+    <tableColumn id="3" xr3:uid="{7A06306A-69AF-482D-910F-86D0EF88F740}" uniqueName="3" name="Column3" queryTableFieldId="3" dataDxfId="119"/>
+    <tableColumn id="4" xr3:uid="{E96F3603-E9D2-4710-BDE5-6FE3E6A378D8}" uniqueName="4" name="Column4" queryTableFieldId="4" dataDxfId="118"/>
+    <tableColumn id="5" xr3:uid="{37151140-CC9F-4EBB-B58D-F87E1081314A}" uniqueName="5" name="Column5" queryTableFieldId="5" dataDxfId="117"/>
+    <tableColumn id="6" xr3:uid="{F0AAEEC2-014D-412A-B58D-24C71FEC9A66}" uniqueName="6" name="Column6" queryTableFieldId="6" dataDxfId="116"/>
+    <tableColumn id="7" xr3:uid="{A4B4F3F0-B14D-498F-B185-AA3E2BAE729A}" uniqueName="7" name="Column7" queryTableFieldId="7" dataDxfId="115"/>
+    <tableColumn id="8" xr3:uid="{0C517BB9-44A4-4BBA-AA88-B86BB679F208}" uniqueName="8" name="Column8" queryTableFieldId="8" dataDxfId="114"/>
   </tableColumns>
   <tableStyleInfo name="TableStyleMedium7" showFirstColumn="0" showLastColumn="0" showRowStripes="1" showColumnStripes="0"/>
 </table>
@@ -5417,12 +5420,12 @@
 <table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="5" xr:uid="{2EB30D60-3074-4922-8217-6B97953C0F87}" name="Table005__Page_4" displayName="Table005__Page_4" ref="A1:F16" tableType="queryTable" totalsRowShown="0">
   <autoFilter ref="A1:F16" xr:uid="{2EB30D60-3074-4922-8217-6B97953C0F87}"/>
   <tableColumns count="6">
-    <tableColumn id="1" xr3:uid="{AB42FEA9-5A85-4A69-B46D-444C53C4B4EF}" uniqueName="1" name="Column1" queryTableFieldId="1" dataDxfId="112"/>
-    <tableColumn id="2" xr3:uid="{0D7919B1-FB5E-4192-8675-3D57B39D9AB0}" uniqueName="2" name="Column2" queryTableFieldId="2" dataDxfId="111"/>
-    <tableColumn id="3" xr3:uid="{94F12F3D-88BF-4BEB-85E7-FF6313F6B88E}" uniqueName="3" name="Column3" queryTableFieldId="3" dataDxfId="110"/>
-    <tableColumn id="4" xr3:uid="{2B04EEA3-DC55-4C69-860F-9571D35E352D}" uniqueName="4" name="Column4" queryTableFieldId="4" dataDxfId="109"/>
-    <tableColumn id="5" xr3:uid="{461C5084-182B-40CC-B479-24798E48D0F4}" uniqueName="5" name="Column5" queryTableFieldId="5" dataDxfId="108"/>
-    <tableColumn id="6" xr3:uid="{258F7EB6-7345-43CA-BF8A-5E088D06FF8F}" uniqueName="6" name="Column6" queryTableFieldId="6" dataDxfId="107"/>
+    <tableColumn id="1" xr3:uid="{AB42FEA9-5A85-4A69-B46D-444C53C4B4EF}" uniqueName="1" name="Column1" queryTableFieldId="1" dataDxfId="113"/>
+    <tableColumn id="2" xr3:uid="{0D7919B1-FB5E-4192-8675-3D57B39D9AB0}" uniqueName="2" name="Column2" queryTableFieldId="2" dataDxfId="112"/>
+    <tableColumn id="3" xr3:uid="{94F12F3D-88BF-4BEB-85E7-FF6313F6B88E}" uniqueName="3" name="Column3" queryTableFieldId="3" dataDxfId="111"/>
+    <tableColumn id="4" xr3:uid="{2B04EEA3-DC55-4C69-860F-9571D35E352D}" uniqueName="4" name="Column4" queryTableFieldId="4" dataDxfId="110"/>
+    <tableColumn id="5" xr3:uid="{461C5084-182B-40CC-B479-24798E48D0F4}" uniqueName="5" name="Column5" queryTableFieldId="5" dataDxfId="109"/>
+    <tableColumn id="6" xr3:uid="{258F7EB6-7345-43CA-BF8A-5E088D06FF8F}" uniqueName="6" name="Column6" queryTableFieldId="6" dataDxfId="108"/>
   </tableColumns>
   <tableStyleInfo name="TableStyleMedium7" showFirstColumn="0" showLastColumn="0" showRowStripes="1" showColumnStripes="0"/>
 </table>
@@ -5432,12 +5435,12 @@
 <table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="6" xr:uid="{BA3E356C-A98F-4646-B7E8-7B0C3904E2A4}" name="Table006__Page_4" displayName="Table006__Page_4" ref="A18:F20" tableType="queryTable" totalsRowShown="0">
   <autoFilter ref="A18:F20" xr:uid="{BA3E356C-A98F-4646-B7E8-7B0C3904E2A4}"/>
   <tableColumns count="6">
-    <tableColumn id="1" xr3:uid="{55987721-40E8-4E11-9B6F-67EE503D78F4}" uniqueName="1" name="Column1" queryTableFieldId="1" dataDxfId="106"/>
-    <tableColumn id="2" xr3:uid="{15260D47-39CC-4501-9656-F8DBE6AD3AB1}" uniqueName="2" name="Column2" queryTableFieldId="2" dataDxfId="105"/>
-    <tableColumn id="3" xr3:uid="{06C8B30C-3DD3-49E6-8BE6-C8A9D39F2FC4}" uniqueName="3" name="Column3" queryTableFieldId="3" dataDxfId="104"/>
-    <tableColumn id="4" xr3:uid="{40A070F6-4BDB-49A7-9394-4D63F3A9E318}" uniqueName="4" name="Column4" queryTableFieldId="4" dataDxfId="103"/>
-    <tableColumn id="5" xr3:uid="{C5E0BAEF-796C-4C71-ACA7-889E63543C2D}" uniqueName="5" name="Column5" queryTableFieldId="5" dataDxfId="102"/>
-    <tableColumn id="6" xr3:uid="{1BA75280-A961-41F1-B113-5935891BA00A}" uniqueName="6" name="Column6" queryTableFieldId="6" dataDxfId="101"/>
+    <tableColumn id="1" xr3:uid="{55987721-40E8-4E11-9B6F-67EE503D78F4}" uniqueName="1" name="Column1" queryTableFieldId="1" dataDxfId="107"/>
+    <tableColumn id="2" xr3:uid="{15260D47-39CC-4501-9656-F8DBE6AD3AB1}" uniqueName="2" name="Column2" queryTableFieldId="2" dataDxfId="106"/>
+    <tableColumn id="3" xr3:uid="{06C8B30C-3DD3-49E6-8BE6-C8A9D39F2FC4}" uniqueName="3" name="Column3" queryTableFieldId="3" dataDxfId="105"/>
+    <tableColumn id="4" xr3:uid="{40A070F6-4BDB-49A7-9394-4D63F3A9E318}" uniqueName="4" name="Column4" queryTableFieldId="4" dataDxfId="104"/>
+    <tableColumn id="5" xr3:uid="{C5E0BAEF-796C-4C71-ACA7-889E63543C2D}" uniqueName="5" name="Column5" queryTableFieldId="5" dataDxfId="103"/>
+    <tableColumn id="6" xr3:uid="{1BA75280-A961-41F1-B113-5935891BA00A}" uniqueName="6" name="Column6" queryTableFieldId="6" dataDxfId="102"/>
   </tableColumns>
   <tableStyleInfo name="TableStyleMedium7" showFirstColumn="0" showLastColumn="0" showRowStripes="1" showColumnStripes="0"/>
 </table>
@@ -5447,18 +5450,18 @@
 <table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="7" xr:uid="{6040FF08-DFFC-4D6C-87C0-7C33D5281777}" name="Table007__Page_5" displayName="Table007__Page_5" ref="A1:L16" tableType="queryTable" totalsRowShown="0">
   <autoFilter ref="A1:L16" xr:uid="{6040FF08-DFFC-4D6C-87C0-7C33D5281777}"/>
   <tableColumns count="12">
-    <tableColumn id="1" xr3:uid="{9561388E-64AE-4A76-863E-A0B2091E2F9F}" uniqueName="1" name="Column1" queryTableFieldId="1" dataDxfId="100"/>
-    <tableColumn id="2" xr3:uid="{151810A9-7DD3-4FD0-91D6-6608DF85A8CF}" uniqueName="2" name="Column2" queryTableFieldId="2" dataDxfId="99"/>
-    <tableColumn id="3" xr3:uid="{94D629BF-F745-493D-8F74-FA7EEFDEAA84}" uniqueName="3" name="Column3" queryTableFieldId="3" dataDxfId="98"/>
-    <tableColumn id="4" xr3:uid="{AE87299A-170F-4661-BD08-B108394E2F7C}" uniqueName="4" name="Column4" queryTableFieldId="4" dataDxfId="97"/>
-    <tableColumn id="5" xr3:uid="{708CB468-5E3F-4D0C-B6BD-C2C44C7191EC}" uniqueName="5" name="Column5" queryTableFieldId="5" dataDxfId="96"/>
-    <tableColumn id="6" xr3:uid="{5D4BD3CB-C344-4155-B3C1-ECC49F86CED1}" uniqueName="6" name="Column6" queryTableFieldId="6" dataDxfId="95"/>
-    <tableColumn id="7" xr3:uid="{61DF1122-5C54-47A3-98F9-27CA1B50CA9D}" uniqueName="7" name="Column7" queryTableFieldId="7" dataDxfId="94"/>
-    <tableColumn id="8" xr3:uid="{130590EE-DDCB-43DB-A020-385B521DA018}" uniqueName="8" name="Column8" queryTableFieldId="8" dataDxfId="93"/>
-    <tableColumn id="9" xr3:uid="{06B903F7-5E22-476D-A116-655599D2C518}" uniqueName="9" name="Column9" queryTableFieldId="9" dataDxfId="92"/>
-    <tableColumn id="10" xr3:uid="{CED96D55-8B0D-492D-B0EC-F3E56EFB2649}" uniqueName="10" name="Column10" queryTableFieldId="10" dataDxfId="91"/>
-    <tableColumn id="11" xr3:uid="{346823E9-F305-4F11-941F-1C42A8AB0C99}" uniqueName="11" name="Column11" queryTableFieldId="11" dataDxfId="90"/>
-    <tableColumn id="12" xr3:uid="{7B421AA8-C9DB-4E35-A456-DF0F56050B79}" uniqueName="12" name="Column12" queryTableFieldId="12" dataDxfId="89"/>
+    <tableColumn id="1" xr3:uid="{9561388E-64AE-4A76-863E-A0B2091E2F9F}" uniqueName="1" name="Column1" queryTableFieldId="1" dataDxfId="101"/>
+    <tableColumn id="2" xr3:uid="{151810A9-7DD3-4FD0-91D6-6608DF85A8CF}" uniqueName="2" name="Column2" queryTableFieldId="2" dataDxfId="100"/>
+    <tableColumn id="3" xr3:uid="{94D629BF-F745-493D-8F74-FA7EEFDEAA84}" uniqueName="3" name="Column3" queryTableFieldId="3" dataDxfId="99"/>
+    <tableColumn id="4" xr3:uid="{AE87299A-170F-4661-BD08-B108394E2F7C}" uniqueName="4" name="Column4" queryTableFieldId="4" dataDxfId="98"/>
+    <tableColumn id="5" xr3:uid="{708CB468-5E3F-4D0C-B6BD-C2C44C7191EC}" uniqueName="5" name="Column5" queryTableFieldId="5" dataDxfId="97"/>
+    <tableColumn id="6" xr3:uid="{5D4BD3CB-C344-4155-B3C1-ECC49F86CED1}" uniqueName="6" name="Column6" queryTableFieldId="6" dataDxfId="96"/>
+    <tableColumn id="7" xr3:uid="{61DF1122-5C54-47A3-98F9-27CA1B50CA9D}" uniqueName="7" name="Column7" queryTableFieldId="7" dataDxfId="95"/>
+    <tableColumn id="8" xr3:uid="{130590EE-DDCB-43DB-A020-385B521DA018}" uniqueName="8" name="Column8" queryTableFieldId="8" dataDxfId="94"/>
+    <tableColumn id="9" xr3:uid="{06B903F7-5E22-476D-A116-655599D2C518}" uniqueName="9" name="Column9" queryTableFieldId="9" dataDxfId="93"/>
+    <tableColumn id="10" xr3:uid="{CED96D55-8B0D-492D-B0EC-F3E56EFB2649}" uniqueName="10" name="Column10" queryTableFieldId="10" dataDxfId="92"/>
+    <tableColumn id="11" xr3:uid="{346823E9-F305-4F11-941F-1C42A8AB0C99}" uniqueName="11" name="Column11" queryTableFieldId="11" dataDxfId="91"/>
+    <tableColumn id="12" xr3:uid="{7B421AA8-C9DB-4E35-A456-DF0F56050B79}" uniqueName="12" name="Column12" queryTableFieldId="12" dataDxfId="90"/>
   </tableColumns>
   <tableStyleInfo name="TableStyleMedium7" showFirstColumn="0" showLastColumn="0" showRowStripes="1" showColumnStripes="0"/>
 </table>
@@ -5468,18 +5471,18 @@
 <table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="8" xr:uid="{DBF54861-4823-4965-9BF8-BF4D83A85FD1}" name="Table008__Page_5" displayName="Table008__Page_5" ref="A18:L20" tableType="queryTable" totalsRowShown="0">
   <autoFilter ref="A18:L20" xr:uid="{DBF54861-4823-4965-9BF8-BF4D83A85FD1}"/>
   <tableColumns count="12">
-    <tableColumn id="1" xr3:uid="{01D3C90B-BA67-46B4-BD1D-5C53486CAE57}" uniqueName="1" name="Column1" queryTableFieldId="1" dataDxfId="88"/>
-    <tableColumn id="2" xr3:uid="{166854EB-0B50-4420-BB3F-7A5A2C9FB7F7}" uniqueName="2" name="Column2" queryTableFieldId="2" dataDxfId="87"/>
-    <tableColumn id="3" xr3:uid="{638857E5-1EB4-4FBE-9FFE-2951F2F4ABD0}" uniqueName="3" name="Column3" queryTableFieldId="3" dataDxfId="86"/>
-    <tableColumn id="4" xr3:uid="{F4EFE2EF-AC84-40F8-BE68-0B6B520F8EA8}" uniqueName="4" name="Column4" queryTableFieldId="4" dataDxfId="85"/>
-    <tableColumn id="5" xr3:uid="{38D026D2-A47E-46EA-BA10-AF890A55BF2B}" uniqueName="5" name="Column5" queryTableFieldId="5" dataDxfId="84"/>
-    <tableColumn id="6" xr3:uid="{025C6DA2-37A6-491F-904E-DDE12948D35B}" uniqueName="6" name="Column6" queryTableFieldId="6" dataDxfId="83"/>
-    <tableColumn id="7" xr3:uid="{AC28B573-67B7-4468-A6A2-F648D17079B6}" uniqueName="7" name="Column7" queryTableFieldId="7" dataDxfId="82"/>
-    <tableColumn id="8" xr3:uid="{F6F06554-210B-472F-95F2-8E89D931E4C1}" uniqueName="8" name="Column8" queryTableFieldId="8" dataDxfId="81"/>
-    <tableColumn id="9" xr3:uid="{F0A8F323-36C1-4290-980B-8F6F5DC6A41E}" uniqueName="9" name="Column9" queryTableFieldId="9" dataDxfId="80"/>
-    <tableColumn id="10" xr3:uid="{25D60007-5007-4174-85F5-572E3C29FE33}" uniqueName="10" name="Column10" queryTableFieldId="10" dataDxfId="79"/>
-    <tableColumn id="11" xr3:uid="{2071EB9B-B14E-4EF0-9B86-0D5FDA96828D}" uniqueName="11" name="Column11" queryTableFieldId="11" dataDxfId="78"/>
-    <tableColumn id="12" xr3:uid="{1660C180-EE6B-48E8-9880-55F02CC623C4}" uniqueName="12" name="Column12" queryTableFieldId="12" dataDxfId="77"/>
+    <tableColumn id="1" xr3:uid="{01D3C90B-BA67-46B4-BD1D-5C53486CAE57}" uniqueName="1" name="Column1" queryTableFieldId="1" dataDxfId="89"/>
+    <tableColumn id="2" xr3:uid="{166854EB-0B50-4420-BB3F-7A5A2C9FB7F7}" uniqueName="2" name="Column2" queryTableFieldId="2" dataDxfId="88"/>
+    <tableColumn id="3" xr3:uid="{638857E5-1EB4-4FBE-9FFE-2951F2F4ABD0}" uniqueName="3" name="Column3" queryTableFieldId="3" dataDxfId="87"/>
+    <tableColumn id="4" xr3:uid="{F4EFE2EF-AC84-40F8-BE68-0B6B520F8EA8}" uniqueName="4" name="Column4" queryTableFieldId="4" dataDxfId="86"/>
+    <tableColumn id="5" xr3:uid="{38D026D2-A47E-46EA-BA10-AF890A55BF2B}" uniqueName="5" name="Column5" queryTableFieldId="5" dataDxfId="85"/>
+    <tableColumn id="6" xr3:uid="{025C6DA2-37A6-491F-904E-DDE12948D35B}" uniqueName="6" name="Column6" queryTableFieldId="6" dataDxfId="84"/>
+    <tableColumn id="7" xr3:uid="{AC28B573-67B7-4468-A6A2-F648D17079B6}" uniqueName="7" name="Column7" queryTableFieldId="7" dataDxfId="83"/>
+    <tableColumn id="8" xr3:uid="{F6F06554-210B-472F-95F2-8E89D931E4C1}" uniqueName="8" name="Column8" queryTableFieldId="8" dataDxfId="82"/>
+    <tableColumn id="9" xr3:uid="{F0A8F323-36C1-4290-980B-8F6F5DC6A41E}" uniqueName="9" name="Column9" queryTableFieldId="9" dataDxfId="81"/>
+    <tableColumn id="10" xr3:uid="{25D60007-5007-4174-85F5-572E3C29FE33}" uniqueName="10" name="Column10" queryTableFieldId="10" dataDxfId="80"/>
+    <tableColumn id="11" xr3:uid="{2071EB9B-B14E-4EF0-9B86-0D5FDA96828D}" uniqueName="11" name="Column11" queryTableFieldId="11" dataDxfId="79"/>
+    <tableColumn id="12" xr3:uid="{1660C180-EE6B-48E8-9880-55F02CC623C4}" uniqueName="12" name="Column12" queryTableFieldId="12" dataDxfId="78"/>
   </tableColumns>
   <tableStyleInfo name="TableStyleMedium7" showFirstColumn="0" showLastColumn="0" showRowStripes="1" showColumnStripes="0"/>
 </table>
@@ -5856,16 +5859,16 @@
       <c r="C2" s="5">
         <v>214000000</v>
       </c>
-      <c r="D2" s="5">
-        <f t="shared" ref="D2:D35" si="0">I2/1.12</f>
+      <c r="D2" s="9">
+        <f>I2/1.12</f>
         <v>18750000</v>
       </c>
       <c r="E2" s="5">
-        <f t="shared" ref="E2:E35" si="1">D2*90%</f>
+        <f t="shared" ref="E2:E35" si="0">D2*90%</f>
         <v>16875000</v>
       </c>
       <c r="F2" s="5">
-        <f t="shared" ref="F2:F35" si="2">D2*70%</f>
+        <f t="shared" ref="F2:F35" si="1">D2*70%</f>
         <v>13125000</v>
       </c>
       <c r="G2" s="3">
@@ -5888,16 +5891,16 @@
       <c r="C3" s="5">
         <v>251000000</v>
       </c>
-      <c r="D3" s="5">
+      <c r="D3" s="9">
+        <f t="shared" ref="D3:D33" si="2">I3/1.12</f>
+        <v>18750000</v>
+      </c>
+      <c r="E3" s="5">
         <f t="shared" si="0"/>
-        <v>18750000</v>
-      </c>
-      <c r="E3" s="5">
+        <v>16875000</v>
+      </c>
+      <c r="F3" s="5">
         <f t="shared" si="1"/>
-        <v>16875000</v>
-      </c>
-      <c r="F3" s="5">
-        <f t="shared" si="2"/>
         <v>13125000</v>
       </c>
       <c r="G3" s="3">
@@ -5920,16 +5923,16 @@
       <c r="C4" s="5">
         <v>251000000</v>
       </c>
-      <c r="D4" s="5">
+      <c r="D4" s="9">
+        <f t="shared" si="2"/>
+        <v>18750000</v>
+      </c>
+      <c r="E4" s="5">
         <f t="shared" si="0"/>
-        <v>18750000</v>
-      </c>
-      <c r="E4" s="5">
+        <v>16875000</v>
+      </c>
+      <c r="F4" s="5">
         <f t="shared" si="1"/>
-        <v>16875000</v>
-      </c>
-      <c r="F4" s="5">
-        <f t="shared" si="2"/>
         <v>13125000</v>
       </c>
       <c r="G4" s="3">
@@ -5952,16 +5955,16 @@
       <c r="C5" s="5">
         <v>251000000</v>
       </c>
-      <c r="D5" s="5">
+      <c r="D5" s="9">
+        <f t="shared" si="2"/>
+        <v>18750000</v>
+      </c>
+      <c r="E5" s="5">
         <f t="shared" si="0"/>
-        <v>18750000</v>
-      </c>
-      <c r="E5" s="5">
+        <v>16875000</v>
+      </c>
+      <c r="F5" s="5">
         <f t="shared" si="1"/>
-        <v>16875000</v>
-      </c>
-      <c r="F5" s="5">
-        <f t="shared" si="2"/>
         <v>13125000</v>
       </c>
       <c r="G5" s="3">
@@ -5984,16 +5987,16 @@
       <c r="C6" s="5">
         <v>307500000</v>
       </c>
-      <c r="D6" s="5">
+      <c r="D6" s="9">
+        <f t="shared" si="2"/>
+        <v>22321428.571428567</v>
+      </c>
+      <c r="E6" s="5">
         <f t="shared" si="0"/>
-        <v>22321428.571428567</v>
-      </c>
-      <c r="E6" s="5">
+        <v>20089285.714285713</v>
+      </c>
+      <c r="F6" s="5">
         <f t="shared" si="1"/>
-        <v>20089285.714285713</v>
-      </c>
-      <c r="F6" s="5">
-        <f t="shared" si="2"/>
         <v>15624999.999999996</v>
       </c>
       <c r="G6" s="3">
@@ -6016,16 +6019,16 @@
       <c r="C7" s="5">
         <v>311500000</v>
       </c>
-      <c r="D7" s="5">
+      <c r="D7" s="9">
+        <f t="shared" si="2"/>
+        <v>20758928.571428567</v>
+      </c>
+      <c r="E7" s="5">
         <f t="shared" si="0"/>
-        <v>20758928.571428567</v>
-      </c>
-      <c r="E7" s="5">
+        <v>18683035.714285713</v>
+      </c>
+      <c r="F7" s="5">
         <f t="shared" si="1"/>
-        <v>18683035.714285713</v>
-      </c>
-      <c r="F7" s="5">
-        <f t="shared" si="2"/>
         <v>14531249.999999996</v>
       </c>
       <c r="G7" s="7">
@@ -6048,16 +6051,16 @@
       <c r="C8" s="5">
         <v>329050000</v>
       </c>
-      <c r="D8" s="5">
+      <c r="D8" s="9">
+        <f t="shared" si="2"/>
+        <v>22053571.428571429</v>
+      </c>
+      <c r="E8" s="5">
         <f t="shared" si="0"/>
-        <v>22053571.428571429</v>
-      </c>
-      <c r="E8" s="5">
+        <v>19848214.285714287</v>
+      </c>
+      <c r="F8" s="5">
         <f t="shared" si="1"/>
-        <v>19848214.285714287</v>
-      </c>
-      <c r="F8" s="5">
-        <f t="shared" si="2"/>
         <v>15437500</v>
       </c>
       <c r="G8" s="7">
@@ -6080,16 +6083,16 @@
       <c r="C9" s="5">
         <v>388500000</v>
       </c>
-      <c r="D9" s="5">
+      <c r="D9" s="9">
+        <f t="shared" si="2"/>
+        <v>29464285.714285709</v>
+      </c>
+      <c r="E9" s="5">
         <f t="shared" si="0"/>
-        <v>29464285.714285709</v>
-      </c>
-      <c r="E9" s="5">
+        <v>26517857.142857138</v>
+      </c>
+      <c r="F9" s="5">
         <f t="shared" si="1"/>
-        <v>26517857.142857138</v>
-      </c>
-      <c r="F9" s="5">
-        <f t="shared" si="2"/>
         <v>20624999.999999996</v>
       </c>
       <c r="G9" s="7">
@@ -6112,16 +6115,16 @@
       <c r="C10" s="5">
         <v>447200000</v>
       </c>
-      <c r="D10" s="5">
+      <c r="D10" s="9">
+        <f t="shared" si="2"/>
+        <v>31249999.999999996</v>
+      </c>
+      <c r="E10" s="5">
         <f t="shared" si="0"/>
-        <v>31249999.999999996</v>
-      </c>
-      <c r="E10" s="5">
+        <v>28124999.999999996</v>
+      </c>
+      <c r="F10" s="5">
         <f t="shared" si="1"/>
-        <v>28124999.999999996</v>
-      </c>
-      <c r="F10" s="5">
-        <f t="shared" si="2"/>
         <v>21874999.999999996</v>
       </c>
       <c r="G10" s="7">
@@ -6144,16 +6147,16 @@
       <c r="C11" s="5">
         <v>405000000</v>
       </c>
-      <c r="D11" s="5">
+      <c r="D11" s="9">
+        <f t="shared" si="2"/>
+        <v>31249999.999999996</v>
+      </c>
+      <c r="E11" s="5">
         <f t="shared" si="0"/>
-        <v>31249999.999999996</v>
-      </c>
-      <c r="E11" s="5">
+        <v>28124999.999999996</v>
+      </c>
+      <c r="F11" s="5">
         <f t="shared" si="1"/>
-        <v>28124999.999999996</v>
-      </c>
-      <c r="F11" s="5">
-        <f t="shared" si="2"/>
         <v>21874999.999999996</v>
       </c>
       <c r="G11" s="7">
@@ -6176,16 +6179,16 @@
       <c r="C12" s="5">
         <v>442000000</v>
       </c>
-      <c r="D12" s="5">
+      <c r="D12" s="9">
+        <f t="shared" si="2"/>
+        <v>33928571.428571425</v>
+      </c>
+      <c r="E12" s="5">
         <f t="shared" si="0"/>
-        <v>33928571.428571425</v>
-      </c>
-      <c r="E12" s="5">
+        <v>30535714.285714284</v>
+      </c>
+      <c r="F12" s="5">
         <f t="shared" si="1"/>
-        <v>30535714.285714284</v>
-      </c>
-      <c r="F12" s="5">
-        <f t="shared" si="2"/>
         <v>23749999.999999996</v>
       </c>
       <c r="G12" s="7">
@@ -6208,16 +6211,16 @@
       <c r="C13" s="5">
         <v>303000000</v>
       </c>
-      <c r="D13" s="5">
+      <c r="D13" s="9">
+        <f t="shared" si="2"/>
+        <v>20535714.285714284</v>
+      </c>
+      <c r="E13" s="5">
         <f t="shared" si="0"/>
-        <v>20535714.285714284</v>
-      </c>
-      <c r="E13" s="5">
+        <v>18482142.857142854</v>
+      </c>
+      <c r="F13" s="5">
         <f t="shared" si="1"/>
-        <v>18482142.857142854</v>
-      </c>
-      <c r="F13" s="5">
-        <f t="shared" si="2"/>
         <v>14374999.999999998</v>
       </c>
       <c r="G13" s="3">
@@ -6240,16 +6243,16 @@
       <c r="C14" s="5">
         <v>263000000</v>
       </c>
-      <c r="D14" s="5">
+      <c r="D14" s="9">
+        <f t="shared" si="2"/>
+        <v>17857142.857142854</v>
+      </c>
+      <c r="E14" s="5">
         <f t="shared" si="0"/>
-        <v>17857142.857142854</v>
-      </c>
-      <c r="E14" s="5">
+        <v>16071428.571428569</v>
+      </c>
+      <c r="F14" s="5">
         <f t="shared" si="1"/>
-        <v>16071428.571428569</v>
-      </c>
-      <c r="F14" s="5">
-        <f t="shared" si="2"/>
         <v>12499999.999999998</v>
       </c>
       <c r="G14" s="3">
@@ -6272,16 +6275,16 @@
       <c r="C15" s="5">
         <v>217000000</v>
       </c>
-      <c r="D15" s="5">
+      <c r="D15" s="9">
+        <f t="shared" si="2"/>
+        <v>11607142.857142856</v>
+      </c>
+      <c r="E15" s="5">
         <f t="shared" si="0"/>
-        <v>11607142.857142856</v>
-      </c>
-      <c r="E15" s="5">
+        <v>10446428.571428571</v>
+      </c>
+      <c r="F15" s="5">
         <f t="shared" si="1"/>
-        <v>10446428.571428571</v>
-      </c>
-      <c r="F15" s="5">
-        <f t="shared" si="2"/>
         <v>8124999.9999999991</v>
       </c>
       <c r="G15" s="3">
@@ -6304,16 +6307,16 @@
       <c r="C16" s="5">
         <v>217000000</v>
       </c>
-      <c r="D16" s="5">
+      <c r="D16" s="9">
+        <f t="shared" si="2"/>
+        <v>11607142.857142856</v>
+      </c>
+      <c r="E16" s="5">
         <f t="shared" si="0"/>
-        <v>11607142.857142856</v>
-      </c>
-      <c r="E16" s="5">
+        <v>10446428.571428571</v>
+      </c>
+      <c r="F16" s="5">
         <f t="shared" si="1"/>
-        <v>10446428.571428571</v>
-      </c>
-      <c r="F16" s="5">
-        <f t="shared" si="2"/>
         <v>8124999.9999999991</v>
       </c>
       <c r="G16" s="3">
@@ -6336,16 +6339,16 @@
       <c r="C17" s="5">
         <v>263000000</v>
       </c>
-      <c r="D17" s="5">
-        <f t="shared" ref="D17" si="3">I17/1.12</f>
+      <c r="D17" s="9">
+        <f t="shared" si="2"/>
         <v>17857142.857142854</v>
       </c>
       <c r="E17" s="5">
-        <f t="shared" si="1"/>
+        <f t="shared" si="0"/>
         <v>16071428.571428569</v>
       </c>
       <c r="F17" s="5">
-        <f t="shared" ref="F17" si="4">D17*70%</f>
+        <f t="shared" ref="F17" si="3">D17*70%</f>
         <v>12499999.999999998</v>
       </c>
       <c r="G17" s="3">
@@ -6368,16 +6371,16 @@
       <c r="C18" s="9">
         <v>303000000</v>
       </c>
-      <c r="D18" s="5">
-        <f t="shared" ref="D18" si="5">I18/1.12</f>
+      <c r="D18" s="9">
+        <f t="shared" si="2"/>
         <v>20535714.285714284</v>
       </c>
       <c r="E18" s="5">
-        <f t="shared" si="1"/>
+        <f t="shared" si="0"/>
         <v>18482142.857142854</v>
       </c>
       <c r="F18" s="5">
-        <f t="shared" ref="F18" si="6">D18*70%</f>
+        <f t="shared" ref="F18" si="4">D18*70%</f>
         <v>14374999.999999998</v>
       </c>
       <c r="G18" s="3">
@@ -6400,16 +6403,16 @@
       <c r="C19" s="5">
         <v>353000000</v>
       </c>
-      <c r="D19" s="5">
+      <c r="D19" s="9">
+        <f t="shared" si="2"/>
+        <v>25892857.142857142</v>
+      </c>
+      <c r="E19" s="5">
         <f t="shared" si="0"/>
-        <v>25892857.142857142</v>
-      </c>
-      <c r="E19" s="5">
+        <v>23303571.428571429</v>
+      </c>
+      <c r="F19" s="5">
         <f t="shared" si="1"/>
-        <v>23303571.428571429</v>
-      </c>
-      <c r="F19" s="5">
-        <f t="shared" si="2"/>
         <v>18124999.999999996</v>
       </c>
       <c r="G19" s="3">
@@ -6432,16 +6435,16 @@
       <c r="C20" s="5">
         <v>318000000</v>
       </c>
-      <c r="D20" s="5">
+      <c r="D20" s="9">
+        <f t="shared" si="2"/>
+        <v>23214285.714285713</v>
+      </c>
+      <c r="E20" s="5">
         <f t="shared" si="0"/>
-        <v>23214285.714285713</v>
-      </c>
-      <c r="E20" s="5">
+        <v>20892857.142857142</v>
+      </c>
+      <c r="F20" s="5">
         <f t="shared" si="1"/>
-        <v>20892857.142857142</v>
-      </c>
-      <c r="F20" s="5">
-        <f t="shared" si="2"/>
         <v>16249999.999999998</v>
       </c>
       <c r="G20" s="3">
@@ -6464,16 +6467,16 @@
       <c r="C21" s="5">
         <v>363000000</v>
       </c>
-      <c r="D21" s="5">
+      <c r="D21" s="9">
+        <f t="shared" si="2"/>
+        <v>26785714.285714284</v>
+      </c>
+      <c r="E21" s="5">
         <f t="shared" si="0"/>
-        <v>26785714.285714284</v>
-      </c>
-      <c r="E21" s="5">
+        <v>24107142.857142854</v>
+      </c>
+      <c r="F21" s="5">
         <f t="shared" si="1"/>
-        <v>24107142.857142854</v>
-      </c>
-      <c r="F21" s="5">
-        <f t="shared" si="2"/>
         <v>18749999.999999996</v>
       </c>
       <c r="G21" s="3">
@@ -6496,16 +6499,16 @@
       <c r="C22" s="5">
         <v>363000000</v>
       </c>
-      <c r="D22" s="5">
+      <c r="D22" s="9">
+        <f t="shared" si="2"/>
+        <v>25892857.142857142</v>
+      </c>
+      <c r="E22" s="5">
         <f t="shared" si="0"/>
-        <v>25892857.142857142</v>
-      </c>
-      <c r="E22" s="5">
+        <v>23303571.428571429</v>
+      </c>
+      <c r="F22" s="5">
         <f t="shared" si="1"/>
-        <v>23303571.428571429</v>
-      </c>
-      <c r="F22" s="5">
-        <f t="shared" si="2"/>
         <v>18124999.999999996</v>
       </c>
       <c r="G22" s="3">
@@ -6528,16 +6531,16 @@
       <c r="C23" s="5">
         <v>363000000</v>
       </c>
-      <c r="D23" s="5">
+      <c r="D23" s="9">
+        <f t="shared" si="2"/>
+        <v>25892857.142857142</v>
+      </c>
+      <c r="E23" s="5">
         <f t="shared" si="0"/>
-        <v>25892857.142857142</v>
-      </c>
-      <c r="E23" s="5">
+        <v>23303571.428571429</v>
+      </c>
+      <c r="F23" s="5">
         <f t="shared" si="1"/>
-        <v>23303571.428571429</v>
-      </c>
-      <c r="F23" s="5">
-        <f t="shared" si="2"/>
         <v>18124999.999999996</v>
       </c>
       <c r="G23" s="3">
@@ -6560,16 +6563,16 @@
       <c r="C24" s="5">
         <v>413000000</v>
       </c>
-      <c r="D24" s="5">
+      <c r="D24" s="9">
+        <f t="shared" si="2"/>
+        <v>30357142.857142854</v>
+      </c>
+      <c r="E24" s="5">
         <f t="shared" si="0"/>
-        <v>30357142.857142854</v>
-      </c>
-      <c r="E24" s="5">
+        <v>27321428.571428571</v>
+      </c>
+      <c r="F24" s="5">
         <f t="shared" si="1"/>
-        <v>27321428.571428571</v>
-      </c>
-      <c r="F24" s="5">
-        <f t="shared" si="2"/>
         <v>21249999.999999996</v>
       </c>
       <c r="G24" s="3">
@@ -6592,16 +6595,16 @@
       <c r="C25" s="5">
         <v>443000000</v>
       </c>
-      <c r="D25" s="5">
+      <c r="D25" s="9">
+        <f t="shared" si="2"/>
+        <v>33035714.285714284</v>
+      </c>
+      <c r="E25" s="5">
         <f t="shared" si="0"/>
-        <v>33035714.285714284</v>
-      </c>
-      <c r="E25" s="5">
+        <v>29732142.857142854</v>
+      </c>
+      <c r="F25" s="5">
         <f t="shared" si="1"/>
-        <v>29732142.857142854</v>
-      </c>
-      <c r="F25" s="5">
-        <f t="shared" si="2"/>
         <v>23124999.999999996</v>
       </c>
       <c r="G25" s="3">
@@ -6624,16 +6627,16 @@
       <c r="C26" s="5">
         <v>443000000</v>
       </c>
-      <c r="D26" s="5">
+      <c r="D26" s="9">
+        <f t="shared" si="2"/>
+        <v>33035714.285714284</v>
+      </c>
+      <c r="E26" s="5">
         <f t="shared" si="0"/>
-        <v>33035714.285714284</v>
-      </c>
-      <c r="E26" s="5">
+        <v>29732142.857142854</v>
+      </c>
+      <c r="F26" s="5">
         <f t="shared" si="1"/>
-        <v>29732142.857142854</v>
-      </c>
-      <c r="F26" s="5">
-        <f t="shared" si="2"/>
         <v>23124999.999999996</v>
       </c>
       <c r="G26" s="3">
@@ -6656,16 +6659,16 @@
       <c r="C27" s="5">
         <v>443000000</v>
       </c>
-      <c r="D27" s="5">
+      <c r="D27" s="9">
+        <f t="shared" si="2"/>
+        <v>33035714.285714284</v>
+      </c>
+      <c r="E27" s="5">
         <f t="shared" si="0"/>
-        <v>33035714.285714284</v>
-      </c>
-      <c r="E27" s="5">
+        <v>29732142.857142854</v>
+      </c>
+      <c r="F27" s="5">
         <f t="shared" si="1"/>
-        <v>29732142.857142854</v>
-      </c>
-      <c r="F27" s="5">
-        <f t="shared" si="2"/>
         <v>23124999.999999996</v>
       </c>
       <c r="G27" s="3">
@@ -6688,16 +6691,16 @@
       <c r="C28" s="5">
         <v>415000000</v>
       </c>
-      <c r="D28" s="5">
+      <c r="D28" s="9">
+        <f t="shared" si="2"/>
+        <v>33035714.285714284</v>
+      </c>
+      <c r="E28" s="5">
         <f t="shared" si="0"/>
-        <v>33035714.285714284</v>
-      </c>
-      <c r="E28" s="5">
+        <v>29732142.857142854</v>
+      </c>
+      <c r="F28" s="5">
         <f t="shared" si="1"/>
-        <v>29732142.857142854</v>
-      </c>
-      <c r="F28" s="5">
-        <f t="shared" si="2"/>
         <v>23124999.999999996</v>
       </c>
       <c r="G28" s="3">
@@ -6720,16 +6723,16 @@
       <c r="C29" s="5">
         <v>415000000</v>
       </c>
-      <c r="D29" s="5">
+      <c r="D29" s="9">
+        <f t="shared" si="2"/>
+        <v>33035714.285714284</v>
+      </c>
+      <c r="E29" s="5">
         <f t="shared" si="0"/>
-        <v>33035714.285714284</v>
-      </c>
-      <c r="E29" s="5">
+        <v>29732142.857142854</v>
+      </c>
+      <c r="F29" s="5">
         <f t="shared" si="1"/>
-        <v>29732142.857142854</v>
-      </c>
-      <c r="F29" s="5">
-        <f t="shared" si="2"/>
         <v>23124999.999999996</v>
       </c>
       <c r="G29" s="3">
@@ -6752,16 +6755,16 @@
       <c r="C30" s="5">
         <v>188300000</v>
       </c>
-      <c r="D30" s="5">
+      <c r="D30" s="9">
+        <f t="shared" si="2"/>
+        <v>11339285.714285715</v>
+      </c>
+      <c r="E30" s="5">
         <f t="shared" si="0"/>
-        <v>11339285.714285715</v>
-      </c>
-      <c r="E30" s="5">
+        <v>10205357.142857144</v>
+      </c>
+      <c r="F30" s="5">
         <f t="shared" si="1"/>
-        <v>10205357.142857144</v>
-      </c>
-      <c r="F30" s="5">
-        <f t="shared" si="2"/>
         <v>7937500</v>
       </c>
       <c r="G30" s="3">
@@ -6784,16 +6787,16 @@
       <c r="C31" s="5">
         <v>188300000</v>
       </c>
-      <c r="D31" s="5">
+      <c r="D31" s="9">
+        <f t="shared" si="2"/>
+        <v>11339285.714285715</v>
+      </c>
+      <c r="E31" s="5">
         <f t="shared" si="0"/>
-        <v>11339285.714285715</v>
-      </c>
-      <c r="E31" s="5">
+        <v>10205357.142857144</v>
+      </c>
+      <c r="F31" s="5">
         <f t="shared" si="1"/>
-        <v>10205357.142857144</v>
-      </c>
-      <c r="F31" s="5">
-        <f t="shared" si="2"/>
         <v>7937500</v>
       </c>
       <c r="G31" s="3">
@@ -6816,16 +6819,16 @@
       <c r="C32" s="5">
         <v>222850000</v>
       </c>
-      <c r="D32" s="5">
+      <c r="D32" s="9">
+        <f t="shared" si="2"/>
+        <v>14285714.285714284</v>
+      </c>
+      <c r="E32" s="5">
         <f t="shared" si="0"/>
-        <v>14285714.285714284</v>
-      </c>
-      <c r="E32" s="5">
+        <v>12857142.857142856</v>
+      </c>
+      <c r="F32" s="5">
         <f t="shared" si="1"/>
-        <v>12857142.857142856</v>
-      </c>
-      <c r="F32" s="5">
-        <f t="shared" si="2"/>
         <v>9999999.9999999981</v>
       </c>
       <c r="G32" s="3">
@@ -6848,16 +6851,16 @@
       <c r="C33" s="5">
         <v>210700000</v>
       </c>
-      <c r="D33" s="5">
+      <c r="D33" s="9">
+        <f t="shared" si="2"/>
+        <v>13124999.999999998</v>
+      </c>
+      <c r="E33" s="5">
         <f t="shared" si="0"/>
-        <v>13124999.999999998</v>
-      </c>
-      <c r="E33" s="5">
+        <v>11812499.999999998</v>
+      </c>
+      <c r="F33" s="5">
         <f t="shared" si="1"/>
-        <v>11812499.999999998</v>
-      </c>
-      <c r="F33" s="5">
-        <f t="shared" si="2"/>
         <v>9187499.9999999981</v>
       </c>
       <c r="G33" s="3">
@@ -6880,16 +6883,16 @@
       <c r="C34" s="5">
         <v>262500000</v>
       </c>
-      <c r="D34" s="5">
+      <c r="D34" s="9">
+        <f t="shared" ref="D34:D65" si="5">I34/1.12</f>
+        <v>16339285.714285713</v>
+      </c>
+      <c r="E34" s="5">
         <f t="shared" si="0"/>
-        <v>16339285.714285713</v>
-      </c>
-      <c r="E34" s="5">
+        <v>14705357.142857142</v>
+      </c>
+      <c r="F34" s="5">
         <f t="shared" si="1"/>
-        <v>14705357.142857142</v>
-      </c>
-      <c r="F34" s="5">
-        <f t="shared" si="2"/>
         <v>11437499.999999998</v>
       </c>
       <c r="G34" s="3">
@@ -6912,16 +6915,16 @@
       <c r="C35" s="5">
         <v>277200000</v>
       </c>
-      <c r="D35" s="5">
+      <c r="D35" s="9">
+        <f t="shared" si="5"/>
+        <v>18660714.285714284</v>
+      </c>
+      <c r="E35" s="5">
         <f t="shared" si="0"/>
-        <v>18660714.285714284</v>
-      </c>
-      <c r="E35" s="5">
+        <v>16794642.857142854</v>
+      </c>
+      <c r="F35" s="5">
         <f t="shared" si="1"/>
-        <v>16794642.857142854</v>
-      </c>
-      <c r="F35" s="5">
-        <f t="shared" si="2"/>
         <v>13062499.999999998</v>
       </c>
       <c r="G35" s="3">
@@ -6944,16 +6947,16 @@
       <c r="C36" s="5">
         <v>291300000</v>
       </c>
-      <c r="D36" s="5">
-        <f t="shared" ref="D36:D57" si="7">I36/1.12</f>
+      <c r="D36" s="9">
+        <f t="shared" si="5"/>
         <v>19642857.142857142</v>
       </c>
       <c r="E36" s="5">
-        <f t="shared" ref="E36:E57" si="8">D36*90%</f>
+        <f t="shared" ref="E36:E57" si="6">D36*90%</f>
         <v>17678571.428571429</v>
       </c>
       <c r="F36" s="5">
-        <f t="shared" ref="F36:F57" si="9">D36*70%</f>
+        <f t="shared" ref="F36:F57" si="7">D36*70%</f>
         <v>13749999.999999998</v>
       </c>
       <c r="G36" s="3">
@@ -6976,16 +6979,16 @@
       <c r="C37" s="5">
         <v>285200000</v>
       </c>
-      <c r="D37" s="5">
+      <c r="D37" s="9">
+        <f t="shared" si="5"/>
+        <v>18303571.428571429</v>
+      </c>
+      <c r="E37" s="5">
+        <f t="shared" si="6"/>
+        <v>16473214.285714287</v>
+      </c>
+      <c r="F37" s="5">
         <f t="shared" si="7"/>
-        <v>18303571.428571429</v>
-      </c>
-      <c r="E37" s="5">
-        <f t="shared" si="8"/>
-        <v>16473214.285714287</v>
-      </c>
-      <c r="F37" s="5">
-        <f t="shared" si="9"/>
         <v>12812500</v>
       </c>
       <c r="G37" s="3">
@@ -7008,16 +7011,16 @@
       <c r="C38" s="9">
         <v>307300000</v>
       </c>
-      <c r="D38" s="5">
-        <f t="shared" ref="D38" si="10">I38/1.12</f>
+      <c r="D38" s="9">
+        <f t="shared" si="5"/>
         <v>19999999.999999996</v>
       </c>
       <c r="E38" s="5">
-        <f t="shared" ref="E38" si="11">D38*90%</f>
+        <f t="shared" ref="E38" si="8">D38*90%</f>
         <v>17999999.999999996</v>
       </c>
       <c r="F38" s="5">
-        <f t="shared" ref="F38" si="12">D38*70%</f>
+        <f t="shared" ref="F38" si="9">D38*70%</f>
         <v>13999999.999999996</v>
       </c>
       <c r="G38" s="20">
@@ -7040,16 +7043,16 @@
       <c r="C39" s="5">
         <v>345650000</v>
       </c>
-      <c r="D39" s="5">
+      <c r="D39" s="9">
+        <f t="shared" si="5"/>
+        <v>22857142.857142854</v>
+      </c>
+      <c r="E39" s="5">
+        <f t="shared" si="6"/>
+        <v>20571428.571428571</v>
+      </c>
+      <c r="F39" s="5">
         <f t="shared" si="7"/>
-        <v>22857142.857142854</v>
-      </c>
-      <c r="E39" s="5">
-        <f t="shared" si="8"/>
-        <v>20571428.571428571</v>
-      </c>
-      <c r="F39" s="5">
-        <f t="shared" si="9"/>
         <v>15999999.999999996</v>
       </c>
       <c r="G39" s="3">
@@ -7072,16 +7075,16 @@
       <c r="C40" s="9">
         <v>307300000</v>
       </c>
-      <c r="D40" s="5">
+      <c r="D40" s="9">
+        <f t="shared" si="5"/>
+        <v>19999999.999999996</v>
+      </c>
+      <c r="E40" s="5">
+        <f t="shared" si="6"/>
+        <v>17999999.999999996</v>
+      </c>
+      <c r="F40" s="5">
         <f t="shared" si="7"/>
-        <v>19999999.999999996</v>
-      </c>
-      <c r="E40" s="5">
-        <f t="shared" si="8"/>
-        <v>17999999.999999996</v>
-      </c>
-      <c r="F40" s="5">
-        <f t="shared" si="9"/>
         <v>13999999.999999996</v>
       </c>
       <c r="G40" s="20">
@@ -7105,15 +7108,15 @@
         <v>399000000</v>
       </c>
       <c r="D41" s="9">
+        <f t="shared" si="5"/>
+        <v>28214285.714285713</v>
+      </c>
+      <c r="E41" s="9">
+        <f t="shared" si="6"/>
+        <v>25392857.142857142</v>
+      </c>
+      <c r="F41" s="9">
         <f t="shared" si="7"/>
-        <v>28214285.714285713</v>
-      </c>
-      <c r="E41" s="9">
-        <f t="shared" si="8"/>
-        <v>25392857.142857142</v>
-      </c>
-      <c r="F41" s="9">
-        <f t="shared" si="9"/>
         <v>19749999.999999996</v>
       </c>
       <c r="G41" s="20">
@@ -7137,15 +7140,15 @@
         <v>459000000</v>
       </c>
       <c r="D42" s="9">
+        <f t="shared" si="5"/>
+        <v>32499999.999999996</v>
+      </c>
+      <c r="E42" s="9">
+        <f t="shared" si="6"/>
+        <v>29249999.999999996</v>
+      </c>
+      <c r="F42" s="9">
         <f t="shared" si="7"/>
-        <v>32499999.999999996</v>
-      </c>
-      <c r="E42" s="9">
-        <f t="shared" si="8"/>
-        <v>29249999.999999996</v>
-      </c>
-      <c r="F42" s="9">
-        <f t="shared" si="9"/>
         <v>22749999.999999996</v>
       </c>
       <c r="G42" s="20">
@@ -7169,15 +7172,15 @@
         <v>449000000</v>
       </c>
       <c r="D43" s="9">
+        <f t="shared" si="5"/>
+        <v>29196428.571428567</v>
+      </c>
+      <c r="E43" s="9">
+        <f t="shared" si="6"/>
+        <v>26276785.714285713</v>
+      </c>
+      <c r="F43" s="9">
         <f t="shared" si="7"/>
-        <v>29196428.571428567</v>
-      </c>
-      <c r="E43" s="9">
-        <f t="shared" si="8"/>
-        <v>26276785.714285713</v>
-      </c>
-      <c r="F43" s="9">
-        <f t="shared" si="9"/>
         <v>20437499.999999996</v>
       </c>
       <c r="G43" s="20">
@@ -7201,15 +7204,15 @@
         <v>499000000</v>
       </c>
       <c r="D44" s="9">
+        <f t="shared" si="5"/>
+        <v>32499999.999999996</v>
+      </c>
+      <c r="E44" s="9">
+        <f t="shared" si="6"/>
+        <v>29249999.999999996</v>
+      </c>
+      <c r="F44" s="9">
         <f t="shared" si="7"/>
-        <v>32499999.999999996</v>
-      </c>
-      <c r="E44" s="9">
-        <f t="shared" si="8"/>
-        <v>29249999.999999996</v>
-      </c>
-      <c r="F44" s="9">
-        <f t="shared" si="9"/>
         <v>22749999.999999996</v>
       </c>
       <c r="G44" s="20">
@@ -7232,16 +7235,16 @@
       <c r="C45" s="5">
         <v>168000000</v>
       </c>
-      <c r="D45" s="5">
+      <c r="D45" s="9">
         <f>I45/1.11</f>
         <v>11261261.261261258</v>
       </c>
       <c r="E45" s="5">
-        <f t="shared" si="8"/>
+        <f t="shared" si="6"/>
         <v>10135135.135135133</v>
       </c>
       <c r="F45" s="5">
-        <f t="shared" si="9"/>
+        <f t="shared" si="7"/>
         <v>7882882.88288288</v>
       </c>
       <c r="G45" s="3">
@@ -7264,16 +7267,16 @@
       <c r="C46" s="23">
         <v>176000000</v>
       </c>
-      <c r="D46" s="5">
-        <f t="shared" ref="D46:D49" si="13">I46/1.11</f>
+      <c r="D46" s="9">
+        <f t="shared" ref="D46:D49" si="10">I46/1.11</f>
         <v>12162162.162162161</v>
       </c>
       <c r="E46" s="5">
-        <f t="shared" si="8"/>
+        <f t="shared" si="6"/>
         <v>10945945.945945945</v>
       </c>
       <c r="F46" s="5">
-        <f t="shared" si="9"/>
+        <f t="shared" si="7"/>
         <v>8513513.513513511</v>
       </c>
       <c r="G46" s="24">
@@ -7296,16 +7299,16 @@
       <c r="C47" s="5">
         <v>155700000</v>
       </c>
-      <c r="D47" s="5">
-        <f t="shared" si="13"/>
+      <c r="D47" s="9">
+        <f t="shared" si="10"/>
         <v>10990990.990990991</v>
       </c>
       <c r="E47" s="5">
-        <f t="shared" si="8"/>
+        <f t="shared" si="6"/>
         <v>9891891.8918918911</v>
       </c>
       <c r="F47" s="5">
-        <f t="shared" si="9"/>
+        <f t="shared" si="7"/>
         <v>7693693.6936936928</v>
       </c>
       <c r="G47" s="3">
@@ -7328,16 +7331,16 @@
       <c r="C48" s="9">
         <v>167800000</v>
       </c>
-      <c r="D48" s="5">
-        <f t="shared" si="13"/>
+      <c r="D48" s="9">
+        <f t="shared" si="10"/>
         <v>7207207.2072072066</v>
       </c>
       <c r="E48" s="9">
-        <f t="shared" si="8"/>
+        <f t="shared" si="6"/>
         <v>6486486.4864864862</v>
       </c>
       <c r="F48" s="9">
-        <f t="shared" si="9"/>
+        <f t="shared" si="7"/>
         <v>5045045.0450450443</v>
       </c>
       <c r="G48" s="20">
@@ -7360,16 +7363,16 @@
       <c r="C49" s="5">
         <v>172600000</v>
       </c>
-      <c r="D49" s="5">
-        <f t="shared" si="13"/>
+      <c r="D49" s="9">
+        <f t="shared" si="10"/>
         <v>7207207.2072072066</v>
       </c>
       <c r="E49" s="5">
-        <f t="shared" si="8"/>
+        <f t="shared" si="6"/>
         <v>6486486.4864864862</v>
       </c>
       <c r="F49" s="5">
-        <f t="shared" si="9"/>
+        <f t="shared" si="7"/>
         <v>5045045.0450450443</v>
       </c>
       <c r="G49" s="3">
@@ -7392,16 +7395,16 @@
       <c r="C50" s="18">
         <v>328000000</v>
       </c>
-      <c r="D50" s="18">
+      <c r="D50" s="9">
+        <f t="shared" si="5"/>
+        <v>17857142.857142854</v>
+      </c>
+      <c r="E50" s="18">
+        <f t="shared" si="6"/>
+        <v>16071428.571428569</v>
+      </c>
+      <c r="F50" s="18">
         <f t="shared" si="7"/>
-        <v>17857142.857142854</v>
-      </c>
-      <c r="E50" s="18">
-        <f t="shared" si="8"/>
-        <v>16071428.571428569</v>
-      </c>
-      <c r="F50" s="18">
-        <f t="shared" si="9"/>
         <v>12499999.999999998</v>
       </c>
       <c r="G50" s="21">
@@ -7425,15 +7428,15 @@
         <v>328000000</v>
       </c>
       <c r="D51" s="9">
+        <f t="shared" si="5"/>
+        <v>17857142.857142854</v>
+      </c>
+      <c r="E51" s="9">
+        <f t="shared" si="6"/>
+        <v>16071428.571428569</v>
+      </c>
+      <c r="F51" s="9">
         <f t="shared" si="7"/>
-        <v>17857142.857142854</v>
-      </c>
-      <c r="E51" s="9">
-        <f t="shared" si="8"/>
-        <v>16071428.571428569</v>
-      </c>
-      <c r="F51" s="9">
-        <f t="shared" si="9"/>
         <v>12499999.999999998</v>
       </c>
       <c r="G51" s="20">
@@ -7457,15 +7460,15 @@
         <v>358000000</v>
       </c>
       <c r="D52" s="9">
+        <f t="shared" si="5"/>
+        <v>22321428.571428571</v>
+      </c>
+      <c r="E52" s="9">
+        <f t="shared" si="6"/>
+        <v>20089285.714285713</v>
+      </c>
+      <c r="F52" s="9">
         <f t="shared" si="7"/>
-        <v>22321428.571428571</v>
-      </c>
-      <c r="E52" s="9">
-        <f t="shared" si="8"/>
-        <v>20089285.714285713</v>
-      </c>
-      <c r="F52" s="9">
-        <f t="shared" si="9"/>
         <v>15624999.999999998</v>
       </c>
       <c r="G52" s="20">
@@ -7489,15 +7492,15 @@
         <v>358000000</v>
       </c>
       <c r="D53" s="9">
+        <f t="shared" si="5"/>
+        <v>22321428.571428571</v>
+      </c>
+      <c r="E53" s="9">
+        <f t="shared" si="6"/>
+        <v>20089285.714285713</v>
+      </c>
+      <c r="F53" s="9">
         <f t="shared" si="7"/>
-        <v>22321428.571428571</v>
-      </c>
-      <c r="E53" s="9">
-        <f t="shared" si="8"/>
-        <v>20089285.714285713</v>
-      </c>
-      <c r="F53" s="9">
-        <f t="shared" si="9"/>
         <v>15624999.999999998</v>
       </c>
       <c r="G53" s="20">
@@ -7520,16 +7523,16 @@
       <c r="C54" s="18">
         <v>348000000</v>
       </c>
-      <c r="D54" s="18">
+      <c r="D54" s="9">
+        <f t="shared" si="5"/>
+        <v>17857142.857142854</v>
+      </c>
+      <c r="E54" s="18">
+        <f t="shared" si="6"/>
+        <v>16071428.571428569</v>
+      </c>
+      <c r="F54" s="18">
         <f t="shared" si="7"/>
-        <v>17857142.857142854</v>
-      </c>
-      <c r="E54" s="18">
-        <f t="shared" si="8"/>
-        <v>16071428.571428569</v>
-      </c>
-      <c r="F54" s="18">
-        <f t="shared" si="9"/>
         <v>12499999.999999998</v>
       </c>
       <c r="G54" s="21">
@@ -7552,16 +7555,16 @@
       <c r="C55" s="18">
         <v>348000000</v>
       </c>
-      <c r="D55" s="18">
+      <c r="D55" s="9">
+        <f t="shared" si="5"/>
+        <v>17857142.857142854</v>
+      </c>
+      <c r="E55" s="18">
+        <f t="shared" si="6"/>
+        <v>16071428.571428569</v>
+      </c>
+      <c r="F55" s="18">
         <f t="shared" si="7"/>
-        <v>17857142.857142854</v>
-      </c>
-      <c r="E55" s="18">
-        <f t="shared" si="8"/>
-        <v>16071428.571428569</v>
-      </c>
-      <c r="F55" s="18">
-        <f t="shared" si="9"/>
         <v>12499999.999999998</v>
       </c>
       <c r="G55" s="21">
@@ -7585,15 +7588,15 @@
         <v>378000000</v>
       </c>
       <c r="D56" s="9">
+        <f t="shared" si="5"/>
+        <v>22321428.571428571</v>
+      </c>
+      <c r="E56" s="9">
+        <f t="shared" si="6"/>
+        <v>20089285.714285713</v>
+      </c>
+      <c r="F56" s="9">
         <f t="shared" si="7"/>
-        <v>22321428.571428571</v>
-      </c>
-      <c r="E56" s="9">
-        <f t="shared" si="8"/>
-        <v>20089285.714285713</v>
-      </c>
-      <c r="F56" s="9">
-        <f t="shared" si="9"/>
         <v>15624999.999999998</v>
       </c>
       <c r="G56" s="20">
@@ -7617,15 +7620,15 @@
         <v>378000000</v>
       </c>
       <c r="D57" s="9">
+        <f t="shared" si="5"/>
+        <v>22321428.571428571</v>
+      </c>
+      <c r="E57" s="9">
+        <f t="shared" si="6"/>
+        <v>20089285.714285713</v>
+      </c>
+      <c r="F57" s="9">
         <f t="shared" si="7"/>
-        <v>22321428.571428571</v>
-      </c>
-      <c r="E57" s="9">
-        <f t="shared" si="8"/>
-        <v>20089285.714285713</v>
-      </c>
-      <c r="F57" s="9">
-        <f t="shared" si="9"/>
         <v>15624999.999999998</v>
       </c>
       <c r="G57" s="21">
@@ -7649,15 +7652,15 @@
         <v>399000000</v>
       </c>
       <c r="D58" s="9">
-        <f t="shared" ref="D58:D65" si="14">I58/1.12</f>
+        <f t="shared" si="5"/>
         <v>22321428.571428571</v>
       </c>
       <c r="E58" s="9">
-        <f t="shared" ref="E58:E65" si="15">D58*90%</f>
+        <f t="shared" ref="E58:E65" si="11">D58*90%</f>
         <v>20089285.714285713</v>
       </c>
       <c r="F58" s="9">
-        <f t="shared" ref="F58:F65" si="16">D58*70%</f>
+        <f t="shared" ref="F58:F65" si="12">D58*70%</f>
         <v>15624999.999999998</v>
       </c>
       <c r="G58" s="21">
@@ -7681,15 +7684,15 @@
         <v>469000000</v>
       </c>
       <c r="D59" s="9">
-        <f t="shared" si="14"/>
+        <f t="shared" si="5"/>
         <v>31249999.999999996</v>
       </c>
       <c r="E59" s="9">
-        <f t="shared" si="15"/>
+        <f t="shared" si="11"/>
         <v>28124999.999999996</v>
       </c>
       <c r="F59" s="9">
-        <f t="shared" si="16"/>
+        <f t="shared" si="12"/>
         <v>21874999.999999996</v>
       </c>
       <c r="G59" s="21">
@@ -7713,15 +7716,15 @@
         <v>459000000</v>
       </c>
       <c r="D60" s="9">
-        <f t="shared" si="14"/>
+        <f t="shared" si="5"/>
         <v>22321428.571428571</v>
       </c>
       <c r="E60" s="9">
-        <f t="shared" si="15"/>
+        <f t="shared" si="11"/>
         <v>20089285.714285713</v>
       </c>
       <c r="F60" s="9">
-        <f t="shared" si="16"/>
+        <f t="shared" si="12"/>
         <v>15624999.999999998</v>
       </c>
       <c r="G60" s="21">
@@ -7745,15 +7748,15 @@
         <v>509000000</v>
       </c>
       <c r="D61" s="9">
-        <f t="shared" si="14"/>
+        <f t="shared" si="5"/>
         <v>31249999.999999996</v>
       </c>
       <c r="E61" s="9">
-        <f t="shared" si="15"/>
+        <f t="shared" si="11"/>
         <v>28124999.999999996</v>
       </c>
       <c r="F61" s="9">
-        <f t="shared" si="16"/>
+        <f t="shared" si="12"/>
         <v>21874999.999999996</v>
       </c>
       <c r="G61" s="21">
@@ -7777,15 +7780,15 @@
         <v>399000000</v>
       </c>
       <c r="D62" s="9">
-        <f t="shared" si="14"/>
+        <f t="shared" si="5"/>
         <v>22321428.571428571</v>
       </c>
       <c r="E62" s="9">
-        <f t="shared" si="15"/>
+        <f t="shared" si="11"/>
         <v>20089285.714285713</v>
       </c>
       <c r="F62" s="9">
-        <f t="shared" si="16"/>
+        <f t="shared" si="12"/>
         <v>15624999.999999998</v>
       </c>
       <c r="G62" s="21">
@@ -7809,15 +7812,15 @@
         <v>469000000</v>
       </c>
       <c r="D63" s="9">
-        <f t="shared" si="14"/>
+        <f t="shared" si="5"/>
         <v>31249999.999999996</v>
       </c>
       <c r="E63" s="9">
-        <f t="shared" si="15"/>
+        <f t="shared" si="11"/>
         <v>28124999.999999996</v>
       </c>
       <c r="F63" s="9">
-        <f t="shared" si="16"/>
+        <f t="shared" si="12"/>
         <v>21874999.999999996</v>
       </c>
       <c r="G63" s="21">
@@ -7841,15 +7844,15 @@
         <v>459000000</v>
       </c>
       <c r="D64" s="9">
-        <f t="shared" si="14"/>
+        <f t="shared" si="5"/>
         <v>22321428.571428571</v>
       </c>
       <c r="E64" s="9">
-        <f t="shared" si="15"/>
+        <f t="shared" si="11"/>
         <v>20089285.714285713</v>
       </c>
       <c r="F64" s="9">
-        <f t="shared" si="16"/>
+        <f t="shared" si="12"/>
         <v>15624999.999999998</v>
       </c>
       <c r="G64" s="21">
@@ -7873,15 +7876,15 @@
         <v>509000000</v>
       </c>
       <c r="D65" s="9">
-        <f t="shared" si="14"/>
+        <f t="shared" si="5"/>
         <v>31249999.999999996</v>
       </c>
       <c r="E65" s="9">
-        <f t="shared" si="15"/>
+        <f t="shared" si="11"/>
         <v>28124999.999999996</v>
       </c>
       <c r="F65" s="9">
-        <f t="shared" si="16"/>
+        <f t="shared" si="12"/>
         <v>21874999.999999996</v>
       </c>
       <c r="G65" s="21">
@@ -7905,15 +7908,15 @@
         <v>303000000</v>
       </c>
       <c r="D66" s="9">
-        <f t="shared" ref="D66:D68" si="17">I66/1.12</f>
+        <f t="shared" ref="D66:D79" si="13">I66/1.12</f>
         <v>20535714.285714284</v>
       </c>
       <c r="E66" s="9">
-        <f t="shared" ref="E66:E68" si="18">D66*90%</f>
+        <f t="shared" ref="E66:E68" si="14">D66*90%</f>
         <v>18482142.857142854</v>
       </c>
       <c r="F66" s="9">
-        <f t="shared" ref="F66:F68" si="19">D66*70%</f>
+        <f t="shared" ref="F66:F68" si="15">D66*70%</f>
         <v>14374999.999999998</v>
       </c>
       <c r="G66" s="3">
@@ -7936,16 +7939,16 @@
       <c r="C67" s="5">
         <v>217000000</v>
       </c>
-      <c r="D67" s="5">
-        <f t="shared" si="17"/>
+      <c r="D67" s="9">
+        <f t="shared" si="13"/>
         <v>11607142.857142856</v>
       </c>
       <c r="E67" s="5">
-        <f t="shared" si="18"/>
+        <f t="shared" si="14"/>
         <v>10446428.571428571</v>
       </c>
       <c r="F67" s="5">
-        <f t="shared" si="19"/>
+        <f t="shared" si="15"/>
         <v>8124999.9999999991</v>
       </c>
       <c r="G67" s="3">
@@ -7968,16 +7971,16 @@
       <c r="C68" s="5">
         <v>263000000</v>
       </c>
-      <c r="D68" s="5">
-        <f t="shared" si="17"/>
+      <c r="D68" s="9">
+        <f t="shared" si="13"/>
         <v>17857142.857142854</v>
       </c>
       <c r="E68" s="5">
-        <f t="shared" si="18"/>
+        <f t="shared" si="14"/>
         <v>16071428.571428569</v>
       </c>
       <c r="F68" s="5">
-        <f t="shared" si="19"/>
+        <f t="shared" si="15"/>
         <v>12499999.999999998</v>
       </c>
       <c r="G68" s="3">
@@ -8000,16 +8003,16 @@
       <c r="C69" s="18">
         <v>155000000</v>
       </c>
-      <c r="D69" s="5">
-        <f t="shared" ref="D69:D71" si="20">I69/1.12</f>
+      <c r="D69" s="9">
+        <f t="shared" si="13"/>
         <v>5357142.8571428563</v>
       </c>
       <c r="E69" s="5">
-        <f t="shared" ref="E69:E71" si="21">D69*90%</f>
+        <f t="shared" ref="E69:E71" si="16">D69*90%</f>
         <v>4821428.5714285709</v>
       </c>
       <c r="F69" s="5">
-        <f t="shared" ref="F69:F71" si="22">D69*70%</f>
+        <f t="shared" ref="F69:F71" si="17">D69*70%</f>
         <v>3749999.9999999991</v>
       </c>
       <c r="G69" s="3">
@@ -8032,16 +8035,16 @@
       <c r="C70" s="18">
         <v>175000000</v>
       </c>
-      <c r="D70" s="5">
-        <f t="shared" si="20"/>
+      <c r="D70" s="9">
+        <f t="shared" si="13"/>
         <v>5357142.8571428563</v>
       </c>
       <c r="E70" s="5">
-        <f t="shared" si="21"/>
+        <f t="shared" si="16"/>
         <v>4821428.5714285709</v>
       </c>
       <c r="F70" s="5">
-        <f t="shared" si="22"/>
+        <f t="shared" si="17"/>
         <v>3749999.9999999991</v>
       </c>
       <c r="G70" s="3">
@@ -8065,15 +8068,15 @@
         <v>389000000</v>
       </c>
       <c r="D71" s="9">
-        <f t="shared" si="20"/>
+        <f t="shared" si="13"/>
         <v>27499999.999999996</v>
       </c>
       <c r="E71" s="9">
-        <f t="shared" si="21"/>
+        <f t="shared" si="16"/>
         <v>24749999.999999996</v>
       </c>
       <c r="F71" s="9">
-        <f t="shared" si="22"/>
+        <f t="shared" si="17"/>
         <v>19249999.999999996</v>
       </c>
       <c r="G71" s="20">
@@ -8097,15 +8100,15 @@
         <v>399000000</v>
       </c>
       <c r="D72" s="9">
-        <f t="shared" ref="D72:D75" si="23">I72/1.12</f>
+        <f t="shared" si="13"/>
         <v>28214285.714285713</v>
       </c>
       <c r="E72" s="9">
-        <f t="shared" ref="E72:E75" si="24">D72*90%</f>
+        <f t="shared" ref="E72:E75" si="18">D72*90%</f>
         <v>25392857.142857142</v>
       </c>
       <c r="F72" s="9">
-        <f t="shared" ref="F72:F75" si="25">D72*70%</f>
+        <f t="shared" ref="F72:F75" si="19">D72*70%</f>
         <v>19749999.999999996</v>
       </c>
       <c r="G72" s="20">
@@ -8129,15 +8132,15 @@
         <v>459000000</v>
       </c>
       <c r="D73" s="9">
-        <f t="shared" si="23"/>
+        <f t="shared" si="13"/>
         <v>32499999.999999996</v>
       </c>
       <c r="E73" s="9">
-        <f t="shared" si="24"/>
+        <f t="shared" si="18"/>
         <v>29249999.999999996</v>
       </c>
       <c r="F73" s="9">
-        <f t="shared" si="25"/>
+        <f t="shared" si="19"/>
         <v>22749999.999999996</v>
       </c>
       <c r="G73" s="20">
@@ -8161,15 +8164,15 @@
         <v>449000000</v>
       </c>
       <c r="D74" s="9">
-        <f t="shared" si="23"/>
+        <f t="shared" si="13"/>
         <v>29196428.571428567</v>
       </c>
       <c r="E74" s="9">
-        <f t="shared" si="24"/>
+        <f t="shared" si="18"/>
         <v>26276785.714285713</v>
       </c>
       <c r="F74" s="9">
-        <f t="shared" si="25"/>
+        <f t="shared" si="19"/>
         <v>20437499.999999996</v>
       </c>
       <c r="G74" s="20">
@@ -8193,15 +8196,15 @@
         <v>499000000</v>
       </c>
       <c r="D75" s="9">
-        <f t="shared" si="23"/>
+        <f t="shared" si="13"/>
         <v>32499999.999999996</v>
       </c>
       <c r="E75" s="9">
-        <f t="shared" si="24"/>
+        <f t="shared" si="18"/>
         <v>29249999.999999996</v>
       </c>
       <c r="F75" s="9">
-        <f t="shared" si="25"/>
+        <f t="shared" si="19"/>
         <v>22749999.999999996</v>
       </c>
       <c r="G75" s="20">
@@ -8225,15 +8228,15 @@
         <v>289000000</v>
       </c>
       <c r="D76" s="9">
-        <f t="shared" ref="D76:D77" si="26">I76/1.12</f>
+        <f t="shared" si="13"/>
         <v>13392857.142857142</v>
       </c>
       <c r="E76" s="9">
-        <f t="shared" ref="E76:E77" si="27">D76*90%</f>
+        <f t="shared" ref="E76:E77" si="20">D76*90%</f>
         <v>12053571.428571427</v>
       </c>
       <c r="F76" s="9">
-        <f t="shared" ref="F76:F77" si="28">D76*70%</f>
+        <f t="shared" ref="F76:F77" si="21">D76*70%</f>
         <v>9374999.9999999981</v>
       </c>
       <c r="G76" s="20">
@@ -8257,15 +8260,15 @@
         <v>319000000</v>
       </c>
       <c r="D77" s="9">
-        <f t="shared" si="26"/>
+        <f t="shared" si="13"/>
         <v>13392857.142857142</v>
       </c>
       <c r="E77" s="9">
-        <f t="shared" si="27"/>
+        <f t="shared" si="20"/>
         <v>12053571.428571427</v>
       </c>
       <c r="F77" s="9">
-        <f t="shared" si="28"/>
+        <f t="shared" si="21"/>
         <v>9374999.9999999981</v>
       </c>
       <c r="G77" s="20">
@@ -8289,15 +8292,15 @@
         <v>299000000</v>
       </c>
       <c r="D78" s="9">
-        <f t="shared" ref="D78:D79" si="29">I78/1.12</f>
+        <f t="shared" si="13"/>
         <v>17857142.857142854</v>
       </c>
       <c r="E78" s="9">
-        <f t="shared" ref="E78:E79" si="30">D78*90%</f>
+        <f t="shared" ref="E78:E79" si="22">D78*90%</f>
         <v>16071428.571428569</v>
       </c>
       <c r="F78" s="9">
-        <f t="shared" ref="F78:F79" si="31">D78*70%</f>
+        <f t="shared" ref="F78:F79" si="23">D78*70%</f>
         <v>12499999.999999998</v>
       </c>
       <c r="G78" s="20">
@@ -8321,15 +8324,15 @@
         <v>339000000</v>
       </c>
       <c r="D79" s="9">
-        <f t="shared" si="29"/>
+        <f t="shared" si="13"/>
         <v>22321428.571428571</v>
       </c>
       <c r="E79" s="9">
-        <f t="shared" si="30"/>
+        <f t="shared" si="22"/>
         <v>20089285.714285713</v>
       </c>
       <c r="F79" s="9">
-        <f t="shared" si="31"/>
+        <f t="shared" si="23"/>
         <v>15624999.999999998</v>
       </c>
       <c r="G79" s="20">
@@ -8345,25 +8348,25 @@
   </sheetData>
   <phoneticPr fontId="4" type="noConversion"/>
   <conditionalFormatting sqref="A1:A1048576">
-    <cfRule type="duplicateValues" dxfId="10" priority="4"/>
+    <cfRule type="duplicateValues" dxfId="11" priority="4"/>
   </conditionalFormatting>
   <conditionalFormatting sqref="A33:A41 A43:A46 A2:A31">
-    <cfRule type="duplicateValues" dxfId="9" priority="16"/>
+    <cfRule type="duplicateValues" dxfId="10" priority="16"/>
   </conditionalFormatting>
   <conditionalFormatting sqref="A33:A46 A2:A31">
-    <cfRule type="duplicateValues" dxfId="8" priority="20"/>
+    <cfRule type="duplicateValues" dxfId="9" priority="20"/>
   </conditionalFormatting>
   <conditionalFormatting sqref="H43:H46">
-    <cfRule type="duplicateValues" dxfId="7" priority="9"/>
-    <cfRule type="duplicateValues" dxfId="6" priority="10"/>
+    <cfRule type="duplicateValues" dxfId="8" priority="9"/>
+    <cfRule type="duplicateValues" dxfId="7" priority="10"/>
   </conditionalFormatting>
   <conditionalFormatting sqref="H51:H54">
-    <cfRule type="duplicateValues" dxfId="5" priority="5"/>
-    <cfRule type="duplicateValues" dxfId="4" priority="6"/>
+    <cfRule type="duplicateValues" dxfId="6" priority="5"/>
+    <cfRule type="duplicateValues" dxfId="5" priority="6"/>
   </conditionalFormatting>
   <conditionalFormatting sqref="H74:H75">
-    <cfRule type="duplicateValues" dxfId="3" priority="1"/>
-    <cfRule type="duplicateValues" dxfId="2" priority="2"/>
+    <cfRule type="duplicateValues" dxfId="4" priority="1"/>
+    <cfRule type="duplicateValues" dxfId="3" priority="2"/>
   </conditionalFormatting>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <pageSetup paperSize="9" orientation="portrait" horizontalDpi="0" verticalDpi="0" r:id="rId1"/>
@@ -10361,10 +10364,10 @@
     </row>
   </sheetData>
   <conditionalFormatting sqref="A2:A33">
-    <cfRule type="duplicateValues" dxfId="1" priority="1"/>
+    <cfRule type="duplicateValues" dxfId="2" priority="1"/>
   </conditionalFormatting>
   <conditionalFormatting sqref="A2:A34">
-    <cfRule type="duplicateValues" dxfId="0" priority="2"/>
+    <cfRule type="duplicateValues" dxfId="1" priority="2"/>
   </conditionalFormatting>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>

</xml_diff>

<commit_message>
UPDATE: New WS and RS September 2026
</commit_message>
<xml_diff>
--- a/gp-app-1.0/Pricelist Car.xlsx
+++ b/gp-app-1.0/Pricelist Car.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\Work\gp-app\gp-app-1.0\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{52799D07-20FD-48B2-BAE3-C136D01F2CE3}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{0A315F8A-08D3-4355-B3C9-5836BD000EAA}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-110" yWindow="-110" windowWidth="19420" windowHeight="11020" tabRatio="861" xr2:uid="{C4C7316A-D95F-426A-ADF9-AD32FA680374}"/>
   </bookViews>
@@ -2772,47 +2772,6 @@
   <dxfs count="156">
     <dxf>
       <font>
-        <b val="0"/>
-        <i val="0"/>
-        <strike val="0"/>
-        <condense val="0"/>
-        <extend val="0"/>
-        <outline val="0"/>
-        <shadow val="0"/>
-        <u val="none"/>
-        <vertAlign val="baseline"/>
-        <sz val="11"/>
-        <color theme="1"/>
-        <name val="Calibri"/>
-        <family val="2"/>
-        <scheme val="minor"/>
-      </font>
-      <numFmt numFmtId="35" formatCode="_-* #,##0.00_-;\-* #,##0.00_-;_-* &quot;-&quot;??_-;_-@_-"/>
-      <fill>
-        <patternFill patternType="none">
-          <fgColor indexed="64"/>
-          <bgColor indexed="65"/>
-        </patternFill>
-      </fill>
-      <border diagonalUp="0" diagonalDown="0">
-        <left style="thin">
-          <color indexed="64"/>
-        </left>
-        <right style="thin">
-          <color indexed="64"/>
-        </right>
-        <top style="thin">
-          <color indexed="64"/>
-        </top>
-        <bottom style="thin">
-          <color indexed="64"/>
-        </bottom>
-        <vertical/>
-        <horizontal/>
-      </border>
-    </dxf>
-    <dxf>
-      <font>
         <color rgb="FF9C0006"/>
       </font>
       <fill>
@@ -3433,6 +3392,47 @@
         <family val="2"/>
         <scheme val="minor"/>
       </font>
+      <fill>
+        <patternFill patternType="none">
+          <fgColor indexed="64"/>
+          <bgColor indexed="65"/>
+        </patternFill>
+      </fill>
+      <border diagonalUp="0" diagonalDown="0">
+        <left style="thin">
+          <color indexed="64"/>
+        </left>
+        <right style="thin">
+          <color indexed="64"/>
+        </right>
+        <top style="thin">
+          <color indexed="64"/>
+        </top>
+        <bottom style="thin">
+          <color indexed="64"/>
+        </bottom>
+        <vertical/>
+        <horizontal/>
+      </border>
+    </dxf>
+    <dxf>
+      <font>
+        <b val="0"/>
+        <i val="0"/>
+        <strike val="0"/>
+        <condense val="0"/>
+        <extend val="0"/>
+        <outline val="0"/>
+        <shadow val="0"/>
+        <u val="none"/>
+        <vertAlign val="baseline"/>
+        <sz val="11"/>
+        <color theme="1"/>
+        <name val="Calibri"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </font>
+      <numFmt numFmtId="35" formatCode="_-* #,##0.00_-;\-* #,##0.00_-;_-* &quot;-&quot;??_-;_-@_-"/>
       <fill>
         <patternFill patternType="none">
           <fgColor indexed="64"/>
@@ -5163,14 +5163,14 @@
     <tableColumn id="1" xr3:uid="{0E6335F2-6B6A-436C-92FA-B48E61551308}" name="Merek/Type" dataDxfId="151"/>
     <tableColumn id="2" xr3:uid="{5A4965DA-398A-4134-90BD-9CE4D8355880}" name="Tipe" dataDxfId="150"/>
     <tableColumn id="3" xr3:uid="{010303D1-E0A2-4DE6-8E87-64ACC3102E09}" name="Harga OTR Awal" dataDxfId="149" dataCellStyle="Comma"/>
-    <tableColumn id="4" xr3:uid="{91C798B0-7964-436A-84A5-7687993F376F}" name="Dealer Margin" dataDxfId="0" dataCellStyle="Comma">
+    <tableColumn id="4" xr3:uid="{91C798B0-7964-436A-84A5-7687993F376F}" name="Dealer Margin" dataDxfId="148" dataCellStyle="Comma">
       <calculatedColumnFormula>I2/1.12</calculatedColumnFormula>
     </tableColumn>
-    <tableColumn id="5" xr3:uid="{CD936623-36F3-4BAA-A615-AF79A61C51E8}" name="Dealer Margin 9 %" dataDxfId="148" dataCellStyle="Comma"/>
-    <tableColumn id="6" xr3:uid="{A36173E8-D9B2-4F38-A572-F5D32CDADEB8}" name="Dealer Margin 7 %" dataDxfId="147" dataCellStyle="Comma"/>
-    <tableColumn id="7" xr3:uid="{7A11B7F5-7683-492A-A8B5-D96984323DDD}" name="Code Unit" dataDxfId="146"/>
-    <tableColumn id="8" xr3:uid="{AF243BB3-2044-4D1E-9F0D-A1EC0D2C15CF}" name="Merk/Type" dataDxfId="145"/>
-    <tableColumn id="9" xr3:uid="{9E0E2E6A-108F-4ACE-959D-9EB0F753BD73}" name="Full Margin" dataDxfId="144"/>
+    <tableColumn id="5" xr3:uid="{CD936623-36F3-4BAA-A615-AF79A61C51E8}" name="Dealer Margin 9 %" dataDxfId="147" dataCellStyle="Comma"/>
+    <tableColumn id="6" xr3:uid="{A36173E8-D9B2-4F38-A572-F5D32CDADEB8}" name="Dealer Margin 7 %" dataDxfId="146" dataCellStyle="Comma"/>
+    <tableColumn id="7" xr3:uid="{7A11B7F5-7683-492A-A8B5-D96984323DDD}" name="Code Unit" dataDxfId="145"/>
+    <tableColumn id="8" xr3:uid="{AF243BB3-2044-4D1E-9F0D-A1EC0D2C15CF}" name="Merk/Type" dataDxfId="144"/>
+    <tableColumn id="9" xr3:uid="{9E0E2E6A-108F-4ACE-959D-9EB0F753BD73}" name="Full Margin" dataDxfId="143"/>
   </tableColumns>
   <tableStyleInfo name="TableStyleMedium2" showFirstColumn="0" showLastColumn="0" showRowStripes="1" showColumnStripes="0"/>
 </table>
@@ -5180,15 +5180,15 @@
 <table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="9" xr:uid="{630D8221-A5B4-4162-BEFC-7BB63825B861}" name="Table009__Page_6" displayName="Table009__Page_6" ref="A1:I16" tableType="queryTable" totalsRowShown="0">
   <autoFilter ref="A1:I16" xr:uid="{630D8221-A5B4-4162-BEFC-7BB63825B861}"/>
   <tableColumns count="9">
-    <tableColumn id="1" xr3:uid="{5980B244-73E4-43AF-B863-305E8B039C33}" uniqueName="1" name="Column1" queryTableFieldId="1" dataDxfId="77"/>
-    <tableColumn id="2" xr3:uid="{549208EE-7E07-4F0F-ACFD-9606CC8F6B50}" uniqueName="2" name="Column2" queryTableFieldId="2" dataDxfId="76"/>
-    <tableColumn id="3" xr3:uid="{086F7B88-A201-47FD-B9A0-0C976108E144}" uniqueName="3" name="Column3" queryTableFieldId="3" dataDxfId="75"/>
-    <tableColumn id="4" xr3:uid="{CC912184-CE02-4DC9-8815-71C4295C86DF}" uniqueName="4" name="Column4" queryTableFieldId="4" dataDxfId="74"/>
-    <tableColumn id="5" xr3:uid="{8F3F2202-7C07-4D43-B483-871C9E242208}" uniqueName="5" name="Column5" queryTableFieldId="5" dataDxfId="73"/>
-    <tableColumn id="6" xr3:uid="{6D2190D6-B434-4BB9-95B1-A29148C453AF}" uniqueName="6" name="Column6" queryTableFieldId="6" dataDxfId="72"/>
-    <tableColumn id="7" xr3:uid="{A33DE0AF-7DA7-4623-87E7-DBA2BF4E404A}" uniqueName="7" name="Column7" queryTableFieldId="7" dataDxfId="71"/>
-    <tableColumn id="8" xr3:uid="{CD689B59-BA44-4F67-9FF9-E08337BE66FD}" uniqueName="8" name="Column8" queryTableFieldId="8" dataDxfId="70"/>
-    <tableColumn id="9" xr3:uid="{744F224A-BA1E-4758-B291-8D5C8D341610}" uniqueName="9" name="Column9" queryTableFieldId="9" dataDxfId="69"/>
+    <tableColumn id="1" xr3:uid="{5980B244-73E4-43AF-B863-305E8B039C33}" uniqueName="1" name="Column1" queryTableFieldId="1" dataDxfId="76"/>
+    <tableColumn id="2" xr3:uid="{549208EE-7E07-4F0F-ACFD-9606CC8F6B50}" uniqueName="2" name="Column2" queryTableFieldId="2" dataDxfId="75"/>
+    <tableColumn id="3" xr3:uid="{086F7B88-A201-47FD-B9A0-0C976108E144}" uniqueName="3" name="Column3" queryTableFieldId="3" dataDxfId="74"/>
+    <tableColumn id="4" xr3:uid="{CC912184-CE02-4DC9-8815-71C4295C86DF}" uniqueName="4" name="Column4" queryTableFieldId="4" dataDxfId="73"/>
+    <tableColumn id="5" xr3:uid="{8F3F2202-7C07-4D43-B483-871C9E242208}" uniqueName="5" name="Column5" queryTableFieldId="5" dataDxfId="72"/>
+    <tableColumn id="6" xr3:uid="{6D2190D6-B434-4BB9-95B1-A29148C453AF}" uniqueName="6" name="Column6" queryTableFieldId="6" dataDxfId="71"/>
+    <tableColumn id="7" xr3:uid="{A33DE0AF-7DA7-4623-87E7-DBA2BF4E404A}" uniqueName="7" name="Column7" queryTableFieldId="7" dataDxfId="70"/>
+    <tableColumn id="8" xr3:uid="{CD689B59-BA44-4F67-9FF9-E08337BE66FD}" uniqueName="8" name="Column8" queryTableFieldId="8" dataDxfId="69"/>
+    <tableColumn id="9" xr3:uid="{744F224A-BA1E-4758-B291-8D5C8D341610}" uniqueName="9" name="Column9" queryTableFieldId="9" dataDxfId="68"/>
   </tableColumns>
   <tableStyleInfo name="TableStyleMedium7" showFirstColumn="0" showLastColumn="0" showRowStripes="1" showColumnStripes="0"/>
 </table>
@@ -5198,15 +5198,15 @@
 <table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="10" xr:uid="{116BBD7B-F856-4C44-8F1F-EA66756E3A0B}" name="Table010__Page_6" displayName="Table010__Page_6" ref="A18:I20" tableType="queryTable" totalsRowShown="0">
   <autoFilter ref="A18:I20" xr:uid="{116BBD7B-F856-4C44-8F1F-EA66756E3A0B}"/>
   <tableColumns count="9">
-    <tableColumn id="1" xr3:uid="{D02866AC-7C8C-4041-B0D6-297717EA2BCA}" uniqueName="1" name="Column1" queryTableFieldId="1" dataDxfId="68"/>
-    <tableColumn id="2" xr3:uid="{F9BA0334-AC0F-4599-91DD-1D3B53530BA2}" uniqueName="2" name="Column2" queryTableFieldId="2" dataDxfId="67"/>
-    <tableColumn id="3" xr3:uid="{2E40CB08-FF90-4211-A5F6-3255AA5CEAED}" uniqueName="3" name="Column3" queryTableFieldId="3" dataDxfId="66"/>
-    <tableColumn id="4" xr3:uid="{951E49DE-3DB8-41C0-8F36-6E5A1649659D}" uniqueName="4" name="Column4" queryTableFieldId="4" dataDxfId="65"/>
-    <tableColumn id="5" xr3:uid="{D7FC7D23-AA29-4FAE-8DF4-B23A11020D8C}" uniqueName="5" name="Column5" queryTableFieldId="5" dataDxfId="64"/>
-    <tableColumn id="6" xr3:uid="{85DA6C7C-BC56-4316-BB56-3D2CA86DF4B0}" uniqueName="6" name="Column6" queryTableFieldId="6" dataDxfId="63"/>
-    <tableColumn id="7" xr3:uid="{47F39228-8CCC-4319-9964-568280350AF4}" uniqueName="7" name="Column7" queryTableFieldId="7" dataDxfId="62"/>
-    <tableColumn id="8" xr3:uid="{781188CD-5AC0-41B9-8575-2EACD4BA90A4}" uniqueName="8" name="Column8" queryTableFieldId="8" dataDxfId="61"/>
-    <tableColumn id="9" xr3:uid="{A2DFBEC8-960F-4613-A8B8-821CF42818AC}" uniqueName="9" name="Column9" queryTableFieldId="9" dataDxfId="60"/>
+    <tableColumn id="1" xr3:uid="{D02866AC-7C8C-4041-B0D6-297717EA2BCA}" uniqueName="1" name="Column1" queryTableFieldId="1" dataDxfId="67"/>
+    <tableColumn id="2" xr3:uid="{F9BA0334-AC0F-4599-91DD-1D3B53530BA2}" uniqueName="2" name="Column2" queryTableFieldId="2" dataDxfId="66"/>
+    <tableColumn id="3" xr3:uid="{2E40CB08-FF90-4211-A5F6-3255AA5CEAED}" uniqueName="3" name="Column3" queryTableFieldId="3" dataDxfId="65"/>
+    <tableColumn id="4" xr3:uid="{951E49DE-3DB8-41C0-8F36-6E5A1649659D}" uniqueName="4" name="Column4" queryTableFieldId="4" dataDxfId="64"/>
+    <tableColumn id="5" xr3:uid="{D7FC7D23-AA29-4FAE-8DF4-B23A11020D8C}" uniqueName="5" name="Column5" queryTableFieldId="5" dataDxfId="63"/>
+    <tableColumn id="6" xr3:uid="{85DA6C7C-BC56-4316-BB56-3D2CA86DF4B0}" uniqueName="6" name="Column6" queryTableFieldId="6" dataDxfId="62"/>
+    <tableColumn id="7" xr3:uid="{47F39228-8CCC-4319-9964-568280350AF4}" uniqueName="7" name="Column7" queryTableFieldId="7" dataDxfId="61"/>
+    <tableColumn id="8" xr3:uid="{781188CD-5AC0-41B9-8575-2EACD4BA90A4}" uniqueName="8" name="Column8" queryTableFieldId="8" dataDxfId="60"/>
+    <tableColumn id="9" xr3:uid="{A2DFBEC8-960F-4613-A8B8-821CF42818AC}" uniqueName="9" name="Column9" queryTableFieldId="9" dataDxfId="59"/>
   </tableColumns>
   <tableStyleInfo name="TableStyleMedium7" showFirstColumn="0" showLastColumn="0" showRowStripes="1" showColumnStripes="0"/>
 </table>
@@ -5216,9 +5216,9 @@
 <table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="11" xr:uid="{D5A80464-2F5E-4F81-BC09-642A89962C82}" name="Table011__Page_7" displayName="Table011__Page_7" ref="A1:C15" tableType="queryTable" totalsRowShown="0">
   <autoFilter ref="A1:C15" xr:uid="{D5A80464-2F5E-4F81-BC09-642A89962C82}"/>
   <tableColumns count="3">
-    <tableColumn id="1" xr3:uid="{384F6B08-E7B1-4ECD-BC7E-1F8C8FC9CD11}" uniqueName="1" name="Column1" queryTableFieldId="1" dataDxfId="59"/>
-    <tableColumn id="2" xr3:uid="{BD116665-54B3-487B-82AD-7E260403FB1A}" uniqueName="2" name="Column2" queryTableFieldId="2" dataDxfId="58"/>
-    <tableColumn id="3" xr3:uid="{A0C72322-3C63-446F-A7B0-E45538411191}" uniqueName="3" name="Column3" queryTableFieldId="3" dataDxfId="57"/>
+    <tableColumn id="1" xr3:uid="{384F6B08-E7B1-4ECD-BC7E-1F8C8FC9CD11}" uniqueName="1" name="Column1" queryTableFieldId="1" dataDxfId="58"/>
+    <tableColumn id="2" xr3:uid="{BD116665-54B3-487B-82AD-7E260403FB1A}" uniqueName="2" name="Column2" queryTableFieldId="2" dataDxfId="57"/>
+    <tableColumn id="3" xr3:uid="{A0C72322-3C63-446F-A7B0-E45538411191}" uniqueName="3" name="Column3" queryTableFieldId="3" dataDxfId="56"/>
   </tableColumns>
   <tableStyleInfo name="TableStyleMedium7" showFirstColumn="0" showLastColumn="0" showRowStripes="1" showColumnStripes="0"/>
 </table>
@@ -5228,9 +5228,9 @@
 <table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="12" xr:uid="{BF5A7D5F-42BD-4927-9517-2459449E72C6}" name="Table012__Page_7" displayName="Table012__Page_7" ref="A17:C19" tableType="queryTable" totalsRowShown="0">
   <autoFilter ref="A17:C19" xr:uid="{BF5A7D5F-42BD-4927-9517-2459449E72C6}"/>
   <tableColumns count="3">
-    <tableColumn id="1" xr3:uid="{92B56AD9-FE6F-4702-B777-811CB1B6E64F}" uniqueName="1" name="Column1" queryTableFieldId="1" dataDxfId="56"/>
-    <tableColumn id="2" xr3:uid="{C37743D7-7886-43A1-BB26-C0F3914426C9}" uniqueName="2" name="Column2" queryTableFieldId="2" dataDxfId="55"/>
-    <tableColumn id="3" xr3:uid="{DFF6BFBF-623A-4318-86AF-C5448FC821A5}" uniqueName="3" name="Column3" queryTableFieldId="3" dataDxfId="54"/>
+    <tableColumn id="1" xr3:uid="{92B56AD9-FE6F-4702-B777-811CB1B6E64F}" uniqueName="1" name="Column1" queryTableFieldId="1" dataDxfId="55"/>
+    <tableColumn id="2" xr3:uid="{C37743D7-7886-43A1-BB26-C0F3914426C9}" uniqueName="2" name="Column2" queryTableFieldId="2" dataDxfId="54"/>
+    <tableColumn id="3" xr3:uid="{DFF6BFBF-623A-4318-86AF-C5448FC821A5}" uniqueName="3" name="Column3" queryTableFieldId="3" dataDxfId="53"/>
   </tableColumns>
   <tableStyleInfo name="TableStyleMedium7" showFirstColumn="0" showLastColumn="0" showRowStripes="1" showColumnStripes="0"/>
 </table>
@@ -5240,11 +5240,11 @@
 <table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="13" xr:uid="{4DAA9679-BE71-4F3A-B608-132984AF6DF1}" name="Table013__Page_8" displayName="Table013__Page_8" ref="A1:E16" tableType="queryTable" totalsRowShown="0">
   <autoFilter ref="A1:E16" xr:uid="{4DAA9679-BE71-4F3A-B608-132984AF6DF1}"/>
   <tableColumns count="5">
-    <tableColumn id="1" xr3:uid="{811DEB23-A3B8-4E1E-AF98-CBD4FE9515C8}" uniqueName="1" name="Column1" queryTableFieldId="1" dataDxfId="53"/>
-    <tableColumn id="2" xr3:uid="{D1233A63-9D37-45F3-9DC7-52977AC06ADC}" uniqueName="2" name="Column2" queryTableFieldId="2" dataDxfId="52"/>
-    <tableColumn id="3" xr3:uid="{400191B1-4CF8-4D78-82E7-FED7CD6730E6}" uniqueName="3" name="Column3" queryTableFieldId="3" dataDxfId="51"/>
-    <tableColumn id="4" xr3:uid="{3D829CC4-4292-4CD0-80B8-3490D4014AC9}" uniqueName="4" name="Column4" queryTableFieldId="4" dataDxfId="50"/>
-    <tableColumn id="5" xr3:uid="{9BC50CF1-EF44-42B4-9129-E887F74428C9}" uniqueName="5" name="Column5" queryTableFieldId="5" dataDxfId="49"/>
+    <tableColumn id="1" xr3:uid="{811DEB23-A3B8-4E1E-AF98-CBD4FE9515C8}" uniqueName="1" name="Column1" queryTableFieldId="1" dataDxfId="52"/>
+    <tableColumn id="2" xr3:uid="{D1233A63-9D37-45F3-9DC7-52977AC06ADC}" uniqueName="2" name="Column2" queryTableFieldId="2" dataDxfId="51"/>
+    <tableColumn id="3" xr3:uid="{400191B1-4CF8-4D78-82E7-FED7CD6730E6}" uniqueName="3" name="Column3" queryTableFieldId="3" dataDxfId="50"/>
+    <tableColumn id="4" xr3:uid="{3D829CC4-4292-4CD0-80B8-3490D4014AC9}" uniqueName="4" name="Column4" queryTableFieldId="4" dataDxfId="49"/>
+    <tableColumn id="5" xr3:uid="{9BC50CF1-EF44-42B4-9129-E887F74428C9}" uniqueName="5" name="Column5" queryTableFieldId="5" dataDxfId="48"/>
   </tableColumns>
   <tableStyleInfo name="TableStyleMedium7" showFirstColumn="0" showLastColumn="0" showRowStripes="1" showColumnStripes="0"/>
 </table>
@@ -5254,11 +5254,11 @@
 <table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="14" xr:uid="{9D3195A8-F1BD-4429-B95A-60FCF241B775}" name="Table014__Page_8" displayName="Table014__Page_8" ref="A18:E21" tableType="queryTable" totalsRowShown="0">
   <autoFilter ref="A18:E21" xr:uid="{9D3195A8-F1BD-4429-B95A-60FCF241B775}"/>
   <tableColumns count="5">
-    <tableColumn id="1" xr3:uid="{98A6121C-2EC1-48CA-8A40-28DAFD66423E}" uniqueName="1" name="Column1" queryTableFieldId="1" dataDxfId="48"/>
-    <tableColumn id="2" xr3:uid="{6B521FB3-E639-4556-B8C5-473A63201BC1}" uniqueName="2" name="Column2" queryTableFieldId="2" dataDxfId="47"/>
-    <tableColumn id="3" xr3:uid="{3D07F9E9-4DA3-41C6-98A7-BC28F0C8BFB5}" uniqueName="3" name="Column3" queryTableFieldId="3" dataDxfId="46"/>
-    <tableColumn id="4" xr3:uid="{89F1E0D5-9B1D-4170-BB1D-3FBA7855FC27}" uniqueName="4" name="Column4" queryTableFieldId="4" dataDxfId="45"/>
-    <tableColumn id="5" xr3:uid="{68E29A0D-4E20-4E2A-A030-157EF3C69E97}" uniqueName="5" name="Column5" queryTableFieldId="5" dataDxfId="44"/>
+    <tableColumn id="1" xr3:uid="{98A6121C-2EC1-48CA-8A40-28DAFD66423E}" uniqueName="1" name="Column1" queryTableFieldId="1" dataDxfId="47"/>
+    <tableColumn id="2" xr3:uid="{6B521FB3-E639-4556-B8C5-473A63201BC1}" uniqueName="2" name="Column2" queryTableFieldId="2" dataDxfId="46"/>
+    <tableColumn id="3" xr3:uid="{3D07F9E9-4DA3-41C6-98A7-BC28F0C8BFB5}" uniqueName="3" name="Column3" queryTableFieldId="3" dataDxfId="45"/>
+    <tableColumn id="4" xr3:uid="{89F1E0D5-9B1D-4170-BB1D-3FBA7855FC27}" uniqueName="4" name="Column4" queryTableFieldId="4" dataDxfId="44"/>
+    <tableColumn id="5" xr3:uid="{68E29A0D-4E20-4E2A-A030-157EF3C69E97}" uniqueName="5" name="Column5" queryTableFieldId="5" dataDxfId="43"/>
   </tableColumns>
   <tableStyleInfo name="TableStyleMedium7" showFirstColumn="0" showLastColumn="0" showRowStripes="1" showColumnStripes="0"/>
 </table>
@@ -5268,12 +5268,12 @@
 <table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="15" xr:uid="{F2B12C92-B774-477F-98C9-509526BBDEE5}" name="Table015__Page_9" displayName="Table015__Page_9" ref="A1:F16" tableType="queryTable" totalsRowShown="0">
   <autoFilter ref="A1:F16" xr:uid="{F2B12C92-B774-477F-98C9-509526BBDEE5}"/>
   <tableColumns count="6">
-    <tableColumn id="1" xr3:uid="{B9D47F1B-922B-4B02-855C-93AF62167342}" uniqueName="1" name="Column1" queryTableFieldId="1" dataDxfId="43"/>
-    <tableColumn id="2" xr3:uid="{9915D8BD-1C99-4D36-BE7E-9EBEAD6D7B12}" uniqueName="2" name="Column2" queryTableFieldId="2" dataDxfId="42"/>
-    <tableColumn id="3" xr3:uid="{D353D58B-6A1D-4079-A9EC-77376B67A375}" uniqueName="3" name="Column3" queryTableFieldId="3" dataDxfId="41"/>
-    <tableColumn id="4" xr3:uid="{ACF53426-7425-4D38-9673-B3197A3F9292}" uniqueName="4" name="Column4" queryTableFieldId="4" dataDxfId="40"/>
-    <tableColumn id="5" xr3:uid="{673A9374-D6DA-46D7-AAD2-6F2220F4ED8C}" uniqueName="5" name="Column5" queryTableFieldId="5" dataDxfId="39"/>
-    <tableColumn id="6" xr3:uid="{37C428F9-0692-44D1-B8CF-2CBC7901020B}" uniqueName="6" name="Column6" queryTableFieldId="6" dataDxfId="38"/>
+    <tableColumn id="1" xr3:uid="{B9D47F1B-922B-4B02-855C-93AF62167342}" uniqueName="1" name="Column1" queryTableFieldId="1" dataDxfId="42"/>
+    <tableColumn id="2" xr3:uid="{9915D8BD-1C99-4D36-BE7E-9EBEAD6D7B12}" uniqueName="2" name="Column2" queryTableFieldId="2" dataDxfId="41"/>
+    <tableColumn id="3" xr3:uid="{D353D58B-6A1D-4079-A9EC-77376B67A375}" uniqueName="3" name="Column3" queryTableFieldId="3" dataDxfId="40"/>
+    <tableColumn id="4" xr3:uid="{ACF53426-7425-4D38-9673-B3197A3F9292}" uniqueName="4" name="Column4" queryTableFieldId="4" dataDxfId="39"/>
+    <tableColumn id="5" xr3:uid="{673A9374-D6DA-46D7-AAD2-6F2220F4ED8C}" uniqueName="5" name="Column5" queryTableFieldId="5" dataDxfId="38"/>
+    <tableColumn id="6" xr3:uid="{37C428F9-0692-44D1-B8CF-2CBC7901020B}" uniqueName="6" name="Column6" queryTableFieldId="6" dataDxfId="37"/>
   </tableColumns>
   <tableStyleInfo name="TableStyleMedium7" showFirstColumn="0" showLastColumn="0" showRowStripes="1" showColumnStripes="0"/>
 </table>
@@ -5283,12 +5283,12 @@
 <table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="16" xr:uid="{3C596C1A-3A31-47DF-B534-2A3593167FFF}" name="Table016__Page_9" displayName="Table016__Page_9" ref="A18:F20" tableType="queryTable" totalsRowShown="0">
   <autoFilter ref="A18:F20" xr:uid="{3C596C1A-3A31-47DF-B534-2A3593167FFF}"/>
   <tableColumns count="6">
-    <tableColumn id="1" xr3:uid="{48EBD4D1-26EB-449F-8D09-DF1A8D9D96A3}" uniqueName="1" name="Column1" queryTableFieldId="1" dataDxfId="37"/>
-    <tableColumn id="2" xr3:uid="{671AE648-452F-44F1-9A65-8468F7B19950}" uniqueName="2" name="Column2" queryTableFieldId="2" dataDxfId="36"/>
-    <tableColumn id="3" xr3:uid="{C3287937-E8A8-4D80-A27C-D2A5C0E44D68}" uniqueName="3" name="Column3" queryTableFieldId="3" dataDxfId="35"/>
-    <tableColumn id="4" xr3:uid="{49CAB777-0355-40CC-9F2D-C41408ED9E98}" uniqueName="4" name="Column4" queryTableFieldId="4" dataDxfId="34"/>
-    <tableColumn id="5" xr3:uid="{A19C49CB-F2CF-4D60-B082-761FE4F0ABC5}" uniqueName="5" name="Column5" queryTableFieldId="5" dataDxfId="33"/>
-    <tableColumn id="6" xr3:uid="{801427E9-2562-451E-AE45-ACF6DAAAFFFB}" uniqueName="6" name="Column6" queryTableFieldId="6" dataDxfId="32"/>
+    <tableColumn id="1" xr3:uid="{48EBD4D1-26EB-449F-8D09-DF1A8D9D96A3}" uniqueName="1" name="Column1" queryTableFieldId="1" dataDxfId="36"/>
+    <tableColumn id="2" xr3:uid="{671AE648-452F-44F1-9A65-8468F7B19950}" uniqueName="2" name="Column2" queryTableFieldId="2" dataDxfId="35"/>
+    <tableColumn id="3" xr3:uid="{C3287937-E8A8-4D80-A27C-D2A5C0E44D68}" uniqueName="3" name="Column3" queryTableFieldId="3" dataDxfId="34"/>
+    <tableColumn id="4" xr3:uid="{49CAB777-0355-40CC-9F2D-C41408ED9E98}" uniqueName="4" name="Column4" queryTableFieldId="4" dataDxfId="33"/>
+    <tableColumn id="5" xr3:uid="{A19C49CB-F2CF-4D60-B082-761FE4F0ABC5}" uniqueName="5" name="Column5" queryTableFieldId="5" dataDxfId="32"/>
+    <tableColumn id="6" xr3:uid="{801427E9-2562-451E-AE45-ACF6DAAAFFFB}" uniqueName="6" name="Column6" queryTableFieldId="6" dataDxfId="31"/>
   </tableColumns>
   <tableStyleInfo name="TableStyleMedium7" showFirstColumn="0" showLastColumn="0" showRowStripes="1" showColumnStripes="0"/>
 </table>
@@ -5298,11 +5298,11 @@
 <table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="17" xr:uid="{510F87AB-8378-4FE2-9EBF-7361BA7DB6B8}" name="Table017__Page_10" displayName="Table017__Page_10" ref="A1:E15" tableType="queryTable" totalsRowShown="0">
   <autoFilter ref="A1:E15" xr:uid="{510F87AB-8378-4FE2-9EBF-7361BA7DB6B8}"/>
   <tableColumns count="5">
-    <tableColumn id="1" xr3:uid="{626476ED-551C-48ED-A0F5-9CB680097EF0}" uniqueName="1" name="Column1" queryTableFieldId="1" dataDxfId="31"/>
-    <tableColumn id="2" xr3:uid="{9215A7DD-9718-48E5-BA20-B6B9989DD0D2}" uniqueName="2" name="Column2" queryTableFieldId="2" dataDxfId="30"/>
-    <tableColumn id="3" xr3:uid="{AE2AC56F-3587-4342-A60B-0B4A30905DD3}" uniqueName="3" name="Column3" queryTableFieldId="3" dataDxfId="29"/>
-    <tableColumn id="4" xr3:uid="{F7BE237D-2C3F-4C27-92EF-2601ABCBA887}" uniqueName="4" name="Column4" queryTableFieldId="4" dataDxfId="28"/>
-    <tableColumn id="5" xr3:uid="{7950C4F9-8FA4-4C6E-B03A-A0235ECC51FF}" uniqueName="5" name="Column5" queryTableFieldId="5" dataDxfId="27"/>
+    <tableColumn id="1" xr3:uid="{626476ED-551C-48ED-A0F5-9CB680097EF0}" uniqueName="1" name="Column1" queryTableFieldId="1" dataDxfId="30"/>
+    <tableColumn id="2" xr3:uid="{9215A7DD-9718-48E5-BA20-B6B9989DD0D2}" uniqueName="2" name="Column2" queryTableFieldId="2" dataDxfId="29"/>
+    <tableColumn id="3" xr3:uid="{AE2AC56F-3587-4342-A60B-0B4A30905DD3}" uniqueName="3" name="Column3" queryTableFieldId="3" dataDxfId="28"/>
+    <tableColumn id="4" xr3:uid="{F7BE237D-2C3F-4C27-92EF-2601ABCBA887}" uniqueName="4" name="Column4" queryTableFieldId="4" dataDxfId="27"/>
+    <tableColumn id="5" xr3:uid="{7950C4F9-8FA4-4C6E-B03A-A0235ECC51FF}" uniqueName="5" name="Column5" queryTableFieldId="5" dataDxfId="26"/>
   </tableColumns>
   <tableStyleInfo name="TableStyleMedium7" showFirstColumn="0" showLastColumn="0" showRowStripes="1" showColumnStripes="0"/>
 </table>
@@ -5312,11 +5312,11 @@
 <table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="18" xr:uid="{14CF879A-74C7-4F0C-8E76-F1430C9579CD}" name="Table018__Page_10" displayName="Table018__Page_10" ref="A17:E19" tableType="queryTable" totalsRowShown="0">
   <autoFilter ref="A17:E19" xr:uid="{14CF879A-74C7-4F0C-8E76-F1430C9579CD}"/>
   <tableColumns count="5">
-    <tableColumn id="1" xr3:uid="{210B1486-2DC9-4D94-98AC-6BEB874B7545}" uniqueName="1" name="Column1" queryTableFieldId="1" dataDxfId="26"/>
-    <tableColumn id="2" xr3:uid="{BB67F395-3AAE-4514-BCCE-DE32693EB37D}" uniqueName="2" name="Column2" queryTableFieldId="2" dataDxfId="25"/>
-    <tableColumn id="3" xr3:uid="{230B22CA-5CA3-4E2D-92CC-C75BC5831FF2}" uniqueName="3" name="Column3" queryTableFieldId="3" dataDxfId="24"/>
-    <tableColumn id="4" xr3:uid="{42788CA6-A70D-442A-9072-79E0D19F0B28}" uniqueName="4" name="Column4" queryTableFieldId="4" dataDxfId="23"/>
-    <tableColumn id="5" xr3:uid="{E37C1038-7442-4E7D-BB43-162AD6FA4195}" uniqueName="5" name="Column5" queryTableFieldId="5" dataDxfId="22"/>
+    <tableColumn id="1" xr3:uid="{210B1486-2DC9-4D94-98AC-6BEB874B7545}" uniqueName="1" name="Column1" queryTableFieldId="1" dataDxfId="25"/>
+    <tableColumn id="2" xr3:uid="{BB67F395-3AAE-4514-BCCE-DE32693EB37D}" uniqueName="2" name="Column2" queryTableFieldId="2" dataDxfId="24"/>
+    <tableColumn id="3" xr3:uid="{230B22CA-5CA3-4E2D-92CC-C75BC5831FF2}" uniqueName="3" name="Column3" queryTableFieldId="3" dataDxfId="23"/>
+    <tableColumn id="4" xr3:uid="{42788CA6-A70D-442A-9072-79E0D19F0B28}" uniqueName="4" name="Column4" queryTableFieldId="4" dataDxfId="22"/>
+    <tableColumn id="5" xr3:uid="{E37C1038-7442-4E7D-BB43-162AD6FA4195}" uniqueName="5" name="Column5" queryTableFieldId="5" dataDxfId="21"/>
   </tableColumns>
   <tableStyleInfo name="TableStyleMedium7" showFirstColumn="0" showLastColumn="0" showRowStripes="1" showColumnStripes="0"/>
 </table>
@@ -5326,13 +5326,13 @@
 <table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="1" xr:uid="{8D8C9D73-217D-4974-B35A-0740746DA27F}" name="Table001__Page_2" displayName="Table001__Page_2" ref="A1:G16" tableType="queryTable" totalsRowShown="0">
   <autoFilter ref="A1:G16" xr:uid="{8D8C9D73-217D-4974-B35A-0740746DA27F}"/>
   <tableColumns count="7">
-    <tableColumn id="1" xr3:uid="{A26CE965-72B2-472B-B9FF-D68F7847F3C5}" uniqueName="1" name="Column1" queryTableFieldId="1" dataDxfId="143"/>
-    <tableColumn id="2" xr3:uid="{375BF78E-5806-424A-B7BD-C63C40843BE9}" uniqueName="2" name="Column2" queryTableFieldId="2" dataDxfId="142"/>
-    <tableColumn id="3" xr3:uid="{CD1FFC74-B097-42B5-B1FA-08D3BD4531B9}" uniqueName="3" name="Column3" queryTableFieldId="3" dataDxfId="141"/>
-    <tableColumn id="4" xr3:uid="{EA6F5C08-47B3-4BE3-8F9B-3167F2B34338}" uniqueName="4" name="Column4" queryTableFieldId="4" dataDxfId="140"/>
-    <tableColumn id="5" xr3:uid="{67D1B145-6151-4A54-9C79-A6B0381CDA09}" uniqueName="5" name="Column5" queryTableFieldId="5" dataDxfId="139"/>
-    <tableColumn id="6" xr3:uid="{E8D8899E-ED32-4A2F-B13D-18F4C289A59B}" uniqueName="6" name="Column6" queryTableFieldId="6" dataDxfId="138"/>
-    <tableColumn id="7" xr3:uid="{CD1BCBB0-10DE-4DDA-903D-C14D16829749}" uniqueName="7" name="Column7" queryTableFieldId="7" dataDxfId="137"/>
+    <tableColumn id="1" xr3:uid="{A26CE965-72B2-472B-B9FF-D68F7847F3C5}" uniqueName="1" name="Column1" queryTableFieldId="1" dataDxfId="142"/>
+    <tableColumn id="2" xr3:uid="{375BF78E-5806-424A-B7BD-C63C40843BE9}" uniqueName="2" name="Column2" queryTableFieldId="2" dataDxfId="141"/>
+    <tableColumn id="3" xr3:uid="{CD1FFC74-B097-42B5-B1FA-08D3BD4531B9}" uniqueName="3" name="Column3" queryTableFieldId="3" dataDxfId="140"/>
+    <tableColumn id="4" xr3:uid="{EA6F5C08-47B3-4BE3-8F9B-3167F2B34338}" uniqueName="4" name="Column4" queryTableFieldId="4" dataDxfId="139"/>
+    <tableColumn id="5" xr3:uid="{67D1B145-6151-4A54-9C79-A6B0381CDA09}" uniqueName="5" name="Column5" queryTableFieldId="5" dataDxfId="138"/>
+    <tableColumn id="6" xr3:uid="{E8D8899E-ED32-4A2F-B13D-18F4C289A59B}" uniqueName="6" name="Column6" queryTableFieldId="6" dataDxfId="137"/>
+    <tableColumn id="7" xr3:uid="{CD1BCBB0-10DE-4DDA-903D-C14D16829749}" uniqueName="7" name="Column7" queryTableFieldId="7" dataDxfId="136"/>
   </tableColumns>
   <tableStyleInfo name="TableStyleMedium7" showFirstColumn="0" showLastColumn="0" showRowStripes="1" showColumnStripes="0"/>
 </table>
@@ -5342,11 +5342,11 @@
 <table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="19" xr:uid="{A8D65B7F-C1B3-4E37-BFF7-03252131F371}" name="Table019__Page_11" displayName="Table019__Page_11" ref="A1:E16" tableType="queryTable" totalsRowShown="0">
   <autoFilter ref="A1:E16" xr:uid="{A8D65B7F-C1B3-4E37-BFF7-03252131F371}"/>
   <tableColumns count="5">
-    <tableColumn id="1" xr3:uid="{60EAA1C9-E43C-458C-A33C-365CF023541D}" uniqueName="1" name="Column1" queryTableFieldId="1" dataDxfId="21"/>
-    <tableColumn id="2" xr3:uid="{BF4ECEAF-8998-4833-A444-7DD2840947AB}" uniqueName="2" name="Column2" queryTableFieldId="2" dataDxfId="20"/>
-    <tableColumn id="3" xr3:uid="{A77E13C5-CB25-43C0-9678-51A378FA64FC}" uniqueName="3" name="Column3" queryTableFieldId="3" dataDxfId="19"/>
-    <tableColumn id="4" xr3:uid="{46713ABC-AA6E-45DD-9BBE-03C863D6B1D1}" uniqueName="4" name="Column4" queryTableFieldId="4" dataDxfId="18"/>
-    <tableColumn id="5" xr3:uid="{85365AB6-280F-40C4-AB42-3455547D61F1}" uniqueName="5" name="Column5" queryTableFieldId="5" dataDxfId="17"/>
+    <tableColumn id="1" xr3:uid="{60EAA1C9-E43C-458C-A33C-365CF023541D}" uniqueName="1" name="Column1" queryTableFieldId="1" dataDxfId="20"/>
+    <tableColumn id="2" xr3:uid="{BF4ECEAF-8998-4833-A444-7DD2840947AB}" uniqueName="2" name="Column2" queryTableFieldId="2" dataDxfId="19"/>
+    <tableColumn id="3" xr3:uid="{A77E13C5-CB25-43C0-9678-51A378FA64FC}" uniqueName="3" name="Column3" queryTableFieldId="3" dataDxfId="18"/>
+    <tableColumn id="4" xr3:uid="{46713ABC-AA6E-45DD-9BBE-03C863D6B1D1}" uniqueName="4" name="Column4" queryTableFieldId="4" dataDxfId="17"/>
+    <tableColumn id="5" xr3:uid="{85365AB6-280F-40C4-AB42-3455547D61F1}" uniqueName="5" name="Column5" queryTableFieldId="5" dataDxfId="16"/>
   </tableColumns>
   <tableStyleInfo name="TableStyleMedium7" showFirstColumn="0" showLastColumn="0" showRowStripes="1" showColumnStripes="0"/>
 </table>
@@ -5356,11 +5356,11 @@
 <table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="21" xr:uid="{0B4290D5-7CEE-4DDC-B997-690EEF6D9589}" name="Table020__Page_11" displayName="Table020__Page_11" ref="A18:E20" tableType="queryTable" totalsRowShown="0">
   <autoFilter ref="A18:E20" xr:uid="{0B4290D5-7CEE-4DDC-B997-690EEF6D9589}"/>
   <tableColumns count="5">
-    <tableColumn id="1" xr3:uid="{344C3D84-8C5A-4C60-ADD3-4EE73F83858B}" uniqueName="1" name="Column1" queryTableFieldId="1" dataDxfId="16"/>
-    <tableColumn id="2" xr3:uid="{3470DF86-5A38-429A-95CF-F5FF5E59449C}" uniqueName="2" name="Column2" queryTableFieldId="2" dataDxfId="15"/>
-    <tableColumn id="3" xr3:uid="{BC1BD851-46F6-4634-95EE-ED117E75EBB6}" uniqueName="3" name="Column3" queryTableFieldId="3" dataDxfId="14"/>
-    <tableColumn id="4" xr3:uid="{FF5D3D34-BBDB-4113-8340-C737255ED1BD}" uniqueName="4" name="Column4" queryTableFieldId="4" dataDxfId="13"/>
-    <tableColumn id="5" xr3:uid="{F05FA152-C9D6-4773-B0A5-5B18B60C7102}" uniqueName="5" name="Column5" queryTableFieldId="5" dataDxfId="12"/>
+    <tableColumn id="1" xr3:uid="{344C3D84-8C5A-4C60-ADD3-4EE73F83858B}" uniqueName="1" name="Column1" queryTableFieldId="1" dataDxfId="15"/>
+    <tableColumn id="2" xr3:uid="{3470DF86-5A38-429A-95CF-F5FF5E59449C}" uniqueName="2" name="Column2" queryTableFieldId="2" dataDxfId="14"/>
+    <tableColumn id="3" xr3:uid="{BC1BD851-46F6-4634-95EE-ED117E75EBB6}" uniqueName="3" name="Column3" queryTableFieldId="3" dataDxfId="13"/>
+    <tableColumn id="4" xr3:uid="{FF5D3D34-BBDB-4113-8340-C737255ED1BD}" uniqueName="4" name="Column4" queryTableFieldId="4" dataDxfId="12"/>
+    <tableColumn id="5" xr3:uid="{F05FA152-C9D6-4773-B0A5-5B18B60C7102}" uniqueName="5" name="Column5" queryTableFieldId="5" dataDxfId="11"/>
   </tableColumns>
   <tableStyleInfo name="TableStyleMedium7" showFirstColumn="0" showLastColumn="0" showRowStripes="1" showColumnStripes="0"/>
 </table>
@@ -5370,13 +5370,13 @@
 <table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="2" xr:uid="{D4474760-F3B7-4070-AE77-2962D090A5AB}" name="Table002__Page_2" displayName="Table002__Page_2" ref="A19:G21" tableType="queryTable" totalsRowShown="0">
   <autoFilter ref="A19:G21" xr:uid="{D4474760-F3B7-4070-AE77-2962D090A5AB}"/>
   <tableColumns count="7">
-    <tableColumn id="1" xr3:uid="{8A3681DA-5FE9-4564-BCAB-75CCDF2C3A51}" uniqueName="1" name="Column1" queryTableFieldId="1" dataDxfId="136"/>
-    <tableColumn id="2" xr3:uid="{44D6563C-A88C-4FEE-9427-B5252DF8FA5D}" uniqueName="2" name="Column6" queryTableFieldId="2" dataDxfId="135"/>
-    <tableColumn id="3" xr3:uid="{2514D758-49E4-4E3E-A628-2B2D894F398E}" uniqueName="3" name="Column2" queryTableFieldId="3" dataDxfId="134"/>
-    <tableColumn id="4" xr3:uid="{062470EA-CB73-435C-8DF3-28DE262C8D69}" uniqueName="4" name="Column3" queryTableFieldId="4" dataDxfId="133"/>
-    <tableColumn id="5" xr3:uid="{CDE500EE-B268-43D9-A30D-9E6CC1608CD0}" uniqueName="5" name="Column4" queryTableFieldId="5" dataDxfId="132"/>
-    <tableColumn id="6" xr3:uid="{699F51E2-9A1B-4953-91BE-8D6434D76B20}" uniqueName="6" name="Column5" queryTableFieldId="6" dataDxfId="131"/>
-    <tableColumn id="7" xr3:uid="{C62D0670-E212-49FF-BA61-22C41F21B60E}" uniqueName="7" name="Column62" queryTableFieldId="7" dataDxfId="130"/>
+    <tableColumn id="1" xr3:uid="{8A3681DA-5FE9-4564-BCAB-75CCDF2C3A51}" uniqueName="1" name="Column1" queryTableFieldId="1" dataDxfId="135"/>
+    <tableColumn id="2" xr3:uid="{44D6563C-A88C-4FEE-9427-B5252DF8FA5D}" uniqueName="2" name="Column6" queryTableFieldId="2" dataDxfId="134"/>
+    <tableColumn id="3" xr3:uid="{2514D758-49E4-4E3E-A628-2B2D894F398E}" uniqueName="3" name="Column2" queryTableFieldId="3" dataDxfId="133"/>
+    <tableColumn id="4" xr3:uid="{062470EA-CB73-435C-8DF3-28DE262C8D69}" uniqueName="4" name="Column3" queryTableFieldId="4" dataDxfId="132"/>
+    <tableColumn id="5" xr3:uid="{CDE500EE-B268-43D9-A30D-9E6CC1608CD0}" uniqueName="5" name="Column4" queryTableFieldId="5" dataDxfId="131"/>
+    <tableColumn id="6" xr3:uid="{699F51E2-9A1B-4953-91BE-8D6434D76B20}" uniqueName="6" name="Column5" queryTableFieldId="6" dataDxfId="130"/>
+    <tableColumn id="7" xr3:uid="{C62D0670-E212-49FF-BA61-22C41F21B60E}" uniqueName="7" name="Column62" queryTableFieldId="7" dataDxfId="129"/>
   </tableColumns>
   <tableStyleInfo name="TableStyleMedium7" showFirstColumn="0" showLastColumn="0" showRowStripes="1" showColumnStripes="0"/>
 </table>
@@ -5386,14 +5386,14 @@
 <table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="3" xr:uid="{EE92A61D-8549-4453-B707-7BA76D39611E}" name="Table003__Page_3" displayName="Table003__Page_3" ref="A1:H16" tableType="queryTable" totalsRowShown="0">
   <autoFilter ref="A1:H16" xr:uid="{EE92A61D-8549-4453-B707-7BA76D39611E}"/>
   <tableColumns count="8">
-    <tableColumn id="1" xr3:uid="{5E78ED26-3040-4033-A95F-3AC09118D17C}" uniqueName="1" name="Column1" queryTableFieldId="1" dataDxfId="129"/>
-    <tableColumn id="2" xr3:uid="{52F60F93-88D4-4F60-A15A-4B2113E53BE2}" uniqueName="2" name="Column2" queryTableFieldId="2" dataDxfId="128"/>
-    <tableColumn id="3" xr3:uid="{2A66B2A9-165C-4995-937F-8E0D8B01B3D8}" uniqueName="3" name="Column3" queryTableFieldId="3" dataDxfId="127"/>
-    <tableColumn id="4" xr3:uid="{937ED0C3-8277-4EC6-BFD2-C6699696538D}" uniqueName="4" name="Column4" queryTableFieldId="4" dataDxfId="126"/>
-    <tableColumn id="5" xr3:uid="{37EAAABA-4FEF-4D28-B237-360AD0A7194A}" uniqueName="5" name="Column5" queryTableFieldId="5" dataDxfId="125"/>
-    <tableColumn id="6" xr3:uid="{6E7D50A0-6329-4797-9F9A-628D251C7CA5}" uniqueName="6" name="Column6" queryTableFieldId="6" dataDxfId="124"/>
-    <tableColumn id="7" xr3:uid="{F8F31C01-9522-488B-915F-110987168D09}" uniqueName="7" name="Column7" queryTableFieldId="7" dataDxfId="123"/>
-    <tableColumn id="8" xr3:uid="{FFD35FDD-AAE7-4F54-8AF3-197380BC0AEB}" uniqueName="8" name="Column8" queryTableFieldId="8" dataDxfId="122"/>
+    <tableColumn id="1" xr3:uid="{5E78ED26-3040-4033-A95F-3AC09118D17C}" uniqueName="1" name="Column1" queryTableFieldId="1" dataDxfId="128"/>
+    <tableColumn id="2" xr3:uid="{52F60F93-88D4-4F60-A15A-4B2113E53BE2}" uniqueName="2" name="Column2" queryTableFieldId="2" dataDxfId="127"/>
+    <tableColumn id="3" xr3:uid="{2A66B2A9-165C-4995-937F-8E0D8B01B3D8}" uniqueName="3" name="Column3" queryTableFieldId="3" dataDxfId="126"/>
+    <tableColumn id="4" xr3:uid="{937ED0C3-8277-4EC6-BFD2-C6699696538D}" uniqueName="4" name="Column4" queryTableFieldId="4" dataDxfId="125"/>
+    <tableColumn id="5" xr3:uid="{37EAAABA-4FEF-4D28-B237-360AD0A7194A}" uniqueName="5" name="Column5" queryTableFieldId="5" dataDxfId="124"/>
+    <tableColumn id="6" xr3:uid="{6E7D50A0-6329-4797-9F9A-628D251C7CA5}" uniqueName="6" name="Column6" queryTableFieldId="6" dataDxfId="123"/>
+    <tableColumn id="7" xr3:uid="{F8F31C01-9522-488B-915F-110987168D09}" uniqueName="7" name="Column7" queryTableFieldId="7" dataDxfId="122"/>
+    <tableColumn id="8" xr3:uid="{FFD35FDD-AAE7-4F54-8AF3-197380BC0AEB}" uniqueName="8" name="Column8" queryTableFieldId="8" dataDxfId="121"/>
   </tableColumns>
   <tableStyleInfo name="TableStyleMedium7" showFirstColumn="0" showLastColumn="0" showRowStripes="1" showColumnStripes="0"/>
 </table>
@@ -5403,14 +5403,14 @@
 <table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="4" xr:uid="{1C7E55B7-7D73-418F-9229-407F52A253A6}" name="Table004__Page_3" displayName="Table004__Page_3" ref="A18:H20" tableType="queryTable" totalsRowShown="0">
   <autoFilter ref="A18:H20" xr:uid="{1C7E55B7-7D73-418F-9229-407F52A253A6}"/>
   <tableColumns count="8">
-    <tableColumn id="1" xr3:uid="{A8A6FCCE-AE43-4EDA-82DC-831809E03401}" uniqueName="1" name="Column1" queryTableFieldId="1" dataDxfId="121"/>
-    <tableColumn id="2" xr3:uid="{0231594E-DA9E-47DE-A01C-22488210A4CF}" uniqueName="2" name="Column2" queryTableFieldId="2" dataDxfId="120"/>
-    <tableColumn id="3" xr3:uid="{7A06306A-69AF-482D-910F-86D0EF88F740}" uniqueName="3" name="Column3" queryTableFieldId="3" dataDxfId="119"/>
-    <tableColumn id="4" xr3:uid="{E96F3603-E9D2-4710-BDE5-6FE3E6A378D8}" uniqueName="4" name="Column4" queryTableFieldId="4" dataDxfId="118"/>
-    <tableColumn id="5" xr3:uid="{37151140-CC9F-4EBB-B58D-F87E1081314A}" uniqueName="5" name="Column5" queryTableFieldId="5" dataDxfId="117"/>
-    <tableColumn id="6" xr3:uid="{F0AAEEC2-014D-412A-B58D-24C71FEC9A66}" uniqueName="6" name="Column6" queryTableFieldId="6" dataDxfId="116"/>
-    <tableColumn id="7" xr3:uid="{A4B4F3F0-B14D-498F-B185-AA3E2BAE729A}" uniqueName="7" name="Column7" queryTableFieldId="7" dataDxfId="115"/>
-    <tableColumn id="8" xr3:uid="{0C517BB9-44A4-4BBA-AA88-B86BB679F208}" uniqueName="8" name="Column8" queryTableFieldId="8" dataDxfId="114"/>
+    <tableColumn id="1" xr3:uid="{A8A6FCCE-AE43-4EDA-82DC-831809E03401}" uniqueName="1" name="Column1" queryTableFieldId="1" dataDxfId="120"/>
+    <tableColumn id="2" xr3:uid="{0231594E-DA9E-47DE-A01C-22488210A4CF}" uniqueName="2" name="Column2" queryTableFieldId="2" dataDxfId="119"/>
+    <tableColumn id="3" xr3:uid="{7A06306A-69AF-482D-910F-86D0EF88F740}" uniqueName="3" name="Column3" queryTableFieldId="3" dataDxfId="118"/>
+    <tableColumn id="4" xr3:uid="{E96F3603-E9D2-4710-BDE5-6FE3E6A378D8}" uniqueName="4" name="Column4" queryTableFieldId="4" dataDxfId="117"/>
+    <tableColumn id="5" xr3:uid="{37151140-CC9F-4EBB-B58D-F87E1081314A}" uniqueName="5" name="Column5" queryTableFieldId="5" dataDxfId="116"/>
+    <tableColumn id="6" xr3:uid="{F0AAEEC2-014D-412A-B58D-24C71FEC9A66}" uniqueName="6" name="Column6" queryTableFieldId="6" dataDxfId="115"/>
+    <tableColumn id="7" xr3:uid="{A4B4F3F0-B14D-498F-B185-AA3E2BAE729A}" uniqueName="7" name="Column7" queryTableFieldId="7" dataDxfId="114"/>
+    <tableColumn id="8" xr3:uid="{0C517BB9-44A4-4BBA-AA88-B86BB679F208}" uniqueName="8" name="Column8" queryTableFieldId="8" dataDxfId="113"/>
   </tableColumns>
   <tableStyleInfo name="TableStyleMedium7" showFirstColumn="0" showLastColumn="0" showRowStripes="1" showColumnStripes="0"/>
 </table>
@@ -5420,12 +5420,12 @@
 <table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="5" xr:uid="{2EB30D60-3074-4922-8217-6B97953C0F87}" name="Table005__Page_4" displayName="Table005__Page_4" ref="A1:F16" tableType="queryTable" totalsRowShown="0">
   <autoFilter ref="A1:F16" xr:uid="{2EB30D60-3074-4922-8217-6B97953C0F87}"/>
   <tableColumns count="6">
-    <tableColumn id="1" xr3:uid="{AB42FEA9-5A85-4A69-B46D-444C53C4B4EF}" uniqueName="1" name="Column1" queryTableFieldId="1" dataDxfId="113"/>
-    <tableColumn id="2" xr3:uid="{0D7919B1-FB5E-4192-8675-3D57B39D9AB0}" uniqueName="2" name="Column2" queryTableFieldId="2" dataDxfId="112"/>
-    <tableColumn id="3" xr3:uid="{94F12F3D-88BF-4BEB-85E7-FF6313F6B88E}" uniqueName="3" name="Column3" queryTableFieldId="3" dataDxfId="111"/>
-    <tableColumn id="4" xr3:uid="{2B04EEA3-DC55-4C69-860F-9571D35E352D}" uniqueName="4" name="Column4" queryTableFieldId="4" dataDxfId="110"/>
-    <tableColumn id="5" xr3:uid="{461C5084-182B-40CC-B479-24798E48D0F4}" uniqueName="5" name="Column5" queryTableFieldId="5" dataDxfId="109"/>
-    <tableColumn id="6" xr3:uid="{258F7EB6-7345-43CA-BF8A-5E088D06FF8F}" uniqueName="6" name="Column6" queryTableFieldId="6" dataDxfId="108"/>
+    <tableColumn id="1" xr3:uid="{AB42FEA9-5A85-4A69-B46D-444C53C4B4EF}" uniqueName="1" name="Column1" queryTableFieldId="1" dataDxfId="112"/>
+    <tableColumn id="2" xr3:uid="{0D7919B1-FB5E-4192-8675-3D57B39D9AB0}" uniqueName="2" name="Column2" queryTableFieldId="2" dataDxfId="111"/>
+    <tableColumn id="3" xr3:uid="{94F12F3D-88BF-4BEB-85E7-FF6313F6B88E}" uniqueName="3" name="Column3" queryTableFieldId="3" dataDxfId="110"/>
+    <tableColumn id="4" xr3:uid="{2B04EEA3-DC55-4C69-860F-9571D35E352D}" uniqueName="4" name="Column4" queryTableFieldId="4" dataDxfId="109"/>
+    <tableColumn id="5" xr3:uid="{461C5084-182B-40CC-B479-24798E48D0F4}" uniqueName="5" name="Column5" queryTableFieldId="5" dataDxfId="108"/>
+    <tableColumn id="6" xr3:uid="{258F7EB6-7345-43CA-BF8A-5E088D06FF8F}" uniqueName="6" name="Column6" queryTableFieldId="6" dataDxfId="107"/>
   </tableColumns>
   <tableStyleInfo name="TableStyleMedium7" showFirstColumn="0" showLastColumn="0" showRowStripes="1" showColumnStripes="0"/>
 </table>
@@ -5435,12 +5435,12 @@
 <table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="6" xr:uid="{BA3E356C-A98F-4646-B7E8-7B0C3904E2A4}" name="Table006__Page_4" displayName="Table006__Page_4" ref="A18:F20" tableType="queryTable" totalsRowShown="0">
   <autoFilter ref="A18:F20" xr:uid="{BA3E356C-A98F-4646-B7E8-7B0C3904E2A4}"/>
   <tableColumns count="6">
-    <tableColumn id="1" xr3:uid="{55987721-40E8-4E11-9B6F-67EE503D78F4}" uniqueName="1" name="Column1" queryTableFieldId="1" dataDxfId="107"/>
-    <tableColumn id="2" xr3:uid="{15260D47-39CC-4501-9656-F8DBE6AD3AB1}" uniqueName="2" name="Column2" queryTableFieldId="2" dataDxfId="106"/>
-    <tableColumn id="3" xr3:uid="{06C8B30C-3DD3-49E6-8BE6-C8A9D39F2FC4}" uniqueName="3" name="Column3" queryTableFieldId="3" dataDxfId="105"/>
-    <tableColumn id="4" xr3:uid="{40A070F6-4BDB-49A7-9394-4D63F3A9E318}" uniqueName="4" name="Column4" queryTableFieldId="4" dataDxfId="104"/>
-    <tableColumn id="5" xr3:uid="{C5E0BAEF-796C-4C71-ACA7-889E63543C2D}" uniqueName="5" name="Column5" queryTableFieldId="5" dataDxfId="103"/>
-    <tableColumn id="6" xr3:uid="{1BA75280-A961-41F1-B113-5935891BA00A}" uniqueName="6" name="Column6" queryTableFieldId="6" dataDxfId="102"/>
+    <tableColumn id="1" xr3:uid="{55987721-40E8-4E11-9B6F-67EE503D78F4}" uniqueName="1" name="Column1" queryTableFieldId="1" dataDxfId="106"/>
+    <tableColumn id="2" xr3:uid="{15260D47-39CC-4501-9656-F8DBE6AD3AB1}" uniqueName="2" name="Column2" queryTableFieldId="2" dataDxfId="105"/>
+    <tableColumn id="3" xr3:uid="{06C8B30C-3DD3-49E6-8BE6-C8A9D39F2FC4}" uniqueName="3" name="Column3" queryTableFieldId="3" dataDxfId="104"/>
+    <tableColumn id="4" xr3:uid="{40A070F6-4BDB-49A7-9394-4D63F3A9E318}" uniqueName="4" name="Column4" queryTableFieldId="4" dataDxfId="103"/>
+    <tableColumn id="5" xr3:uid="{C5E0BAEF-796C-4C71-ACA7-889E63543C2D}" uniqueName="5" name="Column5" queryTableFieldId="5" dataDxfId="102"/>
+    <tableColumn id="6" xr3:uid="{1BA75280-A961-41F1-B113-5935891BA00A}" uniqueName="6" name="Column6" queryTableFieldId="6" dataDxfId="101"/>
   </tableColumns>
   <tableStyleInfo name="TableStyleMedium7" showFirstColumn="0" showLastColumn="0" showRowStripes="1" showColumnStripes="0"/>
 </table>
@@ -5450,18 +5450,18 @@
 <table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="7" xr:uid="{6040FF08-DFFC-4D6C-87C0-7C33D5281777}" name="Table007__Page_5" displayName="Table007__Page_5" ref="A1:L16" tableType="queryTable" totalsRowShown="0">
   <autoFilter ref="A1:L16" xr:uid="{6040FF08-DFFC-4D6C-87C0-7C33D5281777}"/>
   <tableColumns count="12">
-    <tableColumn id="1" xr3:uid="{9561388E-64AE-4A76-863E-A0B2091E2F9F}" uniqueName="1" name="Column1" queryTableFieldId="1" dataDxfId="101"/>
-    <tableColumn id="2" xr3:uid="{151810A9-7DD3-4FD0-91D6-6608DF85A8CF}" uniqueName="2" name="Column2" queryTableFieldId="2" dataDxfId="100"/>
-    <tableColumn id="3" xr3:uid="{94D629BF-F745-493D-8F74-FA7EEFDEAA84}" uniqueName="3" name="Column3" queryTableFieldId="3" dataDxfId="99"/>
-    <tableColumn id="4" xr3:uid="{AE87299A-170F-4661-BD08-B108394E2F7C}" uniqueName="4" name="Column4" queryTableFieldId="4" dataDxfId="98"/>
-    <tableColumn id="5" xr3:uid="{708CB468-5E3F-4D0C-B6BD-C2C44C7191EC}" uniqueName="5" name="Column5" queryTableFieldId="5" dataDxfId="97"/>
-    <tableColumn id="6" xr3:uid="{5D4BD3CB-C344-4155-B3C1-ECC49F86CED1}" uniqueName="6" name="Column6" queryTableFieldId="6" dataDxfId="96"/>
-    <tableColumn id="7" xr3:uid="{61DF1122-5C54-47A3-98F9-27CA1B50CA9D}" uniqueName="7" name="Column7" queryTableFieldId="7" dataDxfId="95"/>
-    <tableColumn id="8" xr3:uid="{130590EE-DDCB-43DB-A020-385B521DA018}" uniqueName="8" name="Column8" queryTableFieldId="8" dataDxfId="94"/>
-    <tableColumn id="9" xr3:uid="{06B903F7-5E22-476D-A116-655599D2C518}" uniqueName="9" name="Column9" queryTableFieldId="9" dataDxfId="93"/>
-    <tableColumn id="10" xr3:uid="{CED96D55-8B0D-492D-B0EC-F3E56EFB2649}" uniqueName="10" name="Column10" queryTableFieldId="10" dataDxfId="92"/>
-    <tableColumn id="11" xr3:uid="{346823E9-F305-4F11-941F-1C42A8AB0C99}" uniqueName="11" name="Column11" queryTableFieldId="11" dataDxfId="91"/>
-    <tableColumn id="12" xr3:uid="{7B421AA8-C9DB-4E35-A456-DF0F56050B79}" uniqueName="12" name="Column12" queryTableFieldId="12" dataDxfId="90"/>
+    <tableColumn id="1" xr3:uid="{9561388E-64AE-4A76-863E-A0B2091E2F9F}" uniqueName="1" name="Column1" queryTableFieldId="1" dataDxfId="100"/>
+    <tableColumn id="2" xr3:uid="{151810A9-7DD3-4FD0-91D6-6608DF85A8CF}" uniqueName="2" name="Column2" queryTableFieldId="2" dataDxfId="99"/>
+    <tableColumn id="3" xr3:uid="{94D629BF-F745-493D-8F74-FA7EEFDEAA84}" uniqueName="3" name="Column3" queryTableFieldId="3" dataDxfId="98"/>
+    <tableColumn id="4" xr3:uid="{AE87299A-170F-4661-BD08-B108394E2F7C}" uniqueName="4" name="Column4" queryTableFieldId="4" dataDxfId="97"/>
+    <tableColumn id="5" xr3:uid="{708CB468-5E3F-4D0C-B6BD-C2C44C7191EC}" uniqueName="5" name="Column5" queryTableFieldId="5" dataDxfId="96"/>
+    <tableColumn id="6" xr3:uid="{5D4BD3CB-C344-4155-B3C1-ECC49F86CED1}" uniqueName="6" name="Column6" queryTableFieldId="6" dataDxfId="95"/>
+    <tableColumn id="7" xr3:uid="{61DF1122-5C54-47A3-98F9-27CA1B50CA9D}" uniqueName="7" name="Column7" queryTableFieldId="7" dataDxfId="94"/>
+    <tableColumn id="8" xr3:uid="{130590EE-DDCB-43DB-A020-385B521DA018}" uniqueName="8" name="Column8" queryTableFieldId="8" dataDxfId="93"/>
+    <tableColumn id="9" xr3:uid="{06B903F7-5E22-476D-A116-655599D2C518}" uniqueName="9" name="Column9" queryTableFieldId="9" dataDxfId="92"/>
+    <tableColumn id="10" xr3:uid="{CED96D55-8B0D-492D-B0EC-F3E56EFB2649}" uniqueName="10" name="Column10" queryTableFieldId="10" dataDxfId="91"/>
+    <tableColumn id="11" xr3:uid="{346823E9-F305-4F11-941F-1C42A8AB0C99}" uniqueName="11" name="Column11" queryTableFieldId="11" dataDxfId="90"/>
+    <tableColumn id="12" xr3:uid="{7B421AA8-C9DB-4E35-A456-DF0F56050B79}" uniqueName="12" name="Column12" queryTableFieldId="12" dataDxfId="89"/>
   </tableColumns>
   <tableStyleInfo name="TableStyleMedium7" showFirstColumn="0" showLastColumn="0" showRowStripes="1" showColumnStripes="0"/>
 </table>
@@ -5471,18 +5471,18 @@
 <table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="8" xr:uid="{DBF54861-4823-4965-9BF8-BF4D83A85FD1}" name="Table008__Page_5" displayName="Table008__Page_5" ref="A18:L20" tableType="queryTable" totalsRowShown="0">
   <autoFilter ref="A18:L20" xr:uid="{DBF54861-4823-4965-9BF8-BF4D83A85FD1}"/>
   <tableColumns count="12">
-    <tableColumn id="1" xr3:uid="{01D3C90B-BA67-46B4-BD1D-5C53486CAE57}" uniqueName="1" name="Column1" queryTableFieldId="1" dataDxfId="89"/>
-    <tableColumn id="2" xr3:uid="{166854EB-0B50-4420-BB3F-7A5A2C9FB7F7}" uniqueName="2" name="Column2" queryTableFieldId="2" dataDxfId="88"/>
-    <tableColumn id="3" xr3:uid="{638857E5-1EB4-4FBE-9FFE-2951F2F4ABD0}" uniqueName="3" name="Column3" queryTableFieldId="3" dataDxfId="87"/>
-    <tableColumn id="4" xr3:uid="{F4EFE2EF-AC84-40F8-BE68-0B6B520F8EA8}" uniqueName="4" name="Column4" queryTableFieldId="4" dataDxfId="86"/>
-    <tableColumn id="5" xr3:uid="{38D026D2-A47E-46EA-BA10-AF890A55BF2B}" uniqueName="5" name="Column5" queryTableFieldId="5" dataDxfId="85"/>
-    <tableColumn id="6" xr3:uid="{025C6DA2-37A6-491F-904E-DDE12948D35B}" uniqueName="6" name="Column6" queryTableFieldId="6" dataDxfId="84"/>
-    <tableColumn id="7" xr3:uid="{AC28B573-67B7-4468-A6A2-F648D17079B6}" uniqueName="7" name="Column7" queryTableFieldId="7" dataDxfId="83"/>
-    <tableColumn id="8" xr3:uid="{F6F06554-210B-472F-95F2-8E89D931E4C1}" uniqueName="8" name="Column8" queryTableFieldId="8" dataDxfId="82"/>
-    <tableColumn id="9" xr3:uid="{F0A8F323-36C1-4290-980B-8F6F5DC6A41E}" uniqueName="9" name="Column9" queryTableFieldId="9" dataDxfId="81"/>
-    <tableColumn id="10" xr3:uid="{25D60007-5007-4174-85F5-572E3C29FE33}" uniqueName="10" name="Column10" queryTableFieldId="10" dataDxfId="80"/>
-    <tableColumn id="11" xr3:uid="{2071EB9B-B14E-4EF0-9B86-0D5FDA96828D}" uniqueName="11" name="Column11" queryTableFieldId="11" dataDxfId="79"/>
-    <tableColumn id="12" xr3:uid="{1660C180-EE6B-48E8-9880-55F02CC623C4}" uniqueName="12" name="Column12" queryTableFieldId="12" dataDxfId="78"/>
+    <tableColumn id="1" xr3:uid="{01D3C90B-BA67-46B4-BD1D-5C53486CAE57}" uniqueName="1" name="Column1" queryTableFieldId="1" dataDxfId="88"/>
+    <tableColumn id="2" xr3:uid="{166854EB-0B50-4420-BB3F-7A5A2C9FB7F7}" uniqueName="2" name="Column2" queryTableFieldId="2" dataDxfId="87"/>
+    <tableColumn id="3" xr3:uid="{638857E5-1EB4-4FBE-9FFE-2951F2F4ABD0}" uniqueName="3" name="Column3" queryTableFieldId="3" dataDxfId="86"/>
+    <tableColumn id="4" xr3:uid="{F4EFE2EF-AC84-40F8-BE68-0B6B520F8EA8}" uniqueName="4" name="Column4" queryTableFieldId="4" dataDxfId="85"/>
+    <tableColumn id="5" xr3:uid="{38D026D2-A47E-46EA-BA10-AF890A55BF2B}" uniqueName="5" name="Column5" queryTableFieldId="5" dataDxfId="84"/>
+    <tableColumn id="6" xr3:uid="{025C6DA2-37A6-491F-904E-DDE12948D35B}" uniqueName="6" name="Column6" queryTableFieldId="6" dataDxfId="83"/>
+    <tableColumn id="7" xr3:uid="{AC28B573-67B7-4468-A6A2-F648D17079B6}" uniqueName="7" name="Column7" queryTableFieldId="7" dataDxfId="82"/>
+    <tableColumn id="8" xr3:uid="{F6F06554-210B-472F-95F2-8E89D931E4C1}" uniqueName="8" name="Column8" queryTableFieldId="8" dataDxfId="81"/>
+    <tableColumn id="9" xr3:uid="{F0A8F323-36C1-4290-980B-8F6F5DC6A41E}" uniqueName="9" name="Column9" queryTableFieldId="9" dataDxfId="80"/>
+    <tableColumn id="10" xr3:uid="{25D60007-5007-4174-85F5-572E3C29FE33}" uniqueName="10" name="Column10" queryTableFieldId="10" dataDxfId="79"/>
+    <tableColumn id="11" xr3:uid="{2071EB9B-B14E-4EF0-9B86-0D5FDA96828D}" uniqueName="11" name="Column11" queryTableFieldId="11" dataDxfId="78"/>
+    <tableColumn id="12" xr3:uid="{1660C180-EE6B-48E8-9880-55F02CC623C4}" uniqueName="12" name="Column12" queryTableFieldId="12" dataDxfId="77"/>
   </tableColumns>
   <tableStyleInfo name="TableStyleMedium7" showFirstColumn="0" showLastColumn="0" showRowStripes="1" showColumnStripes="0"/>
 </table>
@@ -8348,25 +8348,25 @@
   </sheetData>
   <phoneticPr fontId="4" type="noConversion"/>
   <conditionalFormatting sqref="A1:A1048576">
-    <cfRule type="duplicateValues" dxfId="11" priority="4"/>
+    <cfRule type="duplicateValues" dxfId="10" priority="4"/>
   </conditionalFormatting>
   <conditionalFormatting sqref="A33:A41 A43:A46 A2:A31">
-    <cfRule type="duplicateValues" dxfId="10" priority="16"/>
+    <cfRule type="duplicateValues" dxfId="9" priority="16"/>
   </conditionalFormatting>
   <conditionalFormatting sqref="A33:A46 A2:A31">
-    <cfRule type="duplicateValues" dxfId="9" priority="20"/>
+    <cfRule type="duplicateValues" dxfId="8" priority="20"/>
   </conditionalFormatting>
   <conditionalFormatting sqref="H43:H46">
-    <cfRule type="duplicateValues" dxfId="8" priority="9"/>
-    <cfRule type="duplicateValues" dxfId="7" priority="10"/>
+    <cfRule type="duplicateValues" dxfId="7" priority="9"/>
+    <cfRule type="duplicateValues" dxfId="6" priority="10"/>
   </conditionalFormatting>
   <conditionalFormatting sqref="H51:H54">
-    <cfRule type="duplicateValues" dxfId="6" priority="5"/>
-    <cfRule type="duplicateValues" dxfId="5" priority="6"/>
+    <cfRule type="duplicateValues" dxfId="5" priority="5"/>
+    <cfRule type="duplicateValues" dxfId="4" priority="6"/>
   </conditionalFormatting>
   <conditionalFormatting sqref="H74:H75">
-    <cfRule type="duplicateValues" dxfId="4" priority="1"/>
-    <cfRule type="duplicateValues" dxfId="3" priority="2"/>
+    <cfRule type="duplicateValues" dxfId="3" priority="1"/>
+    <cfRule type="duplicateValues" dxfId="2" priority="2"/>
   </conditionalFormatting>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <pageSetup paperSize="9" orientation="portrait" horizontalDpi="0" verticalDpi="0" r:id="rId1"/>
@@ -10364,10 +10364,10 @@
     </row>
   </sheetData>
   <conditionalFormatting sqref="A2:A33">
-    <cfRule type="duplicateValues" dxfId="2" priority="1"/>
+    <cfRule type="duplicateValues" dxfId="1" priority="1"/>
   </conditionalFormatting>
   <conditionalFormatting sqref="A2:A34">
-    <cfRule type="duplicateValues" dxfId="1" priority="2"/>
+    <cfRule type="duplicateValues" dxfId="0" priority="2"/>
   </conditionalFormatting>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>

</xml_diff>

<commit_message>
UPDATE: Added new Merk for Cloud 2026
</commit_message>
<xml_diff>
--- a/gp-app-1.0/Pricelist Car.xlsx
+++ b/gp-app-1.0/Pricelist Car.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\Work\gp-app\gp-app-1.0\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{0A315F8A-08D3-4355-B3C9-5836BD000EAA}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{E0F13263-28F1-410A-90BC-F927B058BAEE}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-110" yWindow="-110" windowWidth="19420" windowHeight="11020" tabRatio="861" xr2:uid="{C4C7316A-D95F-426A-ADF9-AD32FA680374}"/>
   </bookViews>
@@ -490,7 +490,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1450" uniqueCount="651">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1456" uniqueCount="653">
   <si>
     <t>Column1</t>
   </si>
@@ -2523,6 +2523,12 @@
   </si>
   <si>
     <t>New Cloud Pro</t>
+  </si>
+  <si>
+    <t>NEW CLOUD EV LITE 360 KM</t>
+  </si>
+  <si>
+    <t>NEW CLOUD EV PRO 360 KM</t>
   </si>
 </sst>
 </file>
@@ -2720,7 +2726,7 @@
     <xf numFmtId="43" fontId="2" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="25">
+  <cellXfs count="33">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="2" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
     <xf numFmtId="3" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
@@ -2762,6 +2768,14 @@
     <xf numFmtId="0" fontId="2" fillId="2" borderId="9" xfId="3" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="3" xfId="0" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="43" fontId="0" fillId="0" borderId="1" xfId="2" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="43" fontId="0" fillId="0" borderId="4" xfId="0" applyNumberFormat="1" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="8" xfId="0" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="9" xfId="0" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="43" fontId="0" fillId="0" borderId="9" xfId="2" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="43" fontId="0" fillId="0" borderId="10" xfId="0" applyNumberFormat="1" applyFill="1" applyBorder="1"/>
   </cellXfs>
   <cellStyles count="4">
     <cellStyle name="Comma" xfId="2" builtinId="3"/>
@@ -5157,8 +5171,8 @@
 </file>
 
 <file path=xl/tables/table1.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="20" xr:uid="{DF067A72-54A6-48F4-972D-2DE4603D61A4}" name="Table20" displayName="Table20" ref="A1:I79" totalsRowShown="0" headerRowDxfId="155" headerRowBorderDxfId="154" tableBorderDxfId="153" totalsRowBorderDxfId="152">
-  <autoFilter ref="A1:I79" xr:uid="{DF067A72-54A6-48F4-972D-2DE4603D61A4}"/>
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="20" xr:uid="{DF067A72-54A6-48F4-972D-2DE4603D61A4}" name="Table20" displayName="Table20" ref="A1:I81" totalsRowShown="0" headerRowDxfId="155" headerRowBorderDxfId="154" tableBorderDxfId="153" totalsRowBorderDxfId="152">
+  <autoFilter ref="A1:I81" xr:uid="{DF067A72-54A6-48F4-972D-2DE4603D61A4}"/>
   <tableColumns count="9">
     <tableColumn id="1" xr3:uid="{0E6335F2-6B6A-436C-92FA-B48E61551308}" name="Merek/Type" dataDxfId="151"/>
     <tableColumn id="2" xr3:uid="{5A4965DA-398A-4134-90BD-9CE4D8355880}" name="Tipe" dataDxfId="150"/>
@@ -5785,7 +5799,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{3B05C9E0-A64E-40AC-B9F4-C919ED5906CC}">
-  <dimension ref="A1:I79"/>
+  <dimension ref="A1:I81"/>
   <sheetFormatPr defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
   <cols>
     <col min="1" max="1" width="51.453125" bestFit="1" customWidth="1"/>
@@ -8342,6 +8356,70 @@
         <v>571</v>
       </c>
       <c r="I79" s="19">
+        <v>25000000</v>
+      </c>
+    </row>
+    <row r="80" spans="1:9" x14ac:dyDescent="0.35">
+      <c r="A80" s="25" t="s">
+        <v>651</v>
+      </c>
+      <c r="B80" s="26" t="s">
+        <v>649</v>
+      </c>
+      <c r="C80" s="9">
+        <v>299000000</v>
+      </c>
+      <c r="D80" s="27">
+        <f t="shared" ref="D80:D81" si="24">I80/1.12</f>
+        <v>17857142.857142854</v>
+      </c>
+      <c r="E80" s="9">
+        <f t="shared" ref="E80:E81" si="25">D80*90%</f>
+        <v>16071428.571428569</v>
+      </c>
+      <c r="F80" s="9">
+        <f t="shared" ref="F80:F81" si="26">D80*70%</f>
+        <v>12499999.999999998</v>
+      </c>
+      <c r="G80" s="20">
+        <v>274</v>
+      </c>
+      <c r="H80" s="4" t="s">
+        <v>581</v>
+      </c>
+      <c r="I80" s="28">
+        <v>20000000</v>
+      </c>
+    </row>
+    <row r="81" spans="1:9" x14ac:dyDescent="0.35">
+      <c r="A81" s="29" t="s">
+        <v>652</v>
+      </c>
+      <c r="B81" s="30" t="s">
+        <v>650</v>
+      </c>
+      <c r="C81" s="18">
+        <v>339000000</v>
+      </c>
+      <c r="D81" s="31">
+        <f t="shared" si="24"/>
+        <v>22321428.571428571</v>
+      </c>
+      <c r="E81" s="18">
+        <f t="shared" si="25"/>
+        <v>20089285.714285713</v>
+      </c>
+      <c r="F81" s="18">
+        <f t="shared" si="26"/>
+        <v>15624999.999999998</v>
+      </c>
+      <c r="G81" s="21">
+        <v>275</v>
+      </c>
+      <c r="H81" s="17" t="s">
+        <v>571</v>
+      </c>
+      <c r="I81" s="32">
         <v>25000000</v>
       </c>
     </row>

</xml_diff>